<commit_message>
docs(test): refine test cases and record authentication test results
</commit_message>
<xml_diff>
--- a/test/test-cases/CPFriendFinder_TestCases.xlsx
+++ b/test/test-cases/CPFriendFinder_TestCases.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="1" r:id="R94ba4b279b654916"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Scenario Summary" sheetId="2" r:id="R89a5218bc8d94c95"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defect Summary" sheetId="3" r:id="Re969084df431409e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS001" sheetId="4" r:id="Rc78663273fd14d01"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS002" sheetId="5" r:id="R3d681e48ea1b45c1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Case Design &amp; Test Results" sheetId="6" r:id="R833834a9303b4670"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements Traceability" sheetId="7" r:id="R7340ae8b17d7463e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Summary Report" sheetId="8" r:id="Rfce39fe8ae3f41b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution Log" sheetId="9" r:id="R6a8b3ea9962b4e8d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="1" r:id="Ra95ad2d227914695"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Scenario Summary" sheetId="2" r:id="R412769676df149e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defect Summary" sheetId="3" r:id="R8d2856b698fa4ea4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS001" sheetId="4" r:id="R87427b80d2fa4c62"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS002" sheetId="5" r:id="Ra3576b2d5b314952"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Case Design &amp; Test Results" sheetId="6" r:id="R9ad112dcc8f64446"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements Traceability" sheetId="7" r:id="R8ca37dfc005d4356"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Summary Report" sheetId="8" r:id="Rfc2af004083c499b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution Log" sheetId="9" r:id="Rbe423bd2a3b14c4f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -21,7 +21,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="8">
+  <x:fonts count="21">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -68,8 +68,79 @@
       <x:color rgb="FF303030"/>
       <x:name val="Aptos"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF253848"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF253848"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="15"/>
+      <x:color rgb="FF292929"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="15"/>
+      <x:color rgb="FF667788"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="15"/>
+      <x:color rgb="FF52616D"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF52616D"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF253848"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF253848"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF253848"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF52616D"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="15"/>
+      <x:color rgb="FF52616D"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF253848"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="10">
+  <x:fills count="14">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -116,6 +187,26 @@
         <x:fgColor rgb="FFFFFDF4"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE4EBEE"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEEF3F5"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF1F5F7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="2">
     <x:border/>
@@ -124,7 +215,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="43">
+  <x:cellXfs count="89">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -213,6 +304,136 @@
     <x:xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="20" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -508,52 +729,52 @@
         <x:v>30 กันยายน 2569</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="29" customHeight="1">
+    <x:row r="8" ht="35" customHeight="1">
       <x:c r="A8" s="40" t="str">
-        <x:v>โค้ดที่ใช้วางแผนทดสอบ</x:v>
+        <x:v>ส่วนที่ทดสอบ</x:v>
       </x:c>
       <x:c r="B8" s="20" t="str">
-        <x:v>branch backend ของปิยพนธ์ (ก่อนรวมเข้า develop)</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="29" customHeight="1">
+        <x:v>AuthService: สมัครสมาชิกและเข้าสู่ระบบ</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="35" customHeight="1">
       <x:c r="A9" s="40" t="str">
-        <x:v>ขอบเขตเอกสารรอบนี้</x:v>
+        <x:v>รายการที่ออกแบบ</x:v>
       </x:c>
       <x:c r="B9" s="20" t="str">
-        <x:v>ทดสอบ AuthService: สมัครสมาชิก 12 กรณี และเข้าสู่ระบบ 11 กรณี</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="29" customHeight="1">
+        <x:v>Register 12 กรณี และ Login 11 กรณี</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="35" customHeight="1">
       <x:c r="A10" s="40" t="str">
-        <x:v>ผลเดิมที่รันแล้ว</x:v>
+        <x:v>ผลทดสอบเริ่มต้น</x:v>
       </x:c>
       <x:c r="B10" s="20" t="str">
-        <x:v>contextLoads ผ่าน 1 กรณี เมื่อ 30 ก.ย. 2569 (ไม่ใช่ผลของ Register/Login)</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="29" customHeight="1">
+        <x:v>FriendApplicationTests.contextLoads: ผ่าน 1/1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="35" customHeight="1">
       <x:c r="A11" s="40" t="str">
-        <x:v>สถานะของกรณีทดสอบใหม่</x:v>
+        <x:v>ผลทดสอบล่าสุด</x:v>
       </x:c>
       <x:c r="B11" s="20" t="str">
-        <x:v>ยังไม่ได้รันทั้ง 23 กรณี; บันทึกผลหลังรันจริง</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="29" customHeight="1">
+        <x:v>Register ผ่าน 12/12, Login ผ่าน 11/11; รวมผล Maven ผ่าน 25/25</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="35" customHeight="1">
       <x:c r="A12" s="40" t="str">
-        <x:v>วิธีบันทึกผล</x:v>
+        <x:v>วันที่และคำสั่ง</x:v>
       </x:c>
       <x:c r="B12" s="20" t="str">
-        <x:v>กรอก Actual Result และเปลี่ยน Status เมื่อมีผลรัน พร้อมวันเวลาและหลักฐาน</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="29" customHeight="1">
+        <x:v>30 ก.ย. 2569 เวลา 14:14 น. | ./mvnw -Djava.version=21 clean test</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="35" customHeight="1">
       <x:c r="A13" s="40" t="str">
-        <x:v>งานที่จะเพิ่มภายหลัง</x:v>
+        <x:v>ขอบเขตผลการทดสอบ</x:v>
       </x:c>
       <x:c r="B13" s="20" t="str">
-        <x:v>ทดสอบ Controller / API / Integration หลังทีมยืนยัน endpoint และรวมโค้ด</x:v>
+        <x:v>ผลที่บันทึกครอบคลุม Spring context และ AuthService; ยังไม่มีผลทดสอบ API, ฐานข้อมูลจริง หรือ UAT</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="27" customHeight="1">
@@ -614,35 +835,27 @@
     </x:row>
     <x:row r="25" ht="32" customHeight="1">
       <x:c r="A25" s="39" t="str">
-        <x:v>เรื่องที่ต้องตรวจต่อ</x:v>
+        <x:v>ข้อมูลเพิ่มเติม</x:v>
       </x:c>
       <x:c r="B25" s="39" t="str">
-        <x:v>รายละเอียด</x:v>
+        <x:v>ผลจากการรันทดสอบจัดเก็บใน test/reports/ และ target/surefire-reports/</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="32" customHeight="1">
       <x:c r="A26" s="18" t="str">
-        <x:v>เวอร์ชัน Java</x:v>
+        <x:v>ข้อมูลอ้างอิง</x:v>
       </x:c>
       <x:c r="B26" s="18" t="str">
-        <x:v>Backend ตั้ง Java 23 แต่เครื่องทดสอบใช้ Java 21 (รันด้วย -Djava.version=21 ผ่านแล้ว)</x:v>
+        <x:v>รหัส REQ และ UC ภายใน Excel เป็นรหัสสำหรับติดตาม Test Case ในเอกสารนี้</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="32" customHeight="1">
-      <x:c r="A27" s="18" t="str">
-        <x:v>การตรวจสอบข้อมูล</x:v>
-      </x:c>
-      <x:c r="B27" s="18" t="str">
-        <x:v>ปัจจุบัน Service ตรวจข้อมูลเอง; ควรตรวจเรื่อง @Valid กับเพื่อน Backend ก่อนรวมงาน</x:v>
-      </x:c>
+      <x:c r="A27" s="18"/>
+      <x:c r="B27" s="18"/>
     </x:row>
     <x:row r="28" ht="32" customHeight="1">
-      <x:c r="A28" s="18" t="str">
-        <x:v>อ้างอิงซอร์ส</x:v>
-      </x:c>
-      <x:c r="B28" s="18" t="str">
-        <x:v>branch: piyapon_673380050-9_section1_(backend) ใน repo leeLnwCode/CPFriendFinder</x:v>
-      </x:c>
+      <x:c r="A28" s="18"/>
+      <x:c r="B28" s="18"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -740,7 +953,7 @@
       </x:c>
       <x:c r="E5" s="20" t="n">
         <x:f>COUNTIFS('Test Case Design &amp; Test Results'!$B$5:$B$250,B5,'Test Case Design &amp; Test Results'!$J$5:$J$250,"Pass")</x:f>
-        <x:v>0</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="F5" s="20" t="n">
         <x:f>COUNTIFS('Test Case Design &amp; Test Results'!$B$5:$B$250,B5,'Test Case Design &amp; Test Results'!$J$5:$J$250,"Fail")</x:f>
@@ -748,7 +961,7 @@
       </x:c>
       <x:c r="G5" s="20" t="n">
         <x:f>COUNTIFS('Test Case Design &amp; Test Results'!$B$5:$B$250,B5,'Test Case Design &amp; Test Results'!$J$5:$J$250,"No run")</x:f>
-        <x:v>12</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H5" s="20" t="n">
         <x:f>COUNTIFS('Test Case Design &amp; Test Results'!$B$5:$B$250,B5,'Test Case Design &amp; Test Results'!$J$5:$J$250,"Block")</x:f>
@@ -774,7 +987,7 @@
       </x:c>
       <x:c r="E6" s="20" t="n">
         <x:f>COUNTIFS('Test Case Design &amp; Test Results'!$B$5:$B$250,B6,'Test Case Design &amp; Test Results'!$J$5:$J$250,"Pass")</x:f>
-        <x:v>0</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="F6" s="20" t="n">
         <x:f>COUNTIFS('Test Case Design &amp; Test Results'!$B$5:$B$250,B6,'Test Case Design &amp; Test Results'!$J$5:$J$250,"Fail")</x:f>
@@ -782,7 +995,7 @@
       </x:c>
       <x:c r="G6" s="20" t="n">
         <x:f>COUNTIFS('Test Case Design &amp; Test Results'!$B$5:$B$250,B6,'Test Case Design &amp; Test Results'!$J$5:$J$250,"No run")</x:f>
-        <x:v>11</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H6" s="20" t="n">
         <x:f>COUNTIFS('Test Case Design &amp; Test Results'!$B$5:$B$250,B6,'Test Case Design &amp; Test Results'!$J$5:$J$250,"Block")</x:f>
@@ -898,11 +1111,9 @@
     </x:row>
     <x:row r="6" ht="42" customHeight="1">
       <x:c r="A6" s="23" t="str">
-        <x:v>ยังไม่พบข้อบกพร่องที่ยืนยันแล้ว</x:v>
-      </x:c>
-      <x:c r="B6" s="23" t="str">
-        <x:v>ประเด็นที่ต้องคุยกับทีมบันทึกไว้ใน test/reports/review-notes.md</x:v>
-      </x:c>
+        <x:v>ยังไม่มีข้อบกพร่องที่ยืนยันจากชุดทดสอบนี้</x:v>
+      </x:c>
+      <x:c r="B6" s="23"/>
       <x:c r="C6" s="23"/>
       <x:c r="D6" s="23"/>
       <x:c r="E6" s="23"/>
@@ -1015,7 +1226,7 @@
         <x:v>ผลการทดสอบ</x:v>
       </x:c>
       <x:c r="B9" t="str">
-        <x:v>ยังไม่รัน (กรอกผลเมื่อทดสอบจริง)</x:v>
+        <x:v>รันแล้ว 12 รายการ ผ่าน 12 ไม่พบ Fail/Error (30 ก.ย. 2569)</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="34" customHeight="1">
@@ -1225,7 +1436,7 @@
         <x:v>ผลการทดสอบ</x:v>
       </x:c>
       <x:c r="B9" t="str">
-        <x:v>ยังไม่รัน (กรอกผลเมื่อทดสอบจริง)</x:v>
+        <x:v>รันแล้ว 11 รายการ ผ่าน 11 ไม่พบ Fail/Error (30 ก.ย. 2569)</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="34" customHeight="1">
@@ -1470,9 +1681,11 @@
       <x:c r="H5" s="20" t="str">
         <x:v>สมัครสำเร็จ ได้ข้อมูลผู้ใช้กลับมา และบันทึกผู้ใช้ 1 ครั้ง</x:v>
       </x:c>
-      <x:c r="I5" s="42" t="str"/>
+      <x:c r="I5" s="42" t="str">
+        <x:v>ผ่านตามผลที่คาดหวัง โดย JUnit ยืนยันผลของกรณีนี้</x:v>
+      </x:c>
       <x:c r="J5" s="42" t="str">
-        <x:v>No run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K5" s="20" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
@@ -1480,7 +1693,9 @@
       <x:c r="L5" s="20" t="str">
         <x:v>AuthServiceRegisterTest.register_validData_savesUser</x:v>
       </x:c>
-      <x:c r="M5" s="20" t="str"/>
+      <x:c r="M5" s="20" t="str">
+        <x:v>รัน 30 ก.ย. 2569 (ชุดรวม 14:14 น.); ดู Surefire report</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="41" customHeight="1">
       <x:c r="A6" s="20" t="str">
@@ -1507,9 +1722,11 @@
       <x:c r="H6" s="20" t="str">
         <x:v>แจ้ง 'Registration request is required'</x:v>
       </x:c>
-      <x:c r="I6" s="42" t="str"/>
+      <x:c r="I6" s="42" t="str">
+        <x:v>ผ่านตามผลที่คาดหวัง โดย JUnit ยืนยันผลของกรณีนี้</x:v>
+      </x:c>
       <x:c r="J6" s="42" t="str">
-        <x:v>No run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K6" s="20" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
@@ -1517,7 +1734,9 @@
       <x:c r="L6" s="20" t="str">
         <x:v>AuthServiceRegisterTest.register_nullRequest_throwsRequiredRequest</x:v>
       </x:c>
-      <x:c r="M6" s="20" t="str"/>
+      <x:c r="M6" s="20" t="str">
+        <x:v>รัน 30 ก.ย. 2569 (ชุดรวม 14:14 น.); ดู Surefire report</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" ht="41" customHeight="1">
       <x:c r="A7" s="20" t="str">
@@ -1544,9 +1763,11 @@
       <x:c r="H7" s="20" t="str">
         <x:v>แจ้ง 'Email is required'</x:v>
       </x:c>
-      <x:c r="I7" s="42" t="str"/>
+      <x:c r="I7" s="42" t="str">
+        <x:v>ผ่านตามผลที่คาดหวัง โดย JUnit ยืนยันผลของกรณีนี้</x:v>
+      </x:c>
       <x:c r="J7" s="42" t="str">
-        <x:v>No run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K7" s="20" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
@@ -1554,7 +1775,9 @@
       <x:c r="L7" s="20" t="str">
         <x:v>AuthServiceRegisterTest.register_nullEmail_throwsRequiredEmail</x:v>
       </x:c>
-      <x:c r="M7" s="20" t="str"/>
+      <x:c r="M7" s="20" t="str">
+        <x:v>รัน 30 ก.ย. 2569 (ชุดรวม 14:14 น.); ดู Surefire report</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" ht="41" customHeight="1">
       <x:c r="A8" s="20" t="str">
@@ -1581,9 +1804,11 @@
       <x:c r="H8" s="20" t="str">
         <x:v>แจ้ง 'Email is required'</x:v>
       </x:c>
-      <x:c r="I8" s="42" t="str"/>
+      <x:c r="I8" s="42" t="str">
+        <x:v>ผ่านตามผลที่คาดหวัง โดย JUnit ยืนยันผลของกรณีนี้</x:v>
+      </x:c>
       <x:c r="J8" s="42" t="str">
-        <x:v>No run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K8" s="20" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
@@ -1591,7 +1816,9 @@
       <x:c r="L8" s="20" t="str">
         <x:v>AuthServiceRegisterTest.register_blankEmail_throwsRequiredEmail</x:v>
       </x:c>
-      <x:c r="M8" s="20" t="str"/>
+      <x:c r="M8" s="20" t="str">
+        <x:v>รัน 30 ก.ย. 2569 (ชุดรวม 14:14 น.); ดู Surefire report</x:v>
+      </x:c>
     </x:row>
     <x:row r="9" ht="41" customHeight="1">
       <x:c r="A9" s="20" t="str">
@@ -1618,9 +1845,11 @@
       <x:c r="H9" s="20" t="str">
         <x:v>แจ้ง 'Password is required'</x:v>
       </x:c>
-      <x:c r="I9" s="42" t="str"/>
+      <x:c r="I9" s="42" t="str">
+        <x:v>ผ่านตามผลที่คาดหวัง โดย JUnit ยืนยันผลของกรณีนี้</x:v>
+      </x:c>
       <x:c r="J9" s="42" t="str">
-        <x:v>No run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K9" s="20" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
@@ -1628,7 +1857,9 @@
       <x:c r="L9" s="20" t="str">
         <x:v>AuthServiceRegisterTest.register_nullPassword_throwsRequiredPassword</x:v>
       </x:c>
-      <x:c r="M9" s="20" t="str"/>
+      <x:c r="M9" s="20" t="str">
+        <x:v>รัน 30 ก.ย. 2569 (ชุดรวม 14:14 น.); ดู Surefire report</x:v>
+      </x:c>
     </x:row>
     <x:row r="10" ht="41" customHeight="1">
       <x:c r="A10" s="20" t="str">
@@ -1655,9 +1886,11 @@
       <x:c r="H10" s="20" t="str">
         <x:v>แจ้ง 'Password is required'</x:v>
       </x:c>
-      <x:c r="I10" s="42" t="str"/>
+      <x:c r="I10" s="42" t="str">
+        <x:v>ผ่านตามผลที่คาดหวัง โดย JUnit ยืนยันผลของกรณีนี้</x:v>
+      </x:c>
       <x:c r="J10" s="42" t="str">
-        <x:v>No run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K10" s="20" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
@@ -1665,7 +1898,9 @@
       <x:c r="L10" s="20" t="str">
         <x:v>AuthServiceRegisterTest.register_blankPassword_throwsRequiredPassword</x:v>
       </x:c>
-      <x:c r="M10" s="20" t="str"/>
+      <x:c r="M10" s="20" t="str">
+        <x:v>รัน 30 ก.ย. 2569 (ชุดรวม 14:14 น.); ดู Surefire report</x:v>
+      </x:c>
     </x:row>
     <x:row r="11" ht="41" customHeight="1">
       <x:c r="A11" s="20" t="str">
@@ -1692,9 +1927,11 @@
       <x:c r="H11" s="20" t="str">
         <x:v>แจ้ง 'Password must be at least 8 characters'</x:v>
       </x:c>
-      <x:c r="I11" s="42" t="str"/>
+      <x:c r="I11" s="42" t="str">
+        <x:v>ผ่านตามผลที่คาดหวัง โดย JUnit ยืนยันผลของกรณีนี้</x:v>
+      </x:c>
       <x:c r="J11" s="42" t="str">
-        <x:v>No run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K11" s="20" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
@@ -1702,7 +1939,9 @@
       <x:c r="L11" s="20" t="str">
         <x:v>AuthServiceRegisterTest.register_sevenCharacterPassword_rejected</x:v>
       </x:c>
-      <x:c r="M11" s="20" t="str"/>
+      <x:c r="M11" s="20" t="str">
+        <x:v>รัน 30 ก.ย. 2569 (ชุดรวม 14:14 น.); ดู Surefire report</x:v>
+      </x:c>
     </x:row>
     <x:row r="12" ht="41" customHeight="1">
       <x:c r="A12" s="20" t="str">
@@ -1729,9 +1968,11 @@
       <x:c r="H12" s="20" t="str">
         <x:v>ยอมรับรหัสผ่านและบันทึกผู้ใช้ได้</x:v>
       </x:c>
-      <x:c r="I12" s="42" t="str"/>
+      <x:c r="I12" s="42" t="str">
+        <x:v>ผ่านตามผลที่คาดหวัง โดย JUnit ยืนยันผลของกรณีนี้</x:v>
+      </x:c>
       <x:c r="J12" s="42" t="str">
-        <x:v>No run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K12" s="20" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
@@ -1739,7 +1980,9 @@
       <x:c r="L12" s="20" t="str">
         <x:v>AuthServiceRegisterTest.register_eightCharacterPassword_accepted</x:v>
       </x:c>
-      <x:c r="M12" s="20" t="str"/>
+      <x:c r="M12" s="20" t="str">
+        <x:v>รัน 30 ก.ย. 2569 (ชุดรวม 14:14 น.); ดู Surefire report</x:v>
+      </x:c>
     </x:row>
     <x:row r="13" ht="41" customHeight="1">
       <x:c r="A13" s="20" t="str">
@@ -1766,9 +2009,11 @@
       <x:c r="H13" s="20" t="str">
         <x:v>แจ้ง 'Email already exists' และไม่บันทึกผู้ใช้</x:v>
       </x:c>
-      <x:c r="I13" s="42" t="str"/>
+      <x:c r="I13" s="42" t="str">
+        <x:v>ผ่านตามผลที่คาดหวัง โดย JUnit ยืนยันผลของกรณีนี้</x:v>
+      </x:c>
       <x:c r="J13" s="42" t="str">
-        <x:v>No run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K13" s="20" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
@@ -1776,7 +2021,9 @@
       <x:c r="L13" s="20" t="str">
         <x:v>AuthServiceRegisterTest.register_duplicateEmail_rejectedWithoutSaving</x:v>
       </x:c>
-      <x:c r="M13" s="20" t="str"/>
+      <x:c r="M13" s="20" t="str">
+        <x:v>รัน 30 ก.ย. 2569 (ชุดรวม 14:14 น.); ดู Surefire report</x:v>
+      </x:c>
     </x:row>
     <x:row r="14" ht="41" customHeight="1">
       <x:c r="A14" s="20" t="str">
@@ -1803,9 +2050,11 @@
       <x:c r="H14" s="20" t="str">
         <x:v>ตัดช่องว่างและแปลงอีเมลเป็นตัวพิมพ์เล็กก่อนบันทึก</x:v>
       </x:c>
-      <x:c r="I14" s="42" t="str"/>
+      <x:c r="I14" s="42" t="str">
+        <x:v>ผ่านตามผลที่คาดหวัง โดย JUnit ยืนยันผลของกรณีนี้</x:v>
+      </x:c>
       <x:c r="J14" s="42" t="str">
-        <x:v>No run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K14" s="20" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
@@ -1813,7 +2062,9 @@
       <x:c r="L14" s="20" t="str">
         <x:v>AuthServiceRegisterTest.register_spacedUppercaseEmail_normalized</x:v>
       </x:c>
-      <x:c r="M14" s="20" t="str"/>
+      <x:c r="M14" s="20" t="str">
+        <x:v>รัน 30 ก.ย. 2569 (ชุดรวม 14:14 น.); ดู Surefire report</x:v>
+      </x:c>
     </x:row>
     <x:row r="15" ht="41" customHeight="1">
       <x:c r="A15" s="20" t="str">
@@ -1840,9 +2091,11 @@
       <x:c r="H15" s="20" t="str">
         <x:v>เก็บรหัสผ่านที่เข้ารหัสแล้ว และกำหนดสถานะ ACTIVE</x:v>
       </x:c>
-      <x:c r="I15" s="42" t="str"/>
+      <x:c r="I15" s="42" t="str">
+        <x:v>ผ่านตามผลที่คาดหวัง โดย JUnit ยืนยันผลของกรณีนี้</x:v>
+      </x:c>
       <x:c r="J15" s="42" t="str">
-        <x:v>No run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K15" s="20" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
@@ -1850,7 +2103,9 @@
       <x:c r="L15" s="20" t="str">
         <x:v>AuthServiceRegisterTest.register_validData_encodesPasswordAndSetsActive</x:v>
       </x:c>
-      <x:c r="M15" s="20" t="str"/>
+      <x:c r="M15" s="20" t="str">
+        <x:v>รัน 30 ก.ย. 2569 (ชุดรวม 14:14 น.); ดู Surefire report</x:v>
+      </x:c>
     </x:row>
     <x:row r="16" ht="41" customHeight="1">
       <x:c r="A16" s="20" t="str">
@@ -1877,9 +2132,11 @@
       <x:c r="H16" s="20" t="str">
         <x:v>ปฏิเสธข้อมูล และไม่เรียกใช้ Repository/Encoder</x:v>
       </x:c>
-      <x:c r="I16" s="42" t="str"/>
+      <x:c r="I16" s="42" t="str">
+        <x:v>ผ่านตามผลที่คาดหวัง โดย JUnit ยืนยันผลของกรณีนี้</x:v>
+      </x:c>
       <x:c r="J16" s="42" t="str">
-        <x:v>No run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K16" s="20" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
@@ -1887,7 +2144,9 @@
       <x:c r="L16" s="20" t="str">
         <x:v>AuthServiceRegisterTest.register_invalidEmail_doesNotAccessDependencies</x:v>
       </x:c>
-      <x:c r="M16" s="20" t="str"/>
+      <x:c r="M16" s="20" t="str">
+        <x:v>รัน 30 ก.ย. 2569 (ชุดรวม 14:14 น.); ดู Surefire report</x:v>
+      </x:c>
     </x:row>
     <x:row r="17" ht="41" customHeight="1">
       <x:c r="A17" s="20" t="str">
@@ -1914,9 +2173,11 @@
       <x:c r="H17" s="20" t="str">
         <x:v>เข้าสู่ระบบสำเร็จและคืนข้อมูลผู้ใช้</x:v>
       </x:c>
-      <x:c r="I17" s="42" t="str"/>
+      <x:c r="I17" s="42" t="str">
+        <x:v>ผ่านตามผลที่คาดหวัง โดย JUnit ยืนยันผลของกรณีนี้</x:v>
+      </x:c>
       <x:c r="J17" s="42" t="str">
-        <x:v>No run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K17" s="20" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
@@ -1924,7 +2185,9 @@
       <x:c r="L17" s="20" t="str">
         <x:v>AuthServiceLoginTest.login_validCredentials_returnsUser</x:v>
       </x:c>
-      <x:c r="M17" s="20" t="str"/>
+      <x:c r="M17" s="20" t="str">
+        <x:v>รัน 30 ก.ย. 2569 (ชุดรวม 14:14 น.); ดู Surefire report</x:v>
+      </x:c>
     </x:row>
     <x:row r="18" ht="41" customHeight="1">
       <x:c r="A18" s="20" t="str">
@@ -1951,9 +2214,11 @@
       <x:c r="H18" s="20" t="str">
         <x:v>แจ้ง 'Login request is required'</x:v>
       </x:c>
-      <x:c r="I18" s="42" t="str"/>
+      <x:c r="I18" s="42" t="str">
+        <x:v>ผ่านตามผลที่คาดหวัง โดย JUnit ยืนยันผลของกรณีนี้</x:v>
+      </x:c>
       <x:c r="J18" s="42" t="str">
-        <x:v>No run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K18" s="20" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
@@ -1961,7 +2226,9 @@
       <x:c r="L18" s="20" t="str">
         <x:v>AuthServiceLoginTest.login_nullRequest_rejected</x:v>
       </x:c>
-      <x:c r="M18" s="20" t="str"/>
+      <x:c r="M18" s="20" t="str">
+        <x:v>รัน 30 ก.ย. 2569 (ชุดรวม 14:14 น.); ดู Surefire report</x:v>
+      </x:c>
     </x:row>
     <x:row r="19" ht="41" customHeight="1">
       <x:c r="A19" s="20" t="str">
@@ -1988,9 +2255,11 @@
       <x:c r="H19" s="20" t="str">
         <x:v>แจ้ง 'Email is required'</x:v>
       </x:c>
-      <x:c r="I19" s="42" t="str"/>
+      <x:c r="I19" s="42" t="str">
+        <x:v>ผ่านตามผลที่คาดหวัง โดย JUnit ยืนยันผลของกรณีนี้</x:v>
+      </x:c>
       <x:c r="J19" s="42" t="str">
-        <x:v>No run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K19" s="20" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
@@ -1998,7 +2267,9 @@
       <x:c r="L19" s="20" t="str">
         <x:v>AuthServiceLoginTest.login_nullEmail_rejected</x:v>
       </x:c>
-      <x:c r="M19" s="20" t="str"/>
+      <x:c r="M19" s="20" t="str">
+        <x:v>รัน 30 ก.ย. 2569 (ชุดรวม 14:14 น.); ดู Surefire report</x:v>
+      </x:c>
     </x:row>
     <x:row r="20" ht="41" customHeight="1">
       <x:c r="A20" s="20" t="str">
@@ -2025,9 +2296,11 @@
       <x:c r="H20" s="20" t="str">
         <x:v>แจ้ง 'Email is required'</x:v>
       </x:c>
-      <x:c r="I20" s="42" t="str"/>
+      <x:c r="I20" s="42" t="str">
+        <x:v>ผ่านตามผลที่คาดหวัง โดย JUnit ยืนยันผลของกรณีนี้</x:v>
+      </x:c>
       <x:c r="J20" s="42" t="str">
-        <x:v>No run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K20" s="20" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
@@ -2035,7 +2308,9 @@
       <x:c r="L20" s="20" t="str">
         <x:v>AuthServiceLoginTest.login_blankEmail_rejected</x:v>
       </x:c>
-      <x:c r="M20" s="20" t="str"/>
+      <x:c r="M20" s="20" t="str">
+        <x:v>รัน 30 ก.ย. 2569 (ชุดรวม 14:14 น.); ดู Surefire report</x:v>
+      </x:c>
     </x:row>
     <x:row r="21" ht="41" customHeight="1">
       <x:c r="A21" s="20" t="str">
@@ -2062,9 +2337,11 @@
       <x:c r="H21" s="20" t="str">
         <x:v>แจ้ง 'Password is required'</x:v>
       </x:c>
-      <x:c r="I21" s="42" t="str"/>
+      <x:c r="I21" s="42" t="str">
+        <x:v>ผ่านตามผลที่คาดหวัง โดย JUnit ยืนยันผลของกรณีนี้</x:v>
+      </x:c>
       <x:c r="J21" s="42" t="str">
-        <x:v>No run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K21" s="20" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
@@ -2072,7 +2349,9 @@
       <x:c r="L21" s="20" t="str">
         <x:v>AuthServiceLoginTest.login_nullPassword_rejected</x:v>
       </x:c>
-      <x:c r="M21" s="20" t="str"/>
+      <x:c r="M21" s="20" t="str">
+        <x:v>รัน 30 ก.ย. 2569 (ชุดรวม 14:14 น.); ดู Surefire report</x:v>
+      </x:c>
     </x:row>
     <x:row r="22" ht="41" customHeight="1">
       <x:c r="A22" s="20" t="str">
@@ -2099,9 +2378,11 @@
       <x:c r="H22" s="20" t="str">
         <x:v>แจ้ง 'Password is required'</x:v>
       </x:c>
-      <x:c r="I22" s="42" t="str"/>
+      <x:c r="I22" s="42" t="str">
+        <x:v>ผ่านตามผลที่คาดหวัง โดย JUnit ยืนยันผลของกรณีนี้</x:v>
+      </x:c>
       <x:c r="J22" s="42" t="str">
-        <x:v>No run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K22" s="20" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
@@ -2109,7 +2390,9 @@
       <x:c r="L22" s="20" t="str">
         <x:v>AuthServiceLoginTest.login_blankPassword_rejected</x:v>
       </x:c>
-      <x:c r="M22" s="20" t="str"/>
+      <x:c r="M22" s="20" t="str">
+        <x:v>รัน 30 ก.ย. 2569 (ชุดรวม 14:14 น.); ดู Surefire report</x:v>
+      </x:c>
     </x:row>
     <x:row r="23" ht="41" customHeight="1">
       <x:c r="A23" s="20" t="str">
@@ -2136,9 +2419,11 @@
       <x:c r="H23" s="20" t="str">
         <x:v>แจ้ง 'Invalid email or password'</x:v>
       </x:c>
-      <x:c r="I23" s="42" t="str"/>
+      <x:c r="I23" s="42" t="str">
+        <x:v>ผ่านตามผลที่คาดหวัง โดย JUnit ยืนยันผลของกรณีนี้</x:v>
+      </x:c>
       <x:c r="J23" s="42" t="str">
-        <x:v>No run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K23" s="20" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
@@ -2146,7 +2431,9 @@
       <x:c r="L23" s="20" t="str">
         <x:v>AuthServiceLoginTest.login_unknownEmail_rejected</x:v>
       </x:c>
-      <x:c r="M23" s="20" t="str"/>
+      <x:c r="M23" s="20" t="str">
+        <x:v>รัน 30 ก.ย. 2569 (ชุดรวม 14:14 น.); ดู Surefire report</x:v>
+      </x:c>
     </x:row>
     <x:row r="24" ht="41" customHeight="1">
       <x:c r="A24" s="20" t="str">
@@ -2173,9 +2460,11 @@
       <x:c r="H24" s="20" t="str">
         <x:v>แจ้ง 'User account is not active'</x:v>
       </x:c>
-      <x:c r="I24" s="42" t="str"/>
+      <x:c r="I24" s="42" t="str">
+        <x:v>ผ่านตามผลที่คาดหวัง โดย JUnit ยืนยันผลของกรณีนี้</x:v>
+      </x:c>
       <x:c r="J24" s="42" t="str">
-        <x:v>No run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K24" s="20" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
@@ -2183,7 +2472,9 @@
       <x:c r="L24" s="20" t="str">
         <x:v>AuthServiceLoginTest.login_blockedAccount_rejected</x:v>
       </x:c>
-      <x:c r="M24" s="20" t="str"/>
+      <x:c r="M24" s="20" t="str">
+        <x:v>รัน 30 ก.ย. 2569 (ชุดรวม 14:14 น.); ดู Surefire report</x:v>
+      </x:c>
     </x:row>
     <x:row r="25" ht="41" customHeight="1">
       <x:c r="A25" s="20" t="str">
@@ -2210,9 +2501,11 @@
       <x:c r="H25" s="20" t="str">
         <x:v>แจ้ง 'Invalid email or password'</x:v>
       </x:c>
-      <x:c r="I25" s="42" t="str"/>
+      <x:c r="I25" s="42" t="str">
+        <x:v>ผ่านตามผลที่คาดหวัง โดย JUnit ยืนยันผลของกรณีนี้</x:v>
+      </x:c>
       <x:c r="J25" s="42" t="str">
-        <x:v>No run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K25" s="20" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
@@ -2220,7 +2513,9 @@
       <x:c r="L25" s="20" t="str">
         <x:v>AuthServiceLoginTest.login_wrongPassword_rejected</x:v>
       </x:c>
-      <x:c r="M25" s="20" t="str"/>
+      <x:c r="M25" s="20" t="str">
+        <x:v>รัน 30 ก.ย. 2569 (ชุดรวม 14:14 น.); ดู Surefire report</x:v>
+      </x:c>
     </x:row>
     <x:row r="26" ht="41" customHeight="1">
       <x:c r="A26" s="20" t="str">
@@ -2247,9 +2542,11 @@
       <x:c r="H26" s="20" t="str">
         <x:v>ค้นหาด้วยอีเมลที่ตัดช่องว่างและเป็นพิมพ์เล็ก</x:v>
       </x:c>
-      <x:c r="I26" s="42" t="str"/>
+      <x:c r="I26" s="42" t="str">
+        <x:v>ผ่านตามผลที่คาดหวัง โดย JUnit ยืนยันผลของกรณีนี้</x:v>
+      </x:c>
       <x:c r="J26" s="42" t="str">
-        <x:v>No run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K26" s="20" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
@@ -2257,7 +2554,9 @@
       <x:c r="L26" s="20" t="str">
         <x:v>AuthServiceLoginTest.login_spacedUppercaseEmail_normalized</x:v>
       </x:c>
-      <x:c r="M26" s="20" t="str"/>
+      <x:c r="M26" s="20" t="str">
+        <x:v>รัน 30 ก.ย. 2569 (ชุดรวม 14:14 น.); ดู Surefire report</x:v>
+      </x:c>
     </x:row>
     <x:row r="27" ht="41" customHeight="1">
       <x:c r="A27" s="20" t="str">
@@ -2284,9 +2583,11 @@
       <x:c r="H27" s="20" t="str">
         <x:v>ปฏิเสธก่อนตรวจรหัสผ่าน (ไม่เรียก matches)</x:v>
       </x:c>
-      <x:c r="I27" s="42" t="str"/>
+      <x:c r="I27" s="42" t="str">
+        <x:v>ผ่านตามผลที่คาดหวัง โดย JUnit ยืนยันผลของกรณีนี้</x:v>
+      </x:c>
       <x:c r="J27" s="42" t="str">
-        <x:v>No run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K27" s="20" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
@@ -2294,7 +2595,9 @@
       <x:c r="L27" s="20" t="str">
         <x:v>AuthServiceLoginTest.login_blockedAccount_doesNotCheckPassword</x:v>
       </x:c>
-      <x:c r="M27" s="20" t="str"/>
+      <x:c r="M27" s="20" t="str">
+        <x:v>รัน 30 ก.ย. 2569 (ชุดรวม 14:14 น.); ดู Surefire report</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2397,7 +2700,7 @@
         <x:v>AuthService.validateRegistration</x:v>
       </x:c>
       <x:c r="F5" s="20" t="str">
-        <x:v>Planned</x:v>
+        <x:v>ทดสอบผ่าน (Unit)</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="34" customHeight="1">
@@ -2417,7 +2720,7 @@
         <x:v>AuthService.validateRegistration</x:v>
       </x:c>
       <x:c r="F6" s="20" t="str">
-        <x:v>Planned</x:v>
+        <x:v>ทดสอบผ่าน (Unit)</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="34" customHeight="1">
@@ -2437,7 +2740,7 @@
         <x:v>AuthService.register + UserRepository.existsByEmail</x:v>
       </x:c>
       <x:c r="F7" s="20" t="str">
-        <x:v>Planned</x:v>
+        <x:v>ทดสอบผ่าน (Unit)</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="34" customHeight="1">
@@ -2457,7 +2760,7 @@
         <x:v>AuthService.register</x:v>
       </x:c>
       <x:c r="F8" s="20" t="str">
-        <x:v>Planned</x:v>
+        <x:v>ทดสอบผ่าน (Unit)</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="34" customHeight="1">
@@ -2477,7 +2780,7 @@
         <x:v>AuthService.register</x:v>
       </x:c>
       <x:c r="F9" s="20" t="str">
-        <x:v>Planned</x:v>
+        <x:v>ทดสอบผ่าน (Unit)</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="34" customHeight="1">
@@ -2497,7 +2800,7 @@
         <x:v>AuthService.validateLogin</x:v>
       </x:c>
       <x:c r="F10" s="20" t="str">
-        <x:v>Planned</x:v>
+        <x:v>ทดสอบผ่าน (Unit)</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="34" customHeight="1">
@@ -2517,7 +2820,7 @@
         <x:v>AuthService.login</x:v>
       </x:c>
       <x:c r="F11" s="20" t="str">
-        <x:v>Planned</x:v>
+        <x:v>ทดสอบผ่าน (Unit)</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="34" customHeight="1">
@@ -2537,7 +2840,7 @@
         <x:v>AuthService.login</x:v>
       </x:c>
       <x:c r="F12" s="20" t="str">
-        <x:v>Planned</x:v>
+        <x:v>ทดสอบผ่าน (Unit)</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="34" customHeight="1">
@@ -2557,7 +2860,7 @@
         <x:v>AuthService.login</x:v>
       </x:c>
       <x:c r="F13" s="20" t="str">
-        <x:v>Planned</x:v>
+        <x:v>ทดสอบผ่าน (Unit)</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="30" customHeight="1">
@@ -2573,7 +2876,7 @@
         <x:v>หมายเหตุ</x:v>
       </x:c>
       <x:c r="B17" s="18" t="str">
-        <x:v>รหัส REQ และ UC เป็นรหัสชั่วคราวที่ใช้จัด Test Case อ้างอิงโค้ดปัจจุบัน รอเทียบกับ Use Case ของทีมอีกครั้ง</x:v>
+        <x:v>รหัส REQ และ UC ในตารางเป็นรหัสอ้างอิงภายในเอกสารทดสอบ</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2588,19 +2891,23 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="57" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="69" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="35" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="20" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="15" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="15" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="15" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="15" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="33" customHeight="1">
-      <x:c r="A1" s="34" t="str">
-        <x:v>สรุปผลการทดสอบ</x:v>
-      </x:c>
-      <x:c r="B1" s="34"/>
-      <x:c r="C1" s="34"/>
-      <x:c r="D1" s="34"/>
-      <x:c r="E1" s="34"/>
-      <x:c r="F1" s="34"/>
+    <x:row r="1" ht="34" customHeight="1">
+      <x:c r="A1" s="60" t="str">
+        <x:v>สรุปผลการทดสอบ CPFriendFinder</x:v>
+      </x:c>
+      <x:c r="B1" s="61"/>
+      <x:c r="C1" s="61"/>
+      <x:c r="D1" s="61"/>
+      <x:c r="E1" s="61"/>
+      <x:c r="F1" s="61"/>
       <x:c r="G1" s="34"/>
       <x:c r="H1" s="34"/>
       <x:c r="I1" s="34"/>
@@ -2609,74 +2916,76 @@
       <x:c r="L1" s="34"/>
       <x:c r="M1" s="34"/>
     </x:row>
-    <x:row r="2" ht="36" customHeight="1">
-      <x:c r="A2" s="4"/>
-      <x:c r="B2" s="4"/>
-      <x:c r="C2" s="4"/>
-      <x:c r="D2" s="4"/>
-      <x:c r="E2" s="4"/>
-      <x:c r="F2" s="4"/>
-    </x:row>
-    <x:row r="4" ht="34" customHeight="1">
-      <x:c r="A4" s="37" t="str">
-        <x:v>Unit Test: Register และ Login</x:v>
-      </x:c>
-      <x:c r="B4" s="37" t="str">
+    <x:row r="2" ht="25" customHeight="1">
+      <x:c r="A2" s="84" t="str">
+        <x:v>AuthService | 30 กันยายน 2569 เวลา 14:14 น.</x:v>
+      </x:c>
+      <x:c r="B2" s="85"/>
+      <x:c r="C2" s="85"/>
+      <x:c r="D2" s="85"/>
+      <x:c r="E2" s="85"/>
+      <x:c r="F2" s="85"/>
+    </x:row>
+    <x:row r="4" ht="26" customHeight="1">
+      <x:c r="A4" s="44" t="str">
+        <x:v>กรณีทดสอบ Register และ Login</x:v>
+      </x:c>
+      <x:c r="B4" s="44" t="str">
         <x:v>จำนวน</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="28" customHeight="1">
       <x:c r="A5" s="20" t="str">
-        <x:v>Planned cases</x:v>
-      </x:c>
-      <x:c r="B5" s="20" t="n">
+        <x:v>ออกแบบไว้</x:v>
+      </x:c>
+      <x:c r="B5" s="56" t="n">
         <x:f>COUNTA('Test Case Design &amp; Test Results'!$C$5:$C$250)</x:f>
         <x:v>23</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="28" customHeight="1">
       <x:c r="A6" s="20" t="str">
-        <x:v>Actually executed</x:v>
-      </x:c>
-      <x:c r="B6" s="20" t="n">
+        <x:v>รันทดสอบแล้ว</x:v>
+      </x:c>
+      <x:c r="B6" s="56" t="n">
         <x:f>COUNTIF('Test Case Design &amp; Test Results'!$J$5:$J$250,"Pass")+COUNTIF('Test Case Design &amp; Test Results'!$J$5:$J$250,"Fail")+COUNTIF('Test Case Design &amp; Test Results'!$J$5:$J$250,"Block")</x:f>
-        <x:v>0</x:v>
+        <x:v>23</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="28" customHeight="1">
       <x:c r="A7" s="20" t="str">
-        <x:v>Passed</x:v>
-      </x:c>
-      <x:c r="B7" s="20" t="n">
+        <x:v>ผ่าน</x:v>
+      </x:c>
+      <x:c r="B7" s="56" t="n">
         <x:f>COUNTIF('Test Case Design &amp; Test Results'!$J$5:$J$250,"Pass")</x:f>
-        <x:v>0</x:v>
+        <x:v>23</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="28" customHeight="1">
       <x:c r="A8" s="20" t="str">
-        <x:v>Failed</x:v>
-      </x:c>
-      <x:c r="B8" s="20" t="n">
+        <x:v>ไม่ผ่าน</x:v>
+      </x:c>
+      <x:c r="B8" s="56" t="n">
         <x:f>COUNTIF('Test Case Design &amp; Test Results'!$J$5:$J$250,"Fail")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="28" customHeight="1">
       <x:c r="A9" s="20" t="str">
-        <x:v>Blocked</x:v>
-      </x:c>
-      <x:c r="B9" s="20" t="n">
+        <x:v>ทดสอบไม่ได้</x:v>
+      </x:c>
+      <x:c r="B9" s="56" t="n">
         <x:f>COUNTIF('Test Case Design &amp; Test Results'!$J$5:$J$250,"Block")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="28" customHeight="1">
       <x:c r="A10" s="20" t="str">
-        <x:v>No run</x:v>
-      </x:c>
-      <x:c r="B10" s="20" t="n">
+        <x:v>ยังไม่รัน</x:v>
+      </x:c>
+      <x:c r="B10" s="56" t="n">
         <x:f>COUNTIF('Test Case Design &amp; Test Results'!$J$5:$J$250,"No run")</x:f>
-        <x:v>23</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="28" customHeight="1">
@@ -2684,104 +2993,225 @@
       <x:c r="B11" s="20"/>
     </x:row>
     <x:row r="12" ht="28" customHeight="1">
-      <x:c r="A12" s="20"/>
+      <x:c r="A12" s="59" t="str">
+        <x:v>ผลการรัน Maven (ชุดรวม)</x:v>
+      </x:c>
       <x:c r="B12" s="20"/>
+      <x:c r="C12"/>
+      <x:c r="D12"/>
+      <x:c r="E12"/>
+      <x:c r="F12"/>
     </x:row>
     <x:row r="13" ht="27" customHeight="1">
-      <x:c r="A13" s="39" t="str">
-        <x:v>ผลเดิมจากการรัน contextLoads เมื่อ 30 ก.ย. 2569</x:v>
-      </x:c>
-      <x:c r="B13" s="39" t="str">
-        <x:v>จำนวน</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="28" customHeight="1">
+      <x:c r="A13" s="44" t="str">
+        <x:v>ชุดทดสอบ</x:v>
+      </x:c>
+      <x:c r="B13" s="44" t="str">
+        <x:v>รัน</x:v>
+      </x:c>
+      <x:c r="C13" s="49" t="str">
+        <x:v>ผ่าน</x:v>
+      </x:c>
+      <x:c r="D13" s="49" t="str">
+        <x:v>ไม่ผ่าน</x:v>
+      </x:c>
+      <x:c r="E13" s="49" t="str">
+        <x:v>ข้อผิดพลาด</x:v>
+      </x:c>
+      <x:c r="F13" s="49" t="str">
+        <x:v>ข้าม</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="23" customHeight="1">
       <x:c r="A14" s="20" t="str">
-        <x:v>Tests run</x:v>
-      </x:c>
-      <x:c r="B14" s="20" t="n">
+        <x:v>FriendApplicationTests</x:v>
+      </x:c>
+      <x:c r="B14" s="56" t="n">
         <x:v>1</x:v>
       </x:c>
-    </x:row>
-    <x:row r="15" ht="28" customHeight="1">
+      <x:c r="C14" s="57" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D14" s="57" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E14" s="57" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F14" s="57" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="23" customHeight="1">
       <x:c r="A15" s="20" t="str">
-        <x:v>Pass</x:v>
-      </x:c>
-      <x:c r="B15" s="20" t="n">
+        <x:v>AuthServiceRegisterTest</x:v>
+      </x:c>
+      <x:c r="B15" s="56" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="C15" s="57" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="D15" s="57" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E15" s="57" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F15" s="57" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="23" customHeight="1">
+      <x:c r="A16" s="20" t="str">
+        <x:v>AuthServiceLoginTest</x:v>
+      </x:c>
+      <x:c r="B16" s="56" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="C16" s="57" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="D16" s="57" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E16" s="57" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F16" s="57" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="23" customHeight="1">
+      <x:c r="A17" s="20" t="str">
+        <x:v>AuthServiceTest</x:v>
+      </x:c>
+      <x:c r="B17" s="56" t="n">
         <x:v>1</x:v>
       </x:c>
-    </x:row>
-    <x:row r="16" ht="28" customHeight="1">
-      <x:c r="A16" s="20" t="str">
-        <x:v>Fail / Errors / Skipped</x:v>
-      </x:c>
-      <x:c r="B16" s="20" t="str">
-        <x:v>0 / 0 / 0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" ht="28" customHeight="1">
-      <x:c r="A17" s="20"/>
-      <x:c r="B17" s="20"/>
-    </x:row>
-    <x:row r="18" ht="27" customHeight="1">
-      <x:c r="A18" s="39" t="str">
-        <x:v>สถานะ</x:v>
-      </x:c>
-      <x:c r="B18" s="39" t="str">
-        <x:v>ความหมาย</x:v>
+      <x:c r="C17" s="57" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D17" s="57" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E17" s="57" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F17" s="57" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="23" customHeight="1">
+      <x:c r="A18" s="52" t="str">
+        <x:v>รวม</x:v>
+      </x:c>
+      <x:c r="B18" s="52" t="n">
+        <x:f>SUM(B14:B17)</x:f>
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="C18" s="58" t="n">
+        <x:f>SUM(C14:C17)</x:f>
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="D18" s="58" t="n">
+        <x:f>SUM(D14:D17)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E18" s="58" t="n">
+        <x:f>SUM(E14:E17)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F18" s="58" t="n">
+        <x:f>SUM(F14:F17)</x:f>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="26" customHeight="1">
-      <x:c r="A19" s="20" t="str">
-        <x:v>No run</x:v>
-      </x:c>
-      <x:c r="B19" s="20" t="str">
-        <x:v>มี Test Case และ/หรือโค้ดแล้ว แต่ยังไม่รัน/ไม่มีหลักฐานให้ลงผล</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20" ht="26" customHeight="1">
+      <x:c r="A19" s="20"/>
+      <x:c r="B19" s="20"/>
+      <x:c r="C19"/>
+      <x:c r="D19"/>
+      <x:c r="E19"/>
+      <x:c r="F19"/>
+    </x:row>
+    <x:row r="20" ht="25" customHeight="1">
       <x:c r="A20" s="20" t="str">
-        <x:v>Pass</x:v>
+        <x:v>ผลการรัน</x:v>
       </x:c>
       <x:c r="B20" s="20" t="str">
-        <x:v>ต้องมี Actual Result และผลรันจริงพร้อม commit/time</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21" ht="26" customHeight="1">
+        <x:v>BUILD SUCCESS</x:v>
+      </x:c>
+      <x:c r="C20"/>
+      <x:c r="D20"/>
+      <x:c r="E20"/>
+      <x:c r="F20"/>
+    </x:row>
+    <x:row r="21" ht="25" customHeight="1">
       <x:c r="A21" s="20" t="str">
-        <x:v>Fail/Block</x:v>
+        <x:v>ระยะเวลา</x:v>
       </x:c>
       <x:c r="B21" s="20" t="str">
-        <x:v>ลงเหตุผลพร้อม log และผูก Defect ID หากได้รับการยืนยัน</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="22" ht="28" customHeight="1">
-      <x:c r="A22" s="20"/>
-      <x:c r="B22" s="20"/>
-    </x:row>
-    <x:row r="23" ht="28" customHeight="1">
+        <x:v>1 นาที 34 วินาที</x:v>
+      </x:c>
+      <x:c r="C21"/>
+      <x:c r="D21"/>
+      <x:c r="E21"/>
+      <x:c r="F21"/>
+    </x:row>
+    <x:row r="22" ht="25" customHeight="1">
+      <x:c r="A22" s="20" t="str">
+        <x:v>คำสั่ง</x:v>
+      </x:c>
+      <x:c r="B22" s="20" t="str">
+        <x:v>./mvnw -Djava.version=21 clean test</x:v>
+      </x:c>
+      <x:c r="C22"/>
+      <x:c r="D22"/>
+      <x:c r="E22"/>
+      <x:c r="F22"/>
+    </x:row>
+    <x:row r="23" ht="25" customHeight="1">
       <x:c r="A23" s="20"/>
       <x:c r="B23" s="20"/>
-    </x:row>
-    <x:row r="24" ht="27" customHeight="1">
-      <x:c r="A24" s="39" t="str">
-        <x:v>ส่วนที่ยังไม่ได้ทดสอบ</x:v>
-      </x:c>
-      <x:c r="B24" s="39" t="str">
-        <x:v>สถานะ</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="25" ht="28" customHeight="1">
-      <x:c r="A25" s="20" t="str">
-        <x:v>Controller / API / Integration / UAT</x:v>
-      </x:c>
-      <x:c r="B25" s="20" t="str">
-        <x:v>รอรวมและยืนยันการทำงานกับทีม</x:v>
-      </x:c>
+      <x:c r="C23"/>
+      <x:c r="D23"/>
+      <x:c r="E23"/>
+      <x:c r="F23"/>
+    </x:row>
+    <x:row r="24" ht="30" customHeight="1">
+      <x:c r="A24" s="86" t="str">
+        <x:v>กรณีใน Excel</x:v>
+      </x:c>
+      <x:c r="B24" s="74" t="str">
+        <x:v>Register 12 รายการ และ Login 11 รายการ รวม 23 รายการ</x:v>
+      </x:c>
+      <x:c r="C24" s="71"/>
+      <x:c r="D24" s="71"/>
+      <x:c r="E24" s="71"/>
+      <x:c r="F24" s="71"/>
+    </x:row>
+    <x:row r="25" ht="30" customHeight="1">
+      <x:c r="A25" s="87" t="str">
+        <x:v>รายการเพิ่มเติม</x:v>
+      </x:c>
+      <x:c r="B25" s="88" t="str">
+        <x:v>FriendApplicationTests และ AuthServiceTest อย่างละ 1 รายการ รวมผล Maven 25 รายการ</x:v>
+      </x:c>
+      <x:c r="C25" s="71"/>
+      <x:c r="D25" s="71"/>
+      <x:c r="E25" s="71"/>
+      <x:c r="F25" s="71"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:F2"/>
+    <x:mergeCell ref="A1:F1"/>
+    <x:mergeCell ref="A12:F12"/>
+    <x:mergeCell ref="B20:F20"/>
+    <x:mergeCell ref="B21:F21"/>
+    <x:mergeCell ref="B22:F22"/>
+    <x:mergeCell ref="B24:F24"/>
+    <x:mergeCell ref="B25:F25"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -2791,27 +3221,27 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="23" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="49" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="42" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="13" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="13" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="28" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="68" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="19" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="43" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="44" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="12" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="12" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="14" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="24" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="20" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="33" customHeight="1">
-      <x:c r="A1" s="34" t="str">
+    <x:row r="1" ht="32" customHeight="1">
+      <x:c r="A1" s="60" t="str">
         <x:v>ประวัติการรันทดสอบ</x:v>
       </x:c>
-      <x:c r="B1" s="34"/>
-      <x:c r="C1" s="34"/>
-      <x:c r="D1" s="34"/>
-      <x:c r="E1" s="34"/>
-      <x:c r="F1" s="34"/>
-      <x:c r="G1" s="34"/>
-      <x:c r="H1" s="34"/>
+      <x:c r="B1" s="61"/>
+      <x:c r="C1" s="61"/>
+      <x:c r="D1" s="61"/>
+      <x:c r="E1" s="61"/>
+      <x:c r="F1" s="61"/>
+      <x:c r="G1" s="61"/>
+      <x:c r="H1" s="61"/>
       <x:c r="I1" s="34"/>
       <x:c r="J1" s="34"/>
       <x:c r="K1" s="34"/>
@@ -2828,77 +3258,126 @@
       <x:c r="G2" s="4"/>
       <x:c r="H2" s="4"/>
     </x:row>
-    <x:row r="4" ht="34" customHeight="1">
-      <x:c r="A4" s="37" t="str">
-        <x:v>Run ID</x:v>
-      </x:c>
-      <x:c r="B4" s="37" t="str">
+    <x:row r="4" ht="28" customHeight="1">
+      <x:c r="A4" s="44" t="str">
+        <x:v>รอบ</x:v>
+      </x:c>
+      <x:c r="B4" s="44" t="str">
         <x:v>วันและเวลา</x:v>
       </x:c>
-      <x:c r="C4" s="37" t="str">
-        <x:v>branch</x:v>
-      </x:c>
-      <x:c r="D4" s="37" t="str">
+      <x:c r="C4" s="44" t="str">
         <x:v>ชุดทดสอบ</x:v>
       </x:c>
-      <x:c r="E4" s="37" t="str">
+      <x:c r="D4" s="44" t="str">
         <x:v>จำนวน</x:v>
       </x:c>
-      <x:c r="F4" s="37" t="str">
+      <x:c r="E4" s="44" t="str">
         <x:v>ผ่าน</x:v>
       </x:c>
-      <x:c r="G4" s="37" t="str">
-        <x:v>ไม่ผ่าน / error / ข้าม</x:v>
-      </x:c>
-      <x:c r="H4" s="37" t="str">
-        <x:v>หลักฐาน / หมายเหตุ</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="36" customHeight="1">
+      <x:c r="F4" s="44" t="str">
+        <x:v>ไม่ผ่าน</x:v>
+      </x:c>
+      <x:c r="G4" s="44" t="str">
+        <x:v>Error / Skipped</x:v>
+      </x:c>
+      <x:c r="H4" s="44" t="str">
+        <x:v>ผลการรัน</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="29" customHeight="1">
       <x:c r="A5" s="20" t="str">
-        <x:v>BASE-20260930-01</x:v>
+        <x:v>BASE-01</x:v>
       </x:c>
       <x:c r="B5" s="20" t="str">
-        <x:v>2026-09-30 13:06 +07</x:v>
+        <x:v>30 ก.ย. 2569 13:06</x:v>
       </x:c>
       <x:c r="C5" s="20" t="str">
-        <x:v>piyapon_673380050-9_section1_(backend)</x:v>
-      </x:c>
-      <x:c r="D5" s="20" t="str">
         <x:v>FriendApplicationTests.contextLoads</x:v>
+      </x:c>
+      <x:c r="D5" s="20" t="n">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E5" s="20" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="F5" s="20" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G5" s="20" t="str">
-        <x:v>0 / 0 / 0</x:v>
+        <x:v>0 / 0</x:v>
       </x:c>
       <x:c r="H5" s="20" t="str">
-        <x:v>ผล Maven ที่ผู้ทดสอบส่งมา: BUILD SUCCESS; ใช้ยืนยันเฉพาะ Spring context</x:v>
-      </x:c>
+        <x:v>BUILD SUCCESS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="29" customHeight="1">
+      <x:c r="A6" s="18" t="str">
+        <x:v>AUTH-01</x:v>
+      </x:c>
+      <x:c r="B6" s="18" t="str">
+        <x:v>30 ก.ย. 2569 14:14</x:v>
+      </x:c>
+      <x:c r="C6" s="18" t="str">
+        <x:v>JUnit ทุกชุด (รวม 4 คลาส)</x:v>
+      </x:c>
+      <x:c r="D6" s="18" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="E6" s="18" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="F6" s="18" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G6" s="18" t="str">
+        <x:v>0 / 0</x:v>
+      </x:c>
+      <x:c r="H6" s="18" t="str">
+        <x:v>BUILD SUCCESS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="18"/>
+      <x:c r="B7" s="18"/>
+      <x:c r="C7" s="18"/>
+      <x:c r="D7" s="18"/>
+      <x:c r="E7" s="18"/>
+      <x:c r="F7" s="18"/>
+      <x:c r="G7" s="18"/>
+      <x:c r="H7" s="18"/>
     </x:row>
     <x:row r="8" ht="27" customHeight="1">
-      <x:c r="A8" s="39" t="str">
-        <x:v>Next execution</x:v>
-      </x:c>
-      <x:c r="B8" s="39" t="str">
-        <x:v>Status</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9">
-      <x:c r="A9" t="str">
-        <x:v>AuthServiceRegisterTest/AuthServiceLoginTest</x:v>
-      </x:c>
-      <x:c r="B9" t="str">
-        <x:v>No run — ผู้ใช้ต้องรันและบันทึกผลจริงก่อนเปลี่ยนสถานะ</x:v>
-      </x:c>
+      <x:c r="A8" s="64" t="str">
+        <x:v>คำสั่ง</x:v>
+      </x:c>
+      <x:c r="B8" s="78" t="str">
+        <x:v>./mvnw -Djava.version=21 clean test</x:v>
+      </x:c>
+      <x:c r="C8" s="18"/>
+      <x:c r="D8" s="18"/>
+      <x:c r="E8" s="18"/>
+      <x:c r="F8" s="18"/>
+      <x:c r="G8" s="18"/>
+      <x:c r="H8" s="18"/>
+    </x:row>
+    <x:row r="9" ht="44" customHeight="1">
+      <x:c r="A9" s="80" t="str">
+        <x:v>หลักฐาน</x:v>
+      </x:c>
+      <x:c r="B9" s="79" t="str">
+        <x:v>target/surefire-reports/ (ผลทดสอบที่ Maven สร้างในเครื่อง)</x:v>
+      </x:c>
+      <x:c r="C9" s="18"/>
+      <x:c r="D9" s="18"/>
+      <x:c r="E9" s="18"/>
+      <x:c r="F9" s="18"/>
+      <x:c r="G9" s="18"/>
+      <x:c r="H9" s="18"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H2"/>
+    <x:mergeCell ref="A1:H1"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
test(web): add full-context web flow tests and execution results
</commit_message>
<xml_diff>
--- a/test/test-cases/CPFriendFinder_TestCases.xlsx
+++ b/test/test-cases/CPFriendFinder_TestCases.xlsx
@@ -2,17 +2,18 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="1" r:id="Rbca24a2771ec487f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Case Design &amp; Test Results" sheetId="2" r:id="R1c2728ced674451d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Scenario Summary" sheetId="3" r:id="R7061688ca4f64908"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defect Summary" sheetId="4" r:id="Rda678dff42384d12"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS001" sheetId="5" r:id="Ra82380471714483f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS002" sheetId="6" r:id="R9d3bdbdc10de45a4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS003" sheetId="7" r:id="R2c65ec019f9245e7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS004" sheetId="8" r:id="R47b754cd917b4641"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements Traceability" sheetId="9" r:id="R1a3b2e4d26c04c14"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Summary Report" sheetId="10" r:id="R1c1b8cbaf9474b3c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution Log" sheetId="11" r:id="Re72b34a5ae5a4b9c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="1" r:id="R8250022ecbd441ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Case Design &amp; Test Results" sheetId="2" r:id="R741434875c1a4817"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Scenario Summary" sheetId="3" r:id="R309c534f713f4b59"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defect Summary" sheetId="4" r:id="R92b54f913ba94dd0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS001" sheetId="5" r:id="R801a20c1193b434f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS002" sheetId="6" r:id="R0de1a323070f470a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS003" sheetId="7" r:id="R5bc92a2d0f174bcf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS004" sheetId="8" r:id="Rad6f1d07ea4b4119"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements Traceability" sheetId="9" r:id="R00224aa11b39427d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Summary Report" sheetId="10" r:id="R4ca5662d66d949e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution Log" sheetId="11" r:id="Rb1401a685687437c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS005" sheetId="12" r:id="R1845edee92fe474c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -61,7 +62,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="18">
+  <x:cellXfs count="20">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -107,6 +108,10 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -365,7 +370,7 @@
         <x:v>Test scope</x:v>
       </x:c>
       <x:c r="B8" s="8" t="str">
-        <x:v>Registration, login, controller MVC and Spring Security</x:v>
+        <x:v>Authentication (completed); full-context web smoke tests (planned)</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="21" customHeight="1">
@@ -373,7 +378,7 @@
         <x:v>Documented test cases</x:v>
       </x:c>
       <x:c r="B9" s="8" t="str">
-        <x:v>42 (Registration 12; Login 11; Controller 10; Security 9)</x:v>
+        <x:v>50 cases: 42 passed (23 Service, 10 Controller, 9 Security); 8 Web Flow not run</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="21" customHeight="1">
@@ -405,7 +410,7 @@
         <x:v>Coverage boundary</x:v>
       </x:c>
       <x:c r="B13" s="8" t="str">
-        <x:v>Unit tests mock repository/encoder. MVC and security tests mock AuthService; no real-database E2E test.</x:v>
+        <x:v>Service tests mock dependencies. MVC, security and web tests mock AuthService; no real-database E2E test.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="21" customHeight="1">
@@ -469,7 +474,7 @@
         <x:v>JUnit tests</x:v>
       </x:c>
       <x:c r="B22" s="8" t="str">
-        <x:v>src/test/java/com/cp/friend/service/ and controller/</x:v>
+        <x:v>src/test/java/com/cp/friend/ (service, controller and integration)</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="21" customHeight="1">
@@ -520,7 +525,7 @@
     </x:row>
     <x:row r="2" ht="21" customHeight="1">
       <x:c r="A2" s="8" t="str">
-        <x:v>Scope: Authentication  |  Last completed: 2026-09-30 17:09:30</x:v>
+        <x:v>Planned: 50 cases (42 passed + 8 not run) | Last completed full run: 2026-09-30 17:09:30 (43 passed)</x:v>
       </x:c>
       <x:c r="B2" s="8"/>
       <x:c r="C2" s="8"/>
@@ -553,8 +558,8 @@
         <x:v>Designed</x:v>
       </x:c>
       <x:c r="B5" s="15" t="n">
-        <x:f>COUNTA('Test Case Design &amp; Test Results'!$C$5:$C$46)</x:f>
-        <x:v>42</x:v>
+        <x:f>COUNTA('Test Case Design &amp; Test Results'!$C$5:$C$54)</x:f>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C5" s="8"/>
       <x:c r="D5" s="8"/>
@@ -566,7 +571,7 @@
         <x:v>Executed</x:v>
       </x:c>
       <x:c r="B6" s="15" t="n">
-        <x:f>COUNTIF('Test Case Design &amp; Test Results'!$J$5:$J$46,"Pass")+COUNTIF('Test Case Design &amp; Test Results'!$J$5:$J$46,"Fail")</x:f>
+        <x:f>COUNTIF('Test Case Design &amp; Test Results'!$J$5:$J$54,"Pass")+COUNTIF('Test Case Design &amp; Test Results'!$J$5:$J$54,"Fail")</x:f>
         <x:v>42</x:v>
       </x:c>
       <x:c r="C6" s="8"/>
@@ -579,7 +584,7 @@
         <x:v>Passed</x:v>
       </x:c>
       <x:c r="B7" s="15" t="n">
-        <x:f>COUNTIF('Test Case Design &amp; Test Results'!$J$5:$J$46,"Pass")</x:f>
+        <x:f>COUNTIF('Test Case Design &amp; Test Results'!$J$5:$J$54,"Pass")</x:f>
         <x:v>42</x:v>
       </x:c>
       <x:c r="C7" s="8"/>
@@ -592,7 +597,7 @@
         <x:v>Failed</x:v>
       </x:c>
       <x:c r="B8" s="15" t="n">
-        <x:f>COUNTIF('Test Case Design &amp; Test Results'!$J$5:$J$46,"Fail")</x:f>
+        <x:f>COUNTIF('Test Case Design &amp; Test Results'!$J$5:$J$54,"Fail")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="C8" s="8"/>
@@ -605,7 +610,7 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="B9" s="15" t="n">
-        <x:f>COUNTIF('Test Case Design &amp; Test Results'!$J$5:$J$46,"Block")</x:f>
+        <x:f>COUNTIF('Test Case Design &amp; Test Results'!$J$5:$J$54,"Block")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="C9" s="8"/>
@@ -618,8 +623,8 @@
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="B10" s="15" t="n">
-        <x:f>COUNTIF('Test Case Design &amp; Test Results'!$J$5:$J$46,"No run")</x:f>
-        <x:v>0</x:v>
+        <x:f>COUNTIF('Test Case Design &amp; Test Results'!$J$5:$J$54,"No run")</x:f>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="C10" s="8"/>
       <x:c r="D10" s="8"/>
@@ -838,7 +843,7 @@
         <x:v>Documented Cases</x:v>
       </x:c>
       <x:c r="B24" s="8" t="str">
-        <x:v>Registration 12 + Login 11 + Controller 10 + Security 9 = 42</x:v>
+        <x:v>42 completed (Service 23 + Controller 10 + Security 9); 8 WEB cases not run</x:v>
       </x:c>
       <x:c r="C24" s="8"/>
       <x:c r="D24" s="8"/>
@@ -847,10 +852,10 @@
     </x:row>
     <x:row r="25" ht="24" customHeight="1">
       <x:c r="A25" s="8" t="str">
-        <x:v>Additional Context Test</x:v>
+        <x:v>Latest Completed Maven Run</x:v>
       </x:c>
       <x:c r="B25" s="8" t="str">
-        <x:v>FriendApplicationTests = 1; total Maven tests = 43</x:v>
+        <x:v>43/43 passed, including FriendApplicationTests (2026-09-30 17:09:30)</x:v>
       </x:c>
       <x:c r="C25" s="8"/>
       <x:c r="D25" s="8"/>
@@ -1251,6 +1256,270 @@
 </x:worksheet>
 </file>
 
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="39" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="48" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="22" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="16" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" t="str">
+        <x:v>TS005 - Full-Context Web Flow</x:v>
+      </x:c>
+      <x:c r="B1"/>
+      <x:c r="C1"/>
+      <x:c r="D1"/>
+      <x:c r="E1"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2"/>
+      <x:c r="B2"/>
+      <x:c r="C2"/>
+      <x:c r="D2"/>
+      <x:c r="E2"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3"/>
+      <x:c r="B3"/>
+      <x:c r="C3"/>
+      <x:c r="D3"/>
+      <x:c r="E3"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" t="str">
+        <x:v>Scenario ID</x:v>
+      </x:c>
+      <x:c r="B4" t="str">
+        <x:v>TS005</x:v>
+      </x:c>
+      <x:c r="C4"/>
+      <x:c r="D4"/>
+      <x:c r="E4"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" t="str">
+        <x:v>Use Case ID</x:v>
+      </x:c>
+      <x:c r="B5" t="str">
+        <x:v>UC-WEB-01</x:v>
+      </x:c>
+      <x:c r="C5"/>
+      <x:c r="D5"/>
+      <x:c r="E5"/>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" t="str">
+        <x:v>Test Scenario</x:v>
+      </x:c>
+      <x:c r="B6" t="str">
+        <x:v>Full-context pages, static resources and authentication flow</x:v>
+      </x:c>
+      <x:c r="C6"/>
+      <x:c r="D6"/>
+      <x:c r="E6"/>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" t="str">
+        <x:v>JUnit Test Class</x:v>
+      </x:c>
+      <x:c r="B7" t="str">
+        <x:v>WebFlowIntegrationTest</x:v>
+      </x:c>
+      <x:c r="C7"/>
+      <x:c r="D7"/>
+      <x:c r="E7"/>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" t="str">
+        <x:v>Result</x:v>
+      </x:c>
+      <x:c r="B8" t="str">
+        <x:v>Not run (8 planned cases)</x:v>
+      </x:c>
+      <x:c r="C8"/>
+      <x:c r="D8"/>
+      <x:c r="E8"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" t="str">
+        <x:v>Test Date</x:v>
+      </x:c>
+      <x:c r="B9" t="str"/>
+      <x:c r="C9"/>
+      <x:c r="D9"/>
+      <x:c r="E9"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10"/>
+      <x:c r="B10"/>
+      <x:c r="C10"/>
+      <x:c r="D10"/>
+      <x:c r="E10"/>
+    </x:row>
+    <x:row r="11" ht="24" customHeight="1">
+      <x:c r="A11" s="19" t="str">
+        <x:v>Case ID</x:v>
+      </x:c>
+      <x:c r="B11" s="19" t="str">
+        <x:v>Endpoint / Scenario</x:v>
+      </x:c>
+      <x:c r="C11" s="19" t="str">
+        <x:v>Expected Result</x:v>
+      </x:c>
+      <x:c r="D11" s="19" t="str">
+        <x:v>Actual Result</x:v>
+      </x:c>
+      <x:c r="E11" s="19" t="str">
+        <x:v>Status</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="34" customHeight="1">
+      <x:c r="A12" s="19" t="str">
+        <x:v>WEB-001</x:v>
+      </x:c>
+      <x:c r="B12" s="19" t="str">
+        <x:v>GET /login</x:v>
+      </x:c>
+      <x:c r="C12" s="19" t="str">
+        <x:v>200 OK; renders login view</x:v>
+      </x:c>
+      <x:c r="D12" s="19" t="str"/>
+      <x:c r="E12" s="19" t="str">
+        <x:v>No run</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="34" customHeight="1">
+      <x:c r="A13" s="19" t="str">
+        <x:v>WEB-002</x:v>
+      </x:c>
+      <x:c r="B13" s="19" t="str">
+        <x:v>GET /register</x:v>
+      </x:c>
+      <x:c r="C13" s="19" t="str">
+        <x:v>200 OK; renders register view</x:v>
+      </x:c>
+      <x:c r="D13" s="19" t="str"/>
+      <x:c r="E13" s="19" t="str">
+        <x:v>No run</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="34" customHeight="1">
+      <x:c r="A14" s="19" t="str">
+        <x:v>WEB-003</x:v>
+      </x:c>
+      <x:c r="B14" s="19" t="str">
+        <x:v>GET /home</x:v>
+      </x:c>
+      <x:c r="C14" s="19" t="str">
+        <x:v>4xx; anonymous access to protected home denied</x:v>
+      </x:c>
+      <x:c r="D14" s="19" t="str"/>
+      <x:c r="E14" s="19" t="str">
+        <x:v>No run</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="34" customHeight="1">
+      <x:c r="A15" s="19" t="str">
+        <x:v>WEB-004</x:v>
+      </x:c>
+      <x:c r="B15" s="19" t="str">
+        <x:v>GET /css/register.css</x:v>
+      </x:c>
+      <x:c r="C15" s="19" t="str">
+        <x:v>200 OK; stylesheet served</x:v>
+      </x:c>
+      <x:c r="D15" s="19" t="str"/>
+      <x:c r="E15" s="19" t="str">
+        <x:v>No run</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="34" customHeight="1">
+      <x:c r="A16" s="19" t="str">
+        <x:v>WEB-005</x:v>
+      </x:c>
+      <x:c r="B16" s="19" t="str">
+        <x:v>GET /js/register.js</x:v>
+      </x:c>
+      <x:c r="C16" s="19" t="str">
+        <x:v>200 OK; JavaScript served</x:v>
+      </x:c>
+      <x:c r="D16" s="19" t="str"/>
+      <x:c r="E16" s="19" t="str">
+        <x:v>No run</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="34" customHeight="1">
+      <x:c r="A17" s="19" t="str">
+        <x:v>WEB-006</x:v>
+      </x:c>
+      <x:c r="B17" s="19" t="str">
+        <x:v>GET /images/man.jpg</x:v>
+      </x:c>
+      <x:c r="C17" s="19" t="str">
+        <x:v>200 OK; image served</x:v>
+      </x:c>
+      <x:c r="D17" s="19" t="str"/>
+      <x:c r="E17" s="19" t="str">
+        <x:v>No run</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="34" customHeight="1">
+      <x:c r="A18" s="19" t="str">
+        <x:v>WEB-007</x:v>
+      </x:c>
+      <x:c r="B18" s="19" t="str">
+        <x:v>POST /api/auth/register</x:v>
+      </x:c>
+      <x:c r="C18" s="19" t="str">
+        <x:v>201 Created; public user fields; password omitted</x:v>
+      </x:c>
+      <x:c r="D18" s="19" t="str"/>
+      <x:c r="E18" s="19" t="str">
+        <x:v>No run</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="34" customHeight="1">
+      <x:c r="A19" s="19" t="str">
+        <x:v>WEB-008</x:v>
+      </x:c>
+      <x:c r="B19" s="19" t="str">
+        <x:v>POST login / GET auth / POST logout / GET auth</x:v>
+      </x:c>
+      <x:c r="C19" s="19" t="str">
+        <x:v>200 / 200 / 204 / 200; userId saved then cleared</x:v>
+      </x:c>
+      <x:c r="D19" s="19" t="str"/>
+      <x:c r="E19" s="19" t="str">
+        <x:v>No run</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" t="str">
+        <x:v>SEC-009</x:v>
+      </x:c>
+      <x:c r="B20" t="str">
+        <x:v>Malformed login JSON</x:v>
+      </x:c>
+      <x:c r="C20" t="str">
+        <x:v>400 Bad Request</x:v>
+      </x:c>
+      <x:c r="D20" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="E20" t="str">
+        <x:v>anonymousLogin_withMalformedJson_returns400</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
@@ -1289,7 +1558,7 @@
     </x:row>
     <x:row r="2" ht="21" customHeight="1">
       <x:c r="A2" s="8" t="str">
-        <x:v>42 documented test cases; latest full test run: 2026-09-30 17:09:30</x:v>
+        <x:v>50 documented cases: 42 passed, 8 planned; latest completed full run: 2026-09-30 17:09:30 (43/43)</x:v>
       </x:c>
       <x:c r="B2" s="8"/>
       <x:c r="C2" s="8"/>
@@ -3083,34 +3352,316 @@
       </x:c>
     </x:row>
     <x:row r="47" ht="21" customHeight="1">
-      <x:c r="A47" s="8"/>
-      <x:c r="B47" s="8"/>
-      <x:c r="C47" s="8"/>
-      <x:c r="D47" s="8"/>
-      <x:c r="E47" s="8"/>
-      <x:c r="F47" s="8"/>
-      <x:c r="G47" s="8"/>
-      <x:c r="H47" s="8"/>
-      <x:c r="I47" s="8"/>
-      <x:c r="J47" s="8"/>
-      <x:c r="K47" s="8"/>
-      <x:c r="L47" s="8"/>
-      <x:c r="M47" s="8"/>
+      <x:c r="A47" s="8" t="str">
+        <x:v>UC-WEB-01</x:v>
+      </x:c>
+      <x:c r="B47" s="8" t="str">
+        <x:v>TS005</x:v>
+      </x:c>
+      <x:c r="C47" s="8" t="str">
+        <x:v>WEB-001</x:v>
+      </x:c>
+      <x:c r="D47" s="8" t="str">
+        <x:v>Public page</x:v>
+      </x:c>
+      <x:c r="E47" s="8" t="str">
+        <x:v>GET /login</x:v>
+      </x:c>
+      <x:c r="F47" s="8" t="str">
+        <x:v>Anonymous GET request</x:v>
+      </x:c>
+      <x:c r="G47" s="8" t="str">
+        <x:v>Full Spring MVC, SecurityConfig and Thymeleaf</x:v>
+      </x:c>
+      <x:c r="H47" s="8" t="str">
+        <x:v>200 OK; renders login view</x:v>
+      </x:c>
+      <x:c r="I47" s="8" t="str"/>
+      <x:c r="J47" s="8" t="str">
+        <x:v>No run</x:v>
+      </x:c>
+      <x:c r="K47" s="8" t="str">
+        <x:v>SpringBootTest / MockMvc</x:v>
+      </x:c>
+      <x:c r="L47" s="8" t="str">
+        <x:v>WebFlowIntegrationTest.anonymousUser_canOpenLoginPage</x:v>
+      </x:c>
+      <x:c r="M47" s="8" t="str">
+        <x:v>Not executed</x:v>
+      </x:c>
     </x:row>
     <x:row r="48" ht="21" customHeight="1">
-      <x:c r="A48" s="8"/>
-      <x:c r="B48" s="8"/>
-      <x:c r="C48" s="8"/>
-      <x:c r="D48" s="8"/>
-      <x:c r="E48" s="8"/>
-      <x:c r="F48" s="8"/>
-      <x:c r="G48" s="8"/>
-      <x:c r="H48" s="8"/>
-      <x:c r="I48" s="8"/>
-      <x:c r="J48" s="8"/>
-      <x:c r="K48" s="8"/>
-      <x:c r="L48" s="8"/>
-      <x:c r="M48" s="8"/>
+      <x:c r="A48" s="8" t="str">
+        <x:v>UC-WEB-01</x:v>
+      </x:c>
+      <x:c r="B48" s="8" t="str">
+        <x:v>TS005</x:v>
+      </x:c>
+      <x:c r="C48" s="8" t="str">
+        <x:v>WEB-002</x:v>
+      </x:c>
+      <x:c r="D48" s="8" t="str">
+        <x:v>Public page</x:v>
+      </x:c>
+      <x:c r="E48" s="8" t="str">
+        <x:v>GET /register</x:v>
+      </x:c>
+      <x:c r="F48" s="8" t="str">
+        <x:v>Anonymous GET request</x:v>
+      </x:c>
+      <x:c r="G48" s="8" t="str">
+        <x:v>Full Spring MVC, SecurityConfig and Thymeleaf</x:v>
+      </x:c>
+      <x:c r="H48" s="8" t="str">
+        <x:v>200 OK; renders register view</x:v>
+      </x:c>
+      <x:c r="I48" s="8" t="str"/>
+      <x:c r="J48" s="8" t="str">
+        <x:v>No run</x:v>
+      </x:c>
+      <x:c r="K48" s="8" t="str">
+        <x:v>SpringBootTest / MockMvc</x:v>
+      </x:c>
+      <x:c r="L48" s="8" t="str">
+        <x:v>WebFlowIntegrationTest.anonymousUser_canOpenRegistrationPage</x:v>
+      </x:c>
+      <x:c r="M48" s="8" t="str">
+        <x:v>Not executed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" t="str">
+        <x:v>UC-WEB-01</x:v>
+      </x:c>
+      <x:c r="B49" t="str">
+        <x:v>TS005</x:v>
+      </x:c>
+      <x:c r="C49" t="str">
+        <x:v>WEB-003</x:v>
+      </x:c>
+      <x:c r="D49" t="str">
+        <x:v>Access control</x:v>
+      </x:c>
+      <x:c r="E49" t="str">
+        <x:v>GET /home</x:v>
+      </x:c>
+      <x:c r="F49" t="str">
+        <x:v>Anonymous GET request</x:v>
+      </x:c>
+      <x:c r="G49" t="str">
+        <x:v>Full SecurityFilterChain enabled</x:v>
+      </x:c>
+      <x:c r="H49" t="str">
+        <x:v>4xx; anonymous access to protected home denied</x:v>
+      </x:c>
+      <x:c r="I49" t="str"/>
+      <x:c r="J49" t="str">
+        <x:v>No run</x:v>
+      </x:c>
+      <x:c r="K49" t="str">
+        <x:v>SpringBootTest / MockMvc</x:v>
+      </x:c>
+      <x:c r="L49" t="str">
+        <x:v>WebFlowIntegrationTest.anonymousUser_cannotOpenProtectedHomePage</x:v>
+      </x:c>
+      <x:c r="M49" t="str">
+        <x:v>Not executed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" t="str">
+        <x:v>UC-WEB-01</x:v>
+      </x:c>
+      <x:c r="B50" t="str">
+        <x:v>TS005</x:v>
+      </x:c>
+      <x:c r="C50" t="str">
+        <x:v>WEB-004</x:v>
+      </x:c>
+      <x:c r="D50" t="str">
+        <x:v>Static resource</x:v>
+      </x:c>
+      <x:c r="E50" t="str">
+        <x:v>GET /css/register.css</x:v>
+      </x:c>
+      <x:c r="F50" t="str">
+        <x:v>Anonymous GET request</x:v>
+      </x:c>
+      <x:c r="G50" t="str">
+        <x:v>Resource exists; full Spring context</x:v>
+      </x:c>
+      <x:c r="H50" t="str">
+        <x:v>200 OK; stylesheet served</x:v>
+      </x:c>
+      <x:c r="I50" t="str"/>
+      <x:c r="J50" t="str">
+        <x:v>No run</x:v>
+      </x:c>
+      <x:c r="K50" t="str">
+        <x:v>SpringBootTest / MockMvc</x:v>
+      </x:c>
+      <x:c r="L50" t="str">
+        <x:v>WebFlowIntegrationTest.registrationStylesheet_isPubliclyAvailable</x:v>
+      </x:c>
+      <x:c r="M50" t="str">
+        <x:v>Not executed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51" t="str">
+        <x:v>UC-WEB-01</x:v>
+      </x:c>
+      <x:c r="B51" t="str">
+        <x:v>TS005</x:v>
+      </x:c>
+      <x:c r="C51" t="str">
+        <x:v>WEB-005</x:v>
+      </x:c>
+      <x:c r="D51" t="str">
+        <x:v>Static resource</x:v>
+      </x:c>
+      <x:c r="E51" t="str">
+        <x:v>GET /js/register.js</x:v>
+      </x:c>
+      <x:c r="F51" t="str">
+        <x:v>Anonymous GET request</x:v>
+      </x:c>
+      <x:c r="G51" t="str">
+        <x:v>Resource exists; full Spring context</x:v>
+      </x:c>
+      <x:c r="H51" t="str">
+        <x:v>200 OK; JavaScript served</x:v>
+      </x:c>
+      <x:c r="I51" t="str"/>
+      <x:c r="J51" t="str">
+        <x:v>No run</x:v>
+      </x:c>
+      <x:c r="K51" t="str">
+        <x:v>SpringBootTest / MockMvc</x:v>
+      </x:c>
+      <x:c r="L51" t="str">
+        <x:v>WebFlowIntegrationTest.registrationJavascript_isPubliclyAvailable</x:v>
+      </x:c>
+      <x:c r="M51" t="str">
+        <x:v>Not executed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52" t="str">
+        <x:v>UC-WEB-01</x:v>
+      </x:c>
+      <x:c r="B52" t="str">
+        <x:v>TS005</x:v>
+      </x:c>
+      <x:c r="C52" t="str">
+        <x:v>WEB-006</x:v>
+      </x:c>
+      <x:c r="D52" t="str">
+        <x:v>Static resource</x:v>
+      </x:c>
+      <x:c r="E52" t="str">
+        <x:v>GET /images/man.jpg</x:v>
+      </x:c>
+      <x:c r="F52" t="str">
+        <x:v>Anonymous GET request</x:v>
+      </x:c>
+      <x:c r="G52" t="str">
+        <x:v>Resource exists; full Spring context</x:v>
+      </x:c>
+      <x:c r="H52" t="str">
+        <x:v>200 OK; image served</x:v>
+      </x:c>
+      <x:c r="I52" t="str"/>
+      <x:c r="J52" t="str">
+        <x:v>No run</x:v>
+      </x:c>
+      <x:c r="K52" t="str">
+        <x:v>SpringBootTest / MockMvc</x:v>
+      </x:c>
+      <x:c r="L52" t="str">
+        <x:v>WebFlowIntegrationTest.homeImage_isPubliclyAvailable</x:v>
+      </x:c>
+      <x:c r="M52" t="str">
+        <x:v>Not executed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53">
+      <x:c r="A53" t="str">
+        <x:v>UC-WEB-01</x:v>
+      </x:c>
+      <x:c r="B53" t="str">
+        <x:v>TS005</x:v>
+      </x:c>
+      <x:c r="C53" t="str">
+        <x:v>WEB-007</x:v>
+      </x:c>
+      <x:c r="D53" t="str">
+        <x:v>Registration API</x:v>
+      </x:c>
+      <x:c r="E53" t="str">
+        <x:v>POST /api/auth/register</x:v>
+      </x:c>
+      <x:c r="F53" t="str">
+        <x:v>Valid registration JSON</x:v>
+      </x:c>
+      <x:c r="G53" t="str">
+        <x:v>Full Spring context; AuthService mocked</x:v>
+      </x:c>
+      <x:c r="H53" t="str">
+        <x:v>201 Created; public user fields; password omitted</x:v>
+      </x:c>
+      <x:c r="I53" t="str"/>
+      <x:c r="J53" t="str">
+        <x:v>No run</x:v>
+      </x:c>
+      <x:c r="K53" t="str">
+        <x:v>SpringBootTest / MockMvc</x:v>
+      </x:c>
+      <x:c r="L53" t="str">
+        <x:v>WebFlowIntegrationTest.registrationApi_withRealWebContext_returnsPublicUserData</x:v>
+      </x:c>
+      <x:c r="M53" t="str">
+        <x:v>Not executed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54">
+      <x:c r="A54" t="str">
+        <x:v>UC-WEB-01</x:v>
+      </x:c>
+      <x:c r="B54" t="str">
+        <x:v>TS005</x:v>
+      </x:c>
+      <x:c r="C54" t="str">
+        <x:v>WEB-008</x:v>
+      </x:c>
+      <x:c r="D54" t="str">
+        <x:v>Session flow</x:v>
+      </x:c>
+      <x:c r="E54" t="str">
+        <x:v>POST login / GET auth / POST logout / GET auth</x:v>
+      </x:c>
+      <x:c r="F54" t="str">
+        <x:v>Valid login JSON</x:v>
+      </x:c>
+      <x:c r="G54" t="str">
+        <x:v>Full Spring context; AuthService mocked; reuse session</x:v>
+      </x:c>
+      <x:c r="H54" t="str">
+        <x:v>200 / 200 / 204 / 200; userId saved then cleared</x:v>
+      </x:c>
+      <x:c r="I54" t="str"/>
+      <x:c r="J54" t="str">
+        <x:v>No run</x:v>
+      </x:c>
+      <x:c r="K54" t="str">
+        <x:v>SpringBootTest / MockMvc</x:v>
+      </x:c>
+      <x:c r="L54" t="str">
+        <x:v>WebFlowIntegrationTest.loginSessionAndLogout_workAcrossRequests</x:v>
+      </x:c>
+      <x:c r="M54" t="str">
+        <x:v>Not executed</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3211,23 +3762,23 @@
         <x:v>Registration: valid, invalid and duplicate email</x:v>
       </x:c>
       <x:c r="D5" s="15" t="n">
-        <x:f>COUNTIF('Test Case Design &amp; Test Results'!$B$5:$B$46,B5)</x:f>
+        <x:f>COUNTIF('Test Case Design &amp; Test Results'!$B$5:$B$54,B5)</x:f>
         <x:v>12</x:v>
       </x:c>
       <x:c r="E5" s="15" t="n">
-        <x:f>COUNTIFS('Test Case Design &amp; Test Results'!$B$5:$B$46,B5,'Test Case Design &amp; Test Results'!$J$5:$J$46,"Pass")</x:f>
+        <x:f>COUNTIFS('Test Case Design &amp; Test Results'!$B$5:$B$54,B5,'Test Case Design &amp; Test Results'!$J$5:$J$54,"Pass")</x:f>
         <x:v>12</x:v>
       </x:c>
       <x:c r="F5" s="15" t="n">
-        <x:f>COUNTIFS('Test Case Design &amp; Test Results'!$B$5:$B$46,B5,'Test Case Design &amp; Test Results'!$J$5:$J$46,"Fail")</x:f>
+        <x:f>COUNTIFS('Test Case Design &amp; Test Results'!$B$5:$B$54,B5,'Test Case Design &amp; Test Results'!$J$5:$J$54,"Fail")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G5" s="15" t="n">
-        <x:f>COUNTIFS('Test Case Design &amp; Test Results'!$B$5:$B$46,B5,'Test Case Design &amp; Test Results'!$J$5:$J$46,"No run")</x:f>
+        <x:f>COUNTIFS('Test Case Design &amp; Test Results'!$B$5:$B$54,B5,'Test Case Design &amp; Test Results'!$J$5:$J$54,"No run")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="H5" s="15" t="n">
-        <x:f>COUNTIFS('Test Case Design &amp; Test Results'!$B$5:$B$46,B5,'Test Case Design &amp; Test Results'!$J$5:$J$46,"Block")</x:f>
+        <x:f>COUNTIFS('Test Case Design &amp; Test Results'!$B$5:$B$54,B5,'Test Case Design &amp; Test Results'!$J$5:$J$54,"Block")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="I5" s="8" t="str">
@@ -3245,23 +3796,23 @@
         <x:v>Login: valid/invalid credentials and account status</x:v>
       </x:c>
       <x:c r="D6" s="15" t="n">
-        <x:f>COUNTIF('Test Case Design &amp; Test Results'!$B$5:$B$46,B6)</x:f>
+        <x:f>COUNTIF('Test Case Design &amp; Test Results'!$B$5:$B$54,B6)</x:f>
         <x:v>11</x:v>
       </x:c>
       <x:c r="E6" s="15" t="n">
-        <x:f>COUNTIFS('Test Case Design &amp; Test Results'!$B$5:$B$46,B6,'Test Case Design &amp; Test Results'!$J$5:$J$46,"Pass")</x:f>
+        <x:f>COUNTIFS('Test Case Design &amp; Test Results'!$B$5:$B$54,B6,'Test Case Design &amp; Test Results'!$J$5:$J$54,"Pass")</x:f>
         <x:v>11</x:v>
       </x:c>
       <x:c r="F6" s="15" t="n">
-        <x:f>COUNTIFS('Test Case Design &amp; Test Results'!$B$5:$B$46,B6,'Test Case Design &amp; Test Results'!$J$5:$J$46,"Fail")</x:f>
+        <x:f>COUNTIFS('Test Case Design &amp; Test Results'!$B$5:$B$54,B6,'Test Case Design &amp; Test Results'!$J$5:$J$54,"Fail")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G6" s="15" t="n">
-        <x:f>COUNTIFS('Test Case Design &amp; Test Results'!$B$5:$B$46,B6,'Test Case Design &amp; Test Results'!$J$5:$J$46,"No run")</x:f>
+        <x:f>COUNTIFS('Test Case Design &amp; Test Results'!$B$5:$B$54,B6,'Test Case Design &amp; Test Results'!$J$5:$J$54,"No run")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="H6" s="15" t="n">
-        <x:f>COUNTIFS('Test Case Design &amp; Test Results'!$B$5:$B$46,B6,'Test Case Design &amp; Test Results'!$J$5:$J$46,"Block")</x:f>
+        <x:f>COUNTIFS('Test Case Design &amp; Test Results'!$B$5:$B$54,B6,'Test Case Design &amp; Test Results'!$J$5:$J$54,"Block")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="I6" s="8" t="str">
@@ -3279,23 +3830,23 @@
         <x:v>Controller: HTTP responses, JSON and session</x:v>
       </x:c>
       <x:c r="D7" s="15" t="n">
-        <x:f>COUNTIF('Test Case Design &amp; Test Results'!$B$5:$B$46,B7)</x:f>
+        <x:f>COUNTIF('Test Case Design &amp; Test Results'!$B$5:$B$54,B7)</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="E7" s="15" t="n">
-        <x:f>COUNTIFS('Test Case Design &amp; Test Results'!$B$5:$B$46,B7,'Test Case Design &amp; Test Results'!$J$5:$J$46,"Pass")</x:f>
+        <x:f>COUNTIFS('Test Case Design &amp; Test Results'!$B$5:$B$54,B7,'Test Case Design &amp; Test Results'!$J$5:$J$54,"Pass")</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="F7" s="15" t="n">
-        <x:f>COUNTIFS('Test Case Design &amp; Test Results'!$B$5:$B$46,B7,'Test Case Design &amp; Test Results'!$J$5:$J$46,"Fail")</x:f>
+        <x:f>COUNTIFS('Test Case Design &amp; Test Results'!$B$5:$B$54,B7,'Test Case Design &amp; Test Results'!$J$5:$J$54,"Fail")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G7" s="15" t="n">
-        <x:f>COUNTIFS('Test Case Design &amp; Test Results'!$B$5:$B$46,B7,'Test Case Design &amp; Test Results'!$J$5:$J$46,"No run")</x:f>
+        <x:f>COUNTIFS('Test Case Design &amp; Test Results'!$B$5:$B$54,B7,'Test Case Design &amp; Test Results'!$J$5:$J$54,"No run")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="H7" s="15" t="n">
-        <x:f>COUNTIFS('Test Case Design &amp; Test Results'!$B$5:$B$46,B7,'Test Case Design &amp; Test Results'!$J$5:$J$46,"Block")</x:f>
+        <x:f>COUNTIFS('Test Case Design &amp; Test Results'!$B$5:$B$54,B7,'Test Case Design &amp; Test Results'!$J$5:$J$54,"Block")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="I7" s="8" t="str">
@@ -3313,23 +3864,23 @@
         <x:v>Authentication endpoints with Spring Security</x:v>
       </x:c>
       <x:c r="D8" s="15" t="n">
-        <x:f>COUNTIF('Test Case Design &amp; Test Results'!$B$5:$B$46,B8)</x:f>
+        <x:f>COUNTIF('Test Case Design &amp; Test Results'!$B$5:$B$54,B8)</x:f>
         <x:v>9</x:v>
       </x:c>
       <x:c r="E8" s="15" t="n">
-        <x:f>COUNTIFS('Test Case Design &amp; Test Results'!$B$5:$B$46,B8,'Test Case Design &amp; Test Results'!$J$5:$J$46,"Pass")</x:f>
+        <x:f>COUNTIFS('Test Case Design &amp; Test Results'!$B$5:$B$54,B8,'Test Case Design &amp; Test Results'!$J$5:$J$54,"Pass")</x:f>
         <x:v>9</x:v>
       </x:c>
       <x:c r="F8" s="15" t="n">
-        <x:f>COUNTIFS('Test Case Design &amp; Test Results'!$B$5:$B$46,B8,'Test Case Design &amp; Test Results'!$J$5:$J$46,"Fail")</x:f>
+        <x:f>COUNTIFS('Test Case Design &amp; Test Results'!$B$5:$B$54,B8,'Test Case Design &amp; Test Results'!$J$5:$J$54,"Fail")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G8" s="15" t="n">
-        <x:f>COUNTIFS('Test Case Design &amp; Test Results'!$B$5:$B$46,B8,'Test Case Design &amp; Test Results'!$J$5:$J$46,"No run")</x:f>
+        <x:f>COUNTIFS('Test Case Design &amp; Test Results'!$B$5:$B$54,B8,'Test Case Design &amp; Test Results'!$J$5:$J$54,"No run")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="H8" s="15" t="n">
-        <x:f>COUNTIFS('Test Case Design &amp; Test Results'!$B$5:$B$46,B8,'Test Case Design &amp; Test Results'!$J$5:$J$46,"Block")</x:f>
+        <x:f>COUNTIFS('Test Case Design &amp; Test Results'!$B$5:$B$54,B8,'Test Case Design &amp; Test Results'!$J$5:$J$54,"Block")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="I8" s="8" t="str">
@@ -3337,15 +3888,38 @@
       </x:c>
     </x:row>
     <x:row r="9" ht="21" customHeight="1">
-      <x:c r="A9" s="8"/>
-      <x:c r="B9" s="8"/>
-      <x:c r="C9" s="8"/>
-      <x:c r="D9" s="8"/>
-      <x:c r="E9" s="8"/>
-      <x:c r="F9" s="8"/>
-      <x:c r="G9" s="8"/>
-      <x:c r="H9" s="8"/>
-      <x:c r="I9" s="8"/>
+      <x:c r="A9" s="8" t="str">
+        <x:v>UC-WEB-01</x:v>
+      </x:c>
+      <x:c r="B9" s="8" t="str">
+        <x:v>TS005</x:v>
+      </x:c>
+      <x:c r="C9" s="8" t="str">
+        <x:v>Full-context web pages, static resources and authentication flow</x:v>
+      </x:c>
+      <x:c r="D9" s="8" t="n">
+        <x:f>COUNTIF('Test Case Design &amp; Test Results'!$B$5:$B$54,B9)</x:f>
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E9" s="8" t="n">
+        <x:f>COUNTIFS('Test Case Design &amp; Test Results'!$B$5:$B$54,B9,'Test Case Design &amp; Test Results'!$J$5:$J$54,"Pass")</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F9" s="8" t="n">
+        <x:f>COUNTIFS('Test Case Design &amp; Test Results'!$B$5:$B$54,B9,'Test Case Design &amp; Test Results'!$J$5:$J$54,"Fail")</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G9" s="8" t="n">
+        <x:f>COUNTIFS('Test Case Design &amp; Test Results'!$B$5:$B$54,B9,'Test Case Design &amp; Test Results'!$J$5:$J$54,"No run")</x:f>
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="H9" s="8" t="n">
+        <x:f>COUNTIFS('Test Case Design &amp; Test Results'!$B$5:$B$54,B9,'Test Case Design &amp; Test Results'!$J$5:$J$54,"Block")</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I9" s="8" t="str">
+        <x:v>WebFlowIntegrationTest (not run)</x:v>
+      </x:c>
     </x:row>
     <x:row r="10" ht="21" customHeight="1">
       <x:c r="A10" s="8" t="str">
@@ -5374,30 +5948,64 @@
       </x:c>
     </x:row>
     <x:row r="21" ht="21" customHeight="1">
-      <x:c r="A21" s="8"/>
-      <x:c r="B21" s="8"/>
-      <x:c r="C21" s="8"/>
-      <x:c r="D21" s="8"/>
-      <x:c r="E21" s="8"/>
-      <x:c r="F21" s="8"/>
+      <x:c r="A21" s="8" t="str">
+        <x:v>REQ-WEB-01</x:v>
+      </x:c>
+      <x:c r="B21" s="8" t="str">
+        <x:v>Public login/registration pages and static resources</x:v>
+      </x:c>
+      <x:c r="C21" s="8" t="str">
+        <x:v>TS005</x:v>
+      </x:c>
+      <x:c r="D21" s="8" t="str">
+        <x:v>WEB-001, WEB-002, WEB-004 to WEB-006</x:v>
+      </x:c>
+      <x:c r="E21" s="8" t="str">
+        <x:v>PageController / static handlers</x:v>
+      </x:c>
+      <x:c r="F21" s="8" t="str">
+        <x:v>Not run</x:v>
+      </x:c>
     </x:row>
     <x:row r="22" ht="21" customHeight="1">
       <x:c r="A22" s="8" t="str">
-        <x:v>Requirement and use-case IDs are internal identifiers for this test document.</x:v>
-      </x:c>
-      <x:c r="B22" s="8"/>
-      <x:c r="C22" s="8"/>
-      <x:c r="D22" s="8"/>
-      <x:c r="E22" s="8"/>
-      <x:c r="F22" s="8"/>
+        <x:v>REQ-WEB-02</x:v>
+      </x:c>
+      <x:c r="B22" s="8" t="str">
+        <x:v>Require authentication to access the home page</x:v>
+      </x:c>
+      <x:c r="C22" s="8" t="str">
+        <x:v>TS005</x:v>
+      </x:c>
+      <x:c r="D22" s="8" t="str">
+        <x:v>WEB-003</x:v>
+      </x:c>
+      <x:c r="E22" s="8" t="str">
+        <x:v>SecurityConfig / PageController</x:v>
+      </x:c>
+      <x:c r="F22" s="8" t="str">
+        <x:v>Not run</x:v>
+      </x:c>
     </x:row>
     <x:row r="23" ht="21" customHeight="1">
-      <x:c r="A23" s="8"/>
-      <x:c r="B23" s="8"/>
-      <x:c r="C23" s="8"/>
-      <x:c r="D23" s="8"/>
-      <x:c r="E23" s="8"/>
-      <x:c r="F23" s="8"/>
+      <x:c r="A23" s="8" t="str">
+        <x:v>REQ-WEB-03</x:v>
+      </x:c>
+      <x:c r="B23" s="8" t="str">
+        <x:v>Registration, session and logout flow in Spring context</x:v>
+      </x:c>
+      <x:c r="C23" s="8" t="str">
+        <x:v>TS005</x:v>
+      </x:c>
+      <x:c r="D23" s="8" t="str">
+        <x:v>WEB-007 to WEB-008</x:v>
+      </x:c>
+      <x:c r="E23" s="8" t="str">
+        <x:v>AuthController / SecurityConfig</x:v>
+      </x:c>
+      <x:c r="F23" s="8" t="str">
+        <x:v>Not run</x:v>
+      </x:c>
     </x:row>
     <x:row r="24" ht="21" customHeight="1">
       <x:c r="A24" s="8"/>
@@ -5408,7 +6016,9 @@
       <x:c r="F24" s="8"/>
     </x:row>
     <x:row r="25" ht="21" customHeight="1">
-      <x:c r="A25" s="8"/>
+      <x:c r="A25" s="8" t="str">
+        <x:v>Requirement and use-case IDs are internal identifiers for this test document.</x:v>
+      </x:c>
       <x:c r="B25" s="8"/>
       <x:c r="C25" s="8"/>
       <x:c r="D25" s="8"/>

</xml_diff>

<commit_message>
test: complete login service tests
</commit_message>
<xml_diff>
--- a/test/test-cases/CPFriendFinder_TestCases.xlsx
+++ b/test/test-cases/CPFriendFinder_TestCases.xlsx
@@ -2,18 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Scenario Summary" sheetId="1" r:id="R9477e82619e2452b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="2" r:id="R03c8530c28984468"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Case Design &amp; Test Results" sheetId="3" r:id="Ra2814b4e33444dca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS001" sheetId="4" r:id="R37f5eb6329ce4a1b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS002" sheetId="5" r:id="R0ea921762e59475e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS003" sheetId="6" r:id="R09b7223c5d884519"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS004" sheetId="7" r:id="Re30e6d6384f242f8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS005" sheetId="8" r:id="R7530fe118b7a426a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS006" sheetId="9" r:id="Raf70c989dd2240b4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defect Summary" sheetId="10" r:id="R924a22ed9d1f4084"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Summary Report" sheetId="11" r:id="R243745f21771443d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution Log" sheetId="12" r:id="R687d72e7c1194c16"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Scenario Summary" sheetId="1" r:id="Recba8945f3984f78"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="2" r:id="R324bdb53b70e415d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Case Design &amp; Test Results" sheetId="3" r:id="R23d6edf69e824880"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS001" sheetId="4" r:id="R1e452e1eea52491d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS002" sheetId="5" r:id="R40da338c72b54538"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS003" sheetId="6" r:id="Rd873c532642b4fd0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS004" sheetId="7" r:id="Rf552e79d877e4365"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS005" sheetId="8" r:id="R8918426d85ca40aa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS006" sheetId="9" r:id="R9a895c86502b4ab7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defect Summary" sheetId="10" r:id="Rca445e34d02c4373"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Summary Report" sheetId="11" r:id="R46990a198a3d4ca5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution Log" sheetId="12" r:id="R80f83ac4ec5b4384"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision Table" sheetId="13" r:id="R3164514da3774e95"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -369,7 +370,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="282">
+  <x:cellXfs count="287">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1120,6 +1121,19 @@
     <x:xf numFmtId="0" fontId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -1452,7 +1466,7 @@
       </x:c>
       <x:c r="E5" s="259" t="n">
         <x:f>COUNTIFS('Test Case Design &amp; Test Results'!$B$4:$B$80,B5,'Test Case Design &amp; Test Results'!$J$4:$J$80,"Pass")</x:f>
-        <x:v>0</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="F5" s="259" t="n">
         <x:f>COUNTIFS('Test Case Design &amp; Test Results'!$B$4:$B$80,B5,'Test Case Design &amp; Test Results'!$J$4:$J$80,"Fail")</x:f>
@@ -1460,7 +1474,7 @@
       </x:c>
       <x:c r="G5" s="259" t="n">
         <x:f>COUNTIFS('Test Case Design &amp; Test Results'!$B$4:$B$80,B5,'Test Case Design &amp; Test Results'!$J$4:$J$80,"Not Run")+COUNTIFS('Test Case Design &amp; Test Results'!$B$4:$B$80,B5,'Test Case Design &amp; Test Results'!$J$4:$J$80,"Waiting Frontend")</x:f>
-        <x:v>11</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H5" s="260" t="n">
         <x:f>COUNTIFS('Test Case Design &amp; Test Results'!$B$4:$B$80,B5,'Test Case Design &amp; Test Results'!$J$4:$J$80,"Blocked")</x:f>
@@ -4676,12 +4690,18 @@
       </x:c>
       <x:c r="B6" s="270" t="n">
         <x:f>COUNTIF('Test Case Design &amp; Test Results'!$J$4:$J$80,"Pass")+COUNTIF('Test Case Design &amp; Test Results'!$J$4:$J$80,"Fail")+COUNTIF('Test Case Design &amp; Test Results'!$J$4:$J$80,"Blocked")</x:f>
-        <x:v>13</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="C6" s="244"/>
-      <x:c r="D6" s="244"/>
-      <x:c r="E6" s="244"/>
-      <x:c r="F6" s="244"/>
+      <x:c r="D6" s="244" t="str">
+        <x:v>TS002</x:v>
+      </x:c>
+      <x:c r="E6" s="244" t="str">
+        <x:v>11/11 Pass</x:v>
+      </x:c>
+      <x:c r="F6" s="244" t="str">
+        <x:v>25.561 s</x:v>
+      </x:c>
       <x:c r="G6" s="244"/>
       <x:c r="H6" s="244"/>
       <x:c r="I6" s="244"/>
@@ -4696,7 +4716,7 @@
       </x:c>
       <x:c r="B7" s="270" t="n">
         <x:f>COUNTIF('Test Case Design &amp; Test Results'!$J$4:$J$80,"Pass")</x:f>
-        <x:v>13</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="C7" s="244"/>
       <x:c r="D7" s="244"/>
@@ -4736,7 +4756,7 @@
       </x:c>
       <x:c r="B9" s="271" t="n">
         <x:f>COUNTIF('Test Case Design &amp; Test Results'!$J$4:$J$80,"Not Run")+COUNTIF('Test Case Design &amp; Test Results'!$J$4:$J$80,"Waiting Frontend")</x:f>
-        <x:v>35</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="C9" s="244"/>
       <x:c r="D9" s="244"/>
@@ -6263,14 +6283,30 @@
       <x:c r="M5" s="244"/>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
-      <x:c r="A6" s="244"/>
-      <x:c r="B6" s="244"/>
-      <x:c r="C6" s="244"/>
-      <x:c r="D6" s="244"/>
-      <x:c r="E6" s="244"/>
-      <x:c r="F6" s="244"/>
-      <x:c r="G6" s="244"/>
-      <x:c r="H6" s="244"/>
+      <x:c r="A6" s="244" t="str">
+        <x:v>TS002</x:v>
+      </x:c>
+      <x:c r="B6" s="244" t="str">
+        <x:v>2026-10-01 16:29:59 +07:00</x:v>
+      </x:c>
+      <x:c r="C6" s="244" t="str">
+        <x:v>AuthServiceLoginTest</x:v>
+      </x:c>
+      <x:c r="D6" s="244" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E6" s="244" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="F6" s="244" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G6" s="244" t="str">
+        <x:v>0 / 0</x:v>
+      </x:c>
+      <x:c r="H6" s="244" t="str">
+        <x:v>BUILD SUCCESS</x:v>
+      </x:c>
       <x:c r="I6" s="244"/>
       <x:c r="J6" s="244"/>
       <x:c r="K6" s="244"/>
@@ -6307,7 +6343,7 @@
       <x:c r="L8" s="244"/>
       <x:c r="M8" s="244"/>
     </x:row>
-    <x:row r="9">
+    <x:row r="9" ht="15" hidden="0" customHeight="1">
       <x:c r="A9" s="244"/>
       <x:c r="B9" s="244"/>
       <x:c r="C9" s="244"/>
@@ -6322,7 +6358,7 @@
       <x:c r="L9" s="244"/>
       <x:c r="M9" s="244"/>
     </x:row>
-    <x:row r="10">
+    <x:row r="10" ht="15" hidden="0" customHeight="1">
       <x:c r="A10" s="244"/>
       <x:c r="B10" s="244"/>
       <x:c r="C10" s="244"/>
@@ -6376,6 +6412,1690 @@
       <x:c r="F13" s="244"/>
       <x:c r="G13" s="244"/>
       <x:c r="H13" s="244"/>
+      <x:c r="I13" s="244"/>
+      <x:c r="J13" s="244"/>
+      <x:c r="K13" s="244"/>
+      <x:c r="L13" s="244"/>
+      <x:c r="M13" s="244"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="244"/>
+      <x:c r="B14" s="244"/>
+      <x:c r="C14" s="244"/>
+      <x:c r="D14" s="244"/>
+      <x:c r="E14" s="244"/>
+      <x:c r="F14" s="244"/>
+      <x:c r="G14" s="244"/>
+      <x:c r="H14" s="244"/>
+      <x:c r="I14" s="244"/>
+      <x:c r="J14" s="244"/>
+      <x:c r="K14" s="244"/>
+      <x:c r="L14" s="244"/>
+      <x:c r="M14" s="244"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="244"/>
+      <x:c r="B15" s="244"/>
+      <x:c r="C15" s="244"/>
+      <x:c r="D15" s="244"/>
+      <x:c r="E15" s="244"/>
+      <x:c r="F15" s="244"/>
+      <x:c r="G15" s="244"/>
+      <x:c r="H15" s="244"/>
+      <x:c r="I15" s="244"/>
+      <x:c r="J15" s="244"/>
+      <x:c r="K15" s="244"/>
+      <x:c r="L15" s="244"/>
+      <x:c r="M15" s="244"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="244"/>
+      <x:c r="B16" s="244"/>
+      <x:c r="C16" s="244"/>
+      <x:c r="D16" s="244"/>
+      <x:c r="E16" s="244"/>
+      <x:c r="F16" s="244"/>
+      <x:c r="G16" s="244"/>
+      <x:c r="H16" s="244"/>
+      <x:c r="I16" s="244"/>
+      <x:c r="J16" s="244"/>
+      <x:c r="K16" s="244"/>
+      <x:c r="L16" s="244"/>
+      <x:c r="M16" s="244"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="244"/>
+      <x:c r="B17" s="244"/>
+      <x:c r="C17" s="244"/>
+      <x:c r="D17" s="244"/>
+      <x:c r="E17" s="244"/>
+      <x:c r="F17" s="244"/>
+      <x:c r="G17" s="244"/>
+      <x:c r="H17" s="244"/>
+      <x:c r="I17" s="244"/>
+      <x:c r="J17" s="244"/>
+      <x:c r="K17" s="244"/>
+      <x:c r="L17" s="244"/>
+      <x:c r="M17" s="244"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="244"/>
+      <x:c r="B18" s="244"/>
+      <x:c r="C18" s="244"/>
+      <x:c r="D18" s="244"/>
+      <x:c r="E18" s="244"/>
+      <x:c r="F18" s="244"/>
+      <x:c r="G18" s="244"/>
+      <x:c r="H18" s="244"/>
+      <x:c r="I18" s="244"/>
+      <x:c r="J18" s="244"/>
+      <x:c r="K18" s="244"/>
+      <x:c r="L18" s="244"/>
+      <x:c r="M18" s="244"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="244"/>
+      <x:c r="B19" s="244"/>
+      <x:c r="C19" s="244"/>
+      <x:c r="D19" s="244"/>
+      <x:c r="E19" s="244"/>
+      <x:c r="F19" s="244"/>
+      <x:c r="G19" s="244"/>
+      <x:c r="H19" s="244"/>
+      <x:c r="I19" s="244"/>
+      <x:c r="J19" s="244"/>
+      <x:c r="K19" s="244"/>
+      <x:c r="L19" s="244"/>
+      <x:c r="M19" s="244"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="244"/>
+      <x:c r="B20" s="244"/>
+      <x:c r="C20" s="244"/>
+      <x:c r="D20" s="244"/>
+      <x:c r="E20" s="244"/>
+      <x:c r="F20" s="244"/>
+      <x:c r="G20" s="244"/>
+      <x:c r="H20" s="244"/>
+      <x:c r="I20" s="244"/>
+      <x:c r="J20" s="244"/>
+      <x:c r="K20" s="244"/>
+      <x:c r="L20" s="244"/>
+      <x:c r="M20" s="244"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="244"/>
+      <x:c r="B21" s="244"/>
+      <x:c r="C21" s="244"/>
+      <x:c r="D21" s="244"/>
+      <x:c r="E21" s="244"/>
+      <x:c r="F21" s="244"/>
+      <x:c r="G21" s="244"/>
+      <x:c r="H21" s="244"/>
+      <x:c r="I21" s="244"/>
+      <x:c r="J21" s="244"/>
+      <x:c r="K21" s="244"/>
+      <x:c r="L21" s="244"/>
+      <x:c r="M21" s="244"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="244"/>
+      <x:c r="B22" s="244"/>
+      <x:c r="C22" s="244"/>
+      <x:c r="D22" s="244"/>
+      <x:c r="E22" s="244"/>
+      <x:c r="F22" s="244"/>
+      <x:c r="G22" s="244"/>
+      <x:c r="H22" s="244"/>
+      <x:c r="I22" s="244"/>
+      <x:c r="J22" s="244"/>
+      <x:c r="K22" s="244"/>
+      <x:c r="L22" s="244"/>
+      <x:c r="M22" s="244"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="244"/>
+      <x:c r="B23" s="244"/>
+      <x:c r="C23" s="244"/>
+      <x:c r="D23" s="244"/>
+      <x:c r="E23" s="244"/>
+      <x:c r="F23" s="244"/>
+      <x:c r="G23" s="244"/>
+      <x:c r="H23" s="244"/>
+      <x:c r="I23" s="244"/>
+      <x:c r="J23" s="244"/>
+      <x:c r="K23" s="244"/>
+      <x:c r="L23" s="244"/>
+      <x:c r="M23" s="244"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="244"/>
+      <x:c r="B24" s="244"/>
+      <x:c r="C24" s="244"/>
+      <x:c r="D24" s="244"/>
+      <x:c r="E24" s="244"/>
+      <x:c r="F24" s="244"/>
+      <x:c r="G24" s="244"/>
+      <x:c r="H24" s="244"/>
+      <x:c r="I24" s="244"/>
+      <x:c r="J24" s="244"/>
+      <x:c r="K24" s="244"/>
+      <x:c r="L24" s="244"/>
+      <x:c r="M24" s="244"/>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="244"/>
+      <x:c r="B25" s="244"/>
+      <x:c r="C25" s="244"/>
+      <x:c r="D25" s="244"/>
+      <x:c r="E25" s="244"/>
+      <x:c r="F25" s="244"/>
+      <x:c r="G25" s="244"/>
+      <x:c r="H25" s="244"/>
+      <x:c r="I25" s="244"/>
+      <x:c r="J25" s="244"/>
+      <x:c r="K25" s="244"/>
+      <x:c r="L25" s="244"/>
+      <x:c r="M25" s="244"/>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="244"/>
+      <x:c r="B26" s="244"/>
+      <x:c r="C26" s="244"/>
+      <x:c r="D26" s="244"/>
+      <x:c r="E26" s="244"/>
+      <x:c r="F26" s="244"/>
+      <x:c r="G26" s="244"/>
+      <x:c r="H26" s="244"/>
+      <x:c r="I26" s="244"/>
+      <x:c r="J26" s="244"/>
+      <x:c r="K26" s="244"/>
+      <x:c r="L26" s="244"/>
+      <x:c r="M26" s="244"/>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="244"/>
+      <x:c r="B27" s="244"/>
+      <x:c r="C27" s="244"/>
+      <x:c r="D27" s="244"/>
+      <x:c r="E27" s="244"/>
+      <x:c r="F27" s="244"/>
+      <x:c r="G27" s="244"/>
+      <x:c r="H27" s="244"/>
+      <x:c r="I27" s="244"/>
+      <x:c r="J27" s="244"/>
+      <x:c r="K27" s="244"/>
+      <x:c r="L27" s="244"/>
+      <x:c r="M27" s="244"/>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="244"/>
+      <x:c r="B28" s="244"/>
+      <x:c r="C28" s="244"/>
+      <x:c r="D28" s="244"/>
+      <x:c r="E28" s="244"/>
+      <x:c r="F28" s="244"/>
+      <x:c r="G28" s="244"/>
+      <x:c r="H28" s="244"/>
+      <x:c r="I28" s="244"/>
+      <x:c r="J28" s="244"/>
+      <x:c r="K28" s="244"/>
+      <x:c r="L28" s="244"/>
+      <x:c r="M28" s="244"/>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="244"/>
+      <x:c r="B29" s="244"/>
+      <x:c r="C29" s="244"/>
+      <x:c r="D29" s="244"/>
+      <x:c r="E29" s="244"/>
+      <x:c r="F29" s="244"/>
+      <x:c r="G29" s="244"/>
+      <x:c r="H29" s="244"/>
+      <x:c r="I29" s="244"/>
+      <x:c r="J29" s="244"/>
+      <x:c r="K29" s="244"/>
+      <x:c r="L29" s="244"/>
+      <x:c r="M29" s="244"/>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="244"/>
+      <x:c r="B30" s="244"/>
+      <x:c r="C30" s="244"/>
+      <x:c r="D30" s="244"/>
+      <x:c r="E30" s="244"/>
+      <x:c r="F30" s="244"/>
+      <x:c r="G30" s="244"/>
+      <x:c r="H30" s="244"/>
+      <x:c r="I30" s="244"/>
+      <x:c r="J30" s="244"/>
+      <x:c r="K30" s="244"/>
+      <x:c r="L30" s="244"/>
+      <x:c r="M30" s="244"/>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="244"/>
+      <x:c r="B31" s="244"/>
+      <x:c r="C31" s="244"/>
+      <x:c r="D31" s="244"/>
+      <x:c r="E31" s="244"/>
+      <x:c r="F31" s="244"/>
+      <x:c r="G31" s="244"/>
+      <x:c r="H31" s="244"/>
+      <x:c r="I31" s="244"/>
+      <x:c r="J31" s="244"/>
+      <x:c r="K31" s="244"/>
+      <x:c r="L31" s="244"/>
+      <x:c r="M31" s="244"/>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="244"/>
+      <x:c r="B32" s="244"/>
+      <x:c r="C32" s="244"/>
+      <x:c r="D32" s="244"/>
+      <x:c r="E32" s="244"/>
+      <x:c r="F32" s="244"/>
+      <x:c r="G32" s="244"/>
+      <x:c r="H32" s="244"/>
+      <x:c r="I32" s="244"/>
+      <x:c r="J32" s="244"/>
+      <x:c r="K32" s="244"/>
+      <x:c r="L32" s="244"/>
+      <x:c r="M32" s="244"/>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="244"/>
+      <x:c r="B33" s="244"/>
+      <x:c r="C33" s="244"/>
+      <x:c r="D33" s="244"/>
+      <x:c r="E33" s="244"/>
+      <x:c r="F33" s="244"/>
+      <x:c r="G33" s="244"/>
+      <x:c r="H33" s="244"/>
+      <x:c r="I33" s="244"/>
+      <x:c r="J33" s="244"/>
+      <x:c r="K33" s="244"/>
+      <x:c r="L33" s="244"/>
+      <x:c r="M33" s="244"/>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="244"/>
+      <x:c r="B34" s="244"/>
+      <x:c r="C34" s="244"/>
+      <x:c r="D34" s="244"/>
+      <x:c r="E34" s="244"/>
+      <x:c r="F34" s="244"/>
+      <x:c r="G34" s="244"/>
+      <x:c r="H34" s="244"/>
+      <x:c r="I34" s="244"/>
+      <x:c r="J34" s="244"/>
+      <x:c r="K34" s="244"/>
+      <x:c r="L34" s="244"/>
+      <x:c r="M34" s="244"/>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="244"/>
+      <x:c r="B35" s="244"/>
+      <x:c r="C35" s="244"/>
+      <x:c r="D35" s="244"/>
+      <x:c r="E35" s="244"/>
+      <x:c r="F35" s="244"/>
+      <x:c r="G35" s="244"/>
+      <x:c r="H35" s="244"/>
+      <x:c r="I35" s="244"/>
+      <x:c r="J35" s="244"/>
+      <x:c r="K35" s="244"/>
+      <x:c r="L35" s="244"/>
+      <x:c r="M35" s="244"/>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="244"/>
+      <x:c r="B36" s="244"/>
+      <x:c r="C36" s="244"/>
+      <x:c r="D36" s="244"/>
+      <x:c r="E36" s="244"/>
+      <x:c r="F36" s="244"/>
+      <x:c r="G36" s="244"/>
+      <x:c r="H36" s="244"/>
+      <x:c r="I36" s="244"/>
+      <x:c r="J36" s="244"/>
+      <x:c r="K36" s="244"/>
+      <x:c r="L36" s="244"/>
+      <x:c r="M36" s="244"/>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="244"/>
+      <x:c r="B37" s="244"/>
+      <x:c r="C37" s="244"/>
+      <x:c r="D37" s="244"/>
+      <x:c r="E37" s="244"/>
+      <x:c r="F37" s="244"/>
+      <x:c r="G37" s="244"/>
+      <x:c r="H37" s="244"/>
+      <x:c r="I37" s="244"/>
+      <x:c r="J37" s="244"/>
+      <x:c r="K37" s="244"/>
+      <x:c r="L37" s="244"/>
+      <x:c r="M37" s="244"/>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="244"/>
+      <x:c r="B38" s="244"/>
+      <x:c r="C38" s="244"/>
+      <x:c r="D38" s="244"/>
+      <x:c r="E38" s="244"/>
+      <x:c r="F38" s="244"/>
+      <x:c r="G38" s="244"/>
+      <x:c r="H38" s="244"/>
+      <x:c r="I38" s="244"/>
+      <x:c r="J38" s="244"/>
+      <x:c r="K38" s="244"/>
+      <x:c r="L38" s="244"/>
+      <x:c r="M38" s="244"/>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="244"/>
+      <x:c r="B39" s="244"/>
+      <x:c r="C39" s="244"/>
+      <x:c r="D39" s="244"/>
+      <x:c r="E39" s="244"/>
+      <x:c r="F39" s="244"/>
+      <x:c r="G39" s="244"/>
+      <x:c r="H39" s="244"/>
+      <x:c r="I39" s="244"/>
+      <x:c r="J39" s="244"/>
+      <x:c r="K39" s="244"/>
+      <x:c r="L39" s="244"/>
+      <x:c r="M39" s="244"/>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40" s="244"/>
+      <x:c r="B40" s="244"/>
+      <x:c r="C40" s="244"/>
+      <x:c r="D40" s="244"/>
+      <x:c r="E40" s="244"/>
+      <x:c r="F40" s="244"/>
+      <x:c r="G40" s="244"/>
+      <x:c r="H40" s="244"/>
+      <x:c r="I40" s="244"/>
+      <x:c r="J40" s="244"/>
+      <x:c r="K40" s="244"/>
+      <x:c r="L40" s="244"/>
+      <x:c r="M40" s="244"/>
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41" s="244"/>
+      <x:c r="B41" s="244"/>
+      <x:c r="C41" s="244"/>
+      <x:c r="D41" s="244"/>
+      <x:c r="E41" s="244"/>
+      <x:c r="F41" s="244"/>
+      <x:c r="G41" s="244"/>
+      <x:c r="H41" s="244"/>
+      <x:c r="I41" s="244"/>
+      <x:c r="J41" s="244"/>
+      <x:c r="K41" s="244"/>
+      <x:c r="L41" s="244"/>
+      <x:c r="M41" s="244"/>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" s="244"/>
+      <x:c r="B42" s="244"/>
+      <x:c r="C42" s="244"/>
+      <x:c r="D42" s="244"/>
+      <x:c r="E42" s="244"/>
+      <x:c r="F42" s="244"/>
+      <x:c r="G42" s="244"/>
+      <x:c r="H42" s="244"/>
+      <x:c r="I42" s="244"/>
+      <x:c r="J42" s="244"/>
+      <x:c r="K42" s="244"/>
+      <x:c r="L42" s="244"/>
+      <x:c r="M42" s="244"/>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" s="244"/>
+      <x:c r="B43" s="244"/>
+      <x:c r="C43" s="244"/>
+      <x:c r="D43" s="244"/>
+      <x:c r="E43" s="244"/>
+      <x:c r="F43" s="244"/>
+      <x:c r="G43" s="244"/>
+      <x:c r="H43" s="244"/>
+      <x:c r="I43" s="244"/>
+      <x:c r="J43" s="244"/>
+      <x:c r="K43" s="244"/>
+      <x:c r="L43" s="244"/>
+      <x:c r="M43" s="244"/>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" s="244"/>
+      <x:c r="B44" s="244"/>
+      <x:c r="C44" s="244"/>
+      <x:c r="D44" s="244"/>
+      <x:c r="E44" s="244"/>
+      <x:c r="F44" s="244"/>
+      <x:c r="G44" s="244"/>
+      <x:c r="H44" s="244"/>
+      <x:c r="I44" s="244"/>
+      <x:c r="J44" s="244"/>
+      <x:c r="K44" s="244"/>
+      <x:c r="L44" s="244"/>
+      <x:c r="M44" s="244"/>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45" s="244"/>
+      <x:c r="B45" s="244"/>
+      <x:c r="C45" s="244"/>
+      <x:c r="D45" s="244"/>
+      <x:c r="E45" s="244"/>
+      <x:c r="F45" s="244"/>
+      <x:c r="G45" s="244"/>
+      <x:c r="H45" s="244"/>
+      <x:c r="I45" s="244"/>
+      <x:c r="J45" s="244"/>
+      <x:c r="K45" s="244"/>
+      <x:c r="L45" s="244"/>
+      <x:c r="M45" s="244"/>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" s="244"/>
+      <x:c r="B46" s="244"/>
+      <x:c r="C46" s="244"/>
+      <x:c r="D46" s="244"/>
+      <x:c r="E46" s="244"/>
+      <x:c r="F46" s="244"/>
+      <x:c r="G46" s="244"/>
+      <x:c r="H46" s="244"/>
+      <x:c r="I46" s="244"/>
+      <x:c r="J46" s="244"/>
+      <x:c r="K46" s="244"/>
+      <x:c r="L46" s="244"/>
+      <x:c r="M46" s="244"/>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" s="244"/>
+      <x:c r="B47" s="244"/>
+      <x:c r="C47" s="244"/>
+      <x:c r="D47" s="244"/>
+      <x:c r="E47" s="244"/>
+      <x:c r="F47" s="244"/>
+      <x:c r="G47" s="244"/>
+      <x:c r="H47" s="244"/>
+      <x:c r="I47" s="244"/>
+      <x:c r="J47" s="244"/>
+      <x:c r="K47" s="244"/>
+      <x:c r="L47" s="244"/>
+      <x:c r="M47" s="244"/>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" s="244"/>
+      <x:c r="B48" s="244"/>
+      <x:c r="C48" s="244"/>
+      <x:c r="D48" s="244"/>
+      <x:c r="E48" s="244"/>
+      <x:c r="F48" s="244"/>
+      <x:c r="G48" s="244"/>
+      <x:c r="H48" s="244"/>
+      <x:c r="I48" s="244"/>
+      <x:c r="J48" s="244"/>
+      <x:c r="K48" s="244"/>
+      <x:c r="L48" s="244"/>
+      <x:c r="M48" s="244"/>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" s="244"/>
+      <x:c r="B49" s="244"/>
+      <x:c r="C49" s="244"/>
+      <x:c r="D49" s="244"/>
+      <x:c r="E49" s="244"/>
+      <x:c r="F49" s="244"/>
+      <x:c r="G49" s="244"/>
+      <x:c r="H49" s="244"/>
+      <x:c r="I49" s="244"/>
+      <x:c r="J49" s="244"/>
+      <x:c r="K49" s="244"/>
+      <x:c r="L49" s="244"/>
+      <x:c r="M49" s="244"/>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" s="244"/>
+      <x:c r="B50" s="244"/>
+      <x:c r="C50" s="244"/>
+      <x:c r="D50" s="244"/>
+      <x:c r="E50" s="244"/>
+      <x:c r="F50" s="244"/>
+      <x:c r="G50" s="244"/>
+      <x:c r="H50" s="244"/>
+      <x:c r="I50" s="244"/>
+      <x:c r="J50" s="244"/>
+      <x:c r="K50" s="244"/>
+      <x:c r="L50" s="244"/>
+      <x:c r="M50" s="244"/>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51" s="244"/>
+      <x:c r="B51" s="244"/>
+      <x:c r="C51" s="244"/>
+      <x:c r="D51" s="244"/>
+      <x:c r="E51" s="244"/>
+      <x:c r="F51" s="244"/>
+      <x:c r="G51" s="244"/>
+      <x:c r="H51" s="244"/>
+      <x:c r="I51" s="244"/>
+      <x:c r="J51" s="244"/>
+      <x:c r="K51" s="244"/>
+      <x:c r="L51" s="244"/>
+      <x:c r="M51" s="244"/>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52" s="244"/>
+      <x:c r="B52" s="244"/>
+      <x:c r="C52" s="244"/>
+      <x:c r="D52" s="244"/>
+      <x:c r="E52" s="244"/>
+      <x:c r="F52" s="244"/>
+      <x:c r="G52" s="244"/>
+      <x:c r="H52" s="244"/>
+      <x:c r="I52" s="244"/>
+      <x:c r="J52" s="244"/>
+      <x:c r="K52" s="244"/>
+      <x:c r="L52" s="244"/>
+      <x:c r="M52" s="244"/>
+    </x:row>
+    <x:row r="53">
+      <x:c r="A53" s="244"/>
+      <x:c r="B53" s="244"/>
+      <x:c r="C53" s="244"/>
+      <x:c r="D53" s="244"/>
+      <x:c r="E53" s="244"/>
+      <x:c r="F53" s="244"/>
+      <x:c r="G53" s="244"/>
+      <x:c r="H53" s="244"/>
+      <x:c r="I53" s="244"/>
+      <x:c r="J53" s="244"/>
+      <x:c r="K53" s="244"/>
+      <x:c r="L53" s="244"/>
+      <x:c r="M53" s="244"/>
+    </x:row>
+    <x:row r="54">
+      <x:c r="A54" s="244"/>
+      <x:c r="B54" s="244"/>
+      <x:c r="C54" s="244"/>
+      <x:c r="D54" s="244"/>
+      <x:c r="E54" s="244"/>
+      <x:c r="F54" s="244"/>
+      <x:c r="G54" s="244"/>
+      <x:c r="H54" s="244"/>
+      <x:c r="I54" s="244"/>
+      <x:c r="J54" s="244"/>
+      <x:c r="K54" s="244"/>
+      <x:c r="L54" s="244"/>
+      <x:c r="M54" s="244"/>
+    </x:row>
+    <x:row r="55">
+      <x:c r="A55" s="244"/>
+      <x:c r="B55" s="244"/>
+      <x:c r="C55" s="244"/>
+      <x:c r="D55" s="244"/>
+      <x:c r="E55" s="244"/>
+      <x:c r="F55" s="244"/>
+      <x:c r="G55" s="244"/>
+      <x:c r="H55" s="244"/>
+      <x:c r="I55" s="244"/>
+      <x:c r="J55" s="244"/>
+      <x:c r="K55" s="244"/>
+      <x:c r="L55" s="244"/>
+      <x:c r="M55" s="244"/>
+    </x:row>
+    <x:row r="56">
+      <x:c r="A56" s="244"/>
+      <x:c r="B56" s="244"/>
+      <x:c r="C56" s="244"/>
+      <x:c r="D56" s="244"/>
+      <x:c r="E56" s="244"/>
+      <x:c r="F56" s="244"/>
+      <x:c r="G56" s="244"/>
+      <x:c r="H56" s="244"/>
+      <x:c r="I56" s="244"/>
+      <x:c r="J56" s="244"/>
+      <x:c r="K56" s="244"/>
+      <x:c r="L56" s="244"/>
+      <x:c r="M56" s="244"/>
+    </x:row>
+    <x:row r="57">
+      <x:c r="A57" s="244"/>
+      <x:c r="B57" s="244"/>
+      <x:c r="C57" s="244"/>
+      <x:c r="D57" s="244"/>
+      <x:c r="E57" s="244"/>
+      <x:c r="F57" s="244"/>
+      <x:c r="G57" s="244"/>
+      <x:c r="H57" s="244"/>
+      <x:c r="I57" s="244"/>
+      <x:c r="J57" s="244"/>
+      <x:c r="K57" s="244"/>
+      <x:c r="L57" s="244"/>
+      <x:c r="M57" s="244"/>
+    </x:row>
+    <x:row r="58">
+      <x:c r="A58" s="244"/>
+      <x:c r="B58" s="244"/>
+      <x:c r="C58" s="244"/>
+      <x:c r="D58" s="244"/>
+      <x:c r="E58" s="244"/>
+      <x:c r="F58" s="244"/>
+      <x:c r="G58" s="244"/>
+      <x:c r="H58" s="244"/>
+      <x:c r="I58" s="244"/>
+      <x:c r="J58" s="244"/>
+      <x:c r="K58" s="244"/>
+      <x:c r="L58" s="244"/>
+      <x:c r="M58" s="244"/>
+    </x:row>
+    <x:row r="59">
+      <x:c r="A59" s="244"/>
+      <x:c r="B59" s="244"/>
+      <x:c r="C59" s="244"/>
+      <x:c r="D59" s="244"/>
+      <x:c r="E59" s="244"/>
+      <x:c r="F59" s="244"/>
+      <x:c r="G59" s="244"/>
+      <x:c r="H59" s="244"/>
+      <x:c r="I59" s="244"/>
+      <x:c r="J59" s="244"/>
+      <x:c r="K59" s="244"/>
+      <x:c r="L59" s="244"/>
+      <x:c r="M59" s="244"/>
+    </x:row>
+    <x:row r="60">
+      <x:c r="A60" s="244"/>
+      <x:c r="B60" s="244"/>
+      <x:c r="C60" s="244"/>
+      <x:c r="D60" s="244"/>
+      <x:c r="E60" s="244"/>
+      <x:c r="F60" s="244"/>
+      <x:c r="G60" s="244"/>
+      <x:c r="H60" s="244"/>
+      <x:c r="I60" s="244"/>
+      <x:c r="J60" s="244"/>
+      <x:c r="K60" s="244"/>
+      <x:c r="L60" s="244"/>
+      <x:c r="M60" s="244"/>
+    </x:row>
+    <x:row r="61">
+      <x:c r="A61" s="244"/>
+      <x:c r="B61" s="244"/>
+      <x:c r="C61" s="244"/>
+      <x:c r="D61" s="244"/>
+      <x:c r="E61" s="244"/>
+      <x:c r="F61" s="244"/>
+      <x:c r="G61" s="244"/>
+      <x:c r="H61" s="244"/>
+      <x:c r="I61" s="244"/>
+      <x:c r="J61" s="244"/>
+      <x:c r="K61" s="244"/>
+      <x:c r="L61" s="244"/>
+      <x:c r="M61" s="244"/>
+    </x:row>
+    <x:row r="62">
+      <x:c r="A62" s="244"/>
+      <x:c r="B62" s="244"/>
+      <x:c r="C62" s="244"/>
+      <x:c r="D62" s="244"/>
+      <x:c r="E62" s="244"/>
+      <x:c r="F62" s="244"/>
+      <x:c r="G62" s="244"/>
+      <x:c r="H62" s="244"/>
+      <x:c r="I62" s="244"/>
+      <x:c r="J62" s="244"/>
+      <x:c r="K62" s="244"/>
+      <x:c r="L62" s="244"/>
+      <x:c r="M62" s="244"/>
+    </x:row>
+    <x:row r="63">
+      <x:c r="A63" s="244"/>
+      <x:c r="B63" s="244"/>
+      <x:c r="C63" s="244"/>
+      <x:c r="D63" s="244"/>
+      <x:c r="E63" s="244"/>
+      <x:c r="F63" s="244"/>
+      <x:c r="G63" s="244"/>
+      <x:c r="H63" s="244"/>
+      <x:c r="I63" s="244"/>
+      <x:c r="J63" s="244"/>
+      <x:c r="K63" s="244"/>
+      <x:c r="L63" s="244"/>
+      <x:c r="M63" s="244"/>
+    </x:row>
+    <x:row r="64">
+      <x:c r="A64" s="244"/>
+      <x:c r="B64" s="244"/>
+      <x:c r="C64" s="244"/>
+      <x:c r="D64" s="244"/>
+      <x:c r="E64" s="244"/>
+      <x:c r="F64" s="244"/>
+      <x:c r="G64" s="244"/>
+      <x:c r="H64" s="244"/>
+      <x:c r="I64" s="244"/>
+      <x:c r="J64" s="244"/>
+      <x:c r="K64" s="244"/>
+      <x:c r="L64" s="244"/>
+      <x:c r="M64" s="244"/>
+    </x:row>
+    <x:row r="65">
+      <x:c r="A65" s="244"/>
+      <x:c r="B65" s="244"/>
+      <x:c r="C65" s="244"/>
+      <x:c r="D65" s="244"/>
+      <x:c r="E65" s="244"/>
+      <x:c r="F65" s="244"/>
+      <x:c r="G65" s="244"/>
+      <x:c r="H65" s="244"/>
+      <x:c r="I65" s="244"/>
+      <x:c r="J65" s="244"/>
+      <x:c r="K65" s="244"/>
+      <x:c r="L65" s="244"/>
+      <x:c r="M65" s="244"/>
+    </x:row>
+    <x:row r="66">
+      <x:c r="A66" s="244"/>
+      <x:c r="B66" s="244"/>
+      <x:c r="C66" s="244"/>
+      <x:c r="D66" s="244"/>
+      <x:c r="E66" s="244"/>
+      <x:c r="F66" s="244"/>
+      <x:c r="G66" s="244"/>
+      <x:c r="H66" s="244"/>
+      <x:c r="I66" s="244"/>
+      <x:c r="J66" s="244"/>
+      <x:c r="K66" s="244"/>
+      <x:c r="L66" s="244"/>
+      <x:c r="M66" s="244"/>
+    </x:row>
+    <x:row r="67">
+      <x:c r="A67" s="244"/>
+      <x:c r="B67" s="244"/>
+      <x:c r="C67" s="244"/>
+      <x:c r="D67" s="244"/>
+      <x:c r="E67" s="244"/>
+      <x:c r="F67" s="244"/>
+      <x:c r="G67" s="244"/>
+      <x:c r="H67" s="244"/>
+      <x:c r="I67" s="244"/>
+      <x:c r="J67" s="244"/>
+      <x:c r="K67" s="244"/>
+      <x:c r="L67" s="244"/>
+      <x:c r="M67" s="244"/>
+    </x:row>
+    <x:row r="68">
+      <x:c r="A68" s="244"/>
+      <x:c r="B68" s="244"/>
+      <x:c r="C68" s="244"/>
+      <x:c r="D68" s="244"/>
+      <x:c r="E68" s="244"/>
+      <x:c r="F68" s="244"/>
+      <x:c r="G68" s="244"/>
+      <x:c r="H68" s="244"/>
+      <x:c r="I68" s="244"/>
+      <x:c r="J68" s="244"/>
+      <x:c r="K68" s="244"/>
+      <x:c r="L68" s="244"/>
+      <x:c r="M68" s="244"/>
+    </x:row>
+    <x:row r="69">
+      <x:c r="A69" s="244"/>
+      <x:c r="B69" s="244"/>
+      <x:c r="C69" s="244"/>
+      <x:c r="D69" s="244"/>
+      <x:c r="E69" s="244"/>
+      <x:c r="F69" s="244"/>
+      <x:c r="G69" s="244"/>
+      <x:c r="H69" s="244"/>
+      <x:c r="I69" s="244"/>
+      <x:c r="J69" s="244"/>
+      <x:c r="K69" s="244"/>
+      <x:c r="L69" s="244"/>
+      <x:c r="M69" s="244"/>
+    </x:row>
+    <x:row r="70">
+      <x:c r="A70" s="244"/>
+      <x:c r="B70" s="244"/>
+      <x:c r="C70" s="244"/>
+      <x:c r="D70" s="244"/>
+      <x:c r="E70" s="244"/>
+      <x:c r="F70" s="244"/>
+      <x:c r="G70" s="244"/>
+      <x:c r="H70" s="244"/>
+      <x:c r="I70" s="244"/>
+      <x:c r="J70" s="244"/>
+      <x:c r="K70" s="244"/>
+      <x:c r="L70" s="244"/>
+      <x:c r="M70" s="244"/>
+    </x:row>
+    <x:row r="71">
+      <x:c r="A71" s="244"/>
+      <x:c r="B71" s="244"/>
+      <x:c r="C71" s="244"/>
+      <x:c r="D71" s="244"/>
+      <x:c r="E71" s="244"/>
+      <x:c r="F71" s="244"/>
+      <x:c r="G71" s="244"/>
+      <x:c r="H71" s="244"/>
+      <x:c r="I71" s="244"/>
+      <x:c r="J71" s="244"/>
+      <x:c r="K71" s="244"/>
+      <x:c r="L71" s="244"/>
+      <x:c r="M71" s="244"/>
+    </x:row>
+    <x:row r="72">
+      <x:c r="A72" s="244"/>
+      <x:c r="B72" s="244"/>
+      <x:c r="C72" s="244"/>
+      <x:c r="D72" s="244"/>
+      <x:c r="E72" s="244"/>
+      <x:c r="F72" s="244"/>
+      <x:c r="G72" s="244"/>
+      <x:c r="H72" s="244"/>
+      <x:c r="I72" s="244"/>
+      <x:c r="J72" s="244"/>
+      <x:c r="K72" s="244"/>
+      <x:c r="L72" s="244"/>
+      <x:c r="M72" s="244"/>
+    </x:row>
+    <x:row r="73">
+      <x:c r="A73" s="244"/>
+      <x:c r="B73" s="244"/>
+      <x:c r="C73" s="244"/>
+      <x:c r="D73" s="244"/>
+      <x:c r="E73" s="244"/>
+      <x:c r="F73" s="244"/>
+      <x:c r="G73" s="244"/>
+      <x:c r="H73" s="244"/>
+      <x:c r="I73" s="244"/>
+      <x:c r="J73" s="244"/>
+      <x:c r="K73" s="244"/>
+      <x:c r="L73" s="244"/>
+      <x:c r="M73" s="244"/>
+    </x:row>
+    <x:row r="74">
+      <x:c r="A74" s="244"/>
+      <x:c r="B74" s="244"/>
+      <x:c r="C74" s="244"/>
+      <x:c r="D74" s="244"/>
+      <x:c r="E74" s="244"/>
+      <x:c r="F74" s="244"/>
+      <x:c r="G74" s="244"/>
+      <x:c r="H74" s="244"/>
+      <x:c r="I74" s="244"/>
+      <x:c r="J74" s="244"/>
+      <x:c r="K74" s="244"/>
+      <x:c r="L74" s="244"/>
+      <x:c r="M74" s="244"/>
+    </x:row>
+    <x:row r="75">
+      <x:c r="A75" s="244"/>
+      <x:c r="B75" s="244"/>
+      <x:c r="C75" s="244"/>
+      <x:c r="D75" s="244"/>
+      <x:c r="E75" s="244"/>
+      <x:c r="F75" s="244"/>
+      <x:c r="G75" s="244"/>
+      <x:c r="H75" s="244"/>
+      <x:c r="I75" s="244"/>
+      <x:c r="J75" s="244"/>
+      <x:c r="K75" s="244"/>
+      <x:c r="L75" s="244"/>
+      <x:c r="M75" s="244"/>
+    </x:row>
+    <x:row r="76">
+      <x:c r="A76" s="244"/>
+      <x:c r="B76" s="244"/>
+      <x:c r="C76" s="244"/>
+      <x:c r="D76" s="244"/>
+      <x:c r="E76" s="244"/>
+      <x:c r="F76" s="244"/>
+      <x:c r="G76" s="244"/>
+      <x:c r="H76" s="244"/>
+      <x:c r="I76" s="244"/>
+      <x:c r="J76" s="244"/>
+      <x:c r="K76" s="244"/>
+      <x:c r="L76" s="244"/>
+      <x:c r="M76" s="244"/>
+    </x:row>
+    <x:row r="77">
+      <x:c r="A77" s="244"/>
+      <x:c r="B77" s="244"/>
+      <x:c r="C77" s="244"/>
+      <x:c r="D77" s="244"/>
+      <x:c r="E77" s="244"/>
+      <x:c r="F77" s="244"/>
+      <x:c r="G77" s="244"/>
+      <x:c r="H77" s="244"/>
+      <x:c r="I77" s="244"/>
+      <x:c r="J77" s="244"/>
+      <x:c r="K77" s="244"/>
+      <x:c r="L77" s="244"/>
+      <x:c r="M77" s="244"/>
+    </x:row>
+    <x:row r="78">
+      <x:c r="A78" s="244"/>
+      <x:c r="B78" s="244"/>
+      <x:c r="C78" s="244"/>
+      <x:c r="D78" s="244"/>
+      <x:c r="E78" s="244"/>
+      <x:c r="F78" s="244"/>
+      <x:c r="G78" s="244"/>
+      <x:c r="H78" s="244"/>
+      <x:c r="I78" s="244"/>
+      <x:c r="J78" s="244"/>
+      <x:c r="K78" s="244"/>
+      <x:c r="L78" s="244"/>
+      <x:c r="M78" s="244"/>
+    </x:row>
+    <x:row r="79">
+      <x:c r="A79" s="244"/>
+      <x:c r="B79" s="244"/>
+      <x:c r="C79" s="244"/>
+      <x:c r="D79" s="244"/>
+      <x:c r="E79" s="244"/>
+      <x:c r="F79" s="244"/>
+      <x:c r="G79" s="244"/>
+      <x:c r="H79" s="244"/>
+      <x:c r="I79" s="244"/>
+      <x:c r="J79" s="244"/>
+      <x:c r="K79" s="244"/>
+      <x:c r="L79" s="244"/>
+      <x:c r="M79" s="244"/>
+    </x:row>
+    <x:row r="80">
+      <x:c r="A80" s="244"/>
+      <x:c r="B80" s="244"/>
+      <x:c r="C80" s="244"/>
+      <x:c r="D80" s="244"/>
+      <x:c r="E80" s="244"/>
+      <x:c r="F80" s="244"/>
+      <x:c r="G80" s="244"/>
+      <x:c r="H80" s="244"/>
+      <x:c r="I80" s="244"/>
+      <x:c r="J80" s="244"/>
+      <x:c r="K80" s="244"/>
+      <x:c r="L80" s="244"/>
+      <x:c r="M80" s="244"/>
+    </x:row>
+    <x:row r="81">
+      <x:c r="A81" s="244"/>
+      <x:c r="B81" s="244"/>
+      <x:c r="C81" s="244"/>
+      <x:c r="D81" s="244"/>
+      <x:c r="E81" s="244"/>
+      <x:c r="F81" s="244"/>
+      <x:c r="G81" s="244"/>
+      <x:c r="H81" s="244"/>
+      <x:c r="I81" s="244"/>
+      <x:c r="J81" s="244"/>
+      <x:c r="K81" s="244"/>
+      <x:c r="L81" s="244"/>
+      <x:c r="M81" s="244"/>
+    </x:row>
+    <x:row r="82">
+      <x:c r="A82" s="244"/>
+      <x:c r="B82" s="244"/>
+      <x:c r="C82" s="244"/>
+      <x:c r="D82" s="244"/>
+      <x:c r="E82" s="244"/>
+      <x:c r="F82" s="244"/>
+      <x:c r="G82" s="244"/>
+      <x:c r="H82" s="244"/>
+      <x:c r="I82" s="244"/>
+      <x:c r="J82" s="244"/>
+      <x:c r="K82" s="244"/>
+      <x:c r="L82" s="244"/>
+      <x:c r="M82" s="244"/>
+    </x:row>
+    <x:row r="83">
+      <x:c r="A83" s="244"/>
+      <x:c r="B83" s="244"/>
+      <x:c r="C83" s="244"/>
+      <x:c r="D83" s="244"/>
+      <x:c r="E83" s="244"/>
+      <x:c r="F83" s="244"/>
+      <x:c r="G83" s="244"/>
+      <x:c r="H83" s="244"/>
+      <x:c r="I83" s="244"/>
+      <x:c r="J83" s="244"/>
+      <x:c r="K83" s="244"/>
+      <x:c r="L83" s="244"/>
+      <x:c r="M83" s="244"/>
+    </x:row>
+    <x:row r="84">
+      <x:c r="A84" s="244"/>
+      <x:c r="B84" s="244"/>
+      <x:c r="C84" s="244"/>
+      <x:c r="D84" s="244"/>
+      <x:c r="E84" s="244"/>
+      <x:c r="F84" s="244"/>
+      <x:c r="G84" s="244"/>
+      <x:c r="H84" s="244"/>
+      <x:c r="I84" s="244"/>
+      <x:c r="J84" s="244"/>
+      <x:c r="K84" s="244"/>
+      <x:c r="L84" s="244"/>
+      <x:c r="M84" s="244"/>
+    </x:row>
+    <x:row r="85">
+      <x:c r="A85" s="244"/>
+      <x:c r="B85" s="244"/>
+      <x:c r="C85" s="244"/>
+      <x:c r="D85" s="244"/>
+      <x:c r="E85" s="244"/>
+      <x:c r="F85" s="244"/>
+      <x:c r="G85" s="244"/>
+      <x:c r="H85" s="244"/>
+      <x:c r="I85" s="244"/>
+      <x:c r="J85" s="244"/>
+      <x:c r="K85" s="244"/>
+      <x:c r="L85" s="244"/>
+      <x:c r="M85" s="244"/>
+    </x:row>
+    <x:row r="86">
+      <x:c r="A86" s="244"/>
+      <x:c r="B86" s="244"/>
+      <x:c r="C86" s="244"/>
+      <x:c r="D86" s="244"/>
+      <x:c r="E86" s="244"/>
+      <x:c r="F86" s="244"/>
+      <x:c r="G86" s="244"/>
+      <x:c r="H86" s="244"/>
+      <x:c r="I86" s="244"/>
+      <x:c r="J86" s="244"/>
+      <x:c r="K86" s="244"/>
+      <x:c r="L86" s="244"/>
+      <x:c r="M86" s="244"/>
+    </x:row>
+    <x:row r="87">
+      <x:c r="A87" s="244"/>
+      <x:c r="B87" s="244"/>
+      <x:c r="C87" s="244"/>
+      <x:c r="D87" s="244"/>
+      <x:c r="E87" s="244"/>
+      <x:c r="F87" s="244"/>
+      <x:c r="G87" s="244"/>
+      <x:c r="H87" s="244"/>
+      <x:c r="I87" s="244"/>
+      <x:c r="J87" s="244"/>
+      <x:c r="K87" s="244"/>
+      <x:c r="L87" s="244"/>
+      <x:c r="M87" s="244"/>
+    </x:row>
+    <x:row r="88">
+      <x:c r="A88" s="244"/>
+      <x:c r="B88" s="244"/>
+      <x:c r="C88" s="244"/>
+      <x:c r="D88" s="244"/>
+      <x:c r="E88" s="244"/>
+      <x:c r="F88" s="244"/>
+      <x:c r="G88" s="244"/>
+      <x:c r="H88" s="244"/>
+      <x:c r="I88" s="244"/>
+      <x:c r="J88" s="244"/>
+      <x:c r="K88" s="244"/>
+      <x:c r="L88" s="244"/>
+      <x:c r="M88" s="244"/>
+    </x:row>
+    <x:row r="89">
+      <x:c r="A89" s="244"/>
+      <x:c r="B89" s="244"/>
+      <x:c r="C89" s="244"/>
+      <x:c r="D89" s="244"/>
+      <x:c r="E89" s="244"/>
+      <x:c r="F89" s="244"/>
+      <x:c r="G89" s="244"/>
+      <x:c r="H89" s="244"/>
+      <x:c r="I89" s="244"/>
+      <x:c r="J89" s="244"/>
+      <x:c r="K89" s="244"/>
+      <x:c r="L89" s="244"/>
+      <x:c r="M89" s="244"/>
+    </x:row>
+    <x:row r="90">
+      <x:c r="A90" s="244"/>
+      <x:c r="B90" s="244"/>
+      <x:c r="C90" s="244"/>
+      <x:c r="D90" s="244"/>
+      <x:c r="E90" s="244"/>
+      <x:c r="F90" s="244"/>
+      <x:c r="G90" s="244"/>
+      <x:c r="H90" s="244"/>
+      <x:c r="I90" s="244"/>
+      <x:c r="J90" s="244"/>
+      <x:c r="K90" s="244"/>
+      <x:c r="L90" s="244"/>
+      <x:c r="M90" s="244"/>
+    </x:row>
+    <x:row r="91">
+      <x:c r="A91" s="244"/>
+      <x:c r="B91" s="244"/>
+      <x:c r="C91" s="244"/>
+      <x:c r="D91" s="244"/>
+      <x:c r="E91" s="244"/>
+      <x:c r="F91" s="244"/>
+      <x:c r="G91" s="244"/>
+      <x:c r="H91" s="244"/>
+      <x:c r="I91" s="244"/>
+      <x:c r="J91" s="244"/>
+      <x:c r="K91" s="244"/>
+      <x:c r="L91" s="244"/>
+      <x:c r="M91" s="244"/>
+    </x:row>
+    <x:row r="92">
+      <x:c r="A92" s="244"/>
+      <x:c r="B92" s="244"/>
+      <x:c r="C92" s="244"/>
+      <x:c r="D92" s="244"/>
+      <x:c r="E92" s="244"/>
+      <x:c r="F92" s="244"/>
+      <x:c r="G92" s="244"/>
+      <x:c r="H92" s="244"/>
+      <x:c r="I92" s="244"/>
+      <x:c r="J92" s="244"/>
+      <x:c r="K92" s="244"/>
+      <x:c r="L92" s="244"/>
+      <x:c r="M92" s="244"/>
+    </x:row>
+    <x:row r="93">
+      <x:c r="A93" s="244"/>
+      <x:c r="B93" s="244"/>
+      <x:c r="C93" s="244"/>
+      <x:c r="D93" s="244"/>
+      <x:c r="E93" s="244"/>
+      <x:c r="F93" s="244"/>
+      <x:c r="G93" s="244"/>
+      <x:c r="H93" s="244"/>
+      <x:c r="I93" s="244"/>
+      <x:c r="J93" s="244"/>
+      <x:c r="K93" s="244"/>
+      <x:c r="L93" s="244"/>
+      <x:c r="M93" s="244"/>
+    </x:row>
+    <x:row r="94">
+      <x:c r="A94" s="244"/>
+      <x:c r="B94" s="244"/>
+      <x:c r="C94" s="244"/>
+      <x:c r="D94" s="244"/>
+      <x:c r="E94" s="244"/>
+      <x:c r="F94" s="244"/>
+      <x:c r="G94" s="244"/>
+      <x:c r="H94" s="244"/>
+      <x:c r="I94" s="244"/>
+      <x:c r="J94" s="244"/>
+      <x:c r="K94" s="244"/>
+      <x:c r="L94" s="244"/>
+      <x:c r="M94" s="244"/>
+    </x:row>
+    <x:row r="95">
+      <x:c r="A95" s="244"/>
+      <x:c r="B95" s="244"/>
+      <x:c r="C95" s="244"/>
+      <x:c r="D95" s="244"/>
+      <x:c r="E95" s="244"/>
+      <x:c r="F95" s="244"/>
+      <x:c r="G95" s="244"/>
+      <x:c r="H95" s="244"/>
+      <x:c r="I95" s="244"/>
+      <x:c r="J95" s="244"/>
+      <x:c r="K95" s="244"/>
+      <x:c r="L95" s="244"/>
+      <x:c r="M95" s="244"/>
+    </x:row>
+    <x:row r="96">
+      <x:c r="A96" s="244"/>
+      <x:c r="B96" s="244"/>
+      <x:c r="C96" s="244"/>
+      <x:c r="D96" s="244"/>
+      <x:c r="E96" s="244"/>
+      <x:c r="F96" s="244"/>
+      <x:c r="G96" s="244"/>
+      <x:c r="H96" s="244"/>
+      <x:c r="I96" s="244"/>
+      <x:c r="J96" s="244"/>
+      <x:c r="K96" s="244"/>
+      <x:c r="L96" s="244"/>
+      <x:c r="M96" s="244"/>
+    </x:row>
+    <x:row r="97">
+      <x:c r="A97" s="244"/>
+      <x:c r="B97" s="244"/>
+      <x:c r="C97" s="244"/>
+      <x:c r="D97" s="244"/>
+      <x:c r="E97" s="244"/>
+      <x:c r="F97" s="244"/>
+      <x:c r="G97" s="244"/>
+      <x:c r="H97" s="244"/>
+      <x:c r="I97" s="244"/>
+      <x:c r="J97" s="244"/>
+      <x:c r="K97" s="244"/>
+      <x:c r="L97" s="244"/>
+      <x:c r="M97" s="244"/>
+    </x:row>
+    <x:row r="98">
+      <x:c r="A98" s="244"/>
+      <x:c r="B98" s="244"/>
+      <x:c r="C98" s="244"/>
+      <x:c r="D98" s="244"/>
+      <x:c r="E98" s="244"/>
+      <x:c r="F98" s="244"/>
+      <x:c r="G98" s="244"/>
+      <x:c r="H98" s="244"/>
+      <x:c r="I98" s="244"/>
+      <x:c r="J98" s="244"/>
+      <x:c r="K98" s="244"/>
+      <x:c r="L98" s="244"/>
+      <x:c r="M98" s="244"/>
+    </x:row>
+    <x:row r="99">
+      <x:c r="A99" s="244"/>
+      <x:c r="B99" s="244"/>
+      <x:c r="C99" s="244"/>
+      <x:c r="D99" s="244"/>
+      <x:c r="E99" s="244"/>
+      <x:c r="F99" s="244"/>
+      <x:c r="G99" s="244"/>
+      <x:c r="H99" s="244"/>
+      <x:c r="I99" s="244"/>
+      <x:c r="J99" s="244"/>
+      <x:c r="K99" s="244"/>
+      <x:c r="L99" s="244"/>
+      <x:c r="M99" s="244"/>
+    </x:row>
+    <x:row r="100">
+      <x:c r="A100" s="244"/>
+      <x:c r="B100" s="244"/>
+      <x:c r="C100" s="244"/>
+      <x:c r="D100" s="244"/>
+      <x:c r="E100" s="244"/>
+      <x:c r="F100" s="244"/>
+      <x:c r="G100" s="244"/>
+      <x:c r="H100" s="244"/>
+      <x:c r="I100" s="244"/>
+      <x:c r="J100" s="244"/>
+      <x:c r="K100" s="244"/>
+      <x:c r="L100" s="244"/>
+      <x:c r="M100" s="244"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:H1"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="10" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="16" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="38" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="24" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="12" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="44" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="16.799999237060547" hidden="0" customHeight="1">
+      <x:c r="A1" s="243" t="str">
+        <x:v>TS002 Login - Decision Table</x:v>
+      </x:c>
+      <x:c r="B1" s="243"/>
+      <x:c r="C1" s="243"/>
+      <x:c r="D1" s="243"/>
+      <x:c r="E1" s="243"/>
+      <x:c r="F1" s="243"/>
+      <x:c r="G1" s="243"/>
+      <x:c r="H1" s="243"/>
+      <x:c r="I1" s="244"/>
+      <x:c r="J1" s="244"/>
+      <x:c r="K1" s="244"/>
+      <x:c r="L1" s="244"/>
+      <x:c r="M1" s="244"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="244"/>
+      <x:c r="B2" s="244"/>
+      <x:c r="C2" s="244"/>
+      <x:c r="D2" s="244"/>
+      <x:c r="E2" s="244"/>
+      <x:c r="F2" s="244"/>
+      <x:c r="G2" s="244"/>
+      <x:c r="H2" s="244"/>
+      <x:c r="I2" s="244"/>
+      <x:c r="J2" s="244"/>
+      <x:c r="K2" s="244"/>
+      <x:c r="L2" s="244"/>
+      <x:c r="M2" s="244"/>
+    </x:row>
+    <x:row r="3" ht="15" hidden="0" customHeight="1">
+      <x:c r="A3" s="245" t="str">
+        <x:v>Rule</x:v>
+      </x:c>
+      <x:c r="B3" s="246" t="str">
+        <x:v>Email exists</x:v>
+      </x:c>
+      <x:c r="C3" s="246" t="str">
+        <x:v>Account ACTIVE</x:v>
+      </x:c>
+      <x:c r="D3" s="246" t="str">
+        <x:v>Password correct</x:v>
+      </x:c>
+      <x:c r="E3" s="246" t="str">
+        <x:v>Expected action</x:v>
+      </x:c>
+      <x:c r="F3" s="246" t="str">
+        <x:v>Test Case ID</x:v>
+      </x:c>
+      <x:c r="G3" s="246" t="str">
+        <x:v>Result</x:v>
+      </x:c>
+      <x:c r="H3" s="247" t="str">
+        <x:v>JUnit Method</x:v>
+      </x:c>
+      <x:c r="I3" s="244"/>
+      <x:c r="J3" s="244"/>
+      <x:c r="K3" s="244"/>
+      <x:c r="L3" s="244"/>
+      <x:c r="M3" s="244"/>
+    </x:row>
+    <x:row r="4" ht="15" hidden="0" customHeight="1">
+      <x:c r="A4" s="251" t="str">
+        <x:v>R1</x:v>
+      </x:c>
+      <x:c r="B4" s="252" t="str">
+        <x:v>Y</x:v>
+      </x:c>
+      <x:c r="C4" s="252" t="str">
+        <x:v>Y</x:v>
+      </x:c>
+      <x:c r="D4" s="253" t="str">
+        <x:v>Y</x:v>
+      </x:c>
+      <x:c r="E4" s="254" t="str">
+        <x:v>Login success</x:v>
+      </x:c>
+      <x:c r="F4" s="251" t="str">
+        <x:v>LOGIN-001</x:v>
+      </x:c>
+      <x:c r="G4" s="253" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H4" s="254" t="str">
+        <x:v>login_validCredentials_returnsUser</x:v>
+      </x:c>
+      <x:c r="I4" s="244"/>
+      <x:c r="J4" s="244"/>
+      <x:c r="K4" s="244"/>
+      <x:c r="L4" s="244"/>
+      <x:c r="M4" s="244"/>
+    </x:row>
+    <x:row r="5" ht="15" hidden="0" customHeight="1">
+      <x:c r="A5" s="258" t="str">
+        <x:v>R2</x:v>
+      </x:c>
+      <x:c r="B5" s="286" t="str">
+        <x:v>N</x:v>
+      </x:c>
+      <x:c r="C5" s="286" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="D5" s="260" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="E5" s="261" t="str">
+        <x:v>Reject: Invalid email or password</x:v>
+      </x:c>
+      <x:c r="F5" s="258" t="str">
+        <x:v>LOGIN-007</x:v>
+      </x:c>
+      <x:c r="G5" s="260" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H5" s="261" t="str">
+        <x:v>login_unknownEmail_rejected</x:v>
+      </x:c>
+      <x:c r="I5" s="244"/>
+      <x:c r="J5" s="244"/>
+      <x:c r="K5" s="244"/>
+      <x:c r="L5" s="244"/>
+      <x:c r="M5" s="244"/>
+    </x:row>
+    <x:row r="6" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A6" s="258" t="str">
+        <x:v>R3</x:v>
+      </x:c>
+      <x:c r="B6" s="286" t="str">
+        <x:v>Y</x:v>
+      </x:c>
+      <x:c r="C6" s="286" t="str">
+        <x:v>N</x:v>
+      </x:c>
+      <x:c r="D6" s="260" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="E6" s="261" t="str">
+        <x:v>Reject: User account is not active</x:v>
+      </x:c>
+      <x:c r="F6" s="258" t="str">
+        <x:v>LOGIN-008 / LOGIN-011</x:v>
+      </x:c>
+      <x:c r="G6" s="260" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H6" s="261" t="str">
+        <x:v>login_blockedAccount_rejected / login_blockedAccount_doesNotCheckPassword</x:v>
+      </x:c>
+      <x:c r="I6" s="244"/>
+      <x:c r="J6" s="244"/>
+      <x:c r="K6" s="244"/>
+      <x:c r="L6" s="244"/>
+      <x:c r="M6" s="244"/>
+    </x:row>
+    <x:row r="7" ht="15" hidden="0" customHeight="1">
+      <x:c r="A7" s="265" t="str">
+        <x:v>R4</x:v>
+      </x:c>
+      <x:c r="B7" s="266" t="str">
+        <x:v>Y</x:v>
+      </x:c>
+      <x:c r="C7" s="266" t="str">
+        <x:v>Y</x:v>
+      </x:c>
+      <x:c r="D7" s="267" t="str">
+        <x:v>N</x:v>
+      </x:c>
+      <x:c r="E7" s="268" t="str">
+        <x:v>Reject: Invalid email or password</x:v>
+      </x:c>
+      <x:c r="F7" s="265" t="str">
+        <x:v>LOGIN-009</x:v>
+      </x:c>
+      <x:c r="G7" s="267" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H7" s="268" t="str">
+        <x:v>login_wrongPassword_rejected</x:v>
+      </x:c>
+      <x:c r="I7" s="244"/>
+      <x:c r="J7" s="244"/>
+      <x:c r="K7" s="244"/>
+      <x:c r="L7" s="244"/>
+      <x:c r="M7" s="244"/>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="244"/>
+      <x:c r="B8" s="244"/>
+      <x:c r="C8" s="244"/>
+      <x:c r="D8" s="244"/>
+      <x:c r="E8" s="244"/>
+      <x:c r="F8" s="244"/>
+      <x:c r="G8" s="244"/>
+      <x:c r="H8" s="244"/>
+      <x:c r="I8" s="244"/>
+      <x:c r="J8" s="244"/>
+      <x:c r="K8" s="244"/>
+      <x:c r="L8" s="244"/>
+      <x:c r="M8" s="244"/>
+    </x:row>
+    <x:row r="9" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A9" s="245" t="str">
+        <x:v>Validation cases</x:v>
+      </x:c>
+      <x:c r="B9" s="246" t="str">
+        <x:v>Request</x:v>
+      </x:c>
+      <x:c r="C9" s="246" t="str">
+        <x:v>Email</x:v>
+      </x:c>
+      <x:c r="D9" s="246" t="str">
+        <x:v>Password</x:v>
+      </x:c>
+      <x:c r="E9" s="246" t="str">
+        <x:v>Expected</x:v>
+      </x:c>
+      <x:c r="F9" s="246" t="str">
+        <x:v>Test Case ID</x:v>
+      </x:c>
+      <x:c r="G9" s="246" t="str">
+        <x:v>Result</x:v>
+      </x:c>
+      <x:c r="H9" s="247" t="str">
+        <x:v>Method</x:v>
+      </x:c>
+      <x:c r="I9" s="244"/>
+      <x:c r="J9" s="244"/>
+      <x:c r="K9" s="244"/>
+      <x:c r="L9" s="244"/>
+      <x:c r="M9" s="244"/>
+    </x:row>
+    <x:row r="10" ht="15" hidden="0" customHeight="1">
+      <x:c r="A10" s="251" t="str">
+        <x:v>V1</x:v>
+      </x:c>
+      <x:c r="B10" s="252" t="str">
+        <x:v>null</x:v>
+      </x:c>
+      <x:c r="C10" s="252" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="D10" s="253" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="E10" s="254" t="str">
+        <x:v>Reject: Login request is required</x:v>
+      </x:c>
+      <x:c r="F10" s="251" t="str">
+        <x:v>LOGIN-002</x:v>
+      </x:c>
+      <x:c r="G10" s="253" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H10" s="254" t="str">
+        <x:v>login_nullRequest_rejected</x:v>
+      </x:c>
+      <x:c r="I10" s="244"/>
+      <x:c r="J10" s="244"/>
+      <x:c r="K10" s="244"/>
+      <x:c r="L10" s="244"/>
+      <x:c r="M10" s="244"/>
+    </x:row>
+    <x:row r="11" ht="15" hidden="0" customHeight="1">
+      <x:c r="A11" s="258" t="str">
+        <x:v>V2</x:v>
+      </x:c>
+      <x:c r="B11" s="286" t="str">
+        <x:v>present</x:v>
+      </x:c>
+      <x:c r="C11" s="286" t="str">
+        <x:v>null/blank</x:v>
+      </x:c>
+      <x:c r="D11" s="260" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="E11" s="261" t="str">
+        <x:v>Reject: Email is required</x:v>
+      </x:c>
+      <x:c r="F11" s="258" t="str">
+        <x:v>LOGIN-003 / LOGIN-004</x:v>
+      </x:c>
+      <x:c r="G11" s="260" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H11" s="261" t="str">
+        <x:v>login_nullEmail_rejected / login_blankEmail_rejected</x:v>
+      </x:c>
+      <x:c r="I11" s="244"/>
+      <x:c r="J11" s="244"/>
+      <x:c r="K11" s="244"/>
+      <x:c r="L11" s="244"/>
+      <x:c r="M11" s="244"/>
+    </x:row>
+    <x:row r="12" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A12" s="258" t="str">
+        <x:v>V3</x:v>
+      </x:c>
+      <x:c r="B12" s="286" t="str">
+        <x:v>present</x:v>
+      </x:c>
+      <x:c r="C12" s="286" t="str">
+        <x:v>valid</x:v>
+      </x:c>
+      <x:c r="D12" s="260" t="str">
+        <x:v>null/blank</x:v>
+      </x:c>
+      <x:c r="E12" s="261" t="str">
+        <x:v>Reject: Password is required</x:v>
+      </x:c>
+      <x:c r="F12" s="258" t="str">
+        <x:v>LOGIN-005 / LOGIN-006</x:v>
+      </x:c>
+      <x:c r="G12" s="260" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H12" s="261" t="str">
+        <x:v>login_nullPassword_rejected / login_blankPassword_rejected</x:v>
+      </x:c>
+      <x:c r="I12" s="244"/>
+      <x:c r="J12" s="244"/>
+      <x:c r="K12" s="244"/>
+      <x:c r="L12" s="244"/>
+      <x:c r="M12" s="244"/>
+    </x:row>
+    <x:row r="13" ht="15" hidden="0" customHeight="1">
+      <x:c r="A13" s="265" t="str">
+        <x:v>V4</x:v>
+      </x:c>
+      <x:c r="B13" s="266" t="str">
+        <x:v>present</x:v>
+      </x:c>
+      <x:c r="C13" s="266" t="str">
+        <x:v>spaced uppercase</x:v>
+      </x:c>
+      <x:c r="D13" s="267" t="str">
+        <x:v>valid</x:v>
+      </x:c>
+      <x:c r="E13" s="268" t="str">
+        <x:v>Normalize email before lookup</x:v>
+      </x:c>
+      <x:c r="F13" s="265" t="str">
+        <x:v>LOGIN-010</x:v>
+      </x:c>
+      <x:c r="G13" s="267" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H13" s="268" t="str">
+        <x:v>login_spacedUppercaseEmail_normalized</x:v>
+      </x:c>
       <x:c r="I13" s="244"/>
       <x:c r="J13" s="244"/>
       <x:c r="K13" s="244"/>
@@ -7945,7 +9665,7 @@
         <x:v>AuthService.validateLogin</x:v>
       </x:c>
       <x:c r="F10" s="270" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Passed - unit</x:v>
       </x:c>
       <x:c r="G10" s="244"/>
       <x:c r="H10" s="244"/>
@@ -7972,7 +9692,7 @@
         <x:v>AuthService.login</x:v>
       </x:c>
       <x:c r="F11" s="270" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Passed - unit</x:v>
       </x:c>
       <x:c r="G11" s="244"/>
       <x:c r="H11" s="244"/>
@@ -7999,7 +9719,7 @@
         <x:v>AuthService.login</x:v>
       </x:c>
       <x:c r="F12" s="270" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Passed - unit</x:v>
       </x:c>
       <x:c r="G12" s="244"/>
       <x:c r="H12" s="244"/>
@@ -8026,7 +9746,7 @@
         <x:v>AuthService.login</x:v>
       </x:c>
       <x:c r="F13" s="270" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Passed - unit</x:v>
       </x:c>
       <x:c r="G13" s="244"/>
       <x:c r="H13" s="244"/>
@@ -10082,7 +11802,7 @@
         <x:v>2026-10-01 16:21:52 | 13/13 passed | BUILD SUCCESS</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="15" hidden="0" customHeight="1">
+    <x:row r="17" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A17" s="270" t="str">
         <x:v>UC-AUTH-02</x:v>
       </x:c>
@@ -10108,18 +11828,22 @@
         <x:v>เข้าสู่ระบบสำเร็จและคืน User</x:v>
       </x:c>
       <x:c r="I17" s="261" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>ผ่านตาม Expected Result</x:v>
       </x:c>
       <x:c r="J17" s="270" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K17" s="261" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
       </x:c>
-      <x:c r="L17" s="261" t="str"/>
-      <x:c r="M17" s="261" t="str"/>
-    </x:row>
-    <x:row r="18" ht="15" hidden="0" customHeight="1">
+      <x:c r="L17" s="261" t="str">
+        <x:v>AuthServiceLoginTest.login_validCredentials_returnsUser</x:v>
+      </x:c>
+      <x:c r="M17" s="261" t="str">
+        <x:v>2026-10-01 16:29:59 | 11/11 passed | BUILD SUCCESS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A18" s="270" t="str">
         <x:v>UC-AUTH-02</x:v>
       </x:c>
@@ -10145,18 +11869,22 @@
         <x:v>แจ้ง Login request is required</x:v>
       </x:c>
       <x:c r="I18" s="261" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>ผ่านตาม Expected Result</x:v>
       </x:c>
       <x:c r="J18" s="270" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K18" s="261" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
       </x:c>
-      <x:c r="L18" s="261" t="str"/>
-      <x:c r="M18" s="261" t="str"/>
-    </x:row>
-    <x:row r="19" ht="15" hidden="0" customHeight="1">
+      <x:c r="L18" s="261" t="str">
+        <x:v>AuthServiceLoginTest.login_nullRequest_rejected</x:v>
+      </x:c>
+      <x:c r="M18" s="261" t="str">
+        <x:v>2026-10-01 16:29:59 | 11/11 passed | BUILD SUCCESS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A19" s="270" t="str">
         <x:v>UC-AUTH-02</x:v>
       </x:c>
@@ -10182,18 +11910,22 @@
         <x:v>แจ้ง Email is required</x:v>
       </x:c>
       <x:c r="I19" s="261" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>ผ่านตาม Expected Result</x:v>
       </x:c>
       <x:c r="J19" s="270" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K19" s="261" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
       </x:c>
-      <x:c r="L19" s="261" t="str"/>
-      <x:c r="M19" s="261" t="str"/>
-    </x:row>
-    <x:row r="20" ht="15" hidden="0" customHeight="1">
+      <x:c r="L19" s="261" t="str">
+        <x:v>AuthServiceLoginTest.login_nullEmail_rejected</x:v>
+      </x:c>
+      <x:c r="M19" s="261" t="str">
+        <x:v>2026-10-01 16:29:59 | 11/11 passed | BUILD SUCCESS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A20" s="270" t="str">
         <x:v>UC-AUTH-02</x:v>
       </x:c>
@@ -10219,18 +11951,22 @@
         <x:v>แจ้ง Email is required</x:v>
       </x:c>
       <x:c r="I20" s="261" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>ผ่านตาม Expected Result</x:v>
       </x:c>
       <x:c r="J20" s="270" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K20" s="261" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
       </x:c>
-      <x:c r="L20" s="261" t="str"/>
-      <x:c r="M20" s="261" t="str"/>
-    </x:row>
-    <x:row r="21" ht="15" hidden="0" customHeight="1">
+      <x:c r="L20" s="261" t="str">
+        <x:v>AuthServiceLoginTest.login_blankEmail_rejected</x:v>
+      </x:c>
+      <x:c r="M20" s="261" t="str">
+        <x:v>2026-10-01 16:29:59 | 11/11 passed | BUILD SUCCESS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A21" s="270" t="str">
         <x:v>UC-AUTH-02</x:v>
       </x:c>
@@ -10256,18 +11992,22 @@
         <x:v>แจ้ง Password is required</x:v>
       </x:c>
       <x:c r="I21" s="261" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>ผ่านตาม Expected Result</x:v>
       </x:c>
       <x:c r="J21" s="270" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K21" s="261" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
       </x:c>
-      <x:c r="L21" s="261" t="str"/>
-      <x:c r="M21" s="261" t="str"/>
-    </x:row>
-    <x:row r="22" ht="15" hidden="0" customHeight="1">
+      <x:c r="L21" s="261" t="str">
+        <x:v>AuthServiceLoginTest.login_nullPassword_rejected</x:v>
+      </x:c>
+      <x:c r="M21" s="261" t="str">
+        <x:v>2026-10-01 16:29:59 | 11/11 passed | BUILD SUCCESS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A22" s="270" t="str">
         <x:v>UC-AUTH-02</x:v>
       </x:c>
@@ -10293,18 +12033,22 @@
         <x:v>แจ้ง Password is required</x:v>
       </x:c>
       <x:c r="I22" s="261" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>ผ่านตาม Expected Result</x:v>
       </x:c>
       <x:c r="J22" s="270" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K22" s="261" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
       </x:c>
-      <x:c r="L22" s="261" t="str"/>
-      <x:c r="M22" s="261" t="str"/>
-    </x:row>
-    <x:row r="23" ht="15" hidden="0" customHeight="1">
+      <x:c r="L22" s="261" t="str">
+        <x:v>AuthServiceLoginTest.login_blankPassword_rejected</x:v>
+      </x:c>
+      <x:c r="M22" s="261" t="str">
+        <x:v>2026-10-01 16:29:59 | 11/11 passed | BUILD SUCCESS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A23" s="270" t="str">
         <x:v>UC-AUTH-02</x:v>
       </x:c>
@@ -10330,18 +12074,22 @@
         <x:v>แจ้ง Invalid email or password</x:v>
       </x:c>
       <x:c r="I23" s="261" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>ผ่านตาม Expected Result</x:v>
       </x:c>
       <x:c r="J23" s="270" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K23" s="261" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
       </x:c>
-      <x:c r="L23" s="261" t="str"/>
-      <x:c r="M23" s="261" t="str"/>
-    </x:row>
-    <x:row r="24" ht="15" hidden="0" customHeight="1">
+      <x:c r="L23" s="261" t="str">
+        <x:v>AuthServiceLoginTest.login_unknownEmail_rejected</x:v>
+      </x:c>
+      <x:c r="M23" s="261" t="str">
+        <x:v>2026-10-01 16:29:59 | 11/11 passed | BUILD SUCCESS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A24" s="270" t="str">
         <x:v>UC-AUTH-02</x:v>
       </x:c>
@@ -10367,18 +12115,22 @@
         <x:v>แจ้ง User account is not active</x:v>
       </x:c>
       <x:c r="I24" s="261" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>ผ่านตาม Expected Result</x:v>
       </x:c>
       <x:c r="J24" s="270" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K24" s="261" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
       </x:c>
-      <x:c r="L24" s="261" t="str"/>
-      <x:c r="M24" s="261" t="str"/>
-    </x:row>
-    <x:row r="25" ht="15" hidden="0" customHeight="1">
+      <x:c r="L24" s="261" t="str">
+        <x:v>AuthServiceLoginTest.login_blockedAccount_rejected</x:v>
+      </x:c>
+      <x:c r="M24" s="261" t="str">
+        <x:v>2026-10-01 16:29:59 | 11/11 passed | BUILD SUCCESS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A25" s="270" t="str">
         <x:v>UC-AUTH-02</x:v>
       </x:c>
@@ -10404,18 +12156,22 @@
         <x:v>แจ้ง Invalid email or password</x:v>
       </x:c>
       <x:c r="I25" s="261" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>ผ่านตาม Expected Result</x:v>
       </x:c>
       <x:c r="J25" s="270" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K25" s="261" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
       </x:c>
-      <x:c r="L25" s="261" t="str"/>
-      <x:c r="M25" s="261" t="str"/>
-    </x:row>
-    <x:row r="26" ht="15" hidden="0" customHeight="1">
+      <x:c r="L25" s="261" t="str">
+        <x:v>AuthServiceLoginTest.login_wrongPassword_rejected</x:v>
+      </x:c>
+      <x:c r="M25" s="261" t="str">
+        <x:v>2026-10-01 16:29:59 | 11/11 passed | BUILD SUCCESS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A26" s="270" t="str">
         <x:v>UC-AUTH-02</x:v>
       </x:c>
@@ -10441,18 +12197,22 @@
         <x:v>trim + lowercase ก่อนค้นหา</x:v>
       </x:c>
       <x:c r="I26" s="261" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>ผ่านตาม Expected Result</x:v>
       </x:c>
       <x:c r="J26" s="270" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K26" s="261" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
       </x:c>
-      <x:c r="L26" s="261" t="str"/>
-      <x:c r="M26" s="261" t="str"/>
-    </x:row>
-    <x:row r="27" ht="15" hidden="0" customHeight="1">
+      <x:c r="L26" s="261" t="str">
+        <x:v>AuthServiceLoginTest.login_spacedUppercaseEmail_normalized</x:v>
+      </x:c>
+      <x:c r="M26" s="261" t="str">
+        <x:v>2026-10-01 16:29:59 | 11/11 passed | BUILD SUCCESS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A27" s="270" t="str">
         <x:v>UC-AUTH-02</x:v>
       </x:c>
@@ -10478,16 +12238,20 @@
         <x:v>ปฏิเสธก่อนเรียก passwordEncoder.matches</x:v>
       </x:c>
       <x:c r="I27" s="261" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>ผ่านตาม Expected Result</x:v>
       </x:c>
       <x:c r="J27" s="270" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K27" s="261" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
       </x:c>
-      <x:c r="L27" s="261" t="str"/>
-      <x:c r="M27" s="261" t="str"/>
+      <x:c r="L27" s="261" t="str">
+        <x:v>AuthServiceLoginTest.login_blockedAccount_doesNotCheckPassword</x:v>
+      </x:c>
+      <x:c r="M27" s="261" t="str">
+        <x:v>2026-10-01 16:29:59 | 11/11 passed | BUILD SUCCESS</x:v>
+      </x:c>
     </x:row>
     <x:row r="28" ht="15" hidden="0" customHeight="1">
       <x:c r="A28" s="270" t="str">
@@ -11514,7 +13278,7 @@
       <x:c r="L60" s="244"/>
       <x:c r="M60" s="244"/>
     </x:row>
-    <x:row r="61">
+    <x:row r="61" ht="15" hidden="0" customHeight="1">
       <x:c r="A61" s="244"/>
       <x:c r="B61" s="244"/>
       <x:c r="C61" s="244"/>
@@ -11529,7 +13293,7 @@
       <x:c r="L61" s="244"/>
       <x:c r="M61" s="244"/>
     </x:row>
-    <x:row r="62">
+    <x:row r="62" ht="15" hidden="0" customHeight="1">
       <x:c r="A62" s="244"/>
       <x:c r="B62" s="244"/>
       <x:c r="C62" s="244"/>
@@ -11544,7 +13308,7 @@
       <x:c r="L62" s="244"/>
       <x:c r="M62" s="244"/>
     </x:row>
-    <x:row r="63">
+    <x:row r="63" ht="15" hidden="0" customHeight="1">
       <x:c r="A63" s="244"/>
       <x:c r="B63" s="244"/>
       <x:c r="C63" s="244"/>
@@ -11559,7 +13323,7 @@
       <x:c r="L63" s="244"/>
       <x:c r="M63" s="244"/>
     </x:row>
-    <x:row r="64">
+    <x:row r="64" ht="15" hidden="0" customHeight="1">
       <x:c r="A64" s="244"/>
       <x:c r="B64" s="244"/>
       <x:c r="C64" s="244"/>
@@ -11574,7 +13338,7 @@
       <x:c r="L64" s="244"/>
       <x:c r="M64" s="244"/>
     </x:row>
-    <x:row r="65">
+    <x:row r="65" ht="15" hidden="0" customHeight="1">
       <x:c r="A65" s="244"/>
       <x:c r="B65" s="244"/>
       <x:c r="C65" s="244"/>
@@ -11589,7 +13353,7 @@
       <x:c r="L65" s="244"/>
       <x:c r="M65" s="244"/>
     </x:row>
-    <x:row r="66">
+    <x:row r="66" ht="15" hidden="0" customHeight="1">
       <x:c r="A66" s="244"/>
       <x:c r="B66" s="244"/>
       <x:c r="C66" s="244"/>
@@ -11604,7 +13368,7 @@
       <x:c r="L66" s="244"/>
       <x:c r="M66" s="244"/>
     </x:row>
-    <x:row r="67">
+    <x:row r="67" ht="15" hidden="0" customHeight="1">
       <x:c r="A67" s="244"/>
       <x:c r="B67" s="244"/>
       <x:c r="C67" s="244"/>
@@ -11619,7 +13383,7 @@
       <x:c r="L67" s="244"/>
       <x:c r="M67" s="244"/>
     </x:row>
-    <x:row r="68">
+    <x:row r="68" ht="15" hidden="0" customHeight="1">
       <x:c r="A68" s="244"/>
       <x:c r="B68" s="244"/>
       <x:c r="C68" s="244"/>
@@ -11634,7 +13398,7 @@
       <x:c r="L68" s="244"/>
       <x:c r="M68" s="244"/>
     </x:row>
-    <x:row r="69">
+    <x:row r="69" ht="15" hidden="0" customHeight="1">
       <x:c r="A69" s="244"/>
       <x:c r="B69" s="244"/>
       <x:c r="C69" s="244"/>
@@ -11649,7 +13413,7 @@
       <x:c r="L69" s="244"/>
       <x:c r="M69" s="244"/>
     </x:row>
-    <x:row r="70">
+    <x:row r="70" ht="15" hidden="0" customHeight="1">
       <x:c r="A70" s="244"/>
       <x:c r="B70" s="244"/>
       <x:c r="C70" s="244"/>
@@ -13856,7 +15620,7 @@
       <x:c r="L1" s="244"/>
       <x:c r="M1" s="244"/>
     </x:row>
-    <x:row r="2">
+    <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="244"/>
       <x:c r="B2" s="244"/>
       <x:c r="C2" s="244"/>
@@ -14023,7 +15787,7 @@
       <x:c r="L10" s="244"/>
       <x:c r="M10" s="244"/>
     </x:row>
-    <x:row r="11">
+    <x:row r="11" ht="15" hidden="0" customHeight="1">
       <x:c r="A11" s="244"/>
       <x:c r="B11" s="244"/>
       <x:c r="C11" s="244"/>
@@ -14077,7 +15841,7 @@
         <x:v>เข้าสู่ระบบสำเร็จและคืน User</x:v>
       </x:c>
       <x:c r="E13" s="269" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="F13" s="244"/>
       <x:c r="G13" s="244"/>
@@ -14102,7 +15866,7 @@
         <x:v>แจ้ง Login request is required</x:v>
       </x:c>
       <x:c r="E14" s="270" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="F14" s="244"/>
       <x:c r="G14" s="244"/>
@@ -14127,7 +15891,7 @@
         <x:v>แจ้ง Email is required</x:v>
       </x:c>
       <x:c r="E15" s="270" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="F15" s="244"/>
       <x:c r="G15" s="244"/>
@@ -14152,7 +15916,7 @@
         <x:v>แจ้ง Email is required</x:v>
       </x:c>
       <x:c r="E16" s="270" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="F16" s="244"/>
       <x:c r="G16" s="244"/>
@@ -14177,7 +15941,7 @@
         <x:v>แจ้ง Password is required</x:v>
       </x:c>
       <x:c r="E17" s="270" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="F17" s="244"/>
       <x:c r="G17" s="244"/>
@@ -14202,7 +15966,7 @@
         <x:v>แจ้ง Password is required</x:v>
       </x:c>
       <x:c r="E18" s="270" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="F18" s="244"/>
       <x:c r="G18" s="244"/>
@@ -14227,7 +15991,7 @@
         <x:v>แจ้ง Invalid email or password</x:v>
       </x:c>
       <x:c r="E19" s="270" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="F19" s="244"/>
       <x:c r="G19" s="244"/>
@@ -14252,7 +16016,7 @@
         <x:v>แจ้ง User account is not active</x:v>
       </x:c>
       <x:c r="E20" s="270" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="F20" s="244"/>
       <x:c r="G20" s="244"/>
@@ -14277,7 +16041,7 @@
         <x:v>แจ้ง Invalid email or password</x:v>
       </x:c>
       <x:c r="E21" s="270" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="F21" s="244"/>
       <x:c r="G21" s="244"/>
@@ -14302,7 +16066,7 @@
         <x:v>trim + lowercase ก่อนค้นหา</x:v>
       </x:c>
       <x:c r="E22" s="270" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="F22" s="244"/>
       <x:c r="G22" s="244"/>
@@ -14327,7 +16091,7 @@
         <x:v>ปฏิเสธก่อนเรียก passwordEncoder.matches</x:v>
       </x:c>
       <x:c r="E23" s="271" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="F23" s="244"/>
       <x:c r="G23" s="244"/>
@@ -14338,7 +16102,7 @@
       <x:c r="L23" s="244"/>
       <x:c r="M23" s="244"/>
     </x:row>
-    <x:row r="24">
+    <x:row r="24" ht="15" hidden="0" customHeight="1">
       <x:c r="A24" s="244"/>
       <x:c r="B24" s="244"/>
       <x:c r="C24" s="244"/>
@@ -14353,7 +16117,7 @@
       <x:c r="L24" s="244"/>
       <x:c r="M24" s="244"/>
     </x:row>
-    <x:row r="25">
+    <x:row r="25" ht="15" hidden="0" customHeight="1">
       <x:c r="A25" s="244"/>
       <x:c r="B25" s="244"/>
       <x:c r="C25" s="244"/>
@@ -14368,7 +16132,7 @@
       <x:c r="L25" s="244"/>
       <x:c r="M25" s="244"/>
     </x:row>
-    <x:row r="26">
+    <x:row r="26" ht="15" hidden="0" customHeight="1">
       <x:c r="A26" s="244"/>
       <x:c r="B26" s="244"/>
       <x:c r="C26" s="244"/>
@@ -14383,7 +16147,7 @@
       <x:c r="L26" s="244"/>
       <x:c r="M26" s="244"/>
     </x:row>
-    <x:row r="27">
+    <x:row r="27" ht="15" hidden="0" customHeight="1">
       <x:c r="A27" s="244"/>
       <x:c r="B27" s="244"/>
       <x:c r="C27" s="244"/>
@@ -14398,7 +16162,7 @@
       <x:c r="L27" s="244"/>
       <x:c r="M27" s="244"/>
     </x:row>
-    <x:row r="28">
+    <x:row r="28" ht="15" hidden="0" customHeight="1">
       <x:c r="A28" s="244"/>
       <x:c r="B28" s="244"/>
       <x:c r="C28" s="244"/>
@@ -14413,7 +16177,7 @@
       <x:c r="L28" s="244"/>
       <x:c r="M28" s="244"/>
     </x:row>
-    <x:row r="29">
+    <x:row r="29" ht="15" hidden="0" customHeight="1">
       <x:c r="A29" s="244"/>
       <x:c r="B29" s="244"/>
       <x:c r="C29" s="244"/>
@@ -14428,7 +16192,7 @@
       <x:c r="L29" s="244"/>
       <x:c r="M29" s="244"/>
     </x:row>
-    <x:row r="30">
+    <x:row r="30" ht="15" hidden="0" customHeight="1">
       <x:c r="A30" s="244"/>
       <x:c r="B30" s="244"/>
       <x:c r="C30" s="244"/>

</xml_diff>

<commit_message>
test: complete authentication controller tests
</commit_message>
<xml_diff>
--- a/test/test-cases/CPFriendFinder_TestCases.xlsx
+++ b/test/test-cases/CPFriendFinder_TestCases.xlsx
@@ -2,19 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Scenario Summary" sheetId="1" r:id="Recba8945f3984f78"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="2" r:id="R324bdb53b70e415d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Case Design &amp; Test Results" sheetId="3" r:id="R23d6edf69e824880"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS001" sheetId="4" r:id="R1e452e1eea52491d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS002" sheetId="5" r:id="R40da338c72b54538"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS003" sheetId="6" r:id="Rd873c532642b4fd0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS004" sheetId="7" r:id="Rf552e79d877e4365"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS005" sheetId="8" r:id="R8918426d85ca40aa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS006" sheetId="9" r:id="R9a895c86502b4ab7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defect Summary" sheetId="10" r:id="Rca445e34d02c4373"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Summary Report" sheetId="11" r:id="R46990a198a3d4ca5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution Log" sheetId="12" r:id="R80f83ac4ec5b4384"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision Table" sheetId="13" r:id="R3164514da3774e95"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Scenario Summary" sheetId="1" r:id="Rca98c80fc72742c0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="2" r:id="Rc26fca5991e146f4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Case Design &amp; Test Results" sheetId="3" r:id="R8c2bd41287404de7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS001" sheetId="4" r:id="Rd3c45c9a17af4162"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS002" sheetId="5" r:id="R05857e85b3ba4a61"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS003" sheetId="6" r:id="R1012d9e90ad34129"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS004" sheetId="7" r:id="Reac8d4c4773149fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS005" sheetId="8" r:id="Rc921313e9bc74e30"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS006" sheetId="9" r:id="R11dd260787cb4125"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defect Summary" sheetId="10" r:id="Re1906e21dfc14123"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Summary Report" sheetId="11" r:id="R6fe6880f4a48488b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution Log" sheetId="12" r:id="R500f0f5a476f4102"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision Table" sheetId="13" r:id="R9c42a0ddc46b4dae"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1504,7 +1504,7 @@
       </x:c>
       <x:c r="E6" s="259" t="n">
         <x:f>COUNTIFS('Test Case Design &amp; Test Results'!$B$4:$B$80,B6,'Test Case Design &amp; Test Results'!$J$4:$J$80,"Pass")</x:f>
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="F6" s="259" t="n">
         <x:f>COUNTIFS('Test Case Design &amp; Test Results'!$B$4:$B$80,B6,'Test Case Design &amp; Test Results'!$J$4:$J$80,"Fail")</x:f>
@@ -1512,7 +1512,7 @@
       </x:c>
       <x:c r="G6" s="259" t="n">
         <x:f>COUNTIFS('Test Case Design &amp; Test Results'!$B$4:$B$80,B6,'Test Case Design &amp; Test Results'!$J$4:$J$80,"Not Run")+COUNTIFS('Test Case Design &amp; Test Results'!$B$4:$B$80,B6,'Test Case Design &amp; Test Results'!$J$4:$J$80,"Waiting Frontend")</x:f>
-        <x:v>8</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H6" s="260" t="n">
         <x:f>COUNTIFS('Test Case Design &amp; Test Results'!$B$4:$B$80,B6,'Test Case Design &amp; Test Results'!$J$4:$J$80,"Blocked")</x:f>
@@ -4690,7 +4690,7 @@
       </x:c>
       <x:c r="B6" s="270" t="n">
         <x:f>COUNTIF('Test Case Design &amp; Test Results'!$J$4:$J$80,"Pass")+COUNTIF('Test Case Design &amp; Test Results'!$J$4:$J$80,"Fail")+COUNTIF('Test Case Design &amp; Test Results'!$J$4:$J$80,"Blocked")</x:f>
-        <x:v>24</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="C6" s="244"/>
       <x:c r="D6" s="244" t="str">
@@ -4716,12 +4716,18 @@
       </x:c>
       <x:c r="B7" s="270" t="n">
         <x:f>COUNTIF('Test Case Design &amp; Test Results'!$J$4:$J$80,"Pass")</x:f>
-        <x:v>24</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="C7" s="244"/>
-      <x:c r="D7" s="244"/>
-      <x:c r="E7" s="244"/>
-      <x:c r="F7" s="244"/>
+      <x:c r="D7" s="244" t="str">
+        <x:v>TS003</x:v>
+      </x:c>
+      <x:c r="E7" s="244" t="str">
+        <x:v>8/8 Pass</x:v>
+      </x:c>
+      <x:c r="F7" s="244" t="str">
+        <x:v>30.715 s</x:v>
+      </x:c>
       <x:c r="G7" s="244"/>
       <x:c r="H7" s="244"/>
       <x:c r="I7" s="244"/>
@@ -4756,7 +4762,7 @@
       </x:c>
       <x:c r="B9" s="271" t="n">
         <x:f>COUNTIF('Test Case Design &amp; Test Results'!$J$4:$J$80,"Not Run")+COUNTIF('Test Case Design &amp; Test Results'!$J$4:$J$80,"Waiting Frontend")</x:f>
-        <x:v>24</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="C9" s="244"/>
       <x:c r="D9" s="244"/>
@@ -6314,14 +6320,30 @@
       <x:c r="M6" s="244"/>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
-      <x:c r="A7" s="244"/>
-      <x:c r="B7" s="244"/>
-      <x:c r="C7" s="244"/>
-      <x:c r="D7" s="244"/>
-      <x:c r="E7" s="244"/>
-      <x:c r="F7" s="244"/>
-      <x:c r="G7" s="244"/>
-      <x:c r="H7" s="244"/>
+      <x:c r="A7" s="244" t="str">
+        <x:v>TS003</x:v>
+      </x:c>
+      <x:c r="B7" s="244" t="str">
+        <x:v>2026-10-01 16:43:40 +07:00</x:v>
+      </x:c>
+      <x:c r="C7" s="244" t="str">
+        <x:v>AuthControllerMvcTest</x:v>
+      </x:c>
+      <x:c r="D7" s="244" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E7" s="244" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="F7" s="244" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G7" s="244" t="str">
+        <x:v>0 / 0</x:v>
+      </x:c>
+      <x:c r="H7" s="244" t="str">
+        <x:v>BUILD SUCCESS</x:v>
+      </x:c>
       <x:c r="I7" s="244"/>
       <x:c r="J7" s="244"/>
       <x:c r="K7" s="244"/>
@@ -9773,7 +9795,7 @@
         <x:v>AuthController.register</x:v>
       </x:c>
       <x:c r="F14" s="270" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Passed - MVC</x:v>
       </x:c>
       <x:c r="G14" s="244"/>
       <x:c r="H14" s="244"/>
@@ -9800,7 +9822,7 @@
         <x:v>AuthController.login</x:v>
       </x:c>
       <x:c r="F15" s="270" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Passed - MVC</x:v>
       </x:c>
       <x:c r="G15" s="244"/>
       <x:c r="H15" s="244"/>
@@ -9827,7 +9849,7 @@
         <x:v>AuthController.SessionAuth / logout</x:v>
       </x:c>
       <x:c r="F16" s="270" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Passed - MVC</x:v>
       </x:c>
       <x:c r="G16" s="244"/>
       <x:c r="H16" s="244"/>
@@ -10119,7 +10141,7 @@
       <x:c r="L30" s="244"/>
       <x:c r="M30" s="244"/>
     </x:row>
-    <x:row r="31">
+    <x:row r="31" ht="15" hidden="0" customHeight="1">
       <x:c r="A31" s="244"/>
       <x:c r="B31" s="244"/>
       <x:c r="C31" s="244"/>
@@ -10134,7 +10156,7 @@
       <x:c r="L31" s="244"/>
       <x:c r="M31" s="244"/>
     </x:row>
-    <x:row r="32">
+    <x:row r="32" ht="15" hidden="0" customHeight="1">
       <x:c r="A32" s="244"/>
       <x:c r="B32" s="244"/>
       <x:c r="C32" s="244"/>
@@ -10149,7 +10171,7 @@
       <x:c r="L32" s="244"/>
       <x:c r="M32" s="244"/>
     </x:row>
-    <x:row r="33">
+    <x:row r="33" ht="15" hidden="0" customHeight="1">
       <x:c r="A33" s="244"/>
       <x:c r="B33" s="244"/>
       <x:c r="C33" s="244"/>
@@ -10164,7 +10186,7 @@
       <x:c r="L33" s="244"/>
       <x:c r="M33" s="244"/>
     </x:row>
-    <x:row r="34">
+    <x:row r="34" ht="15" hidden="0" customHeight="1">
       <x:c r="A34" s="244"/>
       <x:c r="B34" s="244"/>
       <x:c r="C34" s="244"/>
@@ -10179,7 +10201,7 @@
       <x:c r="L34" s="244"/>
       <x:c r="M34" s="244"/>
     </x:row>
-    <x:row r="35">
+    <x:row r="35" ht="15" hidden="0" customHeight="1">
       <x:c r="A35" s="244"/>
       <x:c r="B35" s="244"/>
       <x:c r="C35" s="244"/>
@@ -10194,7 +10216,7 @@
       <x:c r="L35" s="244"/>
       <x:c r="M35" s="244"/>
     </x:row>
-    <x:row r="36">
+    <x:row r="36" ht="15" hidden="0" customHeight="1">
       <x:c r="A36" s="244"/>
       <x:c r="B36" s="244"/>
       <x:c r="C36" s="244"/>
@@ -10209,7 +10231,7 @@
       <x:c r="L36" s="244"/>
       <x:c r="M36" s="244"/>
     </x:row>
-    <x:row r="37">
+    <x:row r="37" ht="15" hidden="0" customHeight="1">
       <x:c r="A37" s="244"/>
       <x:c r="B37" s="244"/>
       <x:c r="C37" s="244"/>
@@ -10224,7 +10246,7 @@
       <x:c r="L37" s="244"/>
       <x:c r="M37" s="244"/>
     </x:row>
-    <x:row r="38">
+    <x:row r="38" ht="15" hidden="0" customHeight="1">
       <x:c r="A38" s="244"/>
       <x:c r="B38" s="244"/>
       <x:c r="C38" s="244"/>
@@ -10239,7 +10261,7 @@
       <x:c r="L38" s="244"/>
       <x:c r="M38" s="244"/>
     </x:row>
-    <x:row r="39">
+    <x:row r="39" ht="15" hidden="0" customHeight="1">
       <x:c r="A39" s="244"/>
       <x:c r="B39" s="244"/>
       <x:c r="C39" s="244"/>
@@ -10254,7 +10276,7 @@
       <x:c r="L39" s="244"/>
       <x:c r="M39" s="244"/>
     </x:row>
-    <x:row r="40">
+    <x:row r="40" ht="15" hidden="0" customHeight="1">
       <x:c r="A40" s="244"/>
       <x:c r="B40" s="244"/>
       <x:c r="C40" s="244"/>
@@ -12253,7 +12275,7 @@
         <x:v>2026-10-01 16:29:59 | 11/11 passed | BUILD SUCCESS</x:v>
       </x:c>
     </x:row>
-    <x:row r="28" ht="15" hidden="0" customHeight="1">
+    <x:row r="28" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A28" s="270" t="str">
         <x:v>UC-AUTH-03</x:v>
       </x:c>
@@ -12279,18 +12301,22 @@
         <x:v>201 Created + RegisterResponse</x:v>
       </x:c>
       <x:c r="I28" s="261" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>ผ่านตาม Expected Result</x:v>
       </x:c>
       <x:c r="J28" s="270" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K28" s="261" t="str">
         <x:v>MVC Slice Test</x:v>
       </x:c>
-      <x:c r="L28" s="261" t="str"/>
-      <x:c r="M28" s="261" t="str"/>
-    </x:row>
-    <x:row r="29" ht="15" hidden="0" customHeight="1">
+      <x:c r="L28" s="261" t="str">
+        <x:v>AuthControllerMvcTest.register_validRequest_returnsCreated</x:v>
+      </x:c>
+      <x:c r="M28" s="261" t="str">
+        <x:v>2026-10-01 16:43:40 | 8/8 passed | BUILD SUCCESS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A29" s="270" t="str">
         <x:v>UC-AUTH-03</x:v>
       </x:c>
@@ -12316,18 +12342,22 @@
         <x:v>200 OK + LoginResponse + userId ถูกเก็บใน session</x:v>
       </x:c>
       <x:c r="I29" s="261" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>ผ่านตาม Expected Result</x:v>
       </x:c>
       <x:c r="J29" s="270" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K29" s="261" t="str">
         <x:v>MVC Slice Test</x:v>
       </x:c>
-      <x:c r="L29" s="261" t="str"/>
-      <x:c r="M29" s="261" t="str"/>
-    </x:row>
-    <x:row r="30" ht="15" hidden="0" customHeight="1">
+      <x:c r="L29" s="261" t="str">
+        <x:v>AuthControllerMvcTest.login_validRequest_returnsOkAndCreatesSession</x:v>
+      </x:c>
+      <x:c r="M29" s="261" t="str">
+        <x:v>2026-10-01 16:43:40 | 8/8 passed | BUILD SUCCESS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A30" s="270" t="str">
         <x:v>UC-AUTH-03</x:v>
       </x:c>
@@ -12353,18 +12383,22 @@
         <x:v>200 OK + userId=null</x:v>
       </x:c>
       <x:c r="I30" s="261" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>ผ่านตาม Expected Result</x:v>
       </x:c>
       <x:c r="J30" s="270" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K30" s="261" t="str">
         <x:v>MVC Slice Test</x:v>
       </x:c>
-      <x:c r="L30" s="261" t="str"/>
-      <x:c r="M30" s="261" t="str"/>
-    </x:row>
-    <x:row r="31" ht="15" hidden="0" customHeight="1">
+      <x:c r="L30" s="261" t="str">
+        <x:v>AuthControllerMvcTest.sessionAuth_withoutLogin_returnsNullUserId</x:v>
+      </x:c>
+      <x:c r="M30" s="261" t="str">
+        <x:v>2026-10-01 16:43:40 | 8/8 passed | BUILD SUCCESS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A31" s="270" t="str">
         <x:v>UC-AUTH-03</x:v>
       </x:c>
@@ -12390,18 +12424,22 @@
         <x:v>200 OK + userId เดิม</x:v>
       </x:c>
       <x:c r="I31" s="261" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>ผ่านตาม Expected Result</x:v>
       </x:c>
       <x:c r="J31" s="270" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K31" s="261" t="str">
         <x:v>MVC Slice Test</x:v>
       </x:c>
-      <x:c r="L31" s="261" t="str"/>
-      <x:c r="M31" s="261" t="str"/>
-    </x:row>
-    <x:row r="32" ht="15" hidden="0" customHeight="1">
+      <x:c r="L31" s="261" t="str">
+        <x:v>AuthControllerMvcTest.sessionAuth_withSession_returnsUserId</x:v>
+      </x:c>
+      <x:c r="M31" s="261" t="str">
+        <x:v>2026-10-01 16:43:40 | 8/8 passed | BUILD SUCCESS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A32" s="270" t="str">
         <x:v>UC-AUTH-03</x:v>
       </x:c>
@@ -12427,18 +12465,22 @@
         <x:v>204 No Content + session invalidated</x:v>
       </x:c>
       <x:c r="I32" s="261" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>ผ่านตาม Expected Result</x:v>
       </x:c>
       <x:c r="J32" s="270" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K32" s="261" t="str">
         <x:v>MVC Slice Test</x:v>
       </x:c>
-      <x:c r="L32" s="261" t="str"/>
-      <x:c r="M32" s="261" t="str"/>
-    </x:row>
-    <x:row r="33" ht="15" hidden="0" customHeight="1">
+      <x:c r="L32" s="261" t="str">
+        <x:v>AuthControllerMvcTest.logout_invalidatesSession</x:v>
+      </x:c>
+      <x:c r="M32" s="261" t="str">
+        <x:v>2026-10-01 16:43:40 | 8/8 passed | BUILD SUCCESS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A33" s="270" t="str">
         <x:v>UC-AUTH-03</x:v>
       </x:c>
@@ -12455,27 +12497,31 @@
         <x:v>AuthController.register</x:v>
       </x:c>
       <x:c r="F33" s="261" t="str">
-        <x:v>POST register ไม่มี body/JSON ผิดรูป</x:v>
+        <x:v>POST /api/auth/register + malformed JSON</x:v>
       </x:c>
       <x:c r="G33" s="261" t="str">
-        <x:v>MVC binding/serialization</x:v>
+        <x:v>AuthService ต้องไม่ถูกเรียก</x:v>
       </x:c>
       <x:c r="H33" s="261" t="str">
-        <x:v>ได้ 4xx ตาม MVC behavior</x:v>
+        <x:v>400 Bad Request</x:v>
       </x:c>
       <x:c r="I33" s="261" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>ผ่านตาม Expected Result</x:v>
       </x:c>
       <x:c r="J33" s="270" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K33" s="261" t="str">
         <x:v>MVC Slice Test</x:v>
       </x:c>
-      <x:c r="L33" s="261" t="str"/>
-      <x:c r="M33" s="261" t="str"/>
-    </x:row>
-    <x:row r="34" ht="15" hidden="0" customHeight="1">
+      <x:c r="L33" s="261" t="str">
+        <x:v>AuthControllerMvcTest.register_malformedJson_returnsBadRequest</x:v>
+      </x:c>
+      <x:c r="M33" s="261" t="str">
+        <x:v>2026-10-01 16:43:40 | 8/8 passed | BUILD SUCCESS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A34" s="270" t="str">
         <x:v>UC-AUTH-03</x:v>
       </x:c>
@@ -12492,27 +12538,31 @@
         <x:v>AuthController.login</x:v>
       </x:c>
       <x:c r="F34" s="261" t="str">
-        <x:v>POST login ไม่มี body/JSON ผิดรูป</x:v>
+        <x:v>POST /api/auth/login + malformed JSON</x:v>
       </x:c>
       <x:c r="G34" s="261" t="str">
-        <x:v>MVC binding/serialization</x:v>
+        <x:v>AuthService ต้องไม่ถูกเรียก</x:v>
       </x:c>
       <x:c r="H34" s="261" t="str">
-        <x:v>ได้ 4xx ตาม MVC behavior</x:v>
+        <x:v>400 Bad Request</x:v>
       </x:c>
       <x:c r="I34" s="261" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>ผ่านตาม Expected Result</x:v>
       </x:c>
       <x:c r="J34" s="270" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K34" s="261" t="str">
         <x:v>MVC Slice Test</x:v>
       </x:c>
-      <x:c r="L34" s="261" t="str"/>
-      <x:c r="M34" s="261" t="str"/>
-    </x:row>
-    <x:row r="35" ht="15" hidden="0" customHeight="1">
+      <x:c r="L34" s="261" t="str">
+        <x:v>AuthControllerMvcTest.login_malformedJson_returnsBadRequest</x:v>
+      </x:c>
+      <x:c r="M34" s="261" t="str">
+        <x:v>2026-10-01 16:43:40 | 8/8 passed | BUILD SUCCESS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A35" s="270" t="str">
         <x:v>UC-AUTH-03</x:v>
       </x:c>
@@ -12526,28 +12576,32 @@
         <x:v>Response privacy</x:v>
       </x:c>
       <x:c r="E35" s="261" t="str">
-        <x:v>RegisterResponse/LoginResponse</x:v>
+        <x:v>LoginResponse</x:v>
       </x:c>
       <x:c r="F35" s="261" t="str">
-        <x:v>AuthService คืน User ที่มี passwordHash</x:v>
+        <x:v>POST /api/auth/login + valid JSON</x:v>
       </x:c>
       <x:c r="G35" s="261" t="str">
-        <x:v>response serialization</x:v>
+        <x:v>AuthService.login คืน User</x:v>
       </x:c>
       <x:c r="H35" s="261" t="str">
-        <x:v>response ไม่ควรมี passwordHash</x:v>
+        <x:v>response ไม่มี password, passwordHash หรือ password_hash</x:v>
       </x:c>
       <x:c r="I35" s="261" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>ผ่านตาม Expected Result</x:v>
       </x:c>
       <x:c r="J35" s="270" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K35" s="261" t="str">
         <x:v>MVC Slice Test</x:v>
       </x:c>
-      <x:c r="L35" s="261" t="str"/>
-      <x:c r="M35" s="261" t="str"/>
+      <x:c r="L35" s="261" t="str">
+        <x:v>AuthControllerMvcTest.login_responseDoesNotExposePassword</x:v>
+      </x:c>
+      <x:c r="M35" s="261" t="str">
+        <x:v>2026-10-01 16:43:40 | 8/8 passed | BUILD SUCCESS</x:v>
+      </x:c>
     </x:row>
     <x:row r="36" ht="15" hidden="0" customHeight="1">
       <x:c r="A36" s="270" t="str">
@@ -17301,7 +17355,7 @@
       <x:c r="L1" s="244"/>
       <x:c r="M1" s="244"/>
     </x:row>
-    <x:row r="2">
+    <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="244"/>
       <x:c r="B2" s="244"/>
       <x:c r="C2" s="244"/>
@@ -17468,7 +17522,7 @@
       <x:c r="L10" s="244"/>
       <x:c r="M10" s="244"/>
     </x:row>
-    <x:row r="11">
+    <x:row r="11" ht="15" hidden="0" customHeight="1">
       <x:c r="A11" s="244"/>
       <x:c r="B11" s="244"/>
       <x:c r="C11" s="244"/>
@@ -17522,7 +17576,7 @@
         <x:v>201 Created + RegisterResponse</x:v>
       </x:c>
       <x:c r="E13" s="269" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="F13" s="244"/>
       <x:c r="G13" s="244"/>
@@ -17547,7 +17601,7 @@
         <x:v>200 OK + LoginResponse + userId ถูกเก็บใน session</x:v>
       </x:c>
       <x:c r="E14" s="270" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="F14" s="244"/>
       <x:c r="G14" s="244"/>
@@ -17572,7 +17626,7 @@
         <x:v>200 OK + userId=null</x:v>
       </x:c>
       <x:c r="E15" s="270" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="F15" s="244"/>
       <x:c r="G15" s="244"/>
@@ -17597,7 +17651,7 @@
         <x:v>200 OK + userId เดิม</x:v>
       </x:c>
       <x:c r="E16" s="270" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="F16" s="244"/>
       <x:c r="G16" s="244"/>
@@ -17622,7 +17676,7 @@
         <x:v>204 No Content + session invalidated</x:v>
       </x:c>
       <x:c r="E17" s="270" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="F17" s="244"/>
       <x:c r="G17" s="244"/>
@@ -17641,13 +17695,13 @@
         <x:v>Malformed request</x:v>
       </x:c>
       <x:c r="C18" s="256" t="str">
-        <x:v>POST register ไม่มี body/JSON ผิดรูป | MVC binding/serialization</x:v>
+        <x:v>POST /api/auth/register + malformed JSON | AuthService ต้องไม่ถูกเรียก</x:v>
       </x:c>
       <x:c r="D18" s="257" t="str">
-        <x:v>ได้ 4xx ตาม MVC behavior</x:v>
+        <x:v>400 Bad Request</x:v>
       </x:c>
       <x:c r="E18" s="270" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="F18" s="244"/>
       <x:c r="G18" s="244"/>
@@ -17666,13 +17720,13 @@
         <x:v>Malformed request</x:v>
       </x:c>
       <x:c r="C19" s="256" t="str">
-        <x:v>POST login ไม่มี body/JSON ผิดรูป | MVC binding/serialization</x:v>
+        <x:v>POST /api/auth/login + malformed JSON | AuthService ต้องไม่ถูกเรียก</x:v>
       </x:c>
       <x:c r="D19" s="257" t="str">
-        <x:v>ได้ 4xx ตาม MVC behavior</x:v>
+        <x:v>400 Bad Request</x:v>
       </x:c>
       <x:c r="E19" s="270" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="F19" s="244"/>
       <x:c r="G19" s="244"/>
@@ -17691,13 +17745,13 @@
         <x:v>Response privacy</x:v>
       </x:c>
       <x:c r="C20" s="263" t="str">
-        <x:v>AuthService คืน User ที่มี passwordHash | response serialization</x:v>
+        <x:v>POST /api/auth/login + valid JSON | AuthService.login คืน User</x:v>
       </x:c>
       <x:c r="D20" s="264" t="str">
-        <x:v>response ไม่ควรมี passwordHash</x:v>
+        <x:v>response ไม่มี password, passwordHash หรือ password_hash</x:v>
       </x:c>
       <x:c r="E20" s="271" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="F20" s="244"/>
       <x:c r="G20" s="244"/>
@@ -17708,7 +17762,7 @@
       <x:c r="L20" s="244"/>
       <x:c r="M20" s="244"/>
     </x:row>
-    <x:row r="21">
+    <x:row r="21" ht="15" hidden="0" customHeight="1">
       <x:c r="A21" s="244"/>
       <x:c r="B21" s="244"/>
       <x:c r="C21" s="244"/>
@@ -17723,7 +17777,7 @@
       <x:c r="L21" s="244"/>
       <x:c r="M21" s="244"/>
     </x:row>
-    <x:row r="22">
+    <x:row r="22" ht="15" hidden="0" customHeight="1">
       <x:c r="A22" s="244"/>
       <x:c r="B22" s="244"/>
       <x:c r="C22" s="244"/>
@@ -17738,7 +17792,7 @@
       <x:c r="L22" s="244"/>
       <x:c r="M22" s="244"/>
     </x:row>
-    <x:row r="23">
+    <x:row r="23" ht="15" hidden="0" customHeight="1">
       <x:c r="A23" s="244"/>
       <x:c r="B23" s="244"/>
       <x:c r="C23" s="244"/>
@@ -17753,7 +17807,7 @@
       <x:c r="L23" s="244"/>
       <x:c r="M23" s="244"/>
     </x:row>
-    <x:row r="24">
+    <x:row r="24" ht="15" hidden="0" customHeight="1">
       <x:c r="A24" s="244"/>
       <x:c r="B24" s="244"/>
       <x:c r="C24" s="244"/>
@@ -17768,7 +17822,7 @@
       <x:c r="L24" s="244"/>
       <x:c r="M24" s="244"/>
     </x:row>
-    <x:row r="25">
+    <x:row r="25" ht="15" hidden="0" customHeight="1">
       <x:c r="A25" s="244"/>
       <x:c r="B25" s="244"/>
       <x:c r="C25" s="244"/>

</xml_diff>

<commit_message>
test: complete security configuration tests
</commit_message>
<xml_diff>
--- a/test/test-cases/CPFriendFinder_TestCases.xlsx
+++ b/test/test-cases/CPFriendFinder_TestCases.xlsx
@@ -2,19 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Scenario Summary" sheetId="1" r:id="Rca98c80fc72742c0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="2" r:id="Rc26fca5991e146f4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Case Design &amp; Test Results" sheetId="3" r:id="R8c2bd41287404de7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS001" sheetId="4" r:id="Rd3c45c9a17af4162"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS002" sheetId="5" r:id="R05857e85b3ba4a61"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS003" sheetId="6" r:id="R1012d9e90ad34129"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS004" sheetId="7" r:id="Reac8d4c4773149fe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS005" sheetId="8" r:id="Rc921313e9bc74e30"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS006" sheetId="9" r:id="R11dd260787cb4125"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defect Summary" sheetId="10" r:id="Re1906e21dfc14123"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Summary Report" sheetId="11" r:id="R6fe6880f4a48488b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution Log" sheetId="12" r:id="R500f0f5a476f4102"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision Table" sheetId="13" r:id="R9c42a0ddc46b4dae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Scenario Summary" sheetId="1" r:id="R7243b80e31a84036"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="2" r:id="R52aac16da1464c59"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Case Design &amp; Test Results" sheetId="3" r:id="R65b22af242014631"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS001" sheetId="4" r:id="Rc95338479c994bc0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS002" sheetId="5" r:id="Ra6380f9cc3dd409e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS003" sheetId="6" r:id="Rf85a2abb220b4313"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS004" sheetId="7" r:id="R95efdda6f084450a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS005" sheetId="8" r:id="R6141c0d1f4cf4903"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS006" sheetId="9" r:id="Re81420da6a45480a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defect Summary" sheetId="10" r:id="Rcd240c31e64c49b7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Summary Report" sheetId="11" r:id="R14aeb3fee81c4d2e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution Log" sheetId="12" r:id="Re6d1aacf04e24ed7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision Table" sheetId="13" r:id="Rd098b0c8971e4f2d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1542,7 +1542,7 @@
       </x:c>
       <x:c r="E7" s="259" t="n">
         <x:f>COUNTIFS('Test Case Design &amp; Test Results'!$B$4:$B$80,B7,'Test Case Design &amp; Test Results'!$J$4:$J$80,"Pass")</x:f>
-        <x:v>0</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="F7" s="259" t="n">
         <x:f>COUNTIFS('Test Case Design &amp; Test Results'!$B$4:$B$80,B7,'Test Case Design &amp; Test Results'!$J$4:$J$80,"Fail")</x:f>
@@ -1550,7 +1550,7 @@
       </x:c>
       <x:c r="G7" s="259" t="n">
         <x:f>COUNTIFS('Test Case Design &amp; Test Results'!$B$4:$B$80,B7,'Test Case Design &amp; Test Results'!$J$4:$J$80,"Not Run")+COUNTIFS('Test Case Design &amp; Test Results'!$B$4:$B$80,B7,'Test Case Design &amp; Test Results'!$J$4:$J$80,"Waiting Frontend")</x:f>
-        <x:v>7</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H7" s="260" t="n">
         <x:f>COUNTIFS('Test Case Design &amp; Test Results'!$B$4:$B$80,B7,'Test Case Design &amp; Test Results'!$J$4:$J$80,"Blocked")</x:f>
@@ -4690,7 +4690,7 @@
       </x:c>
       <x:c r="B6" s="270" t="n">
         <x:f>COUNTIF('Test Case Design &amp; Test Results'!$J$4:$J$80,"Pass")+COUNTIF('Test Case Design &amp; Test Results'!$J$4:$J$80,"Fail")+COUNTIF('Test Case Design &amp; Test Results'!$J$4:$J$80,"Blocked")</x:f>
-        <x:v>32</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="C6" s="244"/>
       <x:c r="D6" s="244" t="str">
@@ -4716,7 +4716,7 @@
       </x:c>
       <x:c r="B7" s="270" t="n">
         <x:f>COUNTIF('Test Case Design &amp; Test Results'!$J$4:$J$80,"Pass")</x:f>
-        <x:v>32</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="C7" s="244"/>
       <x:c r="D7" s="244" t="str">
@@ -4745,9 +4745,15 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="C8" s="244"/>
-      <x:c r="D8" s="244"/>
-      <x:c r="E8" s="244"/>
-      <x:c r="F8" s="244"/>
+      <x:c r="D8" s="244" t="str">
+        <x:v>TS004</x:v>
+      </x:c>
+      <x:c r="E8" s="244" t="str">
+        <x:v>7/7 Pass</x:v>
+      </x:c>
+      <x:c r="F8" s="244" t="str">
+        <x:v>48.881 s</x:v>
+      </x:c>
       <x:c r="G8" s="244"/>
       <x:c r="H8" s="244"/>
       <x:c r="I8" s="244"/>
@@ -4762,7 +4768,7 @@
       </x:c>
       <x:c r="B9" s="271" t="n">
         <x:f>COUNTIF('Test Case Design &amp; Test Results'!$J$4:$J$80,"Not Run")+COUNTIF('Test Case Design &amp; Test Results'!$J$4:$J$80,"Waiting Frontend")</x:f>
-        <x:v>16</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="C9" s="244"/>
       <x:c r="D9" s="244"/>
@@ -6351,14 +6357,30 @@
       <x:c r="M7" s="244"/>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
-      <x:c r="A8" s="244"/>
-      <x:c r="B8" s="244"/>
-      <x:c r="C8" s="244"/>
-      <x:c r="D8" s="244"/>
-      <x:c r="E8" s="244"/>
-      <x:c r="F8" s="244"/>
-      <x:c r="G8" s="244"/>
-      <x:c r="H8" s="244"/>
+      <x:c r="A8" s="244" t="str">
+        <x:v>TS004</x:v>
+      </x:c>
+      <x:c r="B8" s="244" t="str">
+        <x:v>2026-10-01 17:01:57 +07:00</x:v>
+      </x:c>
+      <x:c r="C8" s="244" t="str">
+        <x:v>AuthSecurityWebMvcTest</x:v>
+      </x:c>
+      <x:c r="D8" s="244" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="E8" s="244" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="F8" s="244" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G8" s="244" t="str">
+        <x:v>0 / 0</x:v>
+      </x:c>
+      <x:c r="H8" s="244" t="str">
+        <x:v>BUILD SUCCESS</x:v>
+      </x:c>
       <x:c r="I8" s="244"/>
       <x:c r="J8" s="244"/>
       <x:c r="K8" s="244"/>
@@ -6395,7 +6417,7 @@
       <x:c r="L10" s="244"/>
       <x:c r="M10" s="244"/>
     </x:row>
-    <x:row r="11">
+    <x:row r="11" ht="15" hidden="0" customHeight="1">
       <x:c r="A11" s="244"/>
       <x:c r="B11" s="244"/>
       <x:c r="C11" s="244"/>
@@ -6410,7 +6432,7 @@
       <x:c r="L11" s="244"/>
       <x:c r="M11" s="244"/>
     </x:row>
-    <x:row r="12">
+    <x:row r="12" ht="15" hidden="0" customHeight="1">
       <x:c r="A12" s="244"/>
       <x:c r="B12" s="244"/>
       <x:c r="C12" s="244"/>
@@ -9876,7 +9898,7 @@
         <x:v>SecurityConfig</x:v>
       </x:c>
       <x:c r="F17" s="270" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Passed - Security MVC</x:v>
       </x:c>
       <x:c r="G17" s="244"/>
       <x:c r="H17" s="244"/>
@@ -9903,7 +9925,7 @@
         <x:v>SecurityConfig</x:v>
       </x:c>
       <x:c r="F18" s="270" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Passed - Security MVC</x:v>
       </x:c>
       <x:c r="G18" s="244"/>
       <x:c r="H18" s="244"/>
@@ -9930,7 +9952,7 @@
         <x:v>SecurityConfig</x:v>
       </x:c>
       <x:c r="F19" s="270" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Passed - Security MVC</x:v>
       </x:c>
       <x:c r="G19" s="244"/>
       <x:c r="H19" s="244"/>
@@ -12603,7 +12625,7 @@
         <x:v>2026-10-01 16:43:40 | 8/8 passed | BUILD SUCCESS</x:v>
       </x:c>
     </x:row>
-    <x:row r="36" ht="15" hidden="0" customHeight="1">
+    <x:row r="36" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A36" s="270" t="str">
         <x:v>UC-AUTH-04</x:v>
       </x:c>
@@ -12626,21 +12648,25 @@
         <x:v>anonymous request</x:v>
       </x:c>
       <x:c r="H36" s="261" t="str">
-        <x:v>route ถูก permitAll ตาม config ปัจจุบัน</x:v>
+        <x:v>security ไม่ตอบ 401 หรือ 403</x:v>
       </x:c>
       <x:c r="I36" s="261" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>ผ่านตาม Expected Result</x:v>
       </x:c>
       <x:c r="J36" s="270" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K36" s="261" t="str">
         <x:v>Security MVC Test</x:v>
       </x:c>
-      <x:c r="L36" s="261" t="str"/>
-      <x:c r="M36" s="261" t="str"/>
-    </x:row>
-    <x:row r="37" ht="15" hidden="0" customHeight="1">
+      <x:c r="L36" s="261" t="str">
+        <x:v>AuthSecurityWebMvcTest.publicPages_areNotBlockedBySecurity</x:v>
+      </x:c>
+      <x:c r="M36" s="261" t="str">
+        <x:v>2026-10-01 17:01:57 | 7/7 passed | BUILD SUCCESS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A37" s="270" t="str">
         <x:v>UC-AUTH-04</x:v>
       </x:c>
@@ -12657,25 +12683,29 @@
         <x:v>SecurityConfig</x:v>
       </x:c>
       <x:c r="F37" s="261" t="str">
-        <x:v>GET/POST /api/**</x:v>
+        <x:v>GET /api/auth</x:v>
       </x:c>
       <x:c r="G37" s="261" t="str">
         <x:v>anonymous request</x:v>
       </x:c>
       <x:c r="H37" s="261" t="str">
-        <x:v>API ถูก permitAll ตาม config ปัจจุบัน</x:v>
+        <x:v>200 OK</x:v>
       </x:c>
       <x:c r="I37" s="261" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>ผ่านตาม Expected Result</x:v>
       </x:c>
       <x:c r="J37" s="270" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K37" s="261" t="str">
         <x:v>Security MVC Test</x:v>
       </x:c>
-      <x:c r="L37" s="261" t="str"/>
-      <x:c r="M37" s="261" t="str"/>
+      <x:c r="L37" s="261" t="str">
+        <x:v>AuthSecurityWebMvcTest.api_isAccessibleWithoutAuthentication</x:v>
+      </x:c>
+      <x:c r="M37" s="261" t="str">
+        <x:v>2026-10-01 17:01:57 | 7/7 passed | BUILD SUCCESS</x:v>
+      </x:c>
     </x:row>
     <x:row r="38" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A38" s="270" t="str">
@@ -12694,27 +12724,31 @@
         <x:v>SecurityConfig</x:v>
       </x:c>
       <x:c r="F38" s="261" t="str">
-        <x:v>POST /api/auth/login/register/logout ไม่มี CSRF token</x:v>
+        <x:v>POST /api/auth/logout ไม่มี CSRF token</x:v>
       </x:c>
       <x:c r="G38" s="261" t="str">
-        <x:v>anonymous/request ตามกรณี</x:v>
+        <x:v>anonymous request</x:v>
       </x:c>
       <x:c r="H38" s="261" t="str">
-        <x:v>ไม่ถูกบล็อกจาก CSRF เพราะ /api/** ถูก ignore</x:v>
+        <x:v>204 No Content; ไม่ถูก CSRF บล็อก</x:v>
       </x:c>
       <x:c r="I38" s="261" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>ผ่านตาม Expected Result</x:v>
       </x:c>
       <x:c r="J38" s="270" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K38" s="261" t="str">
         <x:v>Security MVC Test</x:v>
       </x:c>
-      <x:c r="L38" s="261" t="str"/>
-      <x:c r="M38" s="261" t="str"/>
-    </x:row>
-    <x:row r="39" ht="15" hidden="0" customHeight="1">
+      <x:c r="L38" s="261" t="str">
+        <x:v>AuthSecurityWebMvcTest.apiPost_doesNotRequireCsrfToken</x:v>
+      </x:c>
+      <x:c r="M38" s="261" t="str">
+        <x:v>2026-10-01 17:01:57 | 7/7 passed | BUILD SUCCESS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A39" s="270" t="str">
         <x:v>UC-AUTH-04</x:v>
       </x:c>
@@ -12731,25 +12765,29 @@
         <x:v>SecurityConfig</x:v>
       </x:c>
       <x:c r="F39" s="261" t="str">
-        <x:v>GET /swagger-ui/** หรือ /v3/api-docs/**</x:v>
+        <x:v>GET /swagger-ui/index.html และ /v3/api-docs/openapi</x:v>
       </x:c>
       <x:c r="G39" s="261" t="str">
         <x:v>anonymous request</x:v>
       </x:c>
       <x:c r="H39" s="261" t="str">
-        <x:v>route ถูก permitAll</x:v>
+        <x:v>security ไม่ตอบ 401 หรือ 403</x:v>
       </x:c>
       <x:c r="I39" s="261" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>ผ่านตาม Expected Result</x:v>
       </x:c>
       <x:c r="J39" s="270" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K39" s="261" t="str">
         <x:v>Security MVC Test</x:v>
       </x:c>
-      <x:c r="L39" s="261" t="str"/>
-      <x:c r="M39" s="261" t="str"/>
+      <x:c r="L39" s="261" t="str">
+        <x:v>AuthSecurityWebMvcTest.swaggerRoutes_areNotBlockedBySecurity</x:v>
+      </x:c>
+      <x:c r="M39" s="261" t="str">
+        <x:v>2026-10-01 17:01:57 | 7/7 passed | BUILD SUCCESS</x:v>
+      </x:c>
     </x:row>
     <x:row r="40" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A40" s="270" t="str">
@@ -12768,27 +12806,31 @@
         <x:v>SecurityConfig</x:v>
       </x:c>
       <x:c r="F40" s="261" t="str">
-        <x:v>GET /css/** /js/** /images/** /favicon.ico</x:v>
+        <x:v>GET /css/app.css, /js/app.js, /images/logo.png, /favicon.ico</x:v>
       </x:c>
       <x:c r="G40" s="261" t="str">
         <x:v>anonymous request</x:v>
       </x:c>
       <x:c r="H40" s="261" t="str">
-        <x:v>security ไม่บล็อก route เหล่านี้; resource existence ทดสอบภายหลัง</x:v>
+        <x:v>security ไม่ตอบ 401 หรือ 403</x:v>
       </x:c>
       <x:c r="I40" s="261" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>ผ่านตาม Expected Result</x:v>
       </x:c>
       <x:c r="J40" s="270" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K40" s="261" t="str">
         <x:v>Security MVC Test</x:v>
       </x:c>
-      <x:c r="L40" s="261" t="str"/>
-      <x:c r="M40" s="261" t="str"/>
-    </x:row>
-    <x:row r="41" ht="15" hidden="0" customHeight="1">
+      <x:c r="L40" s="261" t="str">
+        <x:v>AuthSecurityWebMvcTest.staticResources_areNotBlockedBySecurity</x:v>
+      </x:c>
+      <x:c r="M40" s="261" t="str">
+        <x:v>2026-10-01 17:01:57 | 7/7 passed | BUILD SUCCESS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A41" s="270" t="str">
         <x:v>UC-AUTH-04</x:v>
       </x:c>
@@ -12805,27 +12847,31 @@
         <x:v>SecurityConfig</x:v>
       </x:c>
       <x:c r="F41" s="261" t="str">
-        <x:v>GET path ที่ไม่อยู่ใน permitAll</x:v>
+        <x:v>GET /private-test</x:v>
       </x:c>
       <x:c r="G41" s="261" t="str">
         <x:v>anonymous request</x:v>
       </x:c>
       <x:c r="H41" s="261" t="str">
-        <x:v>ต้อง authenticated / ถูกปฏิเสธตาม Spring Security</x:v>
+        <x:v>403 Forbidden</x:v>
       </x:c>
       <x:c r="I41" s="261" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>ผ่านตาม Expected Result</x:v>
       </x:c>
       <x:c r="J41" s="270" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K41" s="261" t="str">
         <x:v>Security MVC Test</x:v>
       </x:c>
-      <x:c r="L41" s="261" t="str"/>
-      <x:c r="M41" s="261" t="str"/>
-    </x:row>
-    <x:row r="42" ht="15" hidden="0" customHeight="1">
+      <x:c r="L41" s="261" t="str">
+        <x:v>AuthSecurityWebMvcTest.unmatchedRoute_requiresAuthentication</x:v>
+      </x:c>
+      <x:c r="M41" s="261" t="str">
+        <x:v>2026-10-01 17:01:57 | 7/7 passed | BUILD SUCCESS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A42" s="270" t="str">
         <x:v>UC-AUTH-04</x:v>
       </x:c>
@@ -12842,25 +12888,29 @@
         <x:v>SecurityConfig</x:v>
       </x:c>
       <x:c r="F42" s="261" t="str">
-        <x:v>request ที่ไม่มี form login/basic credentials</x:v>
+        <x:v>ตรวจ SecurityFilterChain</x:v>
       </x:c>
       <x:c r="G42" s="261" t="str">
-        <x:v>anonymous request</x:v>
+        <x:v>ตรวจ filter ที่ถูกสร้าง</x:v>
       </x:c>
       <x:c r="H42" s="261" t="str">
-        <x:v>formLogin และ httpBasic ถูก disable ตาม config</x:v>
+        <x:v>ไม่มี UsernamePasswordAuthenticationFilter และ BasicAuthenticationFilter</x:v>
       </x:c>
       <x:c r="I42" s="261" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>ผ่านตาม Expected Result</x:v>
       </x:c>
       <x:c r="J42" s="270" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K42" s="261" t="str">
         <x:v>Security MVC Test</x:v>
       </x:c>
-      <x:c r="L42" s="261" t="str"/>
-      <x:c r="M42" s="261" t="str"/>
+      <x:c r="L42" s="261" t="str">
+        <x:v>AuthSecurityWebMvcTest.formLoginAndHttpBasic_areDisabled</x:v>
+      </x:c>
+      <x:c r="M42" s="261" t="str">
+        <x:v>2026-10-01 17:01:57 | 7/7 passed | BUILD SUCCESS</x:v>
+      </x:c>
     </x:row>
     <x:row r="43" ht="15" hidden="0" customHeight="1">
       <x:c r="A43" s="270" t="str">
@@ -19006,7 +19056,7 @@
       <x:c r="L1" s="244"/>
       <x:c r="M1" s="244"/>
     </x:row>
-    <x:row r="2">
+    <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="244"/>
       <x:c r="B2" s="244"/>
       <x:c r="C2" s="244"/>
@@ -19173,7 +19223,7 @@
       <x:c r="L10" s="244"/>
       <x:c r="M10" s="244"/>
     </x:row>
-    <x:row r="11">
+    <x:row r="11" ht="15" hidden="0" customHeight="1">
       <x:c r="A11" s="244"/>
       <x:c r="B11" s="244"/>
       <x:c r="C11" s="244"/>
@@ -19224,10 +19274,10 @@
         <x:v>GET /, /login, /home, /register | anonymous request</x:v>
       </x:c>
       <x:c r="D13" s="250" t="str">
-        <x:v>route ถูก permitAll ตาม config ปัจจุบัน</x:v>
+        <x:v>security ไม่ตอบ 401 หรือ 403</x:v>
       </x:c>
       <x:c r="E13" s="269" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="F13" s="244"/>
       <x:c r="G13" s="244"/>
@@ -19246,13 +19296,13 @@
         <x:v>API access</x:v>
       </x:c>
       <x:c r="C14" s="256" t="str">
-        <x:v>GET/POST /api/** | anonymous request</x:v>
+        <x:v>GET /api/auth | anonymous request</x:v>
       </x:c>
       <x:c r="D14" s="257" t="str">
-        <x:v>API ถูก permitAll ตาม config ปัจจุบัน</x:v>
+        <x:v>200 OK</x:v>
       </x:c>
       <x:c r="E14" s="270" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="F14" s="244"/>
       <x:c r="G14" s="244"/>
@@ -19271,13 +19321,13 @@
         <x:v>CSRF configuration</x:v>
       </x:c>
       <x:c r="C15" s="256" t="str">
-        <x:v>POST /api/auth/login/register/logout ไม่มี CSRF token | anonymous/request ตามกรณี</x:v>
+        <x:v>POST /api/auth/logout ไม่มี CSRF token | anonymous request</x:v>
       </x:c>
       <x:c r="D15" s="257" t="str">
-        <x:v>ไม่ถูกบล็อกจาก CSRF เพราะ /api/** ถูก ignore</x:v>
+        <x:v>204 No Content; ไม่ถูก CSRF บล็อก</x:v>
       </x:c>
       <x:c r="E15" s="270" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="F15" s="244"/>
       <x:c r="G15" s="244"/>
@@ -19296,13 +19346,13 @@
         <x:v>Swagger access</x:v>
       </x:c>
       <x:c r="C16" s="256" t="str">
-        <x:v>GET /swagger-ui/** หรือ /v3/api-docs/** | anonymous request</x:v>
+        <x:v>GET /swagger-ui/index.html และ /v3/api-docs/openapi | anonymous request</x:v>
       </x:c>
       <x:c r="D16" s="257" t="str">
-        <x:v>route ถูก permitAll</x:v>
+        <x:v>security ไม่ตอบ 401 หรือ 403</x:v>
       </x:c>
       <x:c r="E16" s="270" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="F16" s="244"/>
       <x:c r="G16" s="244"/>
@@ -19321,13 +19371,13 @@
         <x:v>Static route access</x:v>
       </x:c>
       <x:c r="C17" s="256" t="str">
-        <x:v>GET /css/** /js/** /images/** /favicon.ico | anonymous request</x:v>
+        <x:v>GET /css/app.css, /js/app.js, /images/logo.png, /favicon.ico | anonymous request</x:v>
       </x:c>
       <x:c r="D17" s="257" t="str">
-        <x:v>security ไม่บล็อก route เหล่านี้; resource existence ทดสอบภายหลัง</x:v>
+        <x:v>security ไม่ตอบ 401 หรือ 403</x:v>
       </x:c>
       <x:c r="E17" s="270" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="F17" s="244"/>
       <x:c r="G17" s="244"/>
@@ -19346,13 +19396,13 @@
         <x:v>Protected fallback</x:v>
       </x:c>
       <x:c r="C18" s="256" t="str">
-        <x:v>GET path ที่ไม่อยู่ใน permitAll | anonymous request</x:v>
+        <x:v>GET /private-test | anonymous request</x:v>
       </x:c>
       <x:c r="D18" s="257" t="str">
-        <x:v>ต้อง authenticated / ถูกปฏิเสธตาม Spring Security</x:v>
+        <x:v>403 Forbidden</x:v>
       </x:c>
       <x:c r="E18" s="270" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="F18" s="244"/>
       <x:c r="G18" s="244"/>
@@ -19371,13 +19421,13 @@
         <x:v>Auth mechanism</x:v>
       </x:c>
       <x:c r="C19" s="263" t="str">
-        <x:v>request ที่ไม่มี form login/basic credentials | anonymous request</x:v>
+        <x:v>ตรวจ SecurityFilterChain | ตรวจ filter ที่ถูกสร้าง</x:v>
       </x:c>
       <x:c r="D19" s="264" t="str">
-        <x:v>formLogin และ httpBasic ถูก disable ตาม config</x:v>
+        <x:v>ไม่มี form login filter และ basic auth filter</x:v>
       </x:c>
       <x:c r="E19" s="271" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="F19" s="244"/>
       <x:c r="G19" s="244"/>
@@ -19388,7 +19438,7 @@
       <x:c r="L19" s="244"/>
       <x:c r="M19" s="244"/>
     </x:row>
-    <x:row r="20">
+    <x:row r="20" ht="15" hidden="0" customHeight="1">
       <x:c r="A20" s="244"/>
       <x:c r="B20" s="244"/>
       <x:c r="C20" s="244"/>
@@ -19403,7 +19453,7 @@
       <x:c r="L20" s="244"/>
       <x:c r="M20" s="244"/>
     </x:row>
-    <x:row r="21">
+    <x:row r="21" ht="15" hidden="0" customHeight="1">
       <x:c r="A21" s="244"/>
       <x:c r="B21" s="244"/>
       <x:c r="C21" s="244"/>
@@ -19418,7 +19468,7 @@
       <x:c r="L21" s="244"/>
       <x:c r="M21" s="244"/>
     </x:row>
-    <x:row r="22">
+    <x:row r="22" ht="15" hidden="0" customHeight="1">
       <x:c r="A22" s="244"/>
       <x:c r="B22" s="244"/>
       <x:c r="C22" s="244"/>
@@ -19433,7 +19483,7 @@
       <x:c r="L22" s="244"/>
       <x:c r="M22" s="244"/>
     </x:row>
-    <x:row r="23">
+    <x:row r="23" ht="15" hidden="0" customHeight="1">
       <x:c r="A23" s="244"/>
       <x:c r="B23" s="244"/>
       <x:c r="C23" s="244"/>
@@ -19448,7 +19498,7 @@
       <x:c r="L23" s="244"/>
       <x:c r="M23" s="244"/>
     </x:row>
-    <x:row r="24">
+    <x:row r="24" ht="15" hidden="0" customHeight="1">
       <x:c r="A24" s="244"/>
       <x:c r="B24" s="244"/>
       <x:c r="C24" s="244"/>

</xml_diff>

<commit_message>
test: complete interest service and controller tests
</commit_message>
<xml_diff>
--- a/test/test-cases/CPFriendFinder_TestCases.xlsx
+++ b/test/test-cases/CPFriendFinder_TestCases.xlsx
@@ -2,19 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Scenario Summary" sheetId="1" r:id="R7243b80e31a84036"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="2" r:id="R52aac16da1464c59"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Case Design &amp; Test Results" sheetId="3" r:id="R65b22af242014631"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS001" sheetId="4" r:id="Rc95338479c994bc0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS002" sheetId="5" r:id="Ra6380f9cc3dd409e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS003" sheetId="6" r:id="Rf85a2abb220b4313"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS004" sheetId="7" r:id="R95efdda6f084450a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS005" sheetId="8" r:id="R6141c0d1f4cf4903"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS006" sheetId="9" r:id="Re81420da6a45480a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defect Summary" sheetId="10" r:id="Rcd240c31e64c49b7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Summary Report" sheetId="11" r:id="R14aeb3fee81c4d2e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution Log" sheetId="12" r:id="Re6d1aacf04e24ed7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision Table" sheetId="13" r:id="Rd098b0c8971e4f2d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Scenario Summary" sheetId="1" r:id="R44fbdd05216d46b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="2" r:id="Rc5c1dc8483c047a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Case Design &amp; Test Results" sheetId="3" r:id="Rf28f50952fe044e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS001" sheetId="4" r:id="R6e8768a45a3f48d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS002" sheetId="5" r:id="Rfca473407a484c01"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS003" sheetId="6" r:id="R7b4ab64554014013"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS004" sheetId="7" r:id="R95cc202aea614200"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS005" sheetId="8" r:id="R4dc4f65d607d45e4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS006" sheetId="9" r:id="R430eb6d86f5c4b60"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defect Summary" sheetId="10" r:id="R5b6cf531b649411b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Summary Report" sheetId="11" r:id="R03990f21f6964d6a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution Log" sheetId="12" r:id="R527e9af607b04ef4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision Table" sheetId="13" r:id="R68208e3b9baf4c9d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1580,7 +1580,7 @@
       </x:c>
       <x:c r="E8" s="259" t="n">
         <x:f>COUNTIFS('Test Case Design &amp; Test Results'!$B$4:$B$80,B8,'Test Case Design &amp; Test Results'!$J$4:$J$80,"Pass")</x:f>
-        <x:v>0</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F8" s="259" t="n">
         <x:f>COUNTIFS('Test Case Design &amp; Test Results'!$B$4:$B$80,B8,'Test Case Design &amp; Test Results'!$J$4:$J$80,"Fail")</x:f>
@@ -1588,7 +1588,7 @@
       </x:c>
       <x:c r="G8" s="259" t="n">
         <x:f>COUNTIFS('Test Case Design &amp; Test Results'!$B$4:$B$80,B8,'Test Case Design &amp; Test Results'!$J$4:$J$80,"Not Run")+COUNTIFS('Test Case Design &amp; Test Results'!$B$4:$B$80,B8,'Test Case Design &amp; Test Results'!$J$4:$J$80,"Waiting Frontend")</x:f>
-        <x:v>4</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H8" s="260" t="n">
         <x:f>COUNTIFS('Test Case Design &amp; Test Results'!$B$4:$B$80,B8,'Test Case Design &amp; Test Results'!$J$4:$J$80,"Blocked")</x:f>
@@ -4690,7 +4690,7 @@
       </x:c>
       <x:c r="B6" s="270" t="n">
         <x:f>COUNTIF('Test Case Design &amp; Test Results'!$J$4:$J$80,"Pass")+COUNTIF('Test Case Design &amp; Test Results'!$J$4:$J$80,"Fail")+COUNTIF('Test Case Design &amp; Test Results'!$J$4:$J$80,"Blocked")</x:f>
-        <x:v>39</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="C6" s="244"/>
       <x:c r="D6" s="244" t="str">
@@ -4716,7 +4716,7 @@
       </x:c>
       <x:c r="B7" s="270" t="n">
         <x:f>COUNTIF('Test Case Design &amp; Test Results'!$J$4:$J$80,"Pass")</x:f>
-        <x:v>39</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="C7" s="244"/>
       <x:c r="D7" s="244" t="str">
@@ -4768,12 +4768,18 @@
       </x:c>
       <x:c r="B9" s="271" t="n">
         <x:f>COUNTIF('Test Case Design &amp; Test Results'!$J$4:$J$80,"Not Run")+COUNTIF('Test Case Design &amp; Test Results'!$J$4:$J$80,"Waiting Frontend")</x:f>
-        <x:v>9</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="C9" s="244"/>
-      <x:c r="D9" s="244"/>
-      <x:c r="E9" s="244"/>
-      <x:c r="F9" s="244"/>
+      <x:c r="D9" s="244" t="str">
+        <x:v>TS005</x:v>
+      </x:c>
+      <x:c r="E9" s="244" t="str">
+        <x:v>4/4 Pass</x:v>
+      </x:c>
+      <x:c r="F9" s="244" t="str">
+        <x:v>56.569 s</x:v>
+      </x:c>
       <x:c r="G9" s="244"/>
       <x:c r="H9" s="244"/>
       <x:c r="I9" s="244"/>
@@ -6388,14 +6394,30 @@
       <x:c r="M8" s="244"/>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
-      <x:c r="A9" s="244"/>
-      <x:c r="B9" s="244"/>
-      <x:c r="C9" s="244"/>
-      <x:c r="D9" s="244"/>
-      <x:c r="E9" s="244"/>
-      <x:c r="F9" s="244"/>
-      <x:c r="G9" s="244"/>
-      <x:c r="H9" s="244"/>
+      <x:c r="A9" s="244" t="str">
+        <x:v>TS005</x:v>
+      </x:c>
+      <x:c r="B9" s="244" t="str">
+        <x:v>2026-10-01 17:20:05 +07:00</x:v>
+      </x:c>
+      <x:c r="C9" s="244" t="str">
+        <x:v>InterestServiceTest + InterestControllerMvcTest</x:v>
+      </x:c>
+      <x:c r="D9" s="244" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E9" s="244" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F9" s="244" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G9" s="244" t="str">
+        <x:v>0 / 0</x:v>
+      </x:c>
+      <x:c r="H9" s="244" t="str">
+        <x:v>BUILD SUCCESS</x:v>
+      </x:c>
       <x:c r="I9" s="244"/>
       <x:c r="J9" s="244"/>
       <x:c r="K9" s="244"/>
@@ -9979,7 +10001,7 @@
         <x:v>InterestService.allInterests</x:v>
       </x:c>
       <x:c r="F20" s="270" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Passed - Unit/MVC</x:v>
       </x:c>
       <x:c r="G20" s="244"/>
       <x:c r="H20" s="244"/>
@@ -10006,7 +10028,7 @@
         <x:v>InterestController.apiInterestAll</x:v>
       </x:c>
       <x:c r="F21" s="270" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Passed - Unit/MVC</x:v>
       </x:c>
       <x:c r="G21" s="244"/>
       <x:c r="H21" s="244"/>
@@ -12912,7 +12934,7 @@
         <x:v>2026-10-01 17:01:57 | 7/7 passed | BUILD SUCCESS</x:v>
       </x:c>
     </x:row>
-    <x:row r="43" ht="15" hidden="0" customHeight="1">
+    <x:row r="43" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A43" s="270" t="str">
         <x:v>UC-INT-01</x:v>
       </x:c>
@@ -12938,18 +12960,22 @@
         <x:v>คืน list เดียวกัน</x:v>
       </x:c>
       <x:c r="I43" s="261" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>ผ่านตาม Expected Result</x:v>
       </x:c>
       <x:c r="J43" s="270" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K43" s="261" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
       </x:c>
-      <x:c r="L43" s="261" t="str"/>
-      <x:c r="M43" s="261" t="str"/>
-    </x:row>
-    <x:row r="44" ht="15" hidden="0" customHeight="1">
+      <x:c r="L43" s="261" t="str">
+        <x:v>InterestServiceTest.allInterests_withData_returnsRepositoryList</x:v>
+      </x:c>
+      <x:c r="M43" s="261" t="str">
+        <x:v>2026-10-01 17:20:05 | 4/4 passed | BUILD SUCCESS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A44" s="270" t="str">
         <x:v>UC-INT-01</x:v>
       </x:c>
@@ -12975,18 +13001,22 @@
         <x:v>คืน empty list</x:v>
       </x:c>
       <x:c r="I44" s="261" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>ผ่านตาม Expected Result</x:v>
       </x:c>
       <x:c r="J44" s="270" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K44" s="261" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
       </x:c>
-      <x:c r="L44" s="261" t="str"/>
-      <x:c r="M44" s="261" t="str"/>
-    </x:row>
-    <x:row r="45" ht="15" hidden="0" customHeight="1">
+      <x:c r="L44" s="261" t="str">
+        <x:v>InterestServiceTest.allInterests_withoutData_returnsEmptyList</x:v>
+      </x:c>
+      <x:c r="M44" s="261" t="str">
+        <x:v>2026-10-01 17:20:05 | 4/4 passed | BUILD SUCCESS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A45" s="270" t="str">
         <x:v>UC-INT-01</x:v>
       </x:c>
@@ -13009,21 +13039,25 @@
         <x:v>InterestService คืน list จำลอง</x:v>
       </x:c>
       <x:c r="H45" s="261" t="str">
-        <x:v>200 OK + list payload</x:v>
+        <x:v>200 OK + name=Music + active=true</x:v>
       </x:c>
       <x:c r="I45" s="261" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>ผ่านตาม Expected Result</x:v>
       </x:c>
       <x:c r="J45" s="270" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K45" s="261" t="str">
-        <x:v>MVC Slice Test</x:v>
-      </x:c>
-      <x:c r="L45" s="261" t="str"/>
-      <x:c r="M45" s="261" t="str"/>
-    </x:row>
-    <x:row r="46" ht="15" hidden="0" customHeight="1">
+        <x:v>Controller MVC Test (standalone MockMvc)</x:v>
+      </x:c>
+      <x:c r="L45" s="261" t="str">
+        <x:v>InterestControllerMvcTest.getInterests_withData_returnsOkAndList</x:v>
+      </x:c>
+      <x:c r="M45" s="261" t="str">
+        <x:v>2026-10-01 17:20:05 | 4/4 passed | BUILD SUCCESS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A46" s="270" t="str">
         <x:v>UC-INT-01</x:v>
       </x:c>
@@ -13046,19 +13080,23 @@
         <x:v>InterestService คืน empty list</x:v>
       </x:c>
       <x:c r="H46" s="261" t="str">
-        <x:v>200 OK + []</x:v>
+        <x:v>200 OK + empty JSON array</x:v>
       </x:c>
       <x:c r="I46" s="261" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>ผ่านตาม Expected Result</x:v>
       </x:c>
       <x:c r="J46" s="270" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K46" s="261" t="str">
-        <x:v>MVC Slice Test</x:v>
-      </x:c>
-      <x:c r="L46" s="261" t="str"/>
-      <x:c r="M46" s="261" t="str"/>
+        <x:v>Controller MVC Test (standalone MockMvc)</x:v>
+      </x:c>
+      <x:c r="L46" s="261" t="str">
+        <x:v>InterestControllerMvcTest.getInterests_withoutData_returnsOkAndEmptyList</x:v>
+      </x:c>
+      <x:c r="M46" s="261" t="str">
+        <x:v>2026-10-01 17:20:05 | 4/4 passed | BUILD SUCCESS</x:v>
+      </x:c>
     </x:row>
     <x:row r="47" ht="15" hidden="0" customHeight="1">
       <x:c r="A47" s="270" t="str">
@@ -20697,7 +20735,7 @@
       <x:c r="L1" s="244"/>
       <x:c r="M1" s="244"/>
     </x:row>
-    <x:row r="2">
+    <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="244"/>
       <x:c r="B2" s="244"/>
       <x:c r="C2" s="244"/>
@@ -20793,7 +20831,7 @@
         <x:v>Test Method</x:v>
       </x:c>
       <x:c r="B7" s="261" t="str">
-        <x:v>JUnit 5 + Mockito / @WebMvcTest + MockMvc</x:v>
+        <x:v>JUnit 5 + Mockito / standalone MockMvc</x:v>
       </x:c>
       <x:c r="C7" s="244"/>
       <x:c r="D7" s="244"/>
@@ -20812,7 +20850,7 @@
         <x:v>Preconditions</x:v>
       </x:c>
       <x:c r="B8" s="261" t="str">
-        <x:v>Unit: mock InterestRepository; MVC: mock InterestService</x:v>
+        <x:v>Unit: mock InterestRepository; Controller: mock InterestService</x:v>
       </x:c>
       <x:c r="C8" s="244"/>
       <x:c r="D8" s="244"/>
@@ -20864,7 +20902,7 @@
       <x:c r="L10" s="244"/>
       <x:c r="M10" s="244"/>
     </x:row>
-    <x:row r="11">
+    <x:row r="11" ht="15" hidden="0" customHeight="1">
       <x:c r="A11" s="244"/>
       <x:c r="B11" s="244"/>
       <x:c r="C11" s="244"/>
@@ -20918,7 +20956,7 @@
         <x:v>คืน list เดียวกัน</x:v>
       </x:c>
       <x:c r="E13" s="269" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="F13" s="244"/>
       <x:c r="G13" s="244"/>
@@ -20943,7 +20981,7 @@
         <x:v>คืน empty list</x:v>
       </x:c>
       <x:c r="E14" s="270" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="F14" s="244"/>
       <x:c r="G14" s="244"/>
@@ -20965,10 +21003,10 @@
         <x:v>GET /api/interest | InterestService คืน list จำลอง</x:v>
       </x:c>
       <x:c r="D15" s="257" t="str">
-        <x:v>200 OK + list payload</x:v>
+        <x:v>200 OK + name=Music + active=true</x:v>
       </x:c>
       <x:c r="E15" s="270" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="F15" s="244"/>
       <x:c r="G15" s="244"/>
@@ -20990,10 +21028,10 @@
         <x:v>GET /api/interest | InterestService คืน empty list</x:v>
       </x:c>
       <x:c r="D16" s="264" t="str">
-        <x:v>200 OK + []</x:v>
+        <x:v>200 OK + empty JSON array</x:v>
       </x:c>
       <x:c r="E16" s="271" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="F16" s="244"/>
       <x:c r="G16" s="244"/>
@@ -21004,7 +21042,7 @@
       <x:c r="L16" s="244"/>
       <x:c r="M16" s="244"/>
     </x:row>
-    <x:row r="17">
+    <x:row r="17" ht="15" hidden="0" customHeight="1">
       <x:c r="A17" s="244"/>
       <x:c r="B17" s="244"/>
       <x:c r="C17" s="244"/>
@@ -21019,7 +21057,7 @@
       <x:c r="L17" s="244"/>
       <x:c r="M17" s="244"/>
     </x:row>
-    <x:row r="18">
+    <x:row r="18" ht="15" hidden="0" customHeight="1">
       <x:c r="A18" s="244"/>
       <x:c r="B18" s="244"/>
       <x:c r="C18" s="244"/>
@@ -21034,7 +21072,7 @@
       <x:c r="L18" s="244"/>
       <x:c r="M18" s="244"/>
     </x:row>
-    <x:row r="19">
+    <x:row r="19" ht="15" hidden="0" customHeight="1">
       <x:c r="A19" s="244"/>
       <x:c r="B19" s="244"/>
       <x:c r="C19" s="244"/>
@@ -21049,7 +21087,7 @@
       <x:c r="L19" s="244"/>
       <x:c r="M19" s="244"/>
     </x:row>
-    <x:row r="20">
+    <x:row r="20" ht="15" hidden="0" customHeight="1">
       <x:c r="A20" s="244"/>
       <x:c r="B20" s="244"/>
       <x:c r="C20" s="244"/>

</xml_diff>

<commit_message>
docs: record final SQA regression results
</commit_message>
<xml_diff>
--- a/test/test-cases/CPFriendFinder_TestCases.xlsx
+++ b/test/test-cases/CPFriendFinder_TestCases.xlsx
@@ -2,28 +2,28 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Scenario Summary" sheetId="1" r:id="R155dd025343844c3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="2" r:id="Ra9783afc30ae4963"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Case Design &amp; Test Results" sheetId="3" r:id="Re2f09161a9a04a1e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS001" sheetId="4" r:id="R7c87c4c44e4f4979"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS002" sheetId="5" r:id="Rf448aa5a6550432c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS003" sheetId="6" r:id="Rf963d1b619de4aba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS004" sheetId="7" r:id="R3b031185f7244887"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS005" sheetId="8" r:id="R1ef2fa5b3ffd4e60"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS006" sheetId="9" r:id="R1c33bd6056b94262"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defect Summary" sheetId="10" r:id="Raa92b7cbe96149a4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Summary Report" sheetId="11" r:id="R8f5e78c2705340f4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution Log" sheetId="12" r:id="R7c8009fb04b84d2d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision Table" sheetId="13" r:id="R63812b47a6b54247"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS007" sheetId="14" r:id="R1bc050d41d694865"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS008" sheetId="15" r:id="R270723ae35b2405d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS009" sheetId="16" r:id="Rea12172f8af54557"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS010" sheetId="17" r:id="R61ac863dd55a4a7b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS011" sheetId="18" r:id="Rd0b522fb11564739"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS012" sheetId="19" r:id="R0c5b5346edce4aa8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS013" sheetId="20" r:id="R00a0a79a0ddc4f83"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS014" sheetId="21" r:id="R3caaa4304c314c99"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS015" sheetId="22" r:id="Rd731d797f39d4205"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Scenario Summary" sheetId="1" r:id="R0277716d87f047de"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="2" r:id="Rc6374cf44bcd42e7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Case Design &amp; Test Results" sheetId="3" r:id="R8512b04b0e5c4881"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS001" sheetId="4" r:id="Ra524785c84b546fb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS002" sheetId="5" r:id="R721b4c90dcd84acf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS003" sheetId="6" r:id="R2aee8885a6924fa4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS004" sheetId="7" r:id="R09d4fa8814834945"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS005" sheetId="8" r:id="Rce5b50276da74cf7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS006" sheetId="9" r:id="R9079c87995644658"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defect Summary" sheetId="10" r:id="Ra4472b3bb9504501"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Summary Report" sheetId="11" r:id="Red682a7bd0964f79"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution Log" sheetId="12" r:id="R703d927b508c46a5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision Table" sheetId="13" r:id="R4c7b7fe1d28e44e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS007" sheetId="14" r:id="Rab3738139aa84959"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS008" sheetId="15" r:id="Rb7167ea83faf4cf4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS009" sheetId="16" r:id="R182113f33df745b9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS010" sheetId="17" r:id="R17bf49a39ed44a6b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS011" sheetId="18" r:id="R3001de88461b41ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS012" sheetId="19" r:id="R4d75c43f17d64817"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS013" sheetId="20" r:id="Rff10755fb0284ec0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS014" sheetId="21" r:id="R9d7bdc4064ed48b7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS015" sheetId="22" r:id="R9e93fbb17e414cb3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1980,13 +1980,13 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="E22" s="287" t="n">
-        <x:v>0</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="F22" s="287" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="G22" s="287" t="n">
-        <x:v>15</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H22" s="287" t="n">
         <x:v>0</x:v>
@@ -2013,13 +2013,13 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="E23" s="287" t="n">
-        <x:v>0</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="F23" s="287" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="G23" s="287" t="n">
-        <x:v>12</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H23" s="287" t="n">
         <x:v>0</x:v>
@@ -2079,13 +2079,13 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E25" s="287" t="n">
-        <x:v>0</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F25" s="287" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="G25" s="287" t="n">
-        <x:v>10</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H25" s="287" t="n">
         <x:v>0</x:v>
@@ -2112,13 +2112,13 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="E26" s="287" t="n">
-        <x:v>0</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="F26" s="287" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="G26" s="287" t="n">
-        <x:v>12</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H26" s="287" t="n">
         <x:v>0</x:v>
@@ -2145,13 +2145,13 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="E27" s="287" t="n">
-        <x:v>0</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="F27" s="287" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="G27" s="287" t="n">
-        <x:v>12</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H27" s="287" t="n">
         <x:v>0</x:v>
@@ -2178,13 +2178,13 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="E28" s="287" t="n">
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="F28" s="287" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="G28" s="287" t="n">
-        <x:v>8</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H28" s="287" t="n">
         <x:v>0</x:v>
@@ -2197,31 +2197,31 @@
       <x:c r="L28" s="244"/>
       <x:c r="M28" s="244"/>
     </x:row>
-    <x:row r="29" ht="34" customHeight="1">
+    <x:row r="29" ht="42" customHeight="1">
       <x:c r="A29" s="287"/>
       <x:c r="B29" s="287" t="str">
         <x:v>Latest Total</x:v>
       </x:c>
       <x:c r="C29" s="287" t="str">
-        <x:v>Test design through TS015 based on current develop; actual results recorded through TS008 + existing Matching tests</x:v>
+        <x:v>Executed coverage through TS015 based on current develop</x:v>
       </x:c>
       <x:c r="D29" s="287" t="n">
         <x:v>171</x:v>
       </x:c>
       <x:c r="E29" s="287" t="n">
-        <x:v>101</x:v>
+        <x:v>170</x:v>
       </x:c>
       <x:c r="F29" s="287" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G29" s="287" t="n">
-        <x:v>69</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H29" s="287" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I29" s="287" t="str">
-        <x:v>Documented executed=102; full Maven regression=103 incl. FriendApplicationTests; only DEF-001 failed</x:v>
+        <x:v>Documented: 171 executed / 170 Pass / 1 Fail. Final Maven regression: 172 tests / 171 Pass / 1 Fail; only DEF-001 failed.</x:v>
       </x:c>
       <x:c r="J29" s="244"/>
       <x:c r="K29" s="244"/>
@@ -3388,7 +3388,7 @@
       <x:c r="L3" s="244"/>
       <x:c r="M3" s="244"/>
     </x:row>
-    <x:row r="4" ht="48" customHeight="1">
+    <x:row r="4" ht="66" customHeight="1">
       <x:c r="A4" s="275" t="str">
         <x:v>DEF-001</x:v>
       </x:c>
@@ -3420,7 +3420,7 @@
         <x:v>UserServiceTest.updateProfile_blankFirstname_clearsFirstname</x:v>
       </x:c>
       <x:c r="K4" s="278" t="str">
-        <x:v>Retest PENDING หลัง Backend แก้; reproduced in full regression 2026-10-07 18:20:44 (103 tests, only this failure)</x:v>
+        <x:v>OPEN / Retest pending after Backend fix. Reproduced in final full regression 2026-10-07 19:24:20 +07:00: 172 tests, 171 Pass, 1 Fail, 0 Errors, 0 Skipped. Only failure: UserServiceTest.updateProfile_blankFirstname_clearsFirstname — expected null, actual 'Old'.</x:v>
       </x:c>
       <x:c r="L4" s="244"/>
       <x:c r="M4" s="244"/>
@@ -5173,13 +5173,13 @@
       </x:c>
       <x:c r="C14" s="287"/>
       <x:c r="D14" s="287" t="str">
-        <x:v>TS008 focused</x:v>
+        <x:v>TS009 Friend Requests</x:v>
       </x:c>
       <x:c r="E14" s="287" t="str">
         <x:v>15/15 Pass</x:v>
       </x:c>
       <x:c r="F14" s="287" t="str">
-        <x:v>14.237 s</x:v>
+        <x:v>12.395 s</x:v>
       </x:c>
       <x:c r="G14" s="244"/>
       <x:c r="H14" s="244"/>
@@ -5194,17 +5194,17 @@
         <x:v>Executed documented cases</x:v>
       </x:c>
       <x:c r="B15" s="287" t="n">
-        <x:v>102</x:v>
+        <x:v>171</x:v>
       </x:c>
       <x:c r="C15" s="287"/>
       <x:c r="D15" s="287" t="str">
-        <x:v>Latest full regression</x:v>
+        <x:v>TS010 Friendship / Discovery</x:v>
       </x:c>
       <x:c r="E15" s="287" t="str">
-        <x:v>103 tests / 102 Pass / 1 Fail</x:v>
+        <x:v>12/12 Pass</x:v>
       </x:c>
       <x:c r="F15" s="287" t="str">
-        <x:v>29.874 s</x:v>
+        <x:v>12.256 s</x:v>
       </x:c>
       <x:c r="G15" s="244"/>
       <x:c r="H15" s="244"/>
@@ -5219,17 +5219,17 @@
         <x:v>Pass</x:v>
       </x:c>
       <x:c r="B16" s="287" t="n">
-        <x:v>101</x:v>
+        <x:v>170</x:v>
       </x:c>
       <x:c r="C16" s="287"/>
       <x:c r="D16" s="287" t="str">
-        <x:v>Known failure</x:v>
+        <x:v>TS012 Notifications</x:v>
       </x:c>
       <x:c r="E16" s="287" t="str">
-        <x:v>DEF-001 / PRO-007</x:v>
+        <x:v>10/10 Pass</x:v>
       </x:c>
       <x:c r="F16" s="287" t="str">
-        <x:v>Expected null; Actual Old</x:v>
+        <x:v>12.299 s</x:v>
       </x:c>
       <x:c r="G16" s="244"/>
       <x:c r="H16" s="244"/>
@@ -5248,13 +5248,13 @@
       </x:c>
       <x:c r="C17" s="287"/>
       <x:c r="D17" s="287" t="str">
-        <x:v>Matching existing tests</x:v>
+        <x:v>TS013 Chat Rooms</x:v>
       </x:c>
       <x:c r="E17" s="287" t="str">
-        <x:v>10/10 Pass</x:v>
+        <x:v>12/12 Pass</x:v>
       </x:c>
       <x:c r="F17" s="287" t="str">
-        <x:v>included in full regression</x:v>
+        <x:v>37.995 s</x:v>
       </x:c>
       <x:c r="G17" s="244"/>
       <x:c r="H17" s="244"/>
@@ -5269,17 +5269,17 @@
         <x:v>Not Run / Planned</x:v>
       </x:c>
       <x:c r="B18" s="287" t="n">
-        <x:v>69</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C18" s="287"/>
       <x:c r="D18" s="287" t="str">
-        <x:v>Full regression time</x:v>
+        <x:v>TS014 Chat Messages</x:v>
       </x:c>
       <x:c r="E18" s="287" t="str">
-        <x:v>2026-10-07 18:20:44 +07:00</x:v>
+        <x:v>12/12 Pass</x:v>
       </x:c>
       <x:c r="F18" s="287" t="str">
-        <x:v>BUILD FAILURE (known defect only)</x:v>
+        <x:v>22.276 s</x:v>
       </x:c>
       <x:c r="G18" s="244"/>
       <x:c r="H18" s="244"/>
@@ -5294,17 +5294,17 @@
         <x:v>Retest</x:v>
       </x:c>
       <x:c r="B19" s="287" t="str">
-        <x:v>PENDING</x:v>
+        <x:v>PENDING — DEF-001</x:v>
       </x:c>
       <x:c r="C19" s="287"/>
       <x:c r="D19" s="287" t="str">
-        <x:v>New regression</x:v>
+        <x:v>TS015 Frontend Contract</x:v>
       </x:c>
       <x:c r="E19" s="287" t="str">
-        <x:v>None detected</x:v>
+        <x:v>8/8 Pass</x:v>
       </x:c>
       <x:c r="F19" s="287" t="str">
-        <x:v>DEF-001 reproduced</x:v>
+        <x:v>15.982 s</x:v>
       </x:c>
       <x:c r="G19" s="244"/>
       <x:c r="H19" s="244"/>
@@ -5314,13 +5314,19 @@
       <x:c r="L19" s="244"/>
       <x:c r="M19" s="244"/>
     </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="244"/>
-      <x:c r="B20" s="244"/>
-      <x:c r="C20" s="244"/>
-      <x:c r="D20" s="244"/>
-      <x:c r="E20" s="244"/>
-      <x:c r="F20" s="244"/>
+    <x:row r="20" ht="30" customHeight="1">
+      <x:c r="A20" s="287"/>
+      <x:c r="B20" s="287"/>
+      <x:c r="C20" s="287"/>
+      <x:c r="D20" s="287" t="str">
+        <x:v>Final full regression</x:v>
+      </x:c>
+      <x:c r="E20" s="287" t="str">
+        <x:v>172 tests / 171 Pass / 1 Fail / 0 Errors / 0 Skipped</x:v>
+      </x:c>
+      <x:c r="F20" s="287" t="str">
+        <x:v>01:09 min</x:v>
+      </x:c>
       <x:c r="G20" s="244"/>
       <x:c r="H20" s="244"/>
       <x:c r="I20" s="244"/>
@@ -5329,13 +5335,19 @@
       <x:c r="L20" s="244"/>
       <x:c r="M20" s="244"/>
     </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="244"/>
-      <x:c r="B21" s="244"/>
-      <x:c r="C21" s="244"/>
-      <x:c r="D21" s="244"/>
-      <x:c r="E21" s="244"/>
-      <x:c r="F21" s="244"/>
+    <x:row r="21" ht="30" customHeight="1">
+      <x:c r="A21" s="287"/>
+      <x:c r="B21" s="287"/>
+      <x:c r="C21" s="287"/>
+      <x:c r="D21" s="287" t="str">
+        <x:v>Finished</x:v>
+      </x:c>
+      <x:c r="E21" s="287" t="str">
+        <x:v>2026-10-07 19:24:20 +07:00</x:v>
+      </x:c>
+      <x:c r="F21" s="287" t="str">
+        <x:v>BUILD FAILURE — DEF-001 only; no new regression</x:v>
+      </x:c>
       <x:c r="G21" s="244"/>
       <x:c r="H21" s="244"/>
       <x:c r="I21" s="244"/>
@@ -6956,105 +6968,217 @@
       <x:c r="L14" s="244"/>
       <x:c r="M14" s="244"/>
     </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="244"/>
-      <x:c r="B15" s="244"/>
-      <x:c r="C15" s="244"/>
-      <x:c r="D15" s="244"/>
-      <x:c r="E15" s="244"/>
-      <x:c r="F15" s="244"/>
-      <x:c r="G15" s="244"/>
-      <x:c r="H15" s="244"/>
+    <x:row r="15" ht="30" customHeight="1">
+      <x:c r="A15" s="287" t="str">
+        <x:v>TS009</x:v>
+      </x:c>
+      <x:c r="B15" s="287" t="str">
+        <x:v>2026-10-07 18:43:45 +07:00</x:v>
+      </x:c>
+      <x:c r="C15" s="287" t="str">
+        <x:v>FriendRequestServiceTest + FriendRequestControllerMvcTest</x:v>
+      </x:c>
+      <x:c r="D15" s="287" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="E15" s="287" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="F15" s="287" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G15" s="287" t="str">
+        <x:v>0 / 0</x:v>
+      </x:c>
+      <x:c r="H15" s="287" t="str">
+        <x:v>BUILD SUCCESS</x:v>
+      </x:c>
       <x:c r="I15" s="244"/>
       <x:c r="J15" s="244"/>
       <x:c r="K15" s="244"/>
       <x:c r="L15" s="244"/>
       <x:c r="M15" s="244"/>
     </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="244"/>
-      <x:c r="B16" s="244"/>
-      <x:c r="C16" s="244"/>
-      <x:c r="D16" s="244"/>
-      <x:c r="E16" s="244"/>
-      <x:c r="F16" s="244"/>
-      <x:c r="G16" s="244"/>
-      <x:c r="H16" s="244"/>
+    <x:row r="16" ht="30" customHeight="1">
+      <x:c r="A16" s="287" t="str">
+        <x:v>TS010</x:v>
+      </x:c>
+      <x:c r="B16" s="287" t="str">
+        <x:v>2026-10-07 18:49:55 +07:00</x:v>
+      </x:c>
+      <x:c r="C16" s="287" t="str">
+        <x:v>FriendshipServiceTest + FriendshipControllerMvcTest + UserDiscoveryServiceTest + UserDiscoveryControllerMvcTest</x:v>
+      </x:c>
+      <x:c r="D16" s="287" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="E16" s="287" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="F16" s="287" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G16" s="287" t="str">
+        <x:v>0 / 0</x:v>
+      </x:c>
+      <x:c r="H16" s="287" t="str">
+        <x:v>BUILD SUCCESS</x:v>
+      </x:c>
       <x:c r="I16" s="244"/>
       <x:c r="J16" s="244"/>
       <x:c r="K16" s="244"/>
       <x:c r="L16" s="244"/>
       <x:c r="M16" s="244"/>
     </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="244"/>
-      <x:c r="B17" s="244"/>
-      <x:c r="C17" s="244"/>
-      <x:c r="D17" s="244"/>
-      <x:c r="E17" s="244"/>
-      <x:c r="F17" s="244"/>
-      <x:c r="G17" s="244"/>
-      <x:c r="H17" s="244"/>
+    <x:row r="17" ht="30" customHeight="1">
+      <x:c r="A17" s="287" t="str">
+        <x:v>TS012</x:v>
+      </x:c>
+      <x:c r="B17" s="287" t="str">
+        <x:v>2026-10-07 19:02:08 +07:00</x:v>
+      </x:c>
+      <x:c r="C17" s="287" t="str">
+        <x:v>NotificationServiceTest + NotificationControllerMvcTest</x:v>
+      </x:c>
+      <x:c r="D17" s="287" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="E17" s="287" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F17" s="287" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G17" s="287" t="str">
+        <x:v>0 / 0</x:v>
+      </x:c>
+      <x:c r="H17" s="287" t="str">
+        <x:v>BUILD SUCCESS</x:v>
+      </x:c>
       <x:c r="I17" s="244"/>
       <x:c r="J17" s="244"/>
       <x:c r="K17" s="244"/>
       <x:c r="L17" s="244"/>
       <x:c r="M17" s="244"/>
     </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="244"/>
-      <x:c r="B18" s="244"/>
-      <x:c r="C18" s="244"/>
-      <x:c r="D18" s="244"/>
-      <x:c r="E18" s="244"/>
-      <x:c r="F18" s="244"/>
-      <x:c r="G18" s="244"/>
-      <x:c r="H18" s="244"/>
+    <x:row r="18" ht="30" customHeight="1">
+      <x:c r="A18" s="287" t="str">
+        <x:v>TS013</x:v>
+      </x:c>
+      <x:c r="B18" s="287" t="str">
+        <x:v>2026-10-07 19:09:36 +07:00</x:v>
+      </x:c>
+      <x:c r="C18" s="287" t="str">
+        <x:v>ChatRoomServiceTest + ChatRoomControllerMvcTest</x:v>
+      </x:c>
+      <x:c r="D18" s="287" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="E18" s="287" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="F18" s="287" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G18" s="287" t="str">
+        <x:v>0 / 0</x:v>
+      </x:c>
+      <x:c r="H18" s="287" t="str">
+        <x:v>BUILD SUCCESS</x:v>
+      </x:c>
       <x:c r="I18" s="244"/>
       <x:c r="J18" s="244"/>
       <x:c r="K18" s="244"/>
       <x:c r="L18" s="244"/>
       <x:c r="M18" s="244"/>
     </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="244"/>
-      <x:c r="B19" s="244"/>
-      <x:c r="C19" s="244"/>
-      <x:c r="D19" s="244"/>
-      <x:c r="E19" s="244"/>
-      <x:c r="F19" s="244"/>
-      <x:c r="G19" s="244"/>
-      <x:c r="H19" s="244"/>
+    <x:row r="19" ht="30" customHeight="1">
+      <x:c r="A19" s="287" t="str">
+        <x:v>TS014</x:v>
+      </x:c>
+      <x:c r="B19" s="287" t="str">
+        <x:v>2026-10-07 19:16:14 +07:00</x:v>
+      </x:c>
+      <x:c r="C19" s="287" t="str">
+        <x:v>ChatMessageServiceTest + ChatMessageControllerMvcTest</x:v>
+      </x:c>
+      <x:c r="D19" s="287" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="E19" s="287" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="F19" s="287" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G19" s="287" t="str">
+        <x:v>0 / 0</x:v>
+      </x:c>
+      <x:c r="H19" s="287" t="str">
+        <x:v>BUILD SUCCESS</x:v>
+      </x:c>
       <x:c r="I19" s="244"/>
       <x:c r="J19" s="244"/>
       <x:c r="K19" s="244"/>
       <x:c r="L19" s="244"/>
       <x:c r="M19" s="244"/>
     </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="244"/>
-      <x:c r="B20" s="244"/>
-      <x:c r="C20" s="244"/>
-      <x:c r="D20" s="244"/>
-      <x:c r="E20" s="244"/>
-      <x:c r="F20" s="244"/>
-      <x:c r="G20" s="244"/>
-      <x:c r="H20" s="244"/>
+    <x:row r="20" ht="30" customHeight="1">
+      <x:c r="A20" s="287" t="str">
+        <x:v>TS015</x:v>
+      </x:c>
+      <x:c r="B20" s="287" t="str">
+        <x:v>2026-10-07 19:20:07 +07:00</x:v>
+      </x:c>
+      <x:c r="C20" s="287" t="str">
+        <x:v>FriendNotificationChatContractTest</x:v>
+      </x:c>
+      <x:c r="D20" s="287" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E20" s="287" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="F20" s="287" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G20" s="287" t="str">
+        <x:v>0 / 0</x:v>
+      </x:c>
+      <x:c r="H20" s="287" t="str">
+        <x:v>BUILD SUCCESS</x:v>
+      </x:c>
       <x:c r="I20" s="244"/>
       <x:c r="J20" s="244"/>
       <x:c r="K20" s="244"/>
       <x:c r="L20" s="244"/>
       <x:c r="M20" s="244"/>
     </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="244"/>
-      <x:c r="B21" s="244"/>
-      <x:c r="C21" s="244"/>
-      <x:c r="D21" s="244"/>
-      <x:c r="E21" s="244"/>
-      <x:c r="F21" s="244"/>
-      <x:c r="G21" s="244"/>
-      <x:c r="H21" s="244"/>
+    <x:row r="21" ht="30" customHeight="1">
+      <x:c r="A21" s="287" t="str">
+        <x:v>REG-20261007-FINAL</x:v>
+      </x:c>
+      <x:c r="B21" s="287" t="str">
+        <x:v>2026-10-07 19:24:20 +07:00</x:v>
+      </x:c>
+      <x:c r="C21" s="287" t="str">
+        <x:v>Final clean full regression after TS009-TS015</x:v>
+      </x:c>
+      <x:c r="D21" s="287" t="n">
+        <x:v>172</x:v>
+      </x:c>
+      <x:c r="E21" s="287" t="n">
+        <x:v>171</x:v>
+      </x:c>
+      <x:c r="F21" s="287" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G21" s="287" t="str">
+        <x:v>0 / 0</x:v>
+      </x:c>
+      <x:c r="H21" s="287" t="str">
+        <x:v>BUILD FAILURE — DEF-001 only</x:v>
+      </x:c>
       <x:c r="I21" s="244"/>
       <x:c r="J21" s="244"/>
       <x:c r="K21" s="244"/>
@@ -10803,12 +10927,12 @@
       <x:c r="D9" s="47"/>
       <x:c r="E9" s="47"/>
     </x:row>
-    <x:row r="10" ht="42" customHeight="1">
+    <x:row r="10" ht="52" customHeight="1">
       <x:c r="A10" s="47" t="str">
         <x:v>Test Data / Stub Return</x:v>
       </x:c>
       <x:c r="B10" s="47" t="str">
-        <x:v>senderId/receiverId/requestId UUID, PENDING/ACCEPTED/DECLINED states, session userId</x:v>
+        <x:v>senderId/receiverId/requestId UUID, PENDING/ACCEPTED/DECLINED states, session userId | Executed: 2026-10-07 18:43:45 +07:00 | 15/15 Pass | BUILD SUCCESS | 12.395 s</x:v>
       </x:c>
       <x:c r="C10" s="47"/>
       <x:c r="D10" s="47"/>
@@ -10852,7 +10976,7 @@
         <x:v>save PENDING request, publish FriendRequestSentEvent, return FriendRequestResponse</x:v>
       </x:c>
       <x:c r="E13" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="34" customHeight="1">
@@ -10869,7 +10993,7 @@
         <x:v>400 BAD_REQUEST: Cannot send a friend request to yourself</x:v>
       </x:c>
       <x:c r="E14" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="34" customHeight="1">
@@ -10886,7 +11010,7 @@
         <x:v>409 CONFLICT: Users are already friends</x:v>
       </x:c>
       <x:c r="E15" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="48" customHeight="1">
@@ -10903,7 +11027,7 @@
         <x:v>409 CONFLICT: A pending friend request already exists</x:v>
       </x:c>
       <x:c r="E16" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="34" customHeight="1">
@@ -10920,7 +11044,7 @@
         <x:v>404 NOT_FOUND: User not found</x:v>
       </x:c>
       <x:c r="E17" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="48" customHeight="1">
@@ -10937,7 +11061,7 @@
         <x:v>return pending incoming responses mapped with sender profile/interests</x:v>
       </x:c>
       <x:c r="E18" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="48" customHeight="1">
@@ -10954,7 +11078,7 @@
         <x:v>return pending outgoing responses mapped with receiver profile/interests</x:v>
       </x:c>
       <x:c r="E19" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="48" customHeight="1">
@@ -10971,7 +11095,7 @@
         <x:v>create Friendship, mark ACCEPTED/respondedAt, publish FriendRequestAcceptedEvent</x:v>
       </x:c>
       <x:c r="E20" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="48" customHeight="1">
@@ -10988,7 +11112,7 @@
         <x:v>mark request ACCEPTED without saving duplicate Friendship</x:v>
       </x:c>
       <x:c r="E21" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="34" customHeight="1">
@@ -11005,7 +11129,7 @@
         <x:v>403 FORBIDDEN: Only the receiver can respond to this request</x:v>
       </x:c>
       <x:c r="E22" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="34" customHeight="1">
@@ -11022,7 +11146,7 @@
         <x:v>409 CONFLICT: Friend request is no longer pending</x:v>
       </x:c>
       <x:c r="E23" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="34" customHeight="1">
@@ -11039,7 +11163,7 @@
         <x:v>404 NOT_FOUND: Friend request not found</x:v>
       </x:c>
       <x:c r="E24" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="34" customHeight="1">
@@ -11056,7 +11180,7 @@
         <x:v>mark DECLINED + respondedAt and return response</x:v>
       </x:c>
       <x:c r="E25" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="34" customHeight="1">
@@ -11073,7 +11197,7 @@
         <x:v>201 Created + FriendRequestResponse</x:v>
       </x:c>
       <x:c r="E26" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="48" customHeight="1">
@@ -11090,7 +11214,7 @@
         <x:v>receiverId null -&gt; 400 VALIDATION_ERROR; missing session -&gt; 401 Unauthorized</x:v>
       </x:c>
       <x:c r="E27" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -11216,12 +11340,12 @@
       <x:c r="D9" s="47"/>
       <x:c r="E9" s="47"/>
     </x:row>
-    <x:row r="10" ht="42" customHeight="1">
+    <x:row r="10" ht="52" customHeight="1">
       <x:c r="A10" s="47" t="str">
         <x:v>Test Data / Stub Return</x:v>
       </x:c>
       <x:c r="B10" s="47" t="str">
-        <x:v>friendId/userId UUID, ACTIVE/BLOCKED candidates, department/year filters</x:v>
+        <x:v>friendId/userId UUID, ACTIVE/BLOCKED candidates, department/year filters | Executed: 2026-10-07 18:49:55 +07:00 | 12/12 Pass | BUILD SUCCESS | 12.256 s</x:v>
       </x:c>
       <x:c r="C10" s="47"/>
       <x:c r="D10" s="47"/>
@@ -11265,7 +11389,7 @@
         <x:v>return FriendResponse list including profile, bio, active interests and createdAt</x:v>
       </x:c>
       <x:c r="E13" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="34" customHeight="1">
@@ -11282,7 +11406,7 @@
         <x:v>404 NOT_FOUND: User not found</x:v>
       </x:c>
       <x:c r="E14" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="34" customHeight="1">
@@ -11299,7 +11423,7 @@
         <x:v>delete friendship successfully</x:v>
       </x:c>
       <x:c r="E15" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="34" customHeight="1">
@@ -11316,7 +11440,7 @@
         <x:v>404 NOT_FOUND: Friendship not found</x:v>
       </x:c>
       <x:c r="E16" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="34" customHeight="1">
@@ -11333,7 +11457,7 @@
         <x:v>200 OK + FriendResponse list</x:v>
       </x:c>
       <x:c r="E17" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="34" customHeight="1">
@@ -11350,7 +11474,7 @@
         <x:v>204 No Content</x:v>
       </x:c>
       <x:c r="E18" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="34" customHeight="1">
@@ -11367,7 +11491,7 @@
         <x:v>return [] without loading candidate users</x:v>
       </x:c>
       <x:c r="E19" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="60" customHeight="1">
@@ -11384,7 +11508,7 @@
         <x:v>exclude self/friends/pending; return only eligible candidate</x:v>
       </x:c>
       <x:c r="E20" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="34" customHeight="1">
@@ -11401,7 +11525,7 @@
         <x:v>exclude non-ACTIVE candidates</x:v>
       </x:c>
       <x:c r="E21" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="48" customHeight="1">
@@ -11418,7 +11542,7 @@
         <x:v>trim + equalsIgnoreCase; matching candidate remains</x:v>
       </x:c>
       <x:c r="E22" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="34" customHeight="1">
@@ -11435,7 +11559,7 @@
         <x:v>return only year=3 candidate</x:v>
       </x:c>
       <x:c r="E23" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="34" customHeight="1">
@@ -11452,7 +11576,7 @@
         <x:v>200 OK; missing session -&gt; 401 Unauthorized</x:v>
       </x:c>
       <x:c r="E24" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -11578,12 +11702,12 @@
       <x:c r="D9" s="47"/>
       <x:c r="E9" s="47"/>
     </x:row>
-    <x:row r="10" ht="42" customHeight="1">
+    <x:row r="10" ht="52" customHeight="1">
       <x:c r="A10" s="47" t="str">
         <x:v>Test Data / Stub Return</x:v>
       </x:c>
       <x:c r="B10" s="47" t="str">
-        <x:v>Interest sets for 0/50/66.67/100% matching, friend/pending exclusion</x:v>
+        <x:v>Interest sets for 0/50/66.67/100% matching, friend/pending exclusion | Executed: 2026-10-07 19:24:20 +07:00 | 10/10 Pass in final full regression</x:v>
       </x:c>
       <x:c r="C10" s="47"/>
       <x:c r="D10" s="47"/>
@@ -11906,12 +12030,12 @@
       <x:c r="D9" s="47"/>
       <x:c r="E9" s="47"/>
     </x:row>
-    <x:row r="10" ht="42" customHeight="1">
+    <x:row r="10" ht="52" customHeight="1">
       <x:c r="A10" s="47" t="str">
         <x:v>Test Data / Stub Return</x:v>
       </x:c>
       <x:c r="B10" s="47" t="str">
-        <x:v>userId/notificationId UUID, unread flag, page/size, FriendRequest events and Message</x:v>
+        <x:v>userId/notificationId UUID, unread flag, page/size, FriendRequest events and Message | Executed: 2026-10-07 19:02:08 +07:00 | 10/10 Pass | BUILD SUCCESS | 12.299 s</x:v>
       </x:c>
       <x:c r="C10" s="47"/>
       <x:c r="D10" s="47"/>
@@ -11955,7 +12079,7 @@
         <x:v>return NotificationResponse content</x:v>
       </x:c>
       <x:c r="E13" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="34" customHeight="1">
@@ -11972,7 +12096,7 @@
         <x:v>return only unread notifications</x:v>
       </x:c>
       <x:c r="E14" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="34" customHeight="1">
@@ -11989,7 +12113,7 @@
         <x:v>page clamps to 0; size clamps to 50</x:v>
       </x:c>
       <x:c r="E15" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="34" customHeight="1">
@@ -12006,7 +12130,7 @@
         <x:v>return 3</x:v>
       </x:c>
       <x:c r="E16" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="34" customHeight="1">
@@ -12023,7 +12147,7 @@
         <x:v>update only notification owned by user</x:v>
       </x:c>
       <x:c r="E17" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="34" customHeight="1">
@@ -12040,7 +12164,7 @@
         <x:v>mark user's notifications read</x:v>
       </x:c>
       <x:c r="E18" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="48" customHeight="1">
@@ -12057,7 +12181,7 @@
         <x:v>save notification and push to /topic/notifications/{userId}</x:v>
       </x:c>
       <x:c r="E19" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="34" customHeight="1">
@@ -12074,7 +12198,7 @@
         <x:v>save and push accepted notification</x:v>
       </x:c>
       <x:c r="E20" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="60" customHeight="1">
@@ -12091,7 +12215,7 @@
         <x:v>reuse/update existing notification instead of creating duplicate; skip sender</x:v>
       </x:c>
       <x:c r="E21" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="48" customHeight="1">
@@ -12108,7 +12232,7 @@
         <x:v>GET -&gt; 200; mark read/read-all -&gt; 204; missing session -&gt; 401</x:v>
       </x:c>
       <x:c r="E22" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -13306,7 +13430,7 @@
         <x:v>FriendRequestService.send</x:v>
       </x:c>
       <x:c r="F46" s="287" t="str">
-        <x:v>Planned / Not Run</x:v>
+        <x:v>Passed - Unit</x:v>
       </x:c>
       <x:c r="G46" s="244"/>
       <x:c r="H46" s="244"/>
@@ -13333,7 +13457,7 @@
         <x:v>FriendRequestService</x:v>
       </x:c>
       <x:c r="F47" s="287" t="str">
-        <x:v>Planned / Not Run</x:v>
+        <x:v>Passed - Unit</x:v>
       </x:c>
       <x:c r="G47" s="244"/>
       <x:c r="H47" s="244"/>
@@ -13360,7 +13484,7 @@
         <x:v>FriendRequestController + CreateFriendRequestRequest</x:v>
       </x:c>
       <x:c r="F48" s="287" t="str">
-        <x:v>Planned / Not Run</x:v>
+        <x:v>Passed - MVC</x:v>
       </x:c>
       <x:c r="G48" s="244"/>
       <x:c r="H48" s="244"/>
@@ -13387,7 +13511,7 @@
         <x:v>FriendshipService + FriendshipController</x:v>
       </x:c>
       <x:c r="F49" s="287" t="str">
-        <x:v>Planned / Not Run</x:v>
+        <x:v>Passed - Unit/MVC</x:v>
       </x:c>
       <x:c r="G49" s="244"/>
       <x:c r="H49" s="244"/>
@@ -13414,7 +13538,7 @@
         <x:v>UserDiscoveryService + UserDiscoveryController</x:v>
       </x:c>
       <x:c r="F50" s="287" t="str">
-        <x:v>Planned / Not Run</x:v>
+        <x:v>Passed - Unit/MVC</x:v>
       </x:c>
       <x:c r="G50" s="244"/>
       <x:c r="H50" s="244"/>
@@ -13495,7 +13619,7 @@
         <x:v>NotificationService + NotificationController</x:v>
       </x:c>
       <x:c r="F53" s="287" t="str">
-        <x:v>Planned / Not Run</x:v>
+        <x:v>Passed - Unit/MVC</x:v>
       </x:c>
       <x:c r="G53" s="244"/>
       <x:c r="H53" s="244"/>
@@ -13522,7 +13646,7 @@
         <x:v>NotificationService + NotificationFactory</x:v>
       </x:c>
       <x:c r="F54" s="287" t="str">
-        <x:v>Planned / Not Run</x:v>
+        <x:v>Passed - Unit/MVC</x:v>
       </x:c>
       <x:c r="G54" s="244"/>
       <x:c r="H54" s="244"/>
@@ -13549,7 +13673,7 @@
         <x:v>ChatRoomService</x:v>
       </x:c>
       <x:c r="F55" s="287" t="str">
-        <x:v>Planned / Not Run</x:v>
+        <x:v>Passed - Unit</x:v>
       </x:c>
       <x:c r="G55" s="244"/>
       <x:c r="H55" s="244"/>
@@ -13576,7 +13700,7 @@
         <x:v>ChatRoomService + ChatRoomController</x:v>
       </x:c>
       <x:c r="F56" s="287" t="str">
-        <x:v>Planned / Not Run</x:v>
+        <x:v>Passed - Unit/MVC</x:v>
       </x:c>
       <x:c r="G56" s="244"/>
       <x:c r="H56" s="244"/>
@@ -13603,7 +13727,7 @@
         <x:v>ChatMessageService</x:v>
       </x:c>
       <x:c r="F57" s="287" t="str">
-        <x:v>Planned / Not Run</x:v>
+        <x:v>Passed - Unit</x:v>
       </x:c>
       <x:c r="G57" s="244"/>
       <x:c r="H57" s="244"/>
@@ -13630,7 +13754,7 @@
         <x:v>ChatMessageController + ChatMessagePayload</x:v>
       </x:c>
       <x:c r="F58" s="287" t="str">
-        <x:v>Planned / Not Run</x:v>
+        <x:v>Passed - MVC</x:v>
       </x:c>
       <x:c r="G58" s="244"/>
       <x:c r="H58" s="244"/>
@@ -13657,7 +13781,7 @@
         <x:v>static/js/friend.js</x:v>
       </x:c>
       <x:c r="F59" s="287" t="str">
-        <x:v>Planned / Not Run</x:v>
+        <x:v>Passed - Contract</x:v>
       </x:c>
       <x:c r="G59" s="244"/>
       <x:c r="H59" s="244"/>
@@ -13684,7 +13808,7 @@
         <x:v>static/js/notification.js</x:v>
       </x:c>
       <x:c r="F60" s="287" t="str">
-        <x:v>Planned / Not Run</x:v>
+        <x:v>Passed - Contract</x:v>
       </x:c>
       <x:c r="G60" s="244"/>
       <x:c r="H60" s="244"/>
@@ -14407,12 +14531,12 @@
       <x:c r="D9" s="47"/>
       <x:c r="E9" s="47"/>
     </x:row>
-    <x:row r="10" ht="42" customHeight="1">
+    <x:row r="10" ht="52" customHeight="1">
       <x:c r="A10" s="47" t="str">
         <x:v>Test Data / Stub Return</x:v>
       </x:c>
       <x:c r="B10" s="47" t="str">
-        <x:v>GROUP/DIRECT rooms, public/private password, interest IDs, member counts, roles, session userId</x:v>
+        <x:v>GROUP/DIRECT rooms, public/private password, interest IDs, member counts, roles, session userId | Executed: 2026-10-07 19:09:36 +07:00 | 12/12 Pass | BUILD SUCCESS | 37.995 s</x:v>
       </x:c>
       <x:c r="C10" s="47"/>
       <x:c r="D10" s="47"/>
@@ -14456,7 +14580,7 @@
         <x:v>GROUP room, trimmed name, maxMembers default 10, owner membership created</x:v>
       </x:c>
       <x:c r="E13" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="34" customHeight="1">
@@ -14473,7 +14597,7 @@
         <x:v>400 BAD_REQUEST: Password is required for private rooms</x:v>
       </x:c>
       <x:c r="E14" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="34" customHeight="1">
@@ -14490,7 +14614,7 @@
         <x:v>store passwordHash, not raw password</x:v>
       </x:c>
       <x:c r="E15" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="48" customHeight="1">
@@ -14507,7 +14631,7 @@
         <x:v>400 BAD_REQUEST: One or more interests do not exist or are inactive</x:v>
       </x:c>
       <x:c r="E16" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="48" customHeight="1">
@@ -14524,7 +14648,7 @@
         <x:v>return intersection only; empty-member rooms excluded</x:v>
       </x:c>
       <x:c r="E17" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="34" customHeight="1">
@@ -14541,7 +14665,7 @@
         <x:v>409 CONFLICT: Already a member of this room</x:v>
       </x:c>
       <x:c r="E18" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="34" customHeight="1">
@@ -14558,7 +14682,7 @@
         <x:v>403 FORBIDDEN: Invalid room password</x:v>
       </x:c>
       <x:c r="E19" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="34" customHeight="1">
@@ -14575,7 +14699,7 @@
         <x:v>409 CONFLICT: Room is full</x:v>
       </x:c>
       <x:c r="E20" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="34" customHeight="1">
@@ -14592,7 +14716,7 @@
         <x:v>404 NOT_FOUND: You are not a member of this room</x:v>
       </x:c>
       <x:c r="E21" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="48" customHeight="1">
@@ -14609,7 +14733,7 @@
         <x:v>403 permission error or 400 maxMembers error</x:v>
       </x:c>
       <x:c r="E22" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="48" customHeight="1">
@@ -14626,7 +14750,7 @@
         <x:v>self -&gt; 400; nonfriend -&gt; 404 'You can only chat directly with friends'</x:v>
       </x:c>
       <x:c r="E23" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="48" customHeight="1">
@@ -14643,7 +14767,7 @@
         <x:v>create -&gt; 201; join/direct -&gt; 200; leave -&gt; 204; protected operations missing session -&gt; 401</x:v>
       </x:c>
       <x:c r="E24" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -14769,12 +14893,12 @@
       <x:c r="D9" s="47"/>
       <x:c r="E9" s="47"/>
     </x:row>
-    <x:row r="10" ht="42" customHeight="1">
+    <x:row r="10" ht="52" customHeight="1">
       <x:c r="A10" s="47" t="str">
         <x:v>Test Data / Stub Return</x:v>
       </x:c>
       <x:c r="B10" s="47" t="str">
-        <x:v>TEXT payloads, room/message/user UUIDs, before Instant, limit boundary, soft-delete ownership</x:v>
+        <x:v>TEXT payloads, room/message/user UUIDs, before Instant, limit boundary, soft-delete ownership | Executed: 2026-10-07 19:16:14 +07:00 | 12/12 Pass | BUILD SUCCESS | 22.276 s</x:v>
       </x:c>
       <x:c r="C10" s="47"/>
       <x:c r="D10" s="47"/>
@@ -14818,7 +14942,7 @@
         <x:v>403 FORBIDDEN: You are not a member of this room</x:v>
       </x:c>
       <x:c r="E13" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="34" customHeight="1">
@@ -14835,7 +14959,7 @@
         <x:v>return [] without MessageRepository history query</x:v>
       </x:c>
       <x:c r="E14" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="48" customHeight="1">
@@ -14852,7 +14976,7 @@
         <x:v>return oldest-&gt;newest and mark lastReadAt</x:v>
       </x:c>
       <x:c r="E15" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="48" customHeight="1">
@@ -14869,7 +14993,7 @@
         <x:v>limit clamps to 1..100 and before query is used</x:v>
       </x:c>
       <x:c r="E16" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="48" customHeight="1">
@@ -14886,7 +15010,7 @@
         <x:v>use correct count query based on lastReadAt</x:v>
       </x:c>
       <x:c r="E17" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="60" customHeight="1">
@@ -14903,7 +15027,7 @@
         <x:v>persist message, broadcast, notifyNewMessage, update sender lastReadAt</x:v>
       </x:c>
       <x:c r="E18" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="48" customHeight="1">
@@ -14920,7 +15044,7 @@
         <x:v>broadcast response with id=null; do not persist or notify</x:v>
       </x:c>
       <x:c r="E19" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="48" customHeight="1">
@@ -14937,7 +15061,7 @@
         <x:v>blank defaults TEXT; invalid -&gt; 400 BAD_REQUEST 'Invalid messageType'</x:v>
       </x:c>
       <x:c r="E20" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="34" customHeight="1">
@@ -14954,7 +15078,7 @@
         <x:v>set deletedAt and save (soft delete)</x:v>
       </x:c>
       <x:c r="E21" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="34" customHeight="1">
@@ -14971,7 +15095,7 @@
         <x:v>403 FORBIDDEN: You can only delete your own messages</x:v>
       </x:c>
       <x:c r="E22" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="34" customHeight="1">
@@ -14988,7 +15112,7 @@
         <x:v>400 BAD_REQUEST: before must be an ISO-8601 instant...</x:v>
       </x:c>
       <x:c r="E23" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="48" customHeight="1">
@@ -15005,7 +15129,7 @@
         <x:v>blank content -&gt; 400 VALIDATION_ERROR; valid session/content -&gt; 201; missing session -&gt; 401</x:v>
       </x:c>
       <x:c r="E24" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -15131,12 +15255,12 @@
       <x:c r="D9" s="47"/>
       <x:c r="E9" s="47"/>
     </x:row>
-    <x:row r="10" ht="42" customHeight="1">
+    <x:row r="10" ht="52" customHeight="1">
       <x:c r="A10" s="47" t="str">
         <x:v>Test Data / Stub Return</x:v>
       </x:c>
       <x:c r="B10" s="47" t="str">
-        <x:v>Expected REST endpoints/methods/credentials/payloads used by friend and notification pages</x:v>
+        <x:v>Expected REST endpoints/methods/credentials/payloads used by friend and notification pages | Executed: 2026-10-07 19:20:07 +07:00 | 8/8 Pass | BUILD SUCCESS | 15.982 s</x:v>
       </x:c>
       <x:c r="C10" s="47"/>
       <x:c r="D10" s="47"/>
@@ -15180,7 +15304,7 @@
         <x:v>frontend retrieves current user and supports id/userId response shape</x:v>
       </x:c>
       <x:c r="E13" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="48" customHeight="1">
@@ -15197,7 +15321,7 @@
         <x:v>friend page uses current Friendship API and expected FriendResponse fields</x:v>
       </x:c>
       <x:c r="E14" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="48" customHeight="1">
@@ -15214,7 +15338,7 @@
         <x:v>opening friend conversation uses current direct-room endpoint and room.id</x:v>
       </x:c>
       <x:c r="E15" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="34" customHeight="1">
@@ -15231,7 +15355,7 @@
         <x:v>message history endpoint/method matches ChatMessageController</x:v>
       </x:c>
       <x:c r="E16" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="48" customHeight="1">
@@ -15248,7 +15372,7 @@
         <x:v>send payload matches ChatMessagePayload REST contract</x:v>
       </x:c>
       <x:c r="E17" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="34" customHeight="1">
@@ -15265,7 +15389,7 @@
         <x:v>notification page loads incoming FriendRequestResponse list</x:v>
       </x:c>
       <x:c r="E18" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="48" customHeight="1">
@@ -15282,7 +15406,7 @@
         <x:v>buttons call current FriendRequestController endpoints</x:v>
       </x:c>
       <x:c r="E19" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="48" customHeight="1">
@@ -15299,7 +15423,7 @@
         <x:v>page loads NotificationResponse and filters NEW_MESSAGE</x:v>
       </x:c>
       <x:c r="E20" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -21288,17 +21412,21 @@
       <x:c r="H148" s="47" t="str">
         <x:v>save PENDING request, publish FriendRequestSentEvent, return FriendRequestResponse</x:v>
       </x:c>
-      <x:c r="I148" s="47"/>
+      <x:c r="I148" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
       <x:c r="J148" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K148" s="47" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
       </x:c>
       <x:c r="L148" s="47" t="str">
-        <x:v>Planned: FriendRequestServiceTest.send_validUsers_savesPendingAndPublishesEvent</x:v>
-      </x:c>
-      <x:c r="M148" s="47"/>
+        <x:v>FriendRequestServiceTest.send_validUsers_savesPendingAndPublishesEvent</x:v>
+      </x:c>
+      <x:c r="M148" s="47" t="str">
+        <x:v>2026-10-07 18:43:45 +07:00 | 15/15 Pass | BUILD SUCCESS | 12.395 s</x:v>
+      </x:c>
     </x:row>
     <x:row r="149" ht="34" customHeight="1">
       <x:c r="A149" s="47" t="str">
@@ -21325,17 +21453,21 @@
       <x:c r="H149" s="47" t="str">
         <x:v>400 BAD_REQUEST: Cannot send a friend request to yourself</x:v>
       </x:c>
-      <x:c r="I149" s="47"/>
+      <x:c r="I149" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
       <x:c r="J149" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K149" s="47" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
       </x:c>
       <x:c r="L149" s="47" t="str">
-        <x:v>Planned: FriendRequestServiceTest.send_toSelf_returnsBadRequest</x:v>
-      </x:c>
-      <x:c r="M149" s="47"/>
+        <x:v>FriendRequestServiceTest.send_toSelf_returnsBadRequest</x:v>
+      </x:c>
+      <x:c r="M149" s="47" t="str">
+        <x:v>2026-10-07 18:43:45 +07:00 | 15/15 Pass | BUILD SUCCESS | 12.395 s</x:v>
+      </x:c>
     </x:row>
     <x:row r="150" ht="34" customHeight="1">
       <x:c r="A150" s="47" t="str">
@@ -21362,17 +21494,21 @@
       <x:c r="H150" s="47" t="str">
         <x:v>409 CONFLICT: Users are already friends</x:v>
       </x:c>
-      <x:c r="I150" s="47"/>
+      <x:c r="I150" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
       <x:c r="J150" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K150" s="47" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
       </x:c>
       <x:c r="L150" s="47" t="str">
-        <x:v>Planned: FriendRequestServiceTest.send_existingFriendship_returnsConflict</x:v>
-      </x:c>
-      <x:c r="M150" s="47"/>
+        <x:v>FriendRequestServiceTest.send_existingFriendship_returnsConflict</x:v>
+      </x:c>
+      <x:c r="M150" s="47" t="str">
+        <x:v>2026-10-07 18:43:45 +07:00 | 15/15 Pass | BUILD SUCCESS | 12.395 s</x:v>
+      </x:c>
     </x:row>
     <x:row r="151" ht="34" customHeight="1">
       <x:c r="A151" s="47" t="str">
@@ -21399,17 +21535,21 @@
       <x:c r="H151" s="47" t="str">
         <x:v>409 CONFLICT: A pending friend request already exists</x:v>
       </x:c>
-      <x:c r="I151" s="47"/>
+      <x:c r="I151" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
       <x:c r="J151" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K151" s="47" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
       </x:c>
       <x:c r="L151" s="47" t="str">
-        <x:v>Planned: FriendRequestServiceTest.send_pendingRequest_returnsConflict</x:v>
-      </x:c>
-      <x:c r="M151" s="47"/>
+        <x:v>FriendRequestServiceTest.send_pendingRequest_returnsConflict</x:v>
+      </x:c>
+      <x:c r="M151" s="47" t="str">
+        <x:v>2026-10-07 18:43:45 +07:00 | 15/15 Pass | BUILD SUCCESS | 12.395 s</x:v>
+      </x:c>
     </x:row>
     <x:row r="152" ht="34" customHeight="1">
       <x:c r="A152" s="47" t="str">
@@ -21436,17 +21576,21 @@
       <x:c r="H152" s="47" t="str">
         <x:v>404 NOT_FOUND: User not found</x:v>
       </x:c>
-      <x:c r="I152" s="47"/>
+      <x:c r="I152" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
       <x:c r="J152" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K152" s="47" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
       </x:c>
       <x:c r="L152" s="47" t="str">
-        <x:v>Planned: FriendRequestServiceTest.send_receiverUnavailable_returnsNotFound</x:v>
-      </x:c>
-      <x:c r="M152" s="47"/>
+        <x:v>FriendRequestServiceTest.send_receiverUnavailable_returnsNotFound</x:v>
+      </x:c>
+      <x:c r="M152" s="47" t="str">
+        <x:v>2026-10-07 18:43:45 +07:00 | 15/15 Pass | BUILD SUCCESS | 12.395 s</x:v>
+      </x:c>
     </x:row>
     <x:row r="153" ht="34" customHeight="1">
       <x:c r="A153" s="47" t="str">
@@ -21473,17 +21617,21 @@
       <x:c r="H153" s="47" t="str">
         <x:v>return pending incoming responses mapped with sender profile/interests</x:v>
       </x:c>
-      <x:c r="I153" s="47"/>
+      <x:c r="I153" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
       <x:c r="J153" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K153" s="47" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
       </x:c>
       <x:c r="L153" s="47" t="str">
-        <x:v>Planned: FriendRequestServiceTest.incoming_returnsPendingRequests</x:v>
-      </x:c>
-      <x:c r="M153" s="47"/>
+        <x:v>FriendRequestServiceTest.incoming_returnsPendingRequests</x:v>
+      </x:c>
+      <x:c r="M153" s="47" t="str">
+        <x:v>2026-10-07 18:43:45 +07:00 | 15/15 Pass | BUILD SUCCESS | 12.395 s</x:v>
+      </x:c>
     </x:row>
     <x:row r="154" ht="34" customHeight="1">
       <x:c r="A154" s="47" t="str">
@@ -21510,17 +21658,21 @@
       <x:c r="H154" s="47" t="str">
         <x:v>return pending outgoing responses mapped with receiver profile/interests</x:v>
       </x:c>
-      <x:c r="I154" s="47"/>
+      <x:c r="I154" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
       <x:c r="J154" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K154" s="47" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
       </x:c>
       <x:c r="L154" s="47" t="str">
-        <x:v>Planned: FriendRequestServiceTest.outgoing_returnsPendingRequests</x:v>
-      </x:c>
-      <x:c r="M154" s="47"/>
+        <x:v>FriendRequestServiceTest.outgoing_returnsPendingRequests</x:v>
+      </x:c>
+      <x:c r="M154" s="47" t="str">
+        <x:v>2026-10-07 18:43:45 +07:00 | 15/15 Pass | BUILD SUCCESS | 12.395 s</x:v>
+      </x:c>
     </x:row>
     <x:row r="155" ht="34" customHeight="1">
       <x:c r="A155" s="47" t="str">
@@ -21547,17 +21699,21 @@
       <x:c r="H155" s="47" t="str">
         <x:v>create Friendship, mark ACCEPTED/respondedAt, publish FriendRequestAcceptedEvent</x:v>
       </x:c>
-      <x:c r="I155" s="47"/>
+      <x:c r="I155" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
       <x:c r="J155" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K155" s="47" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
       </x:c>
       <x:c r="L155" s="47" t="str">
-        <x:v>Planned: FriendRequestServiceTest.accept_validReceiver_createsFriendshipAndPublishesEvent</x:v>
-      </x:c>
-      <x:c r="M155" s="47"/>
+        <x:v>FriendRequestServiceTest.accept_validReceiver_createsFriendshipAndPublishesEvent</x:v>
+      </x:c>
+      <x:c r="M155" s="47" t="str">
+        <x:v>2026-10-07 18:43:45 +07:00 | 15/15 Pass | BUILD SUCCESS | 12.395 s</x:v>
+      </x:c>
     </x:row>
     <x:row r="156" ht="34" customHeight="1">
       <x:c r="A156" s="47" t="str">
@@ -21584,17 +21740,21 @@
       <x:c r="H156" s="47" t="str">
         <x:v>mark request ACCEPTED without saving duplicate Friendship</x:v>
       </x:c>
-      <x:c r="I156" s="47"/>
+      <x:c r="I156" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
       <x:c r="J156" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K156" s="47" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
       </x:c>
       <x:c r="L156" s="47" t="str">
-        <x:v>Planned: FriendRequestServiceTest.accept_existingFriendship_doesNotDuplicate</x:v>
-      </x:c>
-      <x:c r="M156" s="47"/>
+        <x:v>FriendRequestServiceTest.accept_existingFriendship_doesNotDuplicate</x:v>
+      </x:c>
+      <x:c r="M156" s="47" t="str">
+        <x:v>2026-10-07 18:43:45 +07:00 | 15/15 Pass | BUILD SUCCESS | 12.395 s</x:v>
+      </x:c>
     </x:row>
     <x:row r="157" ht="34" customHeight="1">
       <x:c r="A157" s="47" t="str">
@@ -21621,17 +21781,21 @@
       <x:c r="H157" s="47" t="str">
         <x:v>403 FORBIDDEN: Only the receiver can respond to this request</x:v>
       </x:c>
-      <x:c r="I157" s="47"/>
+      <x:c r="I157" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
       <x:c r="J157" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K157" s="47" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
       </x:c>
       <x:c r="L157" s="47" t="str">
-        <x:v>Planned: FriendRequestServiceTest.accept_nonReceiver_returnsForbidden</x:v>
-      </x:c>
-      <x:c r="M157" s="47"/>
+        <x:v>FriendRequestServiceTest.accept_nonReceiver_returnsForbidden</x:v>
+      </x:c>
+      <x:c r="M157" s="47" t="str">
+        <x:v>2026-10-07 18:43:45 +07:00 | 15/15 Pass | BUILD SUCCESS | 12.395 s</x:v>
+      </x:c>
     </x:row>
     <x:row r="158" ht="34" customHeight="1">
       <x:c r="A158" s="47" t="str">
@@ -21658,17 +21822,21 @@
       <x:c r="H158" s="47" t="str">
         <x:v>409 CONFLICT: Friend request is no longer pending</x:v>
       </x:c>
-      <x:c r="I158" s="47"/>
+      <x:c r="I158" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
       <x:c r="J158" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K158" s="47" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
       </x:c>
       <x:c r="L158" s="47" t="str">
-        <x:v>Planned: FriendRequestServiceTest.accept_nonPending_returnsConflict</x:v>
-      </x:c>
-      <x:c r="M158" s="47"/>
+        <x:v>FriendRequestServiceTest.accept_nonPending_returnsConflict</x:v>
+      </x:c>
+      <x:c r="M158" s="47" t="str">
+        <x:v>2026-10-07 18:43:45 +07:00 | 15/15 Pass | BUILD SUCCESS | 12.395 s</x:v>
+      </x:c>
     </x:row>
     <x:row r="159" ht="34" customHeight="1">
       <x:c r="A159" s="47" t="str">
@@ -21695,17 +21863,21 @@
       <x:c r="H159" s="47" t="str">
         <x:v>404 NOT_FOUND: Friend request not found</x:v>
       </x:c>
-      <x:c r="I159" s="47"/>
+      <x:c r="I159" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
       <x:c r="J159" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K159" s="47" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
       </x:c>
       <x:c r="L159" s="47" t="str">
-        <x:v>Planned: FriendRequestServiceTest.accept_missingRequest_returnsNotFound</x:v>
-      </x:c>
-      <x:c r="M159" s="47"/>
+        <x:v>FriendRequestServiceTest.accept_missingRequest_returnsNotFound</x:v>
+      </x:c>
+      <x:c r="M159" s="47" t="str">
+        <x:v>2026-10-07 18:43:45 +07:00 | 15/15 Pass | BUILD SUCCESS | 12.395 s</x:v>
+      </x:c>
     </x:row>
     <x:row r="160" ht="34" customHeight="1">
       <x:c r="A160" s="47" t="str">
@@ -21732,17 +21904,21 @@
       <x:c r="H160" s="47" t="str">
         <x:v>mark DECLINED + respondedAt and return response</x:v>
       </x:c>
-      <x:c r="I160" s="47"/>
+      <x:c r="I160" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
       <x:c r="J160" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K160" s="47" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
       </x:c>
       <x:c r="L160" s="47" t="str">
-        <x:v>Planned: FriendRequestServiceTest.decline_validReceiver_marksDeclined</x:v>
-      </x:c>
-      <x:c r="M160" s="47"/>
+        <x:v>FriendRequestServiceTest.decline_validReceiver_marksDeclined</x:v>
+      </x:c>
+      <x:c r="M160" s="47" t="str">
+        <x:v>2026-10-07 18:43:45 +07:00 | 15/15 Pass | BUILD SUCCESS | 12.395 s</x:v>
+      </x:c>
     </x:row>
     <x:row r="161" ht="34" customHeight="1">
       <x:c r="A161" s="47" t="str">
@@ -21769,17 +21945,21 @@
       <x:c r="H161" s="47" t="str">
         <x:v>201 Created + FriendRequestResponse</x:v>
       </x:c>
-      <x:c r="I161" s="47"/>
+      <x:c r="I161" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
       <x:c r="J161" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K161" s="47" t="str">
         <x:v>Standalone MockMvc</x:v>
       </x:c>
       <x:c r="L161" s="47" t="str">
-        <x:v>Planned: FriendRequestControllerMvcTest.send_validRequest_returnsCreated</x:v>
-      </x:c>
-      <x:c r="M161" s="47"/>
+        <x:v>FriendRequestControllerMvcTest.send_validRequest_returnsCreated</x:v>
+      </x:c>
+      <x:c r="M161" s="47" t="str">
+        <x:v>2026-10-07 18:43:45 +07:00 | 15/15 Pass | BUILD SUCCESS | 12.395 s</x:v>
+      </x:c>
     </x:row>
     <x:row r="162" ht="34" customHeight="1">
       <x:c r="A162" s="47" t="str">
@@ -21806,17 +21986,21 @@
       <x:c r="H162" s="47" t="str">
         <x:v>receiverId null -&gt; 400 VALIDATION_ERROR; missing session -&gt; 401 Unauthorized</x:v>
       </x:c>
-      <x:c r="I162" s="47"/>
+      <x:c r="I162" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
       <x:c r="J162" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K162" s="47" t="str">
         <x:v>Standalone MockMvc</x:v>
       </x:c>
       <x:c r="L162" s="47" t="str">
-        <x:v>Planned: FriendRequestControllerMvcTest.send_invalidInputOrSession_isRejected</x:v>
-      </x:c>
-      <x:c r="M162" s="47"/>
+        <x:v>FriendRequestControllerMvcTest.send_invalidInputOrSession_isRejected</x:v>
+      </x:c>
+      <x:c r="M162" s="47" t="str">
+        <x:v>2026-10-07 18:43:45 +07:00 | 15/15 Pass | BUILD SUCCESS | 12.395 s</x:v>
+      </x:c>
     </x:row>
     <x:row r="163" ht="34" customHeight="1">
       <x:c r="A163" s="47" t="str">
@@ -21843,17 +22027,21 @@
       <x:c r="H163" s="47" t="str">
         <x:v>return FriendResponse list including profile, bio, active interests and createdAt</x:v>
       </x:c>
-      <x:c r="I163" s="47"/>
+      <x:c r="I163" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
       <x:c r="J163" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K163" s="47" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
       </x:c>
       <x:c r="L163" s="47" t="str">
-        <x:v>Planned: FriendshipServiceTest.listFriends_returnsMappedFriends</x:v>
-      </x:c>
-      <x:c r="M163" s="47"/>
+        <x:v>FriendshipServiceTest.listFriends_returnsMappedFriends</x:v>
+      </x:c>
+      <x:c r="M163" s="47" t="str">
+        <x:v>2026-10-07 18:49:55 +07:00 | 12/12 Pass | BUILD SUCCESS | 12.256 s</x:v>
+      </x:c>
     </x:row>
     <x:row r="164" ht="34" customHeight="1">
       <x:c r="A164" s="47" t="str">
@@ -21880,17 +22068,21 @@
       <x:c r="H164" s="47" t="str">
         <x:v>404 NOT_FOUND: User not found</x:v>
       </x:c>
-      <x:c r="I164" s="47"/>
+      <x:c r="I164" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
       <x:c r="J164" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K164" s="47" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
       </x:c>
       <x:c r="L164" s="47" t="str">
-        <x:v>Planned: FriendshipServiceTest.listFriends_inactiveOrMissingUser_returnsNotFound</x:v>
-      </x:c>
-      <x:c r="M164" s="47"/>
+        <x:v>FriendshipServiceTest.listFriends_inactiveOrMissingUser_returnsNotFound</x:v>
+      </x:c>
+      <x:c r="M164" s="47" t="str">
+        <x:v>2026-10-07 18:49:55 +07:00 | 12/12 Pass | BUILD SUCCESS | 12.256 s</x:v>
+      </x:c>
     </x:row>
     <x:row r="165" ht="34" customHeight="1">
       <x:c r="A165" s="47" t="str">
@@ -21917,17 +22109,21 @@
       <x:c r="H165" s="47" t="str">
         <x:v>delete friendship successfully</x:v>
       </x:c>
-      <x:c r="I165" s="47"/>
+      <x:c r="I165" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
       <x:c r="J165" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K165" s="47" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
       </x:c>
       <x:c r="L165" s="47" t="str">
-        <x:v>Planned: FriendshipServiceTest.unfriend_existingFriendship_deletesRelation</x:v>
-      </x:c>
-      <x:c r="M165" s="47"/>
+        <x:v>FriendshipServiceTest.unfriend_existingFriendship_deletesRelation</x:v>
+      </x:c>
+      <x:c r="M165" s="47" t="str">
+        <x:v>2026-10-07 18:49:55 +07:00 | 12/12 Pass | BUILD SUCCESS | 12.256 s</x:v>
+      </x:c>
     </x:row>
     <x:row r="166" ht="34" customHeight="1">
       <x:c r="A166" s="47" t="str">
@@ -21954,17 +22150,21 @@
       <x:c r="H166" s="47" t="str">
         <x:v>404 NOT_FOUND: Friendship not found</x:v>
       </x:c>
-      <x:c r="I166" s="47"/>
+      <x:c r="I166" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
       <x:c r="J166" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K166" s="47" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
       </x:c>
       <x:c r="L166" s="47" t="str">
-        <x:v>Planned: FriendshipServiceTest.unfriend_missingFriendship_returnsNotFound</x:v>
-      </x:c>
-      <x:c r="M166" s="47"/>
+        <x:v>FriendshipServiceTest.unfriend_missingFriendship_returnsNotFound</x:v>
+      </x:c>
+      <x:c r="M166" s="47" t="str">
+        <x:v>2026-10-07 18:49:55 +07:00 | 12/12 Pass | BUILD SUCCESS | 12.256 s</x:v>
+      </x:c>
     </x:row>
     <x:row r="167" ht="34" customHeight="1">
       <x:c r="A167" s="47" t="str">
@@ -21991,17 +22191,21 @@
       <x:c r="H167" s="47" t="str">
         <x:v>200 OK + FriendResponse list</x:v>
       </x:c>
-      <x:c r="I167" s="47"/>
+      <x:c r="I167" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
       <x:c r="J167" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K167" s="47" t="str">
         <x:v>Standalone MockMvc</x:v>
       </x:c>
       <x:c r="L167" s="47" t="str">
-        <x:v>Planned: FriendshipControllerMvcTest.listFriends_withSession_returnsOk</x:v>
-      </x:c>
-      <x:c r="M167" s="47"/>
+        <x:v>FriendshipControllerMvcTest.listFriends_withSession_returnsOk</x:v>
+      </x:c>
+      <x:c r="M167" s="47" t="str">
+        <x:v>2026-10-07 18:49:55 +07:00 | 12/12 Pass | BUILD SUCCESS | 12.256 s</x:v>
+      </x:c>
     </x:row>
     <x:row r="168" ht="34" customHeight="1">
       <x:c r="A168" s="47" t="str">
@@ -22028,17 +22232,21 @@
       <x:c r="H168" s="47" t="str">
         <x:v>204 No Content</x:v>
       </x:c>
-      <x:c r="I168" s="47"/>
+      <x:c r="I168" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
       <x:c r="J168" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K168" s="47" t="str">
         <x:v>Standalone MockMvc</x:v>
       </x:c>
       <x:c r="L168" s="47" t="str">
-        <x:v>Planned: FriendshipControllerMvcTest.unfriend_validRequest_returnsNoContent</x:v>
-      </x:c>
-      <x:c r="M168" s="47"/>
+        <x:v>FriendshipControllerMvcTest.unfriend_validRequest_returnsNoContent</x:v>
+      </x:c>
+      <x:c r="M168" s="47" t="str">
+        <x:v>2026-10-07 18:49:55 +07:00 | 12/12 Pass | BUILD SUCCESS | 12.256 s</x:v>
+      </x:c>
     </x:row>
     <x:row r="169" ht="34" customHeight="1">
       <x:c r="A169" s="47" t="str">
@@ -22065,17 +22273,21 @@
       <x:c r="H169" s="47" t="str">
         <x:v>return [] without loading candidate users</x:v>
       </x:c>
-      <x:c r="I169" s="47"/>
+      <x:c r="I169" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
       <x:c r="J169" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K169" s="47" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
       </x:c>
       <x:c r="L169" s="47" t="str">
-        <x:v>Planned: UserDiscoveryServiceTest.discover_noMatches_returnsEmpty</x:v>
-      </x:c>
-      <x:c r="M169" s="47"/>
+        <x:v>UserDiscoveryServiceTest.discover_noMatches_returnsEmpty</x:v>
+      </x:c>
+      <x:c r="M169" s="47" t="str">
+        <x:v>2026-10-07 18:49:55 +07:00 | 12/12 Pass | BUILD SUCCESS | 12.256 s</x:v>
+      </x:c>
     </x:row>
     <x:row r="170" ht="34" customHeight="1">
       <x:c r="A170" s="47" t="str">
@@ -22102,17 +22314,21 @@
       <x:c r="H170" s="47" t="str">
         <x:v>exclude self/friends/pending; return only eligible candidate</x:v>
       </x:c>
-      <x:c r="I170" s="47"/>
+      <x:c r="I170" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
       <x:c r="J170" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K170" s="47" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
       </x:c>
       <x:c r="L170" s="47" t="str">
-        <x:v>Planned: UserDiscoveryServiceTest.discover_excludesSelfFriendsAndPending</x:v>
-      </x:c>
-      <x:c r="M170" s="47"/>
+        <x:v>UserDiscoveryServiceTest.discover_excludesSelfFriendsAndPending</x:v>
+      </x:c>
+      <x:c r="M170" s="47" t="str">
+        <x:v>2026-10-07 18:49:55 +07:00 | 12/12 Pass | BUILD SUCCESS | 12.256 s</x:v>
+      </x:c>
     </x:row>
     <x:row r="171" ht="34" customHeight="1">
       <x:c r="A171" s="47" t="str">
@@ -22139,17 +22355,21 @@
       <x:c r="H171" s="47" t="str">
         <x:v>exclude non-ACTIVE candidates</x:v>
       </x:c>
-      <x:c r="I171" s="47"/>
+      <x:c r="I171" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
       <x:c r="J171" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K171" s="47" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
       </x:c>
       <x:c r="L171" s="47" t="str">
-        <x:v>Planned: UserDiscoveryServiceTest.discover_excludesInactiveCandidates</x:v>
-      </x:c>
-      <x:c r="M171" s="47"/>
+        <x:v>UserDiscoveryServiceTest.discover_excludesInactiveCandidates</x:v>
+      </x:c>
+      <x:c r="M171" s="47" t="str">
+        <x:v>2026-10-07 18:49:55 +07:00 | 12/12 Pass | BUILD SUCCESS | 12.256 s</x:v>
+      </x:c>
     </x:row>
     <x:row r="172" ht="34" customHeight="1">
       <x:c r="A172" s="47" t="str">
@@ -22176,17 +22396,21 @@
       <x:c r="H172" s="47" t="str">
         <x:v>trim + equalsIgnoreCase; matching candidate remains</x:v>
       </x:c>
-      <x:c r="I172" s="47"/>
+      <x:c r="I172" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
       <x:c r="J172" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K172" s="47" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
       </x:c>
       <x:c r="L172" s="47" t="str">
-        <x:v>Planned: UserDiscoveryServiceTest.discover_departmentFilter_isTrimmedAndCaseInsensitive</x:v>
-      </x:c>
-      <x:c r="M172" s="47"/>
+        <x:v>UserDiscoveryServiceTest.discover_departmentFilter_isTrimmedAndCaseInsensitive</x:v>
+      </x:c>
+      <x:c r="M172" s="47" t="str">
+        <x:v>2026-10-07 18:49:55 +07:00 | 12/12 Pass | BUILD SUCCESS | 12.256 s</x:v>
+      </x:c>
     </x:row>
     <x:row r="173" ht="34" customHeight="1">
       <x:c r="A173" s="47" t="str">
@@ -22213,17 +22437,21 @@
       <x:c r="H173" s="47" t="str">
         <x:v>return only year=3 candidate</x:v>
       </x:c>
-      <x:c r="I173" s="47"/>
+      <x:c r="I173" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
       <x:c r="J173" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K173" s="47" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
       </x:c>
       <x:c r="L173" s="47" t="str">
-        <x:v>Planned: UserDiscoveryServiceTest.discover_yearFilter_returnsMatchingYear</x:v>
-      </x:c>
-      <x:c r="M173" s="47"/>
+        <x:v>UserDiscoveryServiceTest.discover_yearFilter_returnsMatchingYear</x:v>
+      </x:c>
+      <x:c r="M173" s="47" t="str">
+        <x:v>2026-10-07 18:49:55 +07:00 | 12/12 Pass | BUILD SUCCESS | 12.256 s</x:v>
+      </x:c>
     </x:row>
     <x:row r="174" ht="34" customHeight="1">
       <x:c r="A174" s="47" t="str">
@@ -22250,17 +22478,21 @@
       <x:c r="H174" s="47" t="str">
         <x:v>200 OK; missing session -&gt; 401 Unauthorized</x:v>
       </x:c>
-      <x:c r="I174" s="47"/>
+      <x:c r="I174" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
       <x:c r="J174" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K174" s="47" t="str">
         <x:v>Standalone MockMvc</x:v>
       </x:c>
       <x:c r="L174" s="47" t="str">
-        <x:v>Planned: UserDiscoveryControllerMvcTest.discover_filtersAndSession_areHandled</x:v>
-      </x:c>
-      <x:c r="M174" s="47"/>
+        <x:v>UserDiscoveryControllerMvcTest.discover_filtersAndSession_areHandled</x:v>
+      </x:c>
+      <x:c r="M174" s="47" t="str">
+        <x:v>2026-10-07 18:49:55 +07:00 | 12/12 Pass | BUILD SUCCESS | 12.256 s</x:v>
+      </x:c>
     </x:row>
     <x:row r="175" ht="34" customHeight="1">
       <x:c r="A175" s="47" t="str">
@@ -22300,7 +22532,7 @@
         <x:v>MatchingServiceTest.testRecommendFriendsRanked</x:v>
       </x:c>
       <x:c r="M175" s="47" t="str">
-        <x:v>Full regression 2026-10-07 18:20:44 | included in 103 tests</x:v>
+        <x:v>2026-10-07 19:24:20 +07:00 | Matching tests 10/10 Pass in final full regression | overall 172 tests</x:v>
       </x:c>
     </x:row>
     <x:row r="176" ht="34" customHeight="1">
@@ -22341,7 +22573,7 @@
         <x:v>MatchingServiceTest.testExcludeExistingFriendsAndPending</x:v>
       </x:c>
       <x:c r="M176" s="47" t="str">
-        <x:v>Full regression 2026-10-07 18:20:44</x:v>
+        <x:v>2026-10-07 19:24:20 +07:00 | Matching tests 10/10 Pass in final full regression | overall 172 tests</x:v>
       </x:c>
     </x:row>
     <x:row r="177" ht="34" customHeight="1">
@@ -22382,7 +22614,7 @@
         <x:v>MatchingServiceTest.testCalculateCompatibility</x:v>
       </x:c>
       <x:c r="M177" s="47" t="str">
-        <x:v>Full regression 2026-10-07 18:20:44</x:v>
+        <x:v>2026-10-07 19:24:20 +07:00 | Matching tests 10/10 Pass in final full regression | overall 172 tests</x:v>
       </x:c>
     </x:row>
     <x:row r="178" ht="34" customHeight="1">
@@ -22423,7 +22655,7 @@
         <x:v>MatchingServiceTest.testUserNotFoundThrows</x:v>
       </x:c>
       <x:c r="M178" s="47" t="str">
-        <x:v>Full regression 2026-10-07 18:20:44</x:v>
+        <x:v>2026-10-07 19:24:20 +07:00 | Matching tests 10/10 Pass in final full regression | overall 172 tests</x:v>
       </x:c>
     </x:row>
     <x:row r="179" ht="34" customHeight="1">
@@ -22464,7 +22696,7 @@
         <x:v>InterestMatchingStrategyTest.testPartialMatchFromRequirements</x:v>
       </x:c>
       <x:c r="M179" s="47" t="str">
-        <x:v>Full regression 2026-10-07 18:20:44</x:v>
+        <x:v>2026-10-07 19:24:20 +07:00 | Matching tests 10/10 Pass in final full regression | overall 172 tests</x:v>
       </x:c>
     </x:row>
     <x:row r="180" ht="34" customHeight="1">
@@ -22505,7 +22737,7 @@
         <x:v>InterestMatchingStrategyTest.testFullMatch</x:v>
       </x:c>
       <x:c r="M180" s="47" t="str">
-        <x:v>Full regression 2026-10-07 18:20:44</x:v>
+        <x:v>2026-10-07 19:24:20 +07:00 | Matching tests 10/10 Pass in final full regression | overall 172 tests</x:v>
       </x:c>
     </x:row>
     <x:row r="181" ht="34" customHeight="1">
@@ -22546,7 +22778,7 @@
         <x:v>InterestMatchingStrategyTest.testZeroMatch</x:v>
       </x:c>
       <x:c r="M181" s="47" t="str">
-        <x:v>Full regression 2026-10-07 18:20:44</x:v>
+        <x:v>2026-10-07 19:24:20 +07:00 | Matching tests 10/10 Pass in final full regression | overall 172 tests</x:v>
       </x:c>
     </x:row>
     <x:row r="182" ht="34" customHeight="1">
@@ -22587,7 +22819,7 @@
         <x:v>InterestMatchingStrategyTest.testCaseInsensitiveMatching</x:v>
       </x:c>
       <x:c r="M182" s="47" t="str">
-        <x:v>Full regression 2026-10-07 18:20:44</x:v>
+        <x:v>2026-10-07 19:24:20 +07:00 | Matching tests 10/10 Pass in final full regression | overall 172 tests</x:v>
       </x:c>
     </x:row>
     <x:row r="183" ht="34" customHeight="1">
@@ -22628,7 +22860,7 @@
         <x:v>InterestMatchingStrategyTest.testEmptyAndNullScenarios</x:v>
       </x:c>
       <x:c r="M183" s="47" t="str">
-        <x:v>Full regression 2026-10-07 18:20:44</x:v>
+        <x:v>2026-10-07 19:24:20 +07:00 | Matching tests 10/10 Pass in final full regression | overall 172 tests</x:v>
       </x:c>
     </x:row>
     <x:row r="184" ht="34" customHeight="1">
@@ -22669,7 +22901,7 @@
         <x:v>InterestMatchingStrategyTest.testStrategyName</x:v>
       </x:c>
       <x:c r="M184" s="47" t="str">
-        <x:v>Full regression 2026-10-07 18:20:44</x:v>
+        <x:v>2026-10-07 19:24:20 +07:00 | Matching tests 10/10 Pass in final full regression | overall 172 tests</x:v>
       </x:c>
     </x:row>
     <x:row r="185" ht="34" customHeight="1">
@@ -22697,17 +22929,21 @@
       <x:c r="H185" s="47" t="str">
         <x:v>return NotificationResponse content</x:v>
       </x:c>
-      <x:c r="I185" s="47"/>
+      <x:c r="I185" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
       <x:c r="J185" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K185" s="47" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
       </x:c>
       <x:c r="L185" s="47" t="str">
-        <x:v>Planned: NotificationServiceTest.list_allNotifications_mapsResponses</x:v>
-      </x:c>
-      <x:c r="M185" s="47"/>
+        <x:v>NotificationServiceTest.list_allNotifications_mapsResponses</x:v>
+      </x:c>
+      <x:c r="M185" s="47" t="str">
+        <x:v>2026-10-07 19:02:08 +07:00 | 10/10 Pass | BUILD SUCCESS | 12.299 s</x:v>
+      </x:c>
     </x:row>
     <x:row r="186" ht="34" customHeight="1">
       <x:c r="A186" s="47" t="str">
@@ -22734,17 +22970,21 @@
       <x:c r="H186" s="47" t="str">
         <x:v>return only unread notifications</x:v>
       </x:c>
-      <x:c r="I186" s="47"/>
+      <x:c r="I186" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
       <x:c r="J186" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K186" s="47" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
       </x:c>
       <x:c r="L186" s="47" t="str">
-        <x:v>Planned: NotificationServiceTest.list_unreadOnly_usesUnreadRepositoryQuery</x:v>
-      </x:c>
-      <x:c r="M186" s="47"/>
+        <x:v>NotificationServiceTest.list_unreadOnly_usesUnreadRepositoryQuery</x:v>
+      </x:c>
+      <x:c r="M186" s="47" t="str">
+        <x:v>2026-10-07 19:02:08 +07:00 | 10/10 Pass | BUILD SUCCESS | 12.299 s</x:v>
+      </x:c>
     </x:row>
     <x:row r="187" ht="34" customHeight="1">
       <x:c r="A187" s="47" t="str">
@@ -22771,17 +23011,21 @@
       <x:c r="H187" s="47" t="str">
         <x:v>page clamps to 0; size clamps to 50</x:v>
       </x:c>
-      <x:c r="I187" s="47"/>
+      <x:c r="I187" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
       <x:c r="J187" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K187" s="47" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
       </x:c>
       <x:c r="L187" s="47" t="str">
-        <x:v>Planned: NotificationServiceTest.list_outOfRangePagination_isClamped</x:v>
-      </x:c>
-      <x:c r="M187" s="47"/>
+        <x:v>NotificationServiceTest.list_outOfRangePagination_isClamped</x:v>
+      </x:c>
+      <x:c r="M187" s="47" t="str">
+        <x:v>2026-10-07 19:02:08 +07:00 | 10/10 Pass | BUILD SUCCESS | 12.299 s</x:v>
+      </x:c>
     </x:row>
     <x:row r="188" ht="34" customHeight="1">
       <x:c r="A188" s="47" t="str">
@@ -22808,17 +23052,21 @@
       <x:c r="H188" s="47" t="str">
         <x:v>return 3</x:v>
       </x:c>
-      <x:c r="I188" s="47"/>
+      <x:c r="I188" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
       <x:c r="J188" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K188" s="47" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
       </x:c>
       <x:c r="L188" s="47" t="str">
-        <x:v>Planned: NotificationServiceTest.unreadCount_returnsRepositoryCount</x:v>
-      </x:c>
-      <x:c r="M188" s="47"/>
+        <x:v>NotificationServiceTest.unreadCount_returnsRepositoryCount</x:v>
+      </x:c>
+      <x:c r="M188" s="47" t="str">
+        <x:v>2026-10-07 19:02:08 +07:00 | 10/10 Pass | BUILD SUCCESS | 12.299 s</x:v>
+      </x:c>
     </x:row>
     <x:row r="189" ht="34" customHeight="1">
       <x:c r="A189" s="47" t="str">
@@ -22845,17 +23093,21 @@
       <x:c r="H189" s="47" t="str">
         <x:v>update only notification owned by user</x:v>
       </x:c>
-      <x:c r="I189" s="47"/>
+      <x:c r="I189" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
       <x:c r="J189" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K189" s="47" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
       </x:c>
       <x:c r="L189" s="47" t="str">
-        <x:v>Planned: NotificationServiceTest.markAsRead_callsScopedUpdate</x:v>
-      </x:c>
-      <x:c r="M189" s="47"/>
+        <x:v>NotificationServiceTest.markAsRead_callsScopedUpdate</x:v>
+      </x:c>
+      <x:c r="M189" s="47" t="str">
+        <x:v>2026-10-07 19:02:08 +07:00 | 10/10 Pass | BUILD SUCCESS | 12.299 s</x:v>
+      </x:c>
     </x:row>
     <x:row r="190" ht="34" customHeight="1">
       <x:c r="A190" s="47" t="str">
@@ -22882,17 +23134,21 @@
       <x:c r="H190" s="47" t="str">
         <x:v>mark user's notifications read</x:v>
       </x:c>
-      <x:c r="I190" s="47"/>
+      <x:c r="I190" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
       <x:c r="J190" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K190" s="47" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
       </x:c>
       <x:c r="L190" s="47" t="str">
-        <x:v>Planned: NotificationServiceTest.markAllAsRead_callsRepository</x:v>
-      </x:c>
-      <x:c r="M190" s="47"/>
+        <x:v>NotificationServiceTest.markAllAsRead_callsRepository</x:v>
+      </x:c>
+      <x:c r="M190" s="47" t="str">
+        <x:v>2026-10-07 19:02:08 +07:00 | 10/10 Pass | BUILD SUCCESS | 12.299 s</x:v>
+      </x:c>
     </x:row>
     <x:row r="191" ht="34" customHeight="1">
       <x:c r="A191" s="47" t="str">
@@ -22919,17 +23175,21 @@
       <x:c r="H191" s="47" t="str">
         <x:v>save notification and push to /topic/notifications/{userId}</x:v>
       </x:c>
-      <x:c r="I191" s="47"/>
+      <x:c r="I191" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
       <x:c r="J191" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K191" s="47" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
       </x:c>
       <x:c r="L191" s="47" t="str">
-        <x:v>Planned: NotificationServiceTest.onFriendRequestSent_savesAndPushesNotification</x:v>
-      </x:c>
-      <x:c r="M191" s="47"/>
+        <x:v>NotificationServiceTest.onFriendRequestSent_savesAndPushesNotification</x:v>
+      </x:c>
+      <x:c r="M191" s="47" t="str">
+        <x:v>2026-10-07 19:02:08 +07:00 | 10/10 Pass | BUILD SUCCESS | 12.299 s</x:v>
+      </x:c>
     </x:row>
     <x:row r="192" ht="34" customHeight="1">
       <x:c r="A192" s="47" t="str">
@@ -22956,17 +23216,21 @@
       <x:c r="H192" s="47" t="str">
         <x:v>save and push accepted notification</x:v>
       </x:c>
-      <x:c r="I192" s="47"/>
+      <x:c r="I192" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
       <x:c r="J192" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K192" s="47" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
       </x:c>
       <x:c r="L192" s="47" t="str">
-        <x:v>Planned: NotificationServiceTest.onFriendRequestAccepted_savesAndPushesNotification</x:v>
-      </x:c>
-      <x:c r="M192" s="47"/>
+        <x:v>NotificationServiceTest.onFriendRequestAccepted_savesAndPushesNotification</x:v>
+      </x:c>
+      <x:c r="M192" s="47" t="str">
+        <x:v>2026-10-07 19:02:08 +07:00 | 10/10 Pass | BUILD SUCCESS | 12.299 s</x:v>
+      </x:c>
     </x:row>
     <x:row r="193" ht="48" customHeight="1">
       <x:c r="A193" s="47" t="str">
@@ -22993,17 +23257,21 @@
       <x:c r="H193" s="47" t="str">
         <x:v>reuse/update existing notification instead of creating duplicate; skip sender</x:v>
       </x:c>
-      <x:c r="I193" s="47"/>
+      <x:c r="I193" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
       <x:c r="J193" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K193" s="47" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
       </x:c>
       <x:c r="L193" s="47" t="str">
-        <x:v>Planned: NotificationServiceTest.notifyNewMessage_reusesUnreadAndSkipsSender</x:v>
-      </x:c>
-      <x:c r="M193" s="47"/>
+        <x:v>NotificationServiceTest.notifyNewMessage_reusesUnreadAndSkipsSender</x:v>
+      </x:c>
+      <x:c r="M193" s="47" t="str">
+        <x:v>2026-10-07 19:02:08 +07:00 | 10/10 Pass | BUILD SUCCESS | 12.299 s</x:v>
+      </x:c>
     </x:row>
     <x:row r="194" ht="34" customHeight="1">
       <x:c r="A194" s="47" t="str">
@@ -23030,17 +23298,21 @@
       <x:c r="H194" s="47" t="str">
         <x:v>GET -&gt; 200; mark read/read-all -&gt; 204; missing session -&gt; 401</x:v>
       </x:c>
-      <x:c r="I194" s="47"/>
+      <x:c r="I194" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
       <x:c r="J194" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K194" s="47" t="str">
         <x:v>Standalone MockMvc</x:v>
       </x:c>
       <x:c r="L194" s="47" t="str">
-        <x:v>Planned: NotificationControllerMvcTest.notificationEndpoints_enforceStatusAndSession</x:v>
-      </x:c>
-      <x:c r="M194" s="47"/>
+        <x:v>NotificationControllerMvcTest.notificationEndpoints_enforceStatusAndSession</x:v>
+      </x:c>
+      <x:c r="M194" s="47" t="str">
+        <x:v>2026-10-07 19:02:08 +07:00 | 10/10 Pass | BUILD SUCCESS | 12.299 s</x:v>
+      </x:c>
     </x:row>
     <x:row r="195" ht="34" customHeight="1">
       <x:c r="A195" s="47" t="str">
@@ -23067,17 +23339,21 @@
       <x:c r="H195" s="47" t="str">
         <x:v>GROUP room, trimmed name, maxMembers default 10, owner membership created</x:v>
       </x:c>
-      <x:c r="I195" s="47"/>
+      <x:c r="I195" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
       <x:c r="J195" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K195" s="47" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
       </x:c>
       <x:c r="L195" s="47" t="str">
-        <x:v>Planned: ChatRoomServiceTest.createGroupRoom_publicRoom_appliesDefaultsAndOwner</x:v>
-      </x:c>
-      <x:c r="M195" s="47"/>
+        <x:v>ChatRoomServiceTest.createGroupRoom_publicRoom_appliesDefaultsAndOwner</x:v>
+      </x:c>
+      <x:c r="M195" s="47" t="str">
+        <x:v>2026-10-07 19:09:36 +07:00 | 12/12 Pass | BUILD SUCCESS | 37.995 s</x:v>
+      </x:c>
     </x:row>
     <x:row r="196" ht="34" customHeight="1">
       <x:c r="A196" s="47" t="str">
@@ -23104,17 +23380,21 @@
       <x:c r="H196" s="47" t="str">
         <x:v>400 BAD_REQUEST: Password is required for private rooms</x:v>
       </x:c>
-      <x:c r="I196" s="47"/>
+      <x:c r="I196" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
       <x:c r="J196" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K196" s="47" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
       </x:c>
       <x:c r="L196" s="47" t="str">
-        <x:v>Planned: ChatRoomServiceTest.createGroupRoom_privateWithoutPassword_returnsBadRequest</x:v>
-      </x:c>
-      <x:c r="M196" s="47"/>
+        <x:v>ChatRoomServiceTest.createGroupRoom_privateWithoutPassword_returnsBadRequest</x:v>
+      </x:c>
+      <x:c r="M196" s="47" t="str">
+        <x:v>2026-10-07 19:09:36 +07:00 | 12/12 Pass | BUILD SUCCESS | 37.995 s</x:v>
+      </x:c>
     </x:row>
     <x:row r="197" ht="34" customHeight="1">
       <x:c r="A197" s="47" t="str">
@@ -23141,17 +23421,21 @@
       <x:c r="H197" s="47" t="str">
         <x:v>store passwordHash, not raw password</x:v>
       </x:c>
-      <x:c r="I197" s="47"/>
+      <x:c r="I197" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
       <x:c r="J197" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K197" s="47" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
       </x:c>
       <x:c r="L197" s="47" t="str">
-        <x:v>Planned: ChatRoomServiceTest.createGroupRoom_private_encodesPassword</x:v>
-      </x:c>
-      <x:c r="M197" s="47"/>
+        <x:v>ChatRoomServiceTest.createGroupRoom_private_encodesPassword</x:v>
+      </x:c>
+      <x:c r="M197" s="47" t="str">
+        <x:v>2026-10-07 19:09:36 +07:00 | 12/12 Pass | BUILD SUCCESS | 37.995 s</x:v>
+      </x:c>
     </x:row>
     <x:row r="198" ht="34" customHeight="1">
       <x:c r="A198" s="47" t="str">
@@ -23178,17 +23462,21 @@
       <x:c r="H198" s="47" t="str">
         <x:v>400 BAD_REQUEST: One or more interests do not exist or are inactive</x:v>
       </x:c>
-      <x:c r="I198" s="47"/>
+      <x:c r="I198" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
       <x:c r="J198" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K198" s="47" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
       </x:c>
       <x:c r="L198" s="47" t="str">
-        <x:v>Planned: ChatRoomServiceTest.createGroupRoom_invalidInterest_returnsBadRequest</x:v>
-      </x:c>
-      <x:c r="M198" s="47"/>
+        <x:v>ChatRoomServiceTest.createGroupRoom_invalidInterest_returnsBadRequest</x:v>
+      </x:c>
+      <x:c r="M198" s="47" t="str">
+        <x:v>2026-10-07 19:09:36 +07:00 | 12/12 Pass | BUILD SUCCESS | 37.995 s</x:v>
+      </x:c>
     </x:row>
     <x:row r="199" ht="34" customHeight="1">
       <x:c r="A199" s="47" t="str">
@@ -23215,17 +23503,21 @@
       <x:c r="H199" s="47" t="str">
         <x:v>return intersection only; empty-member rooms excluded</x:v>
       </x:c>
-      <x:c r="I199" s="47"/>
+      <x:c r="I199" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
       <x:c r="J199" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K199" s="47" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
       </x:c>
       <x:c r="L199" s="47" t="str">
-        <x:v>Planned: ChatRoomServiceTest.discoverRooms_searchAndInterests_intersectsResults</x:v>
-      </x:c>
-      <x:c r="M199" s="47"/>
+        <x:v>ChatRoomServiceTest.discoverRooms_searchAndInterests_intersectsResults</x:v>
+      </x:c>
+      <x:c r="M199" s="47" t="str">
+        <x:v>2026-10-07 19:09:36 +07:00 | 12/12 Pass | BUILD SUCCESS | 37.995 s</x:v>
+      </x:c>
     </x:row>
     <x:row r="200" ht="34" customHeight="1">
       <x:c r="A200" s="47" t="str">
@@ -23252,17 +23544,21 @@
       <x:c r="H200" s="47" t="str">
         <x:v>409 CONFLICT: Already a member of this room</x:v>
       </x:c>
-      <x:c r="I200" s="47"/>
+      <x:c r="I200" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
       <x:c r="J200" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K200" s="47" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
       </x:c>
       <x:c r="L200" s="47" t="str">
-        <x:v>Planned: ChatRoomServiceTest.joinRoom_existingMember_returnsConflict</x:v>
-      </x:c>
-      <x:c r="M200" s="47"/>
+        <x:v>ChatRoomServiceTest.joinRoom_existingMember_returnsConflict</x:v>
+      </x:c>
+      <x:c r="M200" s="47" t="str">
+        <x:v>2026-10-07 19:09:36 +07:00 | 12/12 Pass | BUILD SUCCESS | 37.995 s</x:v>
+      </x:c>
     </x:row>
     <x:row r="201" ht="34" customHeight="1">
       <x:c r="A201" s="47" t="str">
@@ -23289,17 +23585,21 @@
       <x:c r="H201" s="47" t="str">
         <x:v>403 FORBIDDEN: Invalid room password</x:v>
       </x:c>
-      <x:c r="I201" s="47"/>
+      <x:c r="I201" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
       <x:c r="J201" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K201" s="47" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
       </x:c>
       <x:c r="L201" s="47" t="str">
-        <x:v>Planned: ChatRoomServiceTest.joinRoom_privateWrongPassword_returnsForbidden</x:v>
-      </x:c>
-      <x:c r="M201" s="47"/>
+        <x:v>ChatRoomServiceTest.joinRoom_privateWrongPassword_returnsForbidden</x:v>
+      </x:c>
+      <x:c r="M201" s="47" t="str">
+        <x:v>2026-10-07 19:09:36 +07:00 | 12/12 Pass | BUILD SUCCESS | 37.995 s</x:v>
+      </x:c>
     </x:row>
     <x:row r="202" ht="34" customHeight="1">
       <x:c r="A202" s="47" t="str">
@@ -23326,17 +23626,21 @@
       <x:c r="H202" s="47" t="str">
         <x:v>409 CONFLICT: Room is full</x:v>
       </x:c>
-      <x:c r="I202" s="47"/>
+      <x:c r="I202" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
       <x:c r="J202" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K202" s="47" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
       </x:c>
       <x:c r="L202" s="47" t="str">
-        <x:v>Planned: ChatRoomServiceTest.joinRoom_fullRoom_returnsConflict</x:v>
-      </x:c>
-      <x:c r="M202" s="47"/>
+        <x:v>ChatRoomServiceTest.joinRoom_fullRoom_returnsConflict</x:v>
+      </x:c>
+      <x:c r="M202" s="47" t="str">
+        <x:v>2026-10-07 19:09:36 +07:00 | 12/12 Pass | BUILD SUCCESS | 37.995 s</x:v>
+      </x:c>
     </x:row>
     <x:row r="203" ht="34" customHeight="1">
       <x:c r="A203" s="47" t="str">
@@ -23363,17 +23667,21 @@
       <x:c r="H203" s="47" t="str">
         <x:v>404 NOT_FOUND: You are not a member of this room</x:v>
       </x:c>
-      <x:c r="I203" s="47"/>
+      <x:c r="I203" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
       <x:c r="J203" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K203" s="47" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
       </x:c>
       <x:c r="L203" s="47" t="str">
-        <x:v>Planned: ChatRoomServiceTest.leaveRoom_nonMember_returnsNotFound</x:v>
-      </x:c>
-      <x:c r="M203" s="47"/>
+        <x:v>ChatRoomServiceTest.leaveRoom_nonMember_returnsNotFound</x:v>
+      </x:c>
+      <x:c r="M203" s="47" t="str">
+        <x:v>2026-10-07 19:09:36 +07:00 | 12/12 Pass | BUILD SUCCESS | 37.995 s</x:v>
+      </x:c>
     </x:row>
     <x:row r="204" ht="34" customHeight="1">
       <x:c r="A204" s="47" t="str">
@@ -23400,17 +23708,21 @@
       <x:c r="H204" s="47" t="str">
         <x:v>403 permission error or 400 maxMembers error</x:v>
       </x:c>
-      <x:c r="I204" s="47"/>
+      <x:c r="I204" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
       <x:c r="J204" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K204" s="47" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
       </x:c>
       <x:c r="L204" s="47" t="str">
-        <x:v>Planned: ChatRoomServiceTest.updateRoom_permissionAndMemberLimit_areEnforced</x:v>
-      </x:c>
-      <x:c r="M204" s="47"/>
+        <x:v>ChatRoomServiceTest.updateRoom_permissionAndMemberLimit_areEnforced</x:v>
+      </x:c>
+      <x:c r="M204" s="47" t="str">
+        <x:v>2026-10-07 19:09:36 +07:00 | 12/12 Pass | BUILD SUCCESS | 37.995 s</x:v>
+      </x:c>
     </x:row>
     <x:row r="205" ht="34" customHeight="1">
       <x:c r="A205" s="47" t="str">
@@ -23437,17 +23749,21 @@
       <x:c r="H205" s="47" t="str">
         <x:v>self -&gt; 400; nonfriend -&gt; 404 'You can only chat directly with friends'</x:v>
       </x:c>
-      <x:c r="I205" s="47"/>
+      <x:c r="I205" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
       <x:c r="J205" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K205" s="47" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
       </x:c>
       <x:c r="L205" s="47" t="str">
-        <x:v>Planned: ChatRoomServiceTest.directRoom_selfOrNonFriend_isRejected</x:v>
-      </x:c>
-      <x:c r="M205" s="47"/>
+        <x:v>ChatRoomServiceTest.directRoom_selfOrNonFriend_isRejected</x:v>
+      </x:c>
+      <x:c r="M205" s="47" t="str">
+        <x:v>2026-10-07 19:09:36 +07:00 | 12/12 Pass | BUILD SUCCESS | 37.995 s</x:v>
+      </x:c>
     </x:row>
     <x:row r="206" ht="34" customHeight="1">
       <x:c r="A206" s="47" t="str">
@@ -23474,17 +23790,21 @@
       <x:c r="H206" s="47" t="str">
         <x:v>create -&gt; 201; join/direct -&gt; 200; leave -&gt; 204; protected operations missing session -&gt; 401</x:v>
       </x:c>
-      <x:c r="I206" s="47"/>
+      <x:c r="I206" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
       <x:c r="J206" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K206" s="47" t="str">
         <x:v>Standalone MockMvc</x:v>
       </x:c>
       <x:c r="L206" s="47" t="str">
-        <x:v>Planned: ChatRoomControllerMvcTest.roomEndpoints_statusAndSession_contract</x:v>
-      </x:c>
-      <x:c r="M206" s="47"/>
+        <x:v>ChatRoomControllerMvcTest.roomEndpoints_statusAndSession_contract</x:v>
+      </x:c>
+      <x:c r="M206" s="47" t="str">
+        <x:v>2026-10-07 19:09:36 +07:00 | 12/12 Pass | BUILD SUCCESS | 37.995 s</x:v>
+      </x:c>
     </x:row>
     <x:row r="207" ht="34" customHeight="1">
       <x:c r="A207" s="47" t="str">
@@ -23511,17 +23831,21 @@
       <x:c r="H207" s="47" t="str">
         <x:v>403 FORBIDDEN: You are not a member of this room</x:v>
       </x:c>
-      <x:c r="I207" s="47"/>
+      <x:c r="I207" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
       <x:c r="J207" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K207" s="47" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
       </x:c>
       <x:c r="L207" s="47" t="str">
-        <x:v>Planned: ChatMessageServiceTest.getMessages_nonMember_returnsForbidden</x:v>
-      </x:c>
-      <x:c r="M207" s="47"/>
+        <x:v>ChatMessageServiceTest.getMessages_nonMember_returnsForbidden</x:v>
+      </x:c>
+      <x:c r="M207" s="47" t="str">
+        <x:v>2026-10-07 19:16:14 +07:00 | 12/12 Pass | BUILD SUCCESS | 22.276 s</x:v>
+      </x:c>
     </x:row>
     <x:row r="208" ht="34" customHeight="1">
       <x:c r="A208" s="47" t="str">
@@ -23548,17 +23872,21 @@
       <x:c r="H208" s="47" t="str">
         <x:v>return [] without MessageRepository history query</x:v>
       </x:c>
-      <x:c r="I208" s="47"/>
+      <x:c r="I208" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
       <x:c r="J208" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K208" s="47" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
       </x:c>
       <x:c r="L208" s="47" t="str">
-        <x:v>Planned: ChatMessageServiceTest.getMessages_groupRoom_returnsEmpty</x:v>
-      </x:c>
-      <x:c r="M208" s="47"/>
+        <x:v>ChatMessageServiceTest.getMessages_groupRoom_returnsEmpty</x:v>
+      </x:c>
+      <x:c r="M208" s="47" t="str">
+        <x:v>2026-10-07 19:16:14 +07:00 | 12/12 Pass | BUILD SUCCESS | 22.276 s</x:v>
+      </x:c>
     </x:row>
     <x:row r="209" ht="34" customHeight="1">
       <x:c r="A209" s="47" t="str">
@@ -23585,17 +23913,21 @@
       <x:c r="H209" s="47" t="str">
         <x:v>return oldest-&gt;newest and mark lastReadAt</x:v>
       </x:c>
-      <x:c r="I209" s="47"/>
+      <x:c r="I209" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
       <x:c r="J209" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K209" s="47" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
       </x:c>
       <x:c r="L209" s="47" t="str">
-        <x:v>Planned: ChatMessageServiceTest.getMessages_directRoom_reversesAndMarksRead</x:v>
-      </x:c>
-      <x:c r="M209" s="47"/>
+        <x:v>ChatMessageServiceTest.getMessages_directRoom_reversesAndMarksRead</x:v>
+      </x:c>
+      <x:c r="M209" s="47" t="str">
+        <x:v>2026-10-07 19:16:14 +07:00 | 12/12 Pass | BUILD SUCCESS | 22.276 s</x:v>
+      </x:c>
     </x:row>
     <x:row r="210" ht="34" customHeight="1">
       <x:c r="A210" s="47" t="str">
@@ -23622,17 +23954,21 @@
       <x:c r="H210" s="47" t="str">
         <x:v>limit clamps to 1..100 and before query is used</x:v>
       </x:c>
-      <x:c r="I210" s="47"/>
+      <x:c r="I210" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
       <x:c r="J210" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K210" s="47" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
       </x:c>
       <x:c r="L210" s="47" t="str">
-        <x:v>Planned: ChatMessageServiceTest.getMessages_limitAndBefore_areHandled</x:v>
-      </x:c>
-      <x:c r="M210" s="47"/>
+        <x:v>ChatMessageServiceTest.getMessages_limitAndBefore_areHandled</x:v>
+      </x:c>
+      <x:c r="M210" s="47" t="str">
+        <x:v>2026-10-07 19:16:14 +07:00 | 12/12 Pass | BUILD SUCCESS | 22.276 s</x:v>
+      </x:c>
     </x:row>
     <x:row r="211" ht="34" customHeight="1">
       <x:c r="A211" s="47" t="str">
@@ -23659,17 +23995,21 @@
       <x:c r="H211" s="47" t="str">
         <x:v>use correct count query based on lastReadAt</x:v>
       </x:c>
-      <x:c r="I211" s="47"/>
+      <x:c r="I211" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
       <x:c r="J211" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K211" s="47" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
       </x:c>
       <x:c r="L211" s="47" t="str">
-        <x:v>Planned: ChatMessageServiceTest.unreadCount_usesCorrectRepositoryQuery</x:v>
-      </x:c>
-      <x:c r="M211" s="47"/>
+        <x:v>ChatMessageServiceTest.unreadCount_usesCorrectRepositoryQuery</x:v>
+      </x:c>
+      <x:c r="M211" s="47" t="str">
+        <x:v>2026-10-07 19:16:14 +07:00 | 12/12 Pass | BUILD SUCCESS | 22.276 s</x:v>
+      </x:c>
     </x:row>
     <x:row r="212" ht="34" customHeight="1">
       <x:c r="A212" s="47" t="str">
@@ -23696,17 +24036,21 @@
       <x:c r="H212" s="47" t="str">
         <x:v>persist message, broadcast, notifyNewMessage, update sender lastReadAt</x:v>
       </x:c>
-      <x:c r="I212" s="47"/>
+      <x:c r="I212" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
       <x:c r="J212" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K212" s="47" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
       </x:c>
       <x:c r="L212" s="47" t="str">
-        <x:v>Planned: ChatMessageServiceTest.send_direct_persistsBroadcastsAndNotifies</x:v>
-      </x:c>
-      <x:c r="M212" s="47"/>
+        <x:v>ChatMessageServiceTest.send_direct_persistsBroadcastsAndNotifies</x:v>
+      </x:c>
+      <x:c r="M212" s="47" t="str">
+        <x:v>2026-10-07 19:16:14 +07:00 | 12/12 Pass | BUILD SUCCESS | 22.276 s</x:v>
+      </x:c>
     </x:row>
     <x:row r="213" ht="34" customHeight="1">
       <x:c r="A213" s="47" t="str">
@@ -23733,17 +24077,21 @@
       <x:c r="H213" s="47" t="str">
         <x:v>broadcast response with id=null; do not persist or notify</x:v>
       </x:c>
-      <x:c r="I213" s="47"/>
+      <x:c r="I213" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
       <x:c r="J213" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K213" s="47" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
       </x:c>
       <x:c r="L213" s="47" t="str">
-        <x:v>Planned: ChatMessageServiceTest.send_group_broadcastsWithoutPersistence</x:v>
-      </x:c>
-      <x:c r="M213" s="47"/>
+        <x:v>ChatMessageServiceTest.send_group_broadcastsWithoutPersistence</x:v>
+      </x:c>
+      <x:c r="M213" s="47" t="str">
+        <x:v>2026-10-07 19:16:14 +07:00 | 12/12 Pass | BUILD SUCCESS | 22.276 s</x:v>
+      </x:c>
     </x:row>
     <x:row r="214" ht="34" customHeight="1">
       <x:c r="A214" s="47" t="str">
@@ -23770,17 +24118,21 @@
       <x:c r="H214" s="47" t="str">
         <x:v>blank defaults TEXT; invalid -&gt; 400 BAD_REQUEST 'Invalid messageType'</x:v>
       </x:c>
-      <x:c r="I214" s="47"/>
+      <x:c r="I214" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
       <x:c r="J214" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K214" s="47" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
       </x:c>
       <x:c r="L214" s="47" t="str">
-        <x:v>Planned: ChatMessageServiceTest.send_messageType_defaultAndInvalid_areHandled</x:v>
-      </x:c>
-      <x:c r="M214" s="47"/>
+        <x:v>ChatMessageServiceTest.send_messageType_defaultAndInvalid_areHandled</x:v>
+      </x:c>
+      <x:c r="M214" s="47" t="str">
+        <x:v>2026-10-07 19:16:14 +07:00 | 12/12 Pass | BUILD SUCCESS | 22.276 s</x:v>
+      </x:c>
     </x:row>
     <x:row r="215" ht="34" customHeight="1">
       <x:c r="A215" s="47" t="str">
@@ -23807,17 +24159,21 @@
       <x:c r="H215" s="47" t="str">
         <x:v>set deletedAt and save (soft delete)</x:v>
       </x:c>
-      <x:c r="I215" s="47"/>
+      <x:c r="I215" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
       <x:c r="J215" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K215" s="47" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
       </x:c>
       <x:c r="L215" s="47" t="str">
-        <x:v>Planned: ChatMessageServiceTest.delete_ownMessage_softDeletes</x:v>
-      </x:c>
-      <x:c r="M215" s="47"/>
+        <x:v>ChatMessageServiceTest.delete_ownMessage_softDeletes</x:v>
+      </x:c>
+      <x:c r="M215" s="47" t="str">
+        <x:v>2026-10-07 19:16:14 +07:00 | 12/12 Pass | BUILD SUCCESS | 22.276 s</x:v>
+      </x:c>
     </x:row>
     <x:row r="216" ht="34" customHeight="1">
       <x:c r="A216" s="47" t="str">
@@ -23844,17 +24200,21 @@
       <x:c r="H216" s="47" t="str">
         <x:v>403 FORBIDDEN: You can only delete your own messages</x:v>
       </x:c>
-      <x:c r="I216" s="47"/>
+      <x:c r="I216" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
       <x:c r="J216" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K216" s="47" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
       </x:c>
       <x:c r="L216" s="47" t="str">
-        <x:v>Planned: ChatMessageServiceTest.delete_otherUsersMessage_returnsForbidden</x:v>
-      </x:c>
-      <x:c r="M216" s="47"/>
+        <x:v>ChatMessageServiceTest.delete_otherUsersMessage_returnsForbidden</x:v>
+      </x:c>
+      <x:c r="M216" s="47" t="str">
+        <x:v>2026-10-07 19:16:14 +07:00 | 12/12 Pass | BUILD SUCCESS | 22.276 s</x:v>
+      </x:c>
     </x:row>
     <x:row r="217" ht="34" customHeight="1">
       <x:c r="A217" s="47" t="str">
@@ -23881,17 +24241,21 @@
       <x:c r="H217" s="47" t="str">
         <x:v>400 BAD_REQUEST: before must be an ISO-8601 instant...</x:v>
       </x:c>
-      <x:c r="I217" s="47"/>
+      <x:c r="I217" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
       <x:c r="J217" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K217" s="47" t="str">
         <x:v>Standalone MockMvc</x:v>
       </x:c>
       <x:c r="L217" s="47" t="str">
-        <x:v>Planned: ChatMessageControllerMvcTest.getMessages_invalidBefore_returnsBadRequest</x:v>
-      </x:c>
-      <x:c r="M217" s="47"/>
+        <x:v>ChatMessageControllerMvcTest.getMessages_invalidBefore_returnsBadRequest</x:v>
+      </x:c>
+      <x:c r="M217" s="47" t="str">
+        <x:v>2026-10-07 19:16:14 +07:00 | 12/12 Pass | BUILD SUCCESS | 22.276 s</x:v>
+      </x:c>
     </x:row>
     <x:row r="218" ht="34" customHeight="1">
       <x:c r="A218" s="47" t="str">
@@ -23918,17 +24282,21 @@
       <x:c r="H218" s="47" t="str">
         <x:v>blank content -&gt; 400 VALIDATION_ERROR; valid session/content -&gt; 201; missing session -&gt; 401</x:v>
       </x:c>
-      <x:c r="I218" s="47"/>
+      <x:c r="I218" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
       <x:c r="J218" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K218" s="47" t="str">
         <x:v>Standalone MockMvc</x:v>
       </x:c>
       <x:c r="L218" s="47" t="str">
-        <x:v>Planned: ChatMessageControllerMvcTest.sendMessage_validationAndSession_contract</x:v>
-      </x:c>
-      <x:c r="M218" s="47"/>
+        <x:v>ChatMessageControllerMvcTest.sendMessage_validationAndSession_contract</x:v>
+      </x:c>
+      <x:c r="M218" s="47" t="str">
+        <x:v>2026-10-07 19:16:14 +07:00 | 12/12 Pass | BUILD SUCCESS | 22.276 s</x:v>
+      </x:c>
     </x:row>
     <x:row r="219" ht="34" customHeight="1">
       <x:c r="A219" s="47" t="str">
@@ -23955,17 +24323,21 @@
       <x:c r="H219" s="47" t="str">
         <x:v>frontend retrieves current user and supports id/userId response shape</x:v>
       </x:c>
-      <x:c r="I219" s="47"/>
+      <x:c r="I219" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
       <x:c r="J219" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K219" s="47" t="str">
         <x:v>Frontend contract test</x:v>
       </x:c>
       <x:c r="L219" s="47" t="str">
-        <x:v>Planned: FriendNotificationChatContractTest.friendJs_loadsCurrentUserFromUsersMe</x:v>
-      </x:c>
-      <x:c r="M219" s="47"/>
+        <x:v>FriendNotificationChatContractTest.friendJs_loadsCurrentUserFromUsersMe</x:v>
+      </x:c>
+      <x:c r="M219" s="47" t="str">
+        <x:v>2026-10-07 19:20:07 +07:00 | 8/8 Pass | BUILD SUCCESS | 15.982 s</x:v>
+      </x:c>
     </x:row>
     <x:row r="220" ht="34" customHeight="1">
       <x:c r="A220" s="47" t="str">
@@ -23992,17 +24364,21 @@
       <x:c r="H220" s="47" t="str">
         <x:v>friend page uses current Friendship API and expected FriendResponse fields</x:v>
       </x:c>
-      <x:c r="I220" s="47"/>
+      <x:c r="I220" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
       <x:c r="J220" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K220" s="47" t="str">
         <x:v>Frontend contract test</x:v>
       </x:c>
       <x:c r="L220" s="47" t="str">
-        <x:v>Planned: FriendNotificationChatContractTest.friendJs_callsFriendsApi</x:v>
-      </x:c>
-      <x:c r="M220" s="47"/>
+        <x:v>FriendNotificationChatContractTest.friendJs_callsFriendsApi</x:v>
+      </x:c>
+      <x:c r="M220" s="47" t="str">
+        <x:v>2026-10-07 19:20:07 +07:00 | 8/8 Pass | BUILD SUCCESS | 15.982 s</x:v>
+      </x:c>
     </x:row>
     <x:row r="221" ht="34" customHeight="1">
       <x:c r="A221" s="47" t="str">
@@ -24029,17 +24405,21 @@
       <x:c r="H221" s="47" t="str">
         <x:v>opening friend conversation uses current direct-room endpoint and room.id</x:v>
       </x:c>
-      <x:c r="I221" s="47"/>
+      <x:c r="I221" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
       <x:c r="J221" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K221" s="47" t="str">
         <x:v>Frontend contract test</x:v>
       </x:c>
       <x:c r="L221" s="47" t="str">
-        <x:v>Planned: FriendNotificationChatContractTest.friendJs_opensDirectRoom</x:v>
-      </x:c>
-      <x:c r="M221" s="47"/>
+        <x:v>FriendNotificationChatContractTest.friendJs_opensDirectRoom</x:v>
+      </x:c>
+      <x:c r="M221" s="47" t="str">
+        <x:v>2026-10-07 19:20:07 +07:00 | 8/8 Pass | BUILD SUCCESS | 15.982 s</x:v>
+      </x:c>
     </x:row>
     <x:row r="222" ht="34" customHeight="1">
       <x:c r="A222" s="47" t="str">
@@ -24066,17 +24446,21 @@
       <x:c r="H222" s="47" t="str">
         <x:v>message history endpoint/method matches ChatMessageController</x:v>
       </x:c>
-      <x:c r="I222" s="47"/>
+      <x:c r="I222" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
       <x:c r="J222" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K222" s="47" t="str">
         <x:v>Frontend contract test</x:v>
       </x:c>
       <x:c r="L222" s="47" t="str">
-        <x:v>Planned: FriendNotificationChatContractTest.friendJs_loadsMessageHistory</x:v>
-      </x:c>
-      <x:c r="M222" s="47"/>
+        <x:v>FriendNotificationChatContractTest.friendJs_loadsMessageHistory</x:v>
+      </x:c>
+      <x:c r="M222" s="47" t="str">
+        <x:v>2026-10-07 19:20:07 +07:00 | 8/8 Pass | BUILD SUCCESS | 15.982 s</x:v>
+      </x:c>
     </x:row>
     <x:row r="223" ht="34" customHeight="1">
       <x:c r="A223" s="47" t="str">
@@ -24103,17 +24487,21 @@
       <x:c r="H223" s="47" t="str">
         <x:v>send payload matches ChatMessagePayload REST contract</x:v>
       </x:c>
-      <x:c r="I223" s="47"/>
+      <x:c r="I223" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
       <x:c r="J223" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K223" s="47" t="str">
         <x:v>Frontend contract test</x:v>
       </x:c>
       <x:c r="L223" s="47" t="str">
-        <x:v>Planned: FriendNotificationChatContractTest.friendJs_sendsTextMessage</x:v>
-      </x:c>
-      <x:c r="M223" s="47"/>
+        <x:v>FriendNotificationChatContractTest.friendJs_sendsTextMessage</x:v>
+      </x:c>
+      <x:c r="M223" s="47" t="str">
+        <x:v>2026-10-07 19:20:07 +07:00 | 8/8 Pass | BUILD SUCCESS | 15.982 s</x:v>
+      </x:c>
     </x:row>
     <x:row r="224" ht="34" customHeight="1">
       <x:c r="A224" s="47" t="str">
@@ -24140,17 +24528,21 @@
       <x:c r="H224" s="47" t="str">
         <x:v>notification page loads incoming FriendRequestResponse list</x:v>
       </x:c>
-      <x:c r="I224" s="47"/>
+      <x:c r="I224" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
       <x:c r="J224" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K224" s="47" t="str">
         <x:v>Frontend contract test</x:v>
       </x:c>
       <x:c r="L224" s="47" t="str">
-        <x:v>Planned: FriendNotificationChatContractTest.notificationJs_loadsIncomingFriendRequests</x:v>
-      </x:c>
-      <x:c r="M224" s="47"/>
+        <x:v>FriendNotificationChatContractTest.notificationJs_loadsIncomingFriendRequests</x:v>
+      </x:c>
+      <x:c r="M224" s="47" t="str">
+        <x:v>2026-10-07 19:20:07 +07:00 | 8/8 Pass | BUILD SUCCESS | 15.982 s</x:v>
+      </x:c>
     </x:row>
     <x:row r="225" ht="34" customHeight="1">
       <x:c r="A225" s="47" t="str">
@@ -24177,17 +24569,21 @@
       <x:c r="H225" s="47" t="str">
         <x:v>buttons call current FriendRequestController endpoints</x:v>
       </x:c>
-      <x:c r="I225" s="47"/>
+      <x:c r="I225" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
       <x:c r="J225" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K225" s="47" t="str">
         <x:v>Frontend contract test</x:v>
       </x:c>
       <x:c r="L225" s="47" t="str">
-        <x:v>Planned: FriendNotificationChatContractTest.notificationJs_acceptDecline_endpointsMatch</x:v>
-      </x:c>
-      <x:c r="M225" s="47"/>
+        <x:v>FriendNotificationChatContractTest.notificationJs_acceptDecline_endpointsMatch</x:v>
+      </x:c>
+      <x:c r="M225" s="47" t="str">
+        <x:v>2026-10-07 19:20:07 +07:00 | 8/8 Pass | BUILD SUCCESS | 15.982 s</x:v>
+      </x:c>
     </x:row>
     <x:row r="226" ht="34" customHeight="1">
       <x:c r="A226" s="47" t="str">
@@ -24214,17 +24610,21 @@
       <x:c r="H226" s="47" t="str">
         <x:v>page loads NotificationResponse and filters NEW_MESSAGE</x:v>
       </x:c>
-      <x:c r="I226" s="47"/>
+      <x:c r="I226" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
       <x:c r="J226" s="47" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K226" s="47" t="str">
         <x:v>Frontend contract test</x:v>
       </x:c>
       <x:c r="L226" s="47" t="str">
-        <x:v>Planned: FriendNotificationChatContractTest.notificationJs_loadsMessageNotifications</x:v>
-      </x:c>
-      <x:c r="M226" s="47"/>
+        <x:v>FriendNotificationChatContractTest.notificationJs_loadsMessageNotifications</x:v>
+      </x:c>
+      <x:c r="M226" s="47" t="str">
+        <x:v>2026-10-07 19:20:07 +07:00 | 8/8 Pass | BUILD SUCCESS | 15.982 s</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
docs: record registration interest defect
</commit_message>
<xml_diff>
--- a/test/test-cases/CPFriendFinder_TestCases.xlsx
+++ b/test/test-cases/CPFriendFinder_TestCases.xlsx
@@ -2,28 +2,28 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Scenario Summary" sheetId="1" r:id="R0277716d87f047de"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="2" r:id="Rc6374cf44bcd42e7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Case Design &amp; Test Results" sheetId="3" r:id="R8512b04b0e5c4881"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS001" sheetId="4" r:id="Ra524785c84b546fb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS002" sheetId="5" r:id="R721b4c90dcd84acf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS003" sheetId="6" r:id="R2aee8885a6924fa4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS004" sheetId="7" r:id="R09d4fa8814834945"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS005" sheetId="8" r:id="Rce5b50276da74cf7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS006" sheetId="9" r:id="R9079c87995644658"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defect Summary" sheetId="10" r:id="Ra4472b3bb9504501"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Summary Report" sheetId="11" r:id="Red682a7bd0964f79"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution Log" sheetId="12" r:id="R703d927b508c46a5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision Table" sheetId="13" r:id="R4c7b7fe1d28e44e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS007" sheetId="14" r:id="Rab3738139aa84959"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS008" sheetId="15" r:id="Rb7167ea83faf4cf4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS009" sheetId="16" r:id="R182113f33df745b9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS010" sheetId="17" r:id="R17bf49a39ed44a6b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS011" sheetId="18" r:id="R3001de88461b41ab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS012" sheetId="19" r:id="R4d75c43f17d64817"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS013" sheetId="20" r:id="Rff10755fb0284ec0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS014" sheetId="21" r:id="R9d7bdc4064ed48b7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS015" sheetId="22" r:id="R9e93fbb17e414cb3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Scenario Summary" sheetId="1" r:id="Rf593ce40bb124537"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="2" r:id="R74a3d3f0aca04718"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Case Design &amp; Test Results" sheetId="3" r:id="R746f69606b46409d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS001" sheetId="4" r:id="R1026f8c48f0d4061"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS002" sheetId="5" r:id="R2a98c49883124185"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS003" sheetId="6" r:id="Re13069bfead94e26"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS004" sheetId="7" r:id="R4b45fcfcee4144dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS005" sheetId="8" r:id="R6d38c901a6164eec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS006" sheetId="9" r:id="R3f6600da53944344"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defect Summary" sheetId="10" r:id="R0d3f26b2356443ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Summary Report" sheetId="11" r:id="R42e970f9d0d946e9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution Log" sheetId="12" r:id="R351f1256fdba47a9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision Table" sheetId="13" r:id="Rd93f742e0c494857"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS007" sheetId="14" r:id="Rd92ff503814c40a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS008" sheetId="15" r:id="R76d71515060c4a7e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS009" sheetId="16" r:id="R1dea134e94934d0b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS010" sheetId="17" r:id="Rd7075f8087294168"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS011" sheetId="18" r:id="R56e7808691f54b3a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS012" sheetId="19" r:id="R7eecc66fd5184f62"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS013" sheetId="20" r:id="R7d8f87ce0fe247d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS014" sheetId="21" r:id="R1fc0545afceb4281"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS015" sheetId="22" r:id="Rc6c2741f43024560"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3425,18 +3425,40 @@
       <x:c r="L4" s="244"/>
       <x:c r="M4" s="244"/>
     </x:row>
-    <x:row r="5">
-      <x:c r="A5" s="244"/>
-      <x:c r="B5" s="244"/>
-      <x:c r="C5" s="244"/>
-      <x:c r="D5" s="244"/>
-      <x:c r="E5" s="244"/>
-      <x:c r="F5" s="244"/>
-      <x:c r="G5" s="244"/>
-      <x:c r="H5" s="244"/>
-      <x:c r="I5" s="244"/>
-      <x:c r="J5" s="244"/>
-      <x:c r="K5" s="244"/>
+    <x:row r="5" ht="72" customHeight="1">
+      <x:c r="A5" s="287" t="str">
+        <x:v>DEF-003</x:v>
+      </x:c>
+      <x:c r="B5" s="287" t="str">
+        <x:v>E2E-005</x:v>
+      </x:c>
+      <x:c r="C5" s="287" t="str">
+        <x:v>Selected interests during registration are not saved</x:v>
+      </x:c>
+      <x:c r="D5" s="287" t="str">
+        <x:v>ผู้ใช้เลือก Interest ใน Step 3 และสมัคร/เข้าสู่ระบบสำเร็จ แต่หลัง Login แล้ว GET /api/users/me/interests คืนรายการว่าง</x:v>
+      </x:c>
+      <x:c r="E5" s="287" t="str">
+        <x:v>Selected interests are persisted and returned for the newly registered user</x:v>
+      </x:c>
+      <x:c r="F5" s="287" t="str">
+        <x:v>Interest count = 0</x:v>
+      </x:c>
+      <x:c r="G5" s="287" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="H5" s="287" t="str">
+        <x:v>OPEN</x:v>
+      </x:c>
+      <x:c r="I5" s="287" t="str">
+        <x:v>2026-10-08 +07:00</x:v>
+      </x:c>
+      <x:c r="J5" s="287" t="str">
+        <x:v>Robot Framework E2E-005: register_interest.robot — '0 &gt; 0' should be true.</x:v>
+      </x:c>
+      <x:c r="K5" s="287" t="str">
+        <x:v>Registration succeeds, but selected interests are not persisted. Retest after Frontend/Backend fix.</x:v>
+      </x:c>
       <x:c r="L5" s="244"/>
       <x:c r="M5" s="244"/>
     </x:row>
@@ -5294,7 +5316,7 @@
         <x:v>Retest</x:v>
       </x:c>
       <x:c r="B19" s="287" t="str">
-        <x:v>PENDING — DEF-001</x:v>
+        <x:v>PENDING — DEF-001, DEF-003</x:v>
       </x:c>
       <x:c r="C19" s="287"/>
       <x:c r="D19" s="287" t="str">
@@ -7185,15 +7207,31 @@
       <x:c r="L21" s="244"/>
       <x:c r="M21" s="244"/>
     </x:row>
-    <x:row r="22">
-      <x:c r="A22" s="244"/>
-      <x:c r="B22" s="244"/>
-      <x:c r="C22" s="244"/>
-      <x:c r="D22" s="244"/>
-      <x:c r="E22" s="244"/>
-      <x:c r="F22" s="244"/>
-      <x:c r="G22" s="244"/>
-      <x:c r="H22" s="244"/>
+    <x:row r="22" ht="32" customHeight="1">
+      <x:c r="A22" s="287" t="str">
+        <x:v>E2E-005</x:v>
+      </x:c>
+      <x:c r="B22" s="287" t="str">
+        <x:v>2026-10-08 +07:00</x:v>
+      </x:c>
+      <x:c r="C22" s="287" t="str">
+        <x:v>Robot Framework: register_interest.robot — selected interest persistence after registration</x:v>
+      </x:c>
+      <x:c r="D22" s="287" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E22" s="287" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F22" s="287" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G22" s="287" t="str">
+        <x:v>0 / 0</x:v>
+      </x:c>
+      <x:c r="H22" s="287" t="str">
+        <x:v>FAIL — DEF-003</x:v>
+      </x:c>
       <x:c r="I22" s="244"/>
       <x:c r="J22" s="244"/>
       <x:c r="K22" s="244"/>

</xml_diff>

<commit_message>
docs: close resolved defects after regression
</commit_message>
<xml_diff>
--- a/test/test-cases/CPFriendFinder_TestCases.xlsx
+++ b/test/test-cases/CPFriendFinder_TestCases.xlsx
@@ -2,28 +2,28 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Scenario Summary" sheetId="1" r:id="Rf593ce40bb124537"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="2" r:id="R74a3d3f0aca04718"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Case Design &amp; Test Results" sheetId="3" r:id="R746f69606b46409d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS001" sheetId="4" r:id="R1026f8c48f0d4061"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS002" sheetId="5" r:id="R2a98c49883124185"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS003" sheetId="6" r:id="Re13069bfead94e26"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS004" sheetId="7" r:id="R4b45fcfcee4144dc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS005" sheetId="8" r:id="R6d38c901a6164eec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS006" sheetId="9" r:id="R3f6600da53944344"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defect Summary" sheetId="10" r:id="R0d3f26b2356443ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Summary Report" sheetId="11" r:id="R42e970f9d0d946e9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution Log" sheetId="12" r:id="R351f1256fdba47a9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision Table" sheetId="13" r:id="Rd93f742e0c494857"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS007" sheetId="14" r:id="Rd92ff503814c40a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS008" sheetId="15" r:id="R76d71515060c4a7e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS009" sheetId="16" r:id="R1dea134e94934d0b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS010" sheetId="17" r:id="Rd7075f8087294168"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS011" sheetId="18" r:id="R56e7808691f54b3a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS012" sheetId="19" r:id="R7eecc66fd5184f62"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS013" sheetId="20" r:id="R7d8f87ce0fe247d5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS014" sheetId="21" r:id="R1fc0545afceb4281"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS015" sheetId="22" r:id="Rc6c2741f43024560"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Scenario Summary" sheetId="1" r:id="R18f7e6589ad64ff5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="2" r:id="R577a9dc913df4a64"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Case Design &amp; Test Results" sheetId="3" r:id="R4341521b1e7145e5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS001" sheetId="4" r:id="R17a60e1316994965"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS002" sheetId="5" r:id="R7578590d2107416b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS003" sheetId="6" r:id="R7c261d4cd89243de"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS004" sheetId="7" r:id="R01077d7626914ff4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS005" sheetId="8" r:id="R6d27c36b63994d75"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS006" sheetId="9" r:id="R57fba41917474e1a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defect Summary" sheetId="10" r:id="Rc4ece78952364247"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Summary Report" sheetId="11" r:id="R09618b4b9d494fc4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution Log" sheetId="12" r:id="Rb6aad04fdd03453f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision Table" sheetId="13" r:id="Ref2cde7fba0f4ce0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS007" sheetId="14" r:id="Ra822e6921a8f4940"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS008" sheetId="15" r:id="Rcc82e7d808dd4669"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS009" sheetId="16" r:id="Rf702cfb6aa7f48b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS010" sheetId="17" r:id="R0aa64b4305464d94"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS011" sheetId="18" r:id="Re4cb715a04a343dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS012" sheetId="19" r:id="Rcc3c9ba7797a4289"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS013" sheetId="20" r:id="Re77055a61d1f4bb2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS014" sheetId="21" r:id="R5c5b0efc1e60433d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS015" sheetId="22" r:id="R0701dd83a9864695"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1914,10 +1914,10 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="E20" s="287" t="n">
-        <x:v>11</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="F20" s="287" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G20" s="287" t="n">
         <x:v>0</x:v>
@@ -1926,7 +1926,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I20" s="287" t="str">
-        <x:v>UserService + UserController | DEF-001</x:v>
+        <x:v>UserService + UserController | DEF-001 CLOSED</x:v>
       </x:c>
       <x:c r="J20" s="244"/>
       <x:c r="K20" s="244"/>
@@ -2209,10 +2209,10 @@
         <x:v>171</x:v>
       </x:c>
       <x:c r="E29" s="287" t="n">
-        <x:v>170</x:v>
+        <x:v>171</x:v>
       </x:c>
       <x:c r="F29" s="287" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G29" s="287" t="n">
         <x:v>0</x:v>
@@ -2221,7 +2221,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I29" s="287" t="str">
-        <x:v>Documented: 171 executed / 170 Pass / 1 Fail. Final Maven regression: 172 tests / 171 Pass / 1 Fail; only DEF-001 failed.</x:v>
+        <x:v>Documented: 171 executed / 171 Pass / 0 Fail. Final Maven regression: 174 tests / 174 Pass / 0 Fail / 0 Errors / 0 Skipped. DEF-001 and DEF-003 closed.</x:v>
       </x:c>
       <x:c r="J29" s="244"/>
       <x:c r="K29" s="244"/>
@@ -3411,21 +3411,21 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="H4" s="277" t="str">
-        <x:v>OPEN</x:v>
+        <x:v>CLOSED</x:v>
       </x:c>
       <x:c r="I4" s="276" t="str">
         <x:v>2026-10-07 16:46:16 +07:00</x:v>
       </x:c>
       <x:c r="J4" s="276" t="str">
-        <x:v>UserServiceTest.updateProfile_blankFirstname_clearsFirstname</x:v>
+        <x:v>UserServiceTest.updateProfile_blankFirstname_clearsFirstname passed. Final full regression 2026-10-08 18:02:26 +07:00: 174/174 Pass, 0 Fail, 0 Errors, 0 Skipped.</x:v>
       </x:c>
       <x:c r="K4" s="278" t="str">
-        <x:v>OPEN / Retest pending after Backend fix. Reproduced in final full regression 2026-10-07 19:24:20 +07:00: 172 tests, 171 Pass, 1 Fail, 0 Errors, 0 Skipped. Only failure: UserServiceTest.updateProfile_blankFirstname_clearsFirstname — expected null, actual 'Old'.</x:v>
+        <x:v>CLOSED / Retest passed 2026-10-08 +07:00 after UserService fix. Empty string now clears optional profile string fields while omitted fields remain unchanged.</x:v>
       </x:c>
       <x:c r="L4" s="244"/>
       <x:c r="M4" s="244"/>
     </x:row>
-    <x:row r="5" ht="72" customHeight="1">
+    <x:row r="5" ht="88" customHeight="1">
       <x:c r="A5" s="287" t="str">
         <x:v>DEF-003</x:v>
       </x:c>
@@ -3448,16 +3448,16 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="H5" s="287" t="str">
-        <x:v>OPEN</x:v>
+        <x:v>CLOSED</x:v>
       </x:c>
       <x:c r="I5" s="287" t="str">
         <x:v>2026-10-08 +07:00</x:v>
       </x:c>
       <x:c r="J5" s="287" t="str">
-        <x:v>Robot Framework E2E-005: register_interest.robot — '0 &gt; 0' should be true.</x:v>
+        <x:v>Manual API retest passed. Robot Framework regression: 5/5 Pass including E2E-005. Java targeted regression: 39/39 Pass. Final full regression: 174/174 Pass.</x:v>
       </x:c>
       <x:c r="K5" s="287" t="str">
-        <x:v>Registration succeeds, but selected interests are not persisted. Retest after Frontend/Backend fix.</x:v>
+        <x:v>CLOSED / Retest passed 2026-10-08 +07:00. Selected interests are saved during registration and returned for the newly registered user.</x:v>
       </x:c>
       <x:c r="L5" s="244"/>
       <x:c r="M5" s="244"/>
@@ -5241,7 +5241,7 @@
         <x:v>Pass</x:v>
       </x:c>
       <x:c r="B16" s="287" t="n">
-        <x:v>170</x:v>
+        <x:v>171</x:v>
       </x:c>
       <x:c r="C16" s="287"/>
       <x:c r="D16" s="287" t="str">
@@ -5266,7 +5266,7 @@
         <x:v>Fail</x:v>
       </x:c>
       <x:c r="B17" s="287" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C17" s="287"/>
       <x:c r="D17" s="287" t="str">
@@ -5316,7 +5316,7 @@
         <x:v>Retest</x:v>
       </x:c>
       <x:c r="B19" s="287" t="str">
-        <x:v>PENDING — DEF-001, DEF-003</x:v>
+        <x:v>DEF-001 PASSED / CLOSED; DEF-003 PASSED / CLOSED</x:v>
       </x:c>
       <x:c r="C19" s="287"/>
       <x:c r="D19" s="287" t="str">
@@ -5382,9 +5382,15 @@
       <x:c r="A22" s="244"/>
       <x:c r="B22" s="244"/>
       <x:c r="C22" s="244"/>
-      <x:c r="D22" s="244"/>
-      <x:c r="E22" s="244"/>
-      <x:c r="F22" s="244"/>
+      <x:c r="D22" s="244" t="str">
+        <x:v>DEF-003 Robot retest</x:v>
+      </x:c>
+      <x:c r="E22" s="244" t="str">
+        <x:v>5/5 Pass</x:v>
+      </x:c>
+      <x:c r="F22" s="244" t="str">
+        <x:v>2026-10-08 +07:00</x:v>
+      </x:c>
       <x:c r="G22" s="244"/>
       <x:c r="H22" s="244"/>
       <x:c r="I22" s="244"/>
@@ -5397,9 +5403,15 @@
       <x:c r="A23" s="244"/>
       <x:c r="B23" s="244"/>
       <x:c r="C23" s="244"/>
-      <x:c r="D23" s="244"/>
-      <x:c r="E23" s="244"/>
-      <x:c r="F23" s="244"/>
+      <x:c r="D23" s="244" t="str">
+        <x:v>DEF-003 Java regression</x:v>
+      </x:c>
+      <x:c r="E23" s="244" t="str">
+        <x:v>39/39 Pass</x:v>
+      </x:c>
+      <x:c r="F23" s="244" t="str">
+        <x:v>15:10:48</x:v>
+      </x:c>
       <x:c r="G23" s="244"/>
       <x:c r="H23" s="244"/>
       <x:c r="I23" s="244"/>
@@ -5412,9 +5424,15 @@
       <x:c r="A24" s="244"/>
       <x:c r="B24" s="244"/>
       <x:c r="C24" s="244"/>
-      <x:c r="D24" s="244"/>
-      <x:c r="E24" s="244"/>
-      <x:c r="F24" s="244"/>
+      <x:c r="D24" s="244" t="str">
+        <x:v>Final full regression — 2026-10-08</x:v>
+      </x:c>
+      <x:c r="E24" s="244" t="str">
+        <x:v>174 tests / 174 Pass / 0 Fail / 0 Errors / 0 Skipped</x:v>
+      </x:c>
+      <x:c r="F24" s="244" t="str">
+        <x:v>34.639 s</x:v>
+      </x:c>
       <x:c r="G24" s="244"/>
       <x:c r="H24" s="244"/>
       <x:c r="I24" s="244"/>
@@ -5427,9 +5445,15 @@
       <x:c r="A25" s="244"/>
       <x:c r="B25" s="244"/>
       <x:c r="C25" s="244"/>
-      <x:c r="D25" s="244"/>
-      <x:c r="E25" s="244"/>
-      <x:c r="F25" s="244"/>
+      <x:c r="D25" s="244" t="str">
+        <x:v>Finished</x:v>
+      </x:c>
+      <x:c r="E25" s="244" t="str">
+        <x:v>2026-10-08 18:02:26 +07:00</x:v>
+      </x:c>
+      <x:c r="F25" s="244" t="str">
+        <x:v>BUILD SUCCESS — all tests passed</x:v>
+      </x:c>
       <x:c r="G25" s="244"/>
       <x:c r="H25" s="244"/>
       <x:c r="I25" s="244"/>
@@ -7239,14 +7263,30 @@
       <x:c r="M22" s="244"/>
     </x:row>
     <x:row r="23">
-      <x:c r="A23" s="244"/>
-      <x:c r="B23" s="244"/>
-      <x:c r="C23" s="244"/>
-      <x:c r="D23" s="244"/>
-      <x:c r="E23" s="244"/>
-      <x:c r="F23" s="244"/>
-      <x:c r="G23" s="244"/>
-      <x:c r="H23" s="244"/>
+      <x:c r="A23" s="244" t="str">
+        <x:v>E2E-005-R</x:v>
+      </x:c>
+      <x:c r="B23" s="244" t="str">
+        <x:v>2026-10-08 +07:00</x:v>
+      </x:c>
+      <x:c r="C23" s="287" t="str">
+        <x:v>Robot Framework regression: login_smoke.robot + auth_flow.robot + register_interest.robot</x:v>
+      </x:c>
+      <x:c r="D23" s="244" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E23" s="244" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F23" s="244" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G23" s="244" t="str">
+        <x:v>0 / 0</x:v>
+      </x:c>
+      <x:c r="H23" s="244" t="str">
+        <x:v>PASS — DEF-003 retest</x:v>
+      </x:c>
       <x:c r="I23" s="244"/>
       <x:c r="J23" s="244"/>
       <x:c r="K23" s="244"/>
@@ -7254,14 +7294,30 @@
       <x:c r="M23" s="244"/>
     </x:row>
     <x:row r="24">
-      <x:c r="A24" s="244"/>
-      <x:c r="B24" s="244"/>
-      <x:c r="C24" s="244"/>
-      <x:c r="D24" s="244"/>
-      <x:c r="E24" s="244"/>
-      <x:c r="F24" s="244"/>
-      <x:c r="G24" s="244"/>
-      <x:c r="H24" s="244"/>
+      <x:c r="A24" s="244" t="str">
+        <x:v>REG-DEF003</x:v>
+      </x:c>
+      <x:c r="B24" s="244" t="str">
+        <x:v>2026-10-08 15:10:48 +07:00</x:v>
+      </x:c>
+      <x:c r="C24" s="287" t="str">
+        <x:v>AuthServiceRegisterTest + AuthServiceLoginTest + UserInterestServiceTest + FrontendAuthContractTest</x:v>
+      </x:c>
+      <x:c r="D24" s="244" t="n">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="E24" s="244" t="n">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="F24" s="244" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G24" s="244" t="str">
+        <x:v>0 / 0</x:v>
+      </x:c>
+      <x:c r="H24" s="244" t="str">
+        <x:v>BUILD SUCCESS</x:v>
+      </x:c>
       <x:c r="I24" s="244"/>
       <x:c r="J24" s="244"/>
       <x:c r="K24" s="244"/>
@@ -7269,14 +7325,30 @@
       <x:c r="M24" s="244"/>
     </x:row>
     <x:row r="25">
-      <x:c r="A25" s="244"/>
-      <x:c r="B25" s="244"/>
-      <x:c r="C25" s="244"/>
-      <x:c r="D25" s="244"/>
-      <x:c r="E25" s="244"/>
-      <x:c r="F25" s="244"/>
-      <x:c r="G25" s="244"/>
-      <x:c r="H25" s="244"/>
+      <x:c r="A25" s="244" t="str">
+        <x:v>REG-20261008-FINAL</x:v>
+      </x:c>
+      <x:c r="B25" s="244" t="str">
+        <x:v>2026-10-08 18:02:26 +07:00</x:v>
+      </x:c>
+      <x:c r="C25" s="244" t="str">
+        <x:v>Full Maven regression after DEF-001 and DEF-003 fixes</x:v>
+      </x:c>
+      <x:c r="D25" s="244" t="n">
+        <x:v>174</x:v>
+      </x:c>
+      <x:c r="E25" s="244" t="n">
+        <x:v>174</x:v>
+      </x:c>
+      <x:c r="F25" s="244" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G25" s="244" t="str">
+        <x:v>0 / 0</x:v>
+      </x:c>
+      <x:c r="H25" s="244" t="str">
+        <x:v>BUILD SUCCESS</x:v>
+      </x:c>
       <x:c r="I25" s="244"/>
       <x:c r="J25" s="244"/>
       <x:c r="K25" s="244"/>
@@ -10355,7 +10427,7 @@
         <x:v>ตาม request contract: empty string ต้องล้าง firstname เป็น null</x:v>
       </x:c>
       <x:c r="E19" s="47" t="str">
-        <x:v>Fail</x:v>
+        <x:v>Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="48" customHeight="1">
@@ -13291,7 +13363,7 @@
         <x:v>UpdateProfileRequest + UserService.updateProfile</x:v>
       </x:c>
       <x:c r="F39" s="287" t="str">
-        <x:v>Failed - DEF-001</x:v>
+        <x:v>Passed - DEF-001 retest</x:v>
       </x:c>
       <x:c r="G39" s="244"/>
       <x:c r="H39" s="244"/>
@@ -20590,10 +20662,10 @@
         <x:v>ตาม request contract: empty string ต้องล้าง firstname เป็น null</x:v>
       </x:c>
       <x:c r="I127" s="47" t="str">
-        <x:v>firstname ยังเป็น "Old"</x:v>
+        <x:v>firstname = null</x:v>
       </x:c>
       <x:c r="J127" s="47" t="str">
-        <x:v>Fail</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="K127" s="47" t="str">
         <x:v>Unit test (JUnit 5 / Mockito)</x:v>
@@ -20602,7 +20674,7 @@
         <x:v>UserServiceTest.updateProfile_blankFirstname_clearsFirstname</x:v>
       </x:c>
       <x:c r="M127" s="47" t="str">
-        <x:v>DEF-001 | Retest=PENDING</x:v>
+        <x:v>DEF-001 CLOSED | Full regression 2026-10-08 18:02:26 +07:00 | 174/174 Pass</x:v>
       </x:c>
     </x:row>
     <x:row r="128" ht="34" customHeight="1">

</xml_diff>

<commit_message>
fix: harden WebSocket call flow and add regression coverage
</commit_message>
<xml_diff>
--- a/test/test-cases/CPFriendFinder_TestCases.xlsx
+++ b/test/test-cases/CPFriendFinder_TestCases.xlsx
@@ -2,28 +2,30 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Scenario Summary" sheetId="1" r:id="R18f7e6589ad64ff5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="2" r:id="R577a9dc913df4a64"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Case Design &amp; Test Results" sheetId="3" r:id="R4341521b1e7145e5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS001" sheetId="4" r:id="R17a60e1316994965"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS002" sheetId="5" r:id="R7578590d2107416b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS003" sheetId="6" r:id="R7c261d4cd89243de"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS004" sheetId="7" r:id="R01077d7626914ff4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS005" sheetId="8" r:id="R6d27c36b63994d75"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS006" sheetId="9" r:id="R57fba41917474e1a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defect Summary" sheetId="10" r:id="Rc4ece78952364247"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Summary Report" sheetId="11" r:id="R09618b4b9d494fc4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution Log" sheetId="12" r:id="Rb6aad04fdd03453f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision Table" sheetId="13" r:id="Ref2cde7fba0f4ce0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS007" sheetId="14" r:id="Ra822e6921a8f4940"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS008" sheetId="15" r:id="Rcc82e7d808dd4669"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS009" sheetId="16" r:id="Rf702cfb6aa7f48b0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS010" sheetId="17" r:id="R0aa64b4305464d94"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS011" sheetId="18" r:id="Re4cb715a04a343dc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS012" sheetId="19" r:id="Rcc3c9ba7797a4289"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS013" sheetId="20" r:id="Re77055a61d1f4bb2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS014" sheetId="21" r:id="R5c5b0efc1e60433d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS015" sheetId="22" r:id="R0701dd83a9864695"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Scenario Summary" sheetId="1" r:id="Rddaf593aa2f34481"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="2" r:id="R77fbc5f84ee44632"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Case Design &amp; Test Results" sheetId="3" r:id="R3a2da5c5004f454d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS001" sheetId="4" r:id="R052c87565137416f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS002" sheetId="5" r:id="R51372dac9e064585"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS003" sheetId="6" r:id="Rc8d378e7bac54e7d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS004" sheetId="7" r:id="R12439108764b4ff2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS005" sheetId="8" r:id="R5cd9aa06db5d4637"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS006" sheetId="9" r:id="R67b1eb97781a4b9f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defect Summary" sheetId="10" r:id="R1e36a6327b0048d8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Summary Report" sheetId="11" r:id="R96fd354b95b84fcf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution Log" sheetId="12" r:id="Rcdcd89391b0040b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision Table" sheetId="13" r:id="R200d5e872f2f4e80"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS007" sheetId="14" r:id="Rd22b0caecbe14f89"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS008" sheetId="15" r:id="R7d04c24ee3424eab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS009" sheetId="16" r:id="Ra322be3a7b8b4ead"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS010" sheetId="17" r:id="R48305e86c8b44dec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS011" sheetId="18" r:id="Rb8c2d271b04e4fff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS012" sheetId="19" r:id="Rc8eefda0b19c4694"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS013" sheetId="20" r:id="R55e3ab0d60f2462a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS014" sheetId="21" r:id="R91be70bbb1fa47cc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS015" sheetId="22" r:id="R6a74623246d94671"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS016" sheetId="23" r:id="R578003eb06ef4369"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TS017" sheetId="24" r:id="R4d0710fc9c6c4cb2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -379,7 +381,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="288">
+  <x:cellXfs count="289">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1146,6 +1148,9 @@
     <x:xf numFmtId="0" fontId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="1" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -1360,32 +1365,32 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="16.799999237060547" hidden="0" customHeight="1">
-      <x:c r="A1" s="243" t="str">
+      <x:c r="A1" s="288" t="str">
         <x:v>สรุปสถานการณ์ทดสอบ</x:v>
       </x:c>
-      <x:c r="B1" s="243"/>
-      <x:c r="C1" s="243"/>
-      <x:c r="D1" s="243"/>
-      <x:c r="E1" s="243"/>
-      <x:c r="F1" s="243"/>
-      <x:c r="G1" s="243"/>
-      <x:c r="H1" s="243"/>
-      <x:c r="I1" s="243"/>
+      <x:c r="B1" s="288"/>
+      <x:c r="C1" s="288"/>
+      <x:c r="D1" s="288"/>
+      <x:c r="E1" s="288"/>
+      <x:c r="F1" s="288"/>
+      <x:c r="G1" s="288"/>
+      <x:c r="H1" s="288"/>
+      <x:c r="I1" s="288"/>
       <x:c r="J1" s="244"/>
       <x:c r="K1" s="244"/>
       <x:c r="L1" s="244"/>
       <x:c r="M1" s="244"/>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="244"/>
-      <x:c r="B2" s="244"/>
-      <x:c r="C2" s="244"/>
-      <x:c r="D2" s="244"/>
-      <x:c r="E2" s="244"/>
-      <x:c r="F2" s="244"/>
-      <x:c r="G2" s="244"/>
-      <x:c r="H2" s="244"/>
-      <x:c r="I2" s="244"/>
+      <x:c r="A2" s="287"/>
+      <x:c r="B2" s="287"/>
+      <x:c r="C2" s="287"/>
+      <x:c r="D2" s="287"/>
+      <x:c r="E2" s="287"/>
+      <x:c r="F2" s="287"/>
+      <x:c r="G2" s="287"/>
+      <x:c r="H2" s="287"/>
+      <x:c r="I2" s="287"/>
       <x:c r="J2" s="244"/>
       <x:c r="K2" s="244"/>
       <x:c r="L2" s="244"/>
@@ -1623,15 +1628,15 @@
       <x:c r="M9" s="244"/>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="244"/>
-      <x:c r="B10" s="244"/>
-      <x:c r="C10" s="244"/>
-      <x:c r="D10" s="244"/>
-      <x:c r="E10" s="244"/>
-      <x:c r="F10" s="244"/>
-      <x:c r="G10" s="244"/>
-      <x:c r="H10" s="244"/>
-      <x:c r="I10" s="244"/>
+      <x:c r="A10" s="287"/>
+      <x:c r="B10" s="287"/>
+      <x:c r="C10" s="287"/>
+      <x:c r="D10" s="287"/>
+      <x:c r="E10" s="287"/>
+      <x:c r="F10" s="287"/>
+      <x:c r="G10" s="287"/>
+      <x:c r="H10" s="287"/>
+      <x:c r="I10" s="287"/>
       <x:c r="J10" s="244"/>
       <x:c r="K10" s="244"/>
       <x:c r="L10" s="244"/>
@@ -2198,18 +2203,20 @@
       <x:c r="M28" s="244"/>
     </x:row>
     <x:row r="29" ht="42" customHeight="1">
-      <x:c r="A29" s="287"/>
+      <x:c r="A29" s="287" t="str">
+        <x:v>UC-WS-01 / UC-CALL-01</x:v>
+      </x:c>
       <x:c r="B29" s="287" t="str">
-        <x:v>Latest Total</x:v>
+        <x:v>TS016</x:v>
       </x:c>
       <x:c r="C29" s="287" t="str">
-        <x:v>Executed coverage through TS015 based on current develop</x:v>
+        <x:v>WebSocket / WebRTC Security &amp; Call Signaling</x:v>
       </x:c>
       <x:c r="D29" s="287" t="n">
-        <x:v>171</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="E29" s="287" t="n">
-        <x:v>171</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="F29" s="287" t="n">
         <x:v>0</x:v>
@@ -2221,7 +2228,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I29" s="287" t="str">
-        <x:v>Documented: 171 executed / 171 Pass / 0 Fail. Final Maven regression: 174 tests / 174 Pass / 0 Fail / 0 Errors / 0 Skipped. DEF-001 and DEF-003 closed.</x:v>
+        <x:v>WebSocketAuthChannelInterceptor + ChatMessageService + call.js/friend.js | DEF-002/004/005 CLOSED</x:v>
       </x:c>
       <x:c r="J29" s="244"/>
       <x:c r="K29" s="244"/>
@@ -2229,30 +2236,64 @@
       <x:c r="M29" s="244"/>
     </x:row>
     <x:row r="30">
-      <x:c r="A30" s="244"/>
-      <x:c r="B30" s="244"/>
-      <x:c r="C30" s="244"/>
-      <x:c r="D30" s="244"/>
-      <x:c r="E30" s="244"/>
-      <x:c r="F30" s="244"/>
-      <x:c r="G30" s="244"/>
-      <x:c r="H30" s="244"/>
-      <x:c r="I30" s="244"/>
+      <x:c r="A30" s="287" t="str">
+        <x:v>UC-E2E-01</x:v>
+      </x:c>
+      <x:c r="B30" s="287" t="str">
+        <x:v>TS017</x:v>
+      </x:c>
+      <x:c r="C30" s="287" t="str">
+        <x:v>Robot Framework Browser E2E</x:v>
+      </x:c>
+      <x:c r="D30" s="287" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E30" s="287" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F30" s="287" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G30" s="287" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H30" s="287" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I30" s="287" t="str">
+        <x:v>login_smoke.robot + auth_flow.robot + register_interest.robot</x:v>
+      </x:c>
       <x:c r="J30" s="244"/>
       <x:c r="K30" s="244"/>
       <x:c r="L30" s="244"/>
       <x:c r="M30" s="244"/>
     </x:row>
     <x:row r="31">
-      <x:c r="A31" s="244"/>
-      <x:c r="B31" s="244"/>
-      <x:c r="C31" s="244"/>
-      <x:c r="D31" s="244"/>
-      <x:c r="E31" s="244"/>
-      <x:c r="F31" s="244"/>
-      <x:c r="G31" s="244"/>
-      <x:c r="H31" s="244"/>
-      <x:c r="I31" s="244"/>
+      <x:c r="A31" s="287"/>
+      <x:c r="B31" s="287" t="str">
+        <x:v>Latest Total</x:v>
+      </x:c>
+      <x:c r="C31" s="287" t="str">
+        <x:v>Executed coverage through TS017 on current tester branch</x:v>
+      </x:c>
+      <x:c r="D31" s="287" t="n">
+        <x:v>182</x:v>
+      </x:c>
+      <x:c r="E31" s="287" t="n">
+        <x:v>182</x:v>
+      </x:c>
+      <x:c r="F31" s="287" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G31" s="287" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H31" s="287" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I31" s="287" t="str">
+        <x:v>Documented: 182 executed / 182 Pass / 0 Fail. Final Maven regression: 180/180 Pass. Robot Framework: 5/5 Pass. DEF-001 to DEF-005 documented defects are closed.</x:v>
+      </x:c>
       <x:c r="J31" s="244"/>
       <x:c r="K31" s="244"/>
       <x:c r="L31" s="244"/>
@@ -3320,34 +3361,34 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="243" t="str">
+      <x:c r="A1" s="288" t="str">
         <x:v>Defect Summary</x:v>
       </x:c>
-      <x:c r="B1" s="243"/>
-      <x:c r="C1" s="243"/>
-      <x:c r="D1" s="243"/>
-      <x:c r="E1" s="243"/>
-      <x:c r="F1" s="243"/>
-      <x:c r="G1" s="243"/>
-      <x:c r="H1" s="243"/>
-      <x:c r="I1" s="243"/>
-      <x:c r="J1" s="243"/>
-      <x:c r="K1" s="243"/>
+      <x:c r="B1" s="288"/>
+      <x:c r="C1" s="288"/>
+      <x:c r="D1" s="288"/>
+      <x:c r="E1" s="288"/>
+      <x:c r="F1" s="288"/>
+      <x:c r="G1" s="288"/>
+      <x:c r="H1" s="288"/>
+      <x:c r="I1" s="288"/>
+      <x:c r="J1" s="288"/>
+      <x:c r="K1" s="288"/>
       <x:c r="L1" s="244"/>
       <x:c r="M1" s="244"/>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="244"/>
-      <x:c r="B2" s="244"/>
-      <x:c r="C2" s="244"/>
-      <x:c r="D2" s="244"/>
-      <x:c r="E2" s="244"/>
-      <x:c r="F2" s="244"/>
-      <x:c r="G2" s="244"/>
-      <x:c r="H2" s="244"/>
-      <x:c r="I2" s="244"/>
-      <x:c r="J2" s="244"/>
-      <x:c r="K2" s="244"/>
+      <x:c r="A2" s="287"/>
+      <x:c r="B2" s="287"/>
+      <x:c r="C2" s="287"/>
+      <x:c r="D2" s="287"/>
+      <x:c r="E2" s="287"/>
+      <x:c r="F2" s="287"/>
+      <x:c r="G2" s="287"/>
+      <x:c r="H2" s="287"/>
+      <x:c r="I2" s="287"/>
+      <x:c r="J2" s="287"/>
+      <x:c r="K2" s="287"/>
       <x:c r="L2" s="244"/>
       <x:c r="M2" s="244"/>
     </x:row>
@@ -3417,35 +3458,35 @@
         <x:v>2026-10-07 16:46:16 +07:00</x:v>
       </x:c>
       <x:c r="J4" s="276" t="str">
-        <x:v>UserServiceTest.updateProfile_blankFirstname_clearsFirstname passed. Final full regression 2026-10-08 18:02:26 +07:00: 174/174 Pass, 0 Fail, 0 Errors, 0 Skipped.</x:v>
+        <x:v>UserServiceTest.updateProfile_blankFirstname_clearsFirstname passed. Final regression later remained green.</x:v>
       </x:c>
       <x:c r="K4" s="278" t="str">
-        <x:v>CLOSED / Retest passed 2026-10-08 +07:00 after UserService fix. Empty string now clears optional profile string fields while omitted fields remain unchanged.</x:v>
+        <x:v>CLOSED / Retest passed. Empty string clears optional profile string fields while omitted fields remain unchanged.</x:v>
       </x:c>
       <x:c r="L4" s="244"/>
       <x:c r="M4" s="244"/>
     </x:row>
     <x:row r="5" ht="88" customHeight="1">
       <x:c r="A5" s="287" t="str">
-        <x:v>DEF-003</x:v>
+        <x:v>DEF-002</x:v>
       </x:c>
       <x:c r="B5" s="287" t="str">
-        <x:v>E2E-005</x:v>
+        <x:v>WSA-002</x:v>
       </x:c>
       <x:c r="C5" s="287" t="str">
-        <x:v>Selected interests during registration are not saved</x:v>
+        <x:v>WebSocket CONNECT trusts unverified STOMP login as authenticated user</x:v>
       </x:c>
       <x:c r="D5" s="287" t="str">
-        <x:v>ผู้ใช้เลือก Interest ใน Step 3 และสมัคร/เข้าสู่ระบบสำเร็จ แต่หลัง Login แล้ว GET /api/users/me/interests คืนรายการว่าง</x:v>
+        <x:v>Client ที่ไม่มี authenticated HTTP session สามารถใส่ UUID ใน STOMP login และถูกสร้างเป็น Principal ได้</x:v>
       </x:c>
       <x:c r="E5" s="287" t="str">
-        <x:v>Selected interests are persisted and returned for the newly registered user</x:v>
+        <x:v>Only an authenticated HTTP/session Principal may identify the WebSocket user</x:v>
       </x:c>
       <x:c r="F5" s="287" t="str">
-        <x:v>Interest count = 0</x:v>
+        <x:v>Unverified STOMP login header could become the WebSocket Principal</x:v>
       </x:c>
       <x:c r="G5" s="287" t="str">
-        <x:v>Medium</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="H5" s="287" t="str">
         <x:v>CLOSED</x:v>
@@ -3454,56 +3495,122 @@
         <x:v>2026-10-08 +07:00</x:v>
       </x:c>
       <x:c r="J5" s="287" t="str">
-        <x:v>Manual API retest passed. Robot Framework regression: 5/5 Pass including E2E-005. Java targeted regression: 39/39 Pass. Final full regression: 174/174 Pass.</x:v>
+        <x:v>WebSocketAuthChannelInterceptorTest: 2/2 Pass after fix. Full Maven regression after fix: 176/176 Pass.</x:v>
       </x:c>
       <x:c r="K5" s="287" t="str">
-        <x:v>CLOSED / Retest passed 2026-10-08 +07:00. Selected interests are saved during registration and returned for the newly registered user.</x:v>
+        <x:v>CLOSED / Removed trust in STOMP login. Existing HTTP/session Principal is preserved; unauthenticated CONNECT remains without Principal.</x:v>
       </x:c>
       <x:c r="L5" s="244"/>
       <x:c r="M5" s="244"/>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="244"/>
-      <x:c r="B6" s="244"/>
-      <x:c r="C6" s="244"/>
-      <x:c r="D6" s="244"/>
-      <x:c r="E6" s="244"/>
-      <x:c r="F6" s="244"/>
-      <x:c r="G6" s="244"/>
-      <x:c r="H6" s="244"/>
-      <x:c r="I6" s="244"/>
-      <x:c r="J6" s="244"/>
-      <x:c r="K6" s="244"/>
+      <x:c r="A6" s="287" t="str">
+        <x:v>DEF-003</x:v>
+      </x:c>
+      <x:c r="B6" s="287" t="str">
+        <x:v>E2E-005</x:v>
+      </x:c>
+      <x:c r="C6" s="287" t="str">
+        <x:v>Selected interests during registration are not saved</x:v>
+      </x:c>
+      <x:c r="D6" s="287" t="str">
+        <x:v>ผู้ใช้เลือก Interest ใน Step 3 และสมัคร/เข้าสู่ระบบสำเร็จ แต่หลัง Login แล้ว GET /api/users/me/interests คืนรายการว่าง</x:v>
+      </x:c>
+      <x:c r="E6" s="287" t="str">
+        <x:v>Selected interests are persisted and returned for the newly registered user</x:v>
+      </x:c>
+      <x:c r="F6" s="287" t="str">
+        <x:v>Interest count = 0</x:v>
+      </x:c>
+      <x:c r="G6" s="287" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="H6" s="287" t="str">
+        <x:v>CLOSED</x:v>
+      </x:c>
+      <x:c r="I6" s="287" t="str">
+        <x:v>2026-10-08 +07:00</x:v>
+      </x:c>
+      <x:c r="J6" s="287" t="str">
+        <x:v>Manual API retest passed. Robot Framework regression: 5/5 Pass including E2E-005. Java targeted regression: 39/39 Pass.</x:v>
+      </x:c>
+      <x:c r="K6" s="287" t="str">
+        <x:v>CLOSED / Selected interests are saved during registration and returned for the newly registered user.</x:v>
+      </x:c>
       <x:c r="L6" s="244"/>
       <x:c r="M6" s="244"/>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="244"/>
-      <x:c r="B7" s="244"/>
-      <x:c r="C7" s="244"/>
-      <x:c r="D7" s="244"/>
-      <x:c r="E7" s="244"/>
-      <x:c r="F7" s="244"/>
-      <x:c r="G7" s="244"/>
-      <x:c r="H7" s="244"/>
-      <x:c r="I7" s="244"/>
-      <x:c r="J7" s="244"/>
-      <x:c r="K7" s="244"/>
+      <x:c r="A7" s="287" t="str">
+        <x:v>DEF-004</x:v>
+      </x:c>
+      <x:c r="B7" s="287" t="str">
+        <x:v>CALL-001</x:v>
+      </x:c>
+      <x:c r="C7" s="287" t="str">
+        <x:v>LEAVE signal rejected after room membership ended</x:v>
+      </x:c>
+      <x:c r="D7" s="287" t="str">
+        <x:v>ผู้ใช้เพิ่งออกจากห้องแล้ว client ส่ง WebSocket LEAVE แต่ service ตรวจ active membership ก่อนดู signal type จึงคืน 403</x:v>
+      </x:c>
+      <x:c r="E7" s="287" t="str">
+        <x:v>A user with membership history may relay LEAVE after leaving; a never-member must remain forbidden</x:v>
+      </x:c>
+      <x:c r="F7" s="287" t="str">
+        <x:v>403 FORBIDDEN "You are not a member of this room" for a former member</x:v>
+      </x:c>
+      <x:c r="G7" s="287" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="H7" s="287" t="str">
+        <x:v>CLOSED</x:v>
+      </x:c>
+      <x:c r="I7" s="287" t="str">
+        <x:v>2026-10-08 19:41:47 +07:00</x:v>
+      </x:c>
+      <x:c r="J7" s="287" t="str">
+        <x:v>Reproduced by ChatMessageServiceTest. Focused LEAVE tests passed after fix; full Maven regression: 178/178 Pass.</x:v>
+      </x:c>
+      <x:c r="K7" s="287" t="str">
+        <x:v>CLOSED / LEAVE validates membership history; other call signals still require active membership.</x:v>
+      </x:c>
       <x:c r="L7" s="244"/>
       <x:c r="M7" s="244"/>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="244"/>
-      <x:c r="B8" s="244"/>
-      <x:c r="C8" s="244"/>
-      <x:c r="D8" s="244"/>
-      <x:c r="E8" s="244"/>
-      <x:c r="F8" s="244"/>
-      <x:c r="G8" s="244"/>
-      <x:c r="H8" s="244"/>
-      <x:c r="I8" s="244"/>
-      <x:c r="J8" s="244"/>
-      <x:c r="K8" s="244"/>
+      <x:c r="A8" s="287" t="str">
+        <x:v>DEF-005</x:v>
+      </x:c>
+      <x:c r="B8" s="287" t="str">
+        <x:v>CALL-003 / CALL-004</x:v>
+      </x:c>
+      <x:c r="C8" s="287" t="str">
+        <x:v>Camera MEDIA state is not synchronized between call participants</x:v>
+      </x:c>
+      <x:c r="D8" s="287" t="str">
+        <x:v>การปิด/เปิดกล้องเปลี่ยนเฉพาะ local track/UI และ client ไม่จัดการ incoming MEDIA signal</x:v>
+      </x:c>
+      <x:c r="E8" s="287" t="str">
+        <x:v>Camera state is published through WebSocket and the remote client handles MEDIA to update UI</x:v>
+      </x:c>
+      <x:c r="F8" s="287" t="str">
+        <x:v>No MEDIA publish from camera toggle and no incoming MEDIA handler</x:v>
+      </x:c>
+      <x:c r="G8" s="287" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="H8" s="287" t="str">
+        <x:v>CLOSED</x:v>
+      </x:c>
+      <x:c r="I8" s="287" t="str">
+        <x:v>2026-10-08 20:03:42 +07:00</x:v>
+      </x:c>
+      <x:c r="J8" s="287" t="str">
+        <x:v>CallFrontendContractTest reproduced 2/2 failures; targeted retest passed 2/2. Final Maven regression: 180/180 Pass. Robot regression: 5/5 Pass.</x:v>
+      </x:c>
+      <x:c r="K8" s="287" t="str">
+        <x:v>CLOSED / call.js now publishes and handles MEDIA state; friend.js updates remote video/avatar state.</x:v>
+      </x:c>
       <x:c r="L8" s="244"/>
       <x:c r="M8" s="244"/>
     </x:row>
@@ -4908,14 +5015,14 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="16.799999237060547" hidden="0" customHeight="1">
-      <x:c r="A1" s="243" t="str">
+      <x:c r="A1" s="288" t="str">
         <x:v>Test Summary Report</x:v>
       </x:c>
-      <x:c r="B1" s="243"/>
-      <x:c r="C1" s="243"/>
-      <x:c r="D1" s="243"/>
-      <x:c r="E1" s="243"/>
-      <x:c r="F1" s="243"/>
+      <x:c r="B1" s="288"/>
+      <x:c r="C1" s="288"/>
+      <x:c r="D1" s="288"/>
+      <x:c r="E1" s="288"/>
+      <x:c r="F1" s="288"/>
       <x:c r="G1" s="244"/>
       <x:c r="H1" s="244"/>
       <x:c r="I1" s="244"/>
@@ -4925,12 +5032,12 @@
       <x:c r="M1" s="244"/>
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
-      <x:c r="A2" s="244"/>
-      <x:c r="B2" s="244"/>
-      <x:c r="C2" s="244"/>
-      <x:c r="D2" s="244"/>
-      <x:c r="E2" s="244"/>
-      <x:c r="F2" s="244"/>
+      <x:c r="A2" s="287"/>
+      <x:c r="B2" s="287"/>
+      <x:c r="C2" s="287"/>
+      <x:c r="D2" s="287"/>
+      <x:c r="E2" s="287"/>
+      <x:c r="F2" s="287"/>
       <x:c r="G2" s="244"/>
       <x:c r="H2" s="244"/>
       <x:c r="I2" s="244"/>
@@ -4946,7 +5053,7 @@
       <x:c r="B3" s="247" t="str">
         <x:v>Result</x:v>
       </x:c>
-      <x:c r="C3" s="244"/>
+      <x:c r="C3" s="287"/>
       <x:c r="D3" s="245" t="str">
         <x:v>Run</x:v>
       </x:c>
@@ -4971,7 +5078,7 @@
       <x:c r="B4" s="269" t="str">
         <x:v>develop</x:v>
       </x:c>
-      <x:c r="C4" s="244"/>
+      <x:c r="C4" s="287"/>
       <x:c r="D4" s="279" t="str">
         <x:v>REG-001</x:v>
       </x:c>
@@ -4996,14 +5103,14 @@
       <x:c r="B5" s="270" t="n">
         <x:v>48</x:v>
       </x:c>
-      <x:c r="C5" s="244"/>
-      <x:c r="D5" s="244" t="str">
+      <x:c r="C5" s="287"/>
+      <x:c r="D5" s="287" t="str">
         <x:v>TS001</x:v>
       </x:c>
-      <x:c r="E5" s="244" t="str">
+      <x:c r="E5" s="287" t="str">
         <x:v>13/13 Pass</x:v>
       </x:c>
-      <x:c r="F5" s="244" t="str">
+      <x:c r="F5" s="287" t="str">
         <x:v>44.031 s</x:v>
       </x:c>
       <x:c r="G5" s="244"/>
@@ -5021,14 +5128,14 @@
       <x:c r="B6" s="270" t="n">
         <x:v>43</x:v>
       </x:c>
-      <x:c r="C6" s="244"/>
-      <x:c r="D6" s="244" t="str">
+      <x:c r="C6" s="287"/>
+      <x:c r="D6" s="287" t="str">
         <x:v>TS002</x:v>
       </x:c>
-      <x:c r="E6" s="244" t="str">
+      <x:c r="E6" s="287" t="str">
         <x:v>11/11 Pass</x:v>
       </x:c>
-      <x:c r="F6" s="244" t="str">
+      <x:c r="F6" s="287" t="str">
         <x:v>25.561 s</x:v>
       </x:c>
       <x:c r="G6" s="244"/>
@@ -5046,14 +5153,14 @@
       <x:c r="B7" s="270" t="n">
         <x:v>43</x:v>
       </x:c>
-      <x:c r="C7" s="244"/>
-      <x:c r="D7" s="244" t="str">
+      <x:c r="C7" s="287"/>
+      <x:c r="D7" s="287" t="str">
         <x:v>TS003</x:v>
       </x:c>
-      <x:c r="E7" s="244" t="str">
+      <x:c r="E7" s="287" t="str">
         <x:v>8/8 Pass</x:v>
       </x:c>
-      <x:c r="F7" s="244" t="str">
+      <x:c r="F7" s="287" t="str">
         <x:v>30.715 s</x:v>
       </x:c>
       <x:c r="G7" s="244"/>
@@ -5071,14 +5178,14 @@
       <x:c r="B8" s="270" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="C8" s="244"/>
-      <x:c r="D8" s="244" t="str">
+      <x:c r="C8" s="287"/>
+      <x:c r="D8" s="287" t="str">
         <x:v>TS004</x:v>
       </x:c>
-      <x:c r="E8" s="244" t="str">
+      <x:c r="E8" s="287" t="str">
         <x:v>7/7 Pass</x:v>
       </x:c>
-      <x:c r="F8" s="244" t="str">
+      <x:c r="F8" s="287" t="str">
         <x:v>48.881 s</x:v>
       </x:c>
       <x:c r="G8" s="244"/>
@@ -5096,14 +5203,14 @@
       <x:c r="B9" s="271" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="C9" s="244"/>
-      <x:c r="D9" s="244" t="str">
+      <x:c r="C9" s="287"/>
+      <x:c r="D9" s="287" t="str">
         <x:v>TS005</x:v>
       </x:c>
-      <x:c r="E9" s="244" t="str">
+      <x:c r="E9" s="287" t="str">
         <x:v>4/4 Pass</x:v>
       </x:c>
-      <x:c r="F9" s="244" t="str">
+      <x:c r="F9" s="287" t="str">
         <x:v>56.569 s</x:v>
       </x:c>
       <x:c r="G9" s="244"/>
@@ -5115,12 +5222,12 @@
       <x:c r="M9" s="244"/>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
-      <x:c r="A10" s="244"/>
-      <x:c r="B10" s="244"/>
-      <x:c r="C10" s="244"/>
-      <x:c r="D10" s="244"/>
-      <x:c r="E10" s="244"/>
-      <x:c r="F10" s="244"/>
+      <x:c r="A10" s="287"/>
+      <x:c r="B10" s="287"/>
+      <x:c r="C10" s="287"/>
+      <x:c r="D10" s="287"/>
+      <x:c r="E10" s="287"/>
+      <x:c r="F10" s="287"/>
       <x:c r="G10" s="244"/>
       <x:c r="H10" s="244"/>
       <x:c r="I10" s="244"/>
@@ -5191,7 +5298,7 @@
         <x:v>Designed test cases</x:v>
       </x:c>
       <x:c r="B14" s="287" t="n">
-        <x:v>171</x:v>
+        <x:v>182</x:v>
       </x:c>
       <x:c r="C14" s="287"/>
       <x:c r="D14" s="287" t="str">
@@ -5216,7 +5323,7 @@
         <x:v>Executed documented cases</x:v>
       </x:c>
       <x:c r="B15" s="287" t="n">
-        <x:v>171</x:v>
+        <x:v>182</x:v>
       </x:c>
       <x:c r="C15" s="287"/>
       <x:c r="D15" s="287" t="str">
@@ -5241,7 +5348,7 @@
         <x:v>Pass</x:v>
       </x:c>
       <x:c r="B16" s="287" t="n">
-        <x:v>171</x:v>
+        <x:v>182</x:v>
       </x:c>
       <x:c r="C16" s="287"/>
       <x:c r="D16" s="287" t="str">
@@ -5316,7 +5423,7 @@
         <x:v>Retest</x:v>
       </x:c>
       <x:c r="B19" s="287" t="str">
-        <x:v>DEF-001 PASSED / CLOSED; DEF-003 PASSED / CLOSED</x:v>
+        <x:v>DEF-001, DEF-002, DEF-003, DEF-004, DEF-005 PASSED / CLOSED</x:v>
       </x:c>
       <x:c r="C19" s="287"/>
       <x:c r="D19" s="287" t="str">
@@ -5379,16 +5486,16 @@
       <x:c r="M21" s="244"/>
     </x:row>
     <x:row r="22">
-      <x:c r="A22" s="244"/>
-      <x:c r="B22" s="244"/>
-      <x:c r="C22" s="244"/>
-      <x:c r="D22" s="244" t="str">
+      <x:c r="A22" s="287"/>
+      <x:c r="B22" s="287"/>
+      <x:c r="C22" s="287"/>
+      <x:c r="D22" s="287" t="str">
         <x:v>DEF-003 Robot retest</x:v>
       </x:c>
-      <x:c r="E22" s="244" t="str">
+      <x:c r="E22" s="287" t="str">
         <x:v>5/5 Pass</x:v>
       </x:c>
-      <x:c r="F22" s="244" t="str">
+      <x:c r="F22" s="287" t="str">
         <x:v>2026-10-08 +07:00</x:v>
       </x:c>
       <x:c r="G22" s="244"/>
@@ -5400,16 +5507,16 @@
       <x:c r="M22" s="244"/>
     </x:row>
     <x:row r="23">
-      <x:c r="A23" s="244"/>
-      <x:c r="B23" s="244"/>
-      <x:c r="C23" s="244"/>
-      <x:c r="D23" s="244" t="str">
+      <x:c r="A23" s="287"/>
+      <x:c r="B23" s="287"/>
+      <x:c r="C23" s="287"/>
+      <x:c r="D23" s="287" t="str">
         <x:v>DEF-003 Java regression</x:v>
       </x:c>
-      <x:c r="E23" s="244" t="str">
+      <x:c r="E23" s="287" t="str">
         <x:v>39/39 Pass</x:v>
       </x:c>
-      <x:c r="F23" s="244" t="str">
+      <x:c r="F23" s="287" t="str">
         <x:v>15:10:48</x:v>
       </x:c>
       <x:c r="G23" s="244"/>
@@ -5421,16 +5528,16 @@
       <x:c r="M23" s="244"/>
     </x:row>
     <x:row r="24">
-      <x:c r="A24" s="244"/>
-      <x:c r="B24" s="244"/>
-      <x:c r="C24" s="244"/>
-      <x:c r="D24" s="244" t="str">
+      <x:c r="A24" s="287"/>
+      <x:c r="B24" s="287"/>
+      <x:c r="C24" s="287"/>
+      <x:c r="D24" s="287" t="str">
         <x:v>Final full regression — 2026-10-08</x:v>
       </x:c>
-      <x:c r="E24" s="244" t="str">
+      <x:c r="E24" s="287" t="str">
         <x:v>174 tests / 174 Pass / 0 Fail / 0 Errors / 0 Skipped</x:v>
       </x:c>
-      <x:c r="F24" s="244" t="str">
+      <x:c r="F24" s="287" t="str">
         <x:v>34.639 s</x:v>
       </x:c>
       <x:c r="G24" s="244"/>
@@ -5442,16 +5549,16 @@
       <x:c r="M24" s="244"/>
     </x:row>
     <x:row r="25">
-      <x:c r="A25" s="244"/>
-      <x:c r="B25" s="244"/>
-      <x:c r="C25" s="244"/>
-      <x:c r="D25" s="244" t="str">
+      <x:c r="A25" s="287"/>
+      <x:c r="B25" s="287"/>
+      <x:c r="C25" s="287"/>
+      <x:c r="D25" s="287" t="str">
         <x:v>Finished</x:v>
       </x:c>
-      <x:c r="E25" s="244" t="str">
+      <x:c r="E25" s="287" t="str">
         <x:v>2026-10-08 18:02:26 +07:00</x:v>
       </x:c>
-      <x:c r="F25" s="244" t="str">
+      <x:c r="F25" s="287" t="str">
         <x:v>BUILD SUCCESS — all tests passed</x:v>
       </x:c>
       <x:c r="G25" s="244"/>
@@ -5463,12 +5570,18 @@
       <x:c r="M25" s="244"/>
     </x:row>
     <x:row r="26">
-      <x:c r="A26" s="244"/>
-      <x:c r="B26" s="244"/>
-      <x:c r="C26" s="244"/>
-      <x:c r="D26" s="244"/>
-      <x:c r="E26" s="244"/>
-      <x:c r="F26" s="244"/>
+      <x:c r="A26" s="287"/>
+      <x:c r="B26" s="287"/>
+      <x:c r="C26" s="287"/>
+      <x:c r="D26" s="287" t="str">
+        <x:v>WebSocket auth targeted retest</x:v>
+      </x:c>
+      <x:c r="E26" s="287" t="str">
+        <x:v>2/2 Pass</x:v>
+      </x:c>
+      <x:c r="F26" s="287" t="str">
+        <x:v>2026-10-08 +07:00</x:v>
+      </x:c>
       <x:c r="G26" s="244"/>
       <x:c r="H26" s="244"/>
       <x:c r="I26" s="244"/>
@@ -5478,12 +5591,18 @@
       <x:c r="M26" s="244"/>
     </x:row>
     <x:row r="27">
-      <x:c r="A27" s="244"/>
-      <x:c r="B27" s="244"/>
-      <x:c r="C27" s="244"/>
-      <x:c r="D27" s="244"/>
-      <x:c r="E27" s="244"/>
-      <x:c r="F27" s="244"/>
+      <x:c r="A27" s="287"/>
+      <x:c r="B27" s="287"/>
+      <x:c r="C27" s="287"/>
+      <x:c r="D27" s="287" t="str">
+        <x:v>LEAVE signaling targeted retest</x:v>
+      </x:c>
+      <x:c r="E27" s="287" t="str">
+        <x:v>2/2 Pass</x:v>
+      </x:c>
+      <x:c r="F27" s="287" t="str">
+        <x:v>2026-10-08 +07:00</x:v>
+      </x:c>
       <x:c r="G27" s="244"/>
       <x:c r="H27" s="244"/>
       <x:c r="I27" s="244"/>
@@ -5493,12 +5612,18 @@
       <x:c r="M27" s="244"/>
     </x:row>
     <x:row r="28">
-      <x:c r="A28" s="244"/>
-      <x:c r="B28" s="244"/>
-      <x:c r="C28" s="244"/>
-      <x:c r="D28" s="244"/>
-      <x:c r="E28" s="244"/>
-      <x:c r="F28" s="244"/>
+      <x:c r="A28" s="287"/>
+      <x:c r="B28" s="287"/>
+      <x:c r="C28" s="287"/>
+      <x:c r="D28" s="287" t="str">
+        <x:v>Full Maven regression — after DEF-004</x:v>
+      </x:c>
+      <x:c r="E28" s="287" t="str">
+        <x:v>178/178 Pass</x:v>
+      </x:c>
+      <x:c r="F28" s="287" t="str">
+        <x:v>2026-10-08 19:51:02 +07:00</x:v>
+      </x:c>
       <x:c r="G28" s="244"/>
       <x:c r="H28" s="244"/>
       <x:c r="I28" s="244"/>
@@ -5508,12 +5633,18 @@
       <x:c r="M28" s="244"/>
     </x:row>
     <x:row r="29">
-      <x:c r="A29" s="244"/>
-      <x:c r="B29" s="244"/>
-      <x:c r="C29" s="244"/>
-      <x:c r="D29" s="244"/>
-      <x:c r="E29" s="244"/>
-      <x:c r="F29" s="244"/>
+      <x:c r="A29" s="287"/>
+      <x:c r="B29" s="287"/>
+      <x:c r="C29" s="287"/>
+      <x:c r="D29" s="287" t="str">
+        <x:v>MEDIA frontend contract retest</x:v>
+      </x:c>
+      <x:c r="E29" s="287" t="str">
+        <x:v>2/2 Pass</x:v>
+      </x:c>
+      <x:c r="F29" s="287" t="str">
+        <x:v>2026-10-08 20:14:49 +07:00</x:v>
+      </x:c>
       <x:c r="G29" s="244"/>
       <x:c r="H29" s="244"/>
       <x:c r="I29" s="244"/>
@@ -5523,12 +5654,18 @@
       <x:c r="M29" s="244"/>
     </x:row>
     <x:row r="30">
-      <x:c r="A30" s="244"/>
-      <x:c r="B30" s="244"/>
-      <x:c r="C30" s="244"/>
-      <x:c r="D30" s="244"/>
-      <x:c r="E30" s="244"/>
-      <x:c r="F30" s="244"/>
+      <x:c r="A30" s="287"/>
+      <x:c r="B30" s="287"/>
+      <x:c r="C30" s="287"/>
+      <x:c r="D30" s="287" t="str">
+        <x:v>Final full Maven regression</x:v>
+      </x:c>
+      <x:c r="E30" s="287" t="str">
+        <x:v>180/180 Pass</x:v>
+      </x:c>
+      <x:c r="F30" s="287" t="str">
+        <x:v>2026-10-08 20:16:01 +07:00</x:v>
+      </x:c>
       <x:c r="G30" s="244"/>
       <x:c r="H30" s="244"/>
       <x:c r="I30" s="244"/>
@@ -5538,12 +5675,18 @@
       <x:c r="M30" s="244"/>
     </x:row>
     <x:row r="31">
-      <x:c r="A31" s="244"/>
-      <x:c r="B31" s="244"/>
-      <x:c r="C31" s="244"/>
-      <x:c r="D31" s="244"/>
-      <x:c r="E31" s="244"/>
-      <x:c r="F31" s="244"/>
+      <x:c r="A31" s="287"/>
+      <x:c r="B31" s="287"/>
+      <x:c r="C31" s="287"/>
+      <x:c r="D31" s="287" t="str">
+        <x:v>Final Robot Framework regression</x:v>
+      </x:c>
+      <x:c r="E31" s="287" t="str">
+        <x:v>5/5 Pass</x:v>
+      </x:c>
+      <x:c r="F31" s="287" t="str">
+        <x:v>2026-10-08 +07:00</x:v>
+      </x:c>
       <x:c r="G31" s="244"/>
       <x:c r="H31" s="244"/>
       <x:c r="I31" s="244"/>
@@ -5553,12 +5696,18 @@
       <x:c r="M31" s="244"/>
     </x:row>
     <x:row r="32">
-      <x:c r="A32" s="244"/>
-      <x:c r="B32" s="244"/>
-      <x:c r="C32" s="244"/>
-      <x:c r="D32" s="244"/>
-      <x:c r="E32" s="244"/>
-      <x:c r="F32" s="244"/>
+      <x:c r="A32" s="287"/>
+      <x:c r="B32" s="287"/>
+      <x:c r="C32" s="287"/>
+      <x:c r="D32" s="287" t="str">
+        <x:v>Final status</x:v>
+      </x:c>
+      <x:c r="E32" s="287" t="str">
+        <x:v>BUILD SUCCESS / E2E PASS</x:v>
+      </x:c>
+      <x:c r="F32" s="287" t="str">
+        <x:v>All documented defects closed</x:v>
+      </x:c>
       <x:c r="G32" s="244"/>
       <x:c r="H32" s="244"/>
       <x:c r="I32" s="244"/>
@@ -6611,16 +6760,16 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="16.799999237060547" hidden="0" customHeight="1">
-      <x:c r="A1" s="243" t="str">
+      <x:c r="A1" s="288" t="str">
         <x:v>Execution Log</x:v>
       </x:c>
-      <x:c r="B1" s="243"/>
-      <x:c r="C1" s="243"/>
-      <x:c r="D1" s="243"/>
-      <x:c r="E1" s="243"/>
-      <x:c r="F1" s="243"/>
-      <x:c r="G1" s="243"/>
-      <x:c r="H1" s="243"/>
+      <x:c r="B1" s="288"/>
+      <x:c r="C1" s="288"/>
+      <x:c r="D1" s="288"/>
+      <x:c r="E1" s="288"/>
+      <x:c r="F1" s="288"/>
+      <x:c r="G1" s="288"/>
+      <x:c r="H1" s="288"/>
       <x:c r="I1" s="244"/>
       <x:c r="J1" s="244"/>
       <x:c r="K1" s="244"/>
@@ -6628,14 +6777,14 @@
       <x:c r="M1" s="244"/>
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
-      <x:c r="A2" s="244"/>
-      <x:c r="B2" s="244"/>
-      <x:c r="C2" s="244"/>
-      <x:c r="D2" s="244"/>
-      <x:c r="E2" s="244"/>
-      <x:c r="F2" s="244"/>
-      <x:c r="G2" s="244"/>
-      <x:c r="H2" s="244"/>
+      <x:c r="A2" s="287"/>
+      <x:c r="B2" s="287"/>
+      <x:c r="C2" s="287"/>
+      <x:c r="D2" s="287"/>
+      <x:c r="E2" s="287"/>
+      <x:c r="F2" s="287"/>
+      <x:c r="G2" s="287"/>
+      <x:c r="H2" s="287"/>
       <x:c r="I2" s="244"/>
       <x:c r="J2" s="244"/>
       <x:c r="K2" s="244"/>
@@ -6705,28 +6854,28 @@
       <x:c r="M4" s="244"/>
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
-      <x:c r="A5" s="244" t="str">
+      <x:c r="A5" s="287" t="str">
         <x:v>TS001</x:v>
       </x:c>
-      <x:c r="B5" s="244" t="str">
+      <x:c r="B5" s="287" t="str">
         <x:v>2026-10-01 16:21:52 +07:00</x:v>
       </x:c>
-      <x:c r="C5" s="244" t="str">
+      <x:c r="C5" s="287" t="str">
         <x:v>AuthServiceRegisterTest</x:v>
       </x:c>
-      <x:c r="D5" s="244" t="n">
+      <x:c r="D5" s="287" t="n">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="E5" s="244" t="n">
+      <x:c r="E5" s="287" t="n">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="F5" s="244" t="n">
+      <x:c r="F5" s="287" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="G5" s="244" t="str">
+      <x:c r="G5" s="287" t="str">
         <x:v>0 / 0</x:v>
       </x:c>
-      <x:c r="H5" s="244" t="str">
+      <x:c r="H5" s="287" t="str">
         <x:v>BUILD SUCCESS</x:v>
       </x:c>
       <x:c r="I5" s="244"/>
@@ -6736,28 +6885,28 @@
       <x:c r="M5" s="244"/>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
-      <x:c r="A6" s="244" t="str">
+      <x:c r="A6" s="287" t="str">
         <x:v>TS002</x:v>
       </x:c>
-      <x:c r="B6" s="244" t="str">
+      <x:c r="B6" s="287" t="str">
         <x:v>2026-10-01 16:29:59 +07:00</x:v>
       </x:c>
-      <x:c r="C6" s="244" t="str">
+      <x:c r="C6" s="287" t="str">
         <x:v>AuthServiceLoginTest</x:v>
       </x:c>
-      <x:c r="D6" s="244" t="n">
+      <x:c r="D6" s="287" t="n">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="E6" s="244" t="n">
+      <x:c r="E6" s="287" t="n">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="F6" s="244" t="n">
+      <x:c r="F6" s="287" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="G6" s="244" t="str">
+      <x:c r="G6" s="287" t="str">
         <x:v>0 / 0</x:v>
       </x:c>
-      <x:c r="H6" s="244" t="str">
+      <x:c r="H6" s="287" t="str">
         <x:v>BUILD SUCCESS</x:v>
       </x:c>
       <x:c r="I6" s="244"/>
@@ -6767,28 +6916,28 @@
       <x:c r="M6" s="244"/>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
-      <x:c r="A7" s="244" t="str">
+      <x:c r="A7" s="287" t="str">
         <x:v>TS003</x:v>
       </x:c>
-      <x:c r="B7" s="244" t="str">
+      <x:c r="B7" s="287" t="str">
         <x:v>2026-10-01 16:43:40 +07:00</x:v>
       </x:c>
-      <x:c r="C7" s="244" t="str">
+      <x:c r="C7" s="287" t="str">
         <x:v>AuthControllerMvcTest</x:v>
       </x:c>
-      <x:c r="D7" s="244" t="n">
+      <x:c r="D7" s="287" t="n">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="E7" s="244" t="n">
+      <x:c r="E7" s="287" t="n">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="F7" s="244" t="n">
+      <x:c r="F7" s="287" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="G7" s="244" t="str">
+      <x:c r="G7" s="287" t="str">
         <x:v>0 / 0</x:v>
       </x:c>
-      <x:c r="H7" s="244" t="str">
+      <x:c r="H7" s="287" t="str">
         <x:v>BUILD SUCCESS</x:v>
       </x:c>
       <x:c r="I7" s="244"/>
@@ -6798,28 +6947,28 @@
       <x:c r="M7" s="244"/>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
-      <x:c r="A8" s="244" t="str">
+      <x:c r="A8" s="287" t="str">
         <x:v>TS004</x:v>
       </x:c>
-      <x:c r="B8" s="244" t="str">
+      <x:c r="B8" s="287" t="str">
         <x:v>2026-10-01 17:01:57 +07:00</x:v>
       </x:c>
-      <x:c r="C8" s="244" t="str">
+      <x:c r="C8" s="287" t="str">
         <x:v>AuthSecurityWebMvcTest</x:v>
       </x:c>
-      <x:c r="D8" s="244" t="n">
+      <x:c r="D8" s="287" t="n">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="E8" s="244" t="n">
+      <x:c r="E8" s="287" t="n">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="F8" s="244" t="n">
+      <x:c r="F8" s="287" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="G8" s="244" t="str">
+      <x:c r="G8" s="287" t="str">
         <x:v>0 / 0</x:v>
       </x:c>
-      <x:c r="H8" s="244" t="str">
+      <x:c r="H8" s="287" t="str">
         <x:v>BUILD SUCCESS</x:v>
       </x:c>
       <x:c r="I8" s="244"/>
@@ -6829,28 +6978,28 @@
       <x:c r="M8" s="244"/>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
-      <x:c r="A9" s="244" t="str">
+      <x:c r="A9" s="287" t="str">
         <x:v>TS005</x:v>
       </x:c>
-      <x:c r="B9" s="244" t="str">
+      <x:c r="B9" s="287" t="str">
         <x:v>2026-10-01 17:20:05 +07:00</x:v>
       </x:c>
-      <x:c r="C9" s="244" t="str">
+      <x:c r="C9" s="287" t="str">
         <x:v>InterestServiceTest + InterestControllerMvcTest</x:v>
       </x:c>
-      <x:c r="D9" s="244" t="n">
+      <x:c r="D9" s="287" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="E9" s="244" t="n">
+      <x:c r="E9" s="287" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="F9" s="244" t="n">
+      <x:c r="F9" s="287" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="G9" s="244" t="str">
+      <x:c r="G9" s="287" t="str">
         <x:v>0 / 0</x:v>
       </x:c>
-      <x:c r="H9" s="244" t="str">
+      <x:c r="H9" s="287" t="str">
         <x:v>BUILD SUCCESS</x:v>
       </x:c>
       <x:c r="I9" s="244"/>
@@ -7263,28 +7412,28 @@
       <x:c r="M22" s="244"/>
     </x:row>
     <x:row r="23">
-      <x:c r="A23" s="244" t="str">
+      <x:c r="A23" s="287" t="str">
         <x:v>E2E-005-R</x:v>
       </x:c>
-      <x:c r="B23" s="244" t="str">
+      <x:c r="B23" s="287" t="str">
         <x:v>2026-10-08 +07:00</x:v>
       </x:c>
       <x:c r="C23" s="287" t="str">
         <x:v>Robot Framework regression: login_smoke.robot + auth_flow.robot + register_interest.robot</x:v>
       </x:c>
-      <x:c r="D23" s="244" t="n">
+      <x:c r="D23" s="287" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="E23" s="244" t="n">
+      <x:c r="E23" s="287" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="F23" s="244" t="n">
+      <x:c r="F23" s="287" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="G23" s="244" t="str">
+      <x:c r="G23" s="287" t="str">
         <x:v>0 / 0</x:v>
       </x:c>
-      <x:c r="H23" s="244" t="str">
+      <x:c r="H23" s="287" t="str">
         <x:v>PASS — DEF-003 retest</x:v>
       </x:c>
       <x:c r="I23" s="244"/>
@@ -7294,28 +7443,28 @@
       <x:c r="M23" s="244"/>
     </x:row>
     <x:row r="24">
-      <x:c r="A24" s="244" t="str">
+      <x:c r="A24" s="287" t="str">
         <x:v>REG-DEF003</x:v>
       </x:c>
-      <x:c r="B24" s="244" t="str">
+      <x:c r="B24" s="287" t="str">
         <x:v>2026-10-08 15:10:48 +07:00</x:v>
       </x:c>
       <x:c r="C24" s="287" t="str">
         <x:v>AuthServiceRegisterTest + AuthServiceLoginTest + UserInterestServiceTest + FrontendAuthContractTest</x:v>
       </x:c>
-      <x:c r="D24" s="244" t="n">
+      <x:c r="D24" s="287" t="n">
         <x:v>39</x:v>
       </x:c>
-      <x:c r="E24" s="244" t="n">
+      <x:c r="E24" s="287" t="n">
         <x:v>39</x:v>
       </x:c>
-      <x:c r="F24" s="244" t="n">
+      <x:c r="F24" s="287" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="G24" s="244" t="str">
+      <x:c r="G24" s="287" t="str">
         <x:v>0 / 0</x:v>
       </x:c>
-      <x:c r="H24" s="244" t="str">
+      <x:c r="H24" s="287" t="str">
         <x:v>BUILD SUCCESS</x:v>
       </x:c>
       <x:c r="I24" s="244"/>
@@ -7325,28 +7474,28 @@
       <x:c r="M24" s="244"/>
     </x:row>
     <x:row r="25">
-      <x:c r="A25" s="244" t="str">
+      <x:c r="A25" s="287" t="str">
         <x:v>REG-20261008-FINAL</x:v>
       </x:c>
-      <x:c r="B25" s="244" t="str">
+      <x:c r="B25" s="287" t="str">
         <x:v>2026-10-08 18:02:26 +07:00</x:v>
       </x:c>
-      <x:c r="C25" s="244" t="str">
+      <x:c r="C25" s="287" t="str">
         <x:v>Full Maven regression after DEF-001 and DEF-003 fixes</x:v>
       </x:c>
-      <x:c r="D25" s="244" t="n">
+      <x:c r="D25" s="287" t="n">
         <x:v>174</x:v>
       </x:c>
-      <x:c r="E25" s="244" t="n">
+      <x:c r="E25" s="287" t="n">
         <x:v>174</x:v>
       </x:c>
-      <x:c r="F25" s="244" t="n">
+      <x:c r="F25" s="287" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="G25" s="244" t="str">
+      <x:c r="G25" s="287" t="str">
         <x:v>0 / 0</x:v>
       </x:c>
-      <x:c r="H25" s="244" t="str">
+      <x:c r="H25" s="287" t="str">
         <x:v>BUILD SUCCESS</x:v>
       </x:c>
       <x:c r="I25" s="244"/>
@@ -7356,14 +7505,30 @@
       <x:c r="M25" s="244"/>
     </x:row>
     <x:row r="26">
-      <x:c r="A26" s="244"/>
-      <x:c r="B26" s="244"/>
-      <x:c r="C26" s="244"/>
-      <x:c r="D26" s="244"/>
-      <x:c r="E26" s="244"/>
-      <x:c r="F26" s="244"/>
-      <x:c r="G26" s="244"/>
-      <x:c r="H26" s="244"/>
+      <x:c r="A26" s="287" t="str">
+        <x:v>WS-AUTH-REPRO</x:v>
+      </x:c>
+      <x:c r="B26" s="287" t="str">
+        <x:v>2026-10-08 +07:00</x:v>
+      </x:c>
+      <x:c r="C26" s="287" t="str">
+        <x:v>WebSocketAuthChannelInterceptorTest.connect_withoutAuthenticatedPrincipal_mustNotTrustLoginHeader</x:v>
+      </x:c>
+      <x:c r="D26" s="287" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E26" s="287" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F26" s="287" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G26" s="287" t="str">
+        <x:v>0 / 0</x:v>
+      </x:c>
+      <x:c r="H26" s="287" t="str">
+        <x:v>BUILD FAILURE — DEF-002 reproduced</x:v>
+      </x:c>
       <x:c r="I26" s="244"/>
       <x:c r="J26" s="244"/>
       <x:c r="K26" s="244"/>
@@ -7371,14 +7536,30 @@
       <x:c r="M26" s="244"/>
     </x:row>
     <x:row r="27">
-      <x:c r="A27" s="244"/>
-      <x:c r="B27" s="244"/>
-      <x:c r="C27" s="244"/>
-      <x:c r="D27" s="244"/>
-      <x:c r="E27" s="244"/>
-      <x:c r="F27" s="244"/>
-      <x:c r="G27" s="244"/>
-      <x:c r="H27" s="244"/>
+      <x:c r="A27" s="287" t="str">
+        <x:v>WS-AUTH-RETEST</x:v>
+      </x:c>
+      <x:c r="B27" s="287" t="str">
+        <x:v>2026-10-08 +07:00</x:v>
+      </x:c>
+      <x:c r="C27" s="287" t="str">
+        <x:v>WebSocketAuthChannelInterceptorTest</x:v>
+      </x:c>
+      <x:c r="D27" s="287" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E27" s="287" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F27" s="287" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G27" s="287" t="str">
+        <x:v>0 / 0</x:v>
+      </x:c>
+      <x:c r="H27" s="287" t="str">
+        <x:v>BUILD SUCCESS — DEF-002 retest</x:v>
+      </x:c>
       <x:c r="I27" s="244"/>
       <x:c r="J27" s="244"/>
       <x:c r="K27" s="244"/>
@@ -7386,14 +7567,30 @@
       <x:c r="M27" s="244"/>
     </x:row>
     <x:row r="28">
-      <x:c r="A28" s="244"/>
-      <x:c r="B28" s="244"/>
-      <x:c r="C28" s="244"/>
-      <x:c r="D28" s="244"/>
-      <x:c r="E28" s="244"/>
-      <x:c r="F28" s="244"/>
-      <x:c r="G28" s="244"/>
-      <x:c r="H28" s="244"/>
+      <x:c r="A28" s="287" t="str">
+        <x:v>REG-WS-AUTH</x:v>
+      </x:c>
+      <x:c r="B28" s="287" t="str">
+        <x:v>2026-10-08 19:19:08 +07:00</x:v>
+      </x:c>
+      <x:c r="C28" s="287" t="str">
+        <x:v>Full Maven regression after WebSocket authentication fix</x:v>
+      </x:c>
+      <x:c r="D28" s="287" t="n">
+        <x:v>176</x:v>
+      </x:c>
+      <x:c r="E28" s="287" t="n">
+        <x:v>176</x:v>
+      </x:c>
+      <x:c r="F28" s="287" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G28" s="287" t="str">
+        <x:v>0 / 0</x:v>
+      </x:c>
+      <x:c r="H28" s="287" t="str">
+        <x:v>BUILD SUCCESS</x:v>
+      </x:c>
       <x:c r="I28" s="244"/>
       <x:c r="J28" s="244"/>
       <x:c r="K28" s="244"/>
@@ -7401,14 +7598,30 @@
       <x:c r="M28" s="244"/>
     </x:row>
     <x:row r="29">
-      <x:c r="A29" s="244"/>
-      <x:c r="B29" s="244"/>
-      <x:c r="C29" s="244"/>
-      <x:c r="D29" s="244"/>
-      <x:c r="E29" s="244"/>
-      <x:c r="F29" s="244"/>
-      <x:c r="G29" s="244"/>
-      <x:c r="H29" s="244"/>
+      <x:c r="A29" s="287" t="str">
+        <x:v>CALL-LEAVE-REPRO</x:v>
+      </x:c>
+      <x:c r="B29" s="287" t="str">
+        <x:v>2026-10-08 19:44:37 +07:00</x:v>
+      </x:c>
+      <x:c r="C29" s="287" t="str">
+        <x:v>ChatMessageServiceTest — former member LEAVE + never-member LEAVE</x:v>
+      </x:c>
+      <x:c r="D29" s="287" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E29" s="287" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F29" s="287" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G29" s="287" t="str">
+        <x:v>0 / 0</x:v>
+      </x:c>
+      <x:c r="H29" s="287" t="str">
+        <x:v>BUILD FAILURE — DEF-004 reproduced</x:v>
+      </x:c>
       <x:c r="I29" s="244"/>
       <x:c r="J29" s="244"/>
       <x:c r="K29" s="244"/>
@@ -7416,14 +7629,30 @@
       <x:c r="M29" s="244"/>
     </x:row>
     <x:row r="30">
-      <x:c r="A30" s="244"/>
-      <x:c r="B30" s="244"/>
-      <x:c r="C30" s="244"/>
-      <x:c r="D30" s="244"/>
-      <x:c r="E30" s="244"/>
-      <x:c r="F30" s="244"/>
-      <x:c r="G30" s="244"/>
-      <x:c r="H30" s="244"/>
+      <x:c r="A30" s="287" t="str">
+        <x:v>CALL-LEAVE-RETEST</x:v>
+      </x:c>
+      <x:c r="B30" s="287" t="str">
+        <x:v>2026-10-08 +07:00</x:v>
+      </x:c>
+      <x:c r="C30" s="287" t="str">
+        <x:v>ChatMessageServiceTest — LEAVE signaling targeted retest</x:v>
+      </x:c>
+      <x:c r="D30" s="287" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E30" s="287" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F30" s="287" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G30" s="287" t="str">
+        <x:v>0 / 0</x:v>
+      </x:c>
+      <x:c r="H30" s="287" t="str">
+        <x:v>BUILD SUCCESS — DEF-004 retest</x:v>
+      </x:c>
       <x:c r="I30" s="244"/>
       <x:c r="J30" s="244"/>
       <x:c r="K30" s="244"/>
@@ -7431,14 +7660,30 @@
       <x:c r="M30" s="244"/>
     </x:row>
     <x:row r="31">
-      <x:c r="A31" s="244"/>
-      <x:c r="B31" s="244"/>
-      <x:c r="C31" s="244"/>
-      <x:c r="D31" s="244"/>
-      <x:c r="E31" s="244"/>
-      <x:c r="F31" s="244"/>
-      <x:c r="G31" s="244"/>
-      <x:c r="H31" s="244"/>
+      <x:c r="A31" s="287" t="str">
+        <x:v>REG-20261008-178</x:v>
+      </x:c>
+      <x:c r="B31" s="287" t="str">
+        <x:v>2026-10-08 19:51:02 +07:00</x:v>
+      </x:c>
+      <x:c r="C31" s="287" t="str">
+        <x:v>Full Maven regression after DEF-004 fix</x:v>
+      </x:c>
+      <x:c r="D31" s="287" t="n">
+        <x:v>178</x:v>
+      </x:c>
+      <x:c r="E31" s="287" t="n">
+        <x:v>178</x:v>
+      </x:c>
+      <x:c r="F31" s="287" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G31" s="287" t="str">
+        <x:v>0 / 0</x:v>
+      </x:c>
+      <x:c r="H31" s="287" t="str">
+        <x:v>BUILD SUCCESS</x:v>
+      </x:c>
       <x:c r="I31" s="244"/>
       <x:c r="J31" s="244"/>
       <x:c r="K31" s="244"/>
@@ -7446,14 +7691,30 @@
       <x:c r="M31" s="244"/>
     </x:row>
     <x:row r="32">
-      <x:c r="A32" s="244"/>
-      <x:c r="B32" s="244"/>
-      <x:c r="C32" s="244"/>
-      <x:c r="D32" s="244"/>
-      <x:c r="E32" s="244"/>
-      <x:c r="F32" s="244"/>
-      <x:c r="G32" s="244"/>
-      <x:c r="H32" s="244"/>
+      <x:c r="A32" s="287" t="str">
+        <x:v>CALL-MEDIA-REPRO</x:v>
+      </x:c>
+      <x:c r="B32" s="287" t="str">
+        <x:v>2026-10-08 20:03:42 +07:00</x:v>
+      </x:c>
+      <x:c r="C32" s="287" t="str">
+        <x:v>CallFrontendContractTest</x:v>
+      </x:c>
+      <x:c r="D32" s="287" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E32" s="287" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F32" s="287" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G32" s="287" t="str">
+        <x:v>0 / 0</x:v>
+      </x:c>
+      <x:c r="H32" s="287" t="str">
+        <x:v>BUILD FAILURE — DEF-005 reproduced</x:v>
+      </x:c>
       <x:c r="I32" s="244"/>
       <x:c r="J32" s="244"/>
       <x:c r="K32" s="244"/>
@@ -7461,14 +7722,30 @@
       <x:c r="M32" s="244"/>
     </x:row>
     <x:row r="33">
-      <x:c r="A33" s="244"/>
-      <x:c r="B33" s="244"/>
-      <x:c r="C33" s="244"/>
-      <x:c r="D33" s="244"/>
-      <x:c r="E33" s="244"/>
-      <x:c r="F33" s="244"/>
-      <x:c r="G33" s="244"/>
-      <x:c r="H33" s="244"/>
+      <x:c r="A33" s="287" t="str">
+        <x:v>CALL-MEDIA-RETEST</x:v>
+      </x:c>
+      <x:c r="B33" s="287" t="str">
+        <x:v>2026-10-08 20:14:49 +07:00</x:v>
+      </x:c>
+      <x:c r="C33" s="287" t="str">
+        <x:v>CallFrontendContractTest</x:v>
+      </x:c>
+      <x:c r="D33" s="287" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E33" s="287" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F33" s="287" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G33" s="287" t="str">
+        <x:v>0 / 0</x:v>
+      </x:c>
+      <x:c r="H33" s="287" t="str">
+        <x:v>BUILD SUCCESS — DEF-005 retest</x:v>
+      </x:c>
       <x:c r="I33" s="244"/>
       <x:c r="J33" s="244"/>
       <x:c r="K33" s="244"/>
@@ -7476,14 +7753,30 @@
       <x:c r="M33" s="244"/>
     </x:row>
     <x:row r="34">
-      <x:c r="A34" s="244"/>
-      <x:c r="B34" s="244"/>
-      <x:c r="C34" s="244"/>
-      <x:c r="D34" s="244"/>
-      <x:c r="E34" s="244"/>
-      <x:c r="F34" s="244"/>
-      <x:c r="G34" s="244"/>
-      <x:c r="H34" s="244"/>
+      <x:c r="A34" s="287" t="str">
+        <x:v>REG-20261008-180</x:v>
+      </x:c>
+      <x:c r="B34" s="287" t="str">
+        <x:v>2026-10-08 20:16:01 +07:00</x:v>
+      </x:c>
+      <x:c r="C34" s="287" t="str">
+        <x:v>Final full Maven regression + Robot Framework browser regression 5/5</x:v>
+      </x:c>
+      <x:c r="D34" s="287" t="n">
+        <x:v>180</x:v>
+      </x:c>
+      <x:c r="E34" s="287" t="n">
+        <x:v>180</x:v>
+      </x:c>
+      <x:c r="F34" s="287" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G34" s="287" t="str">
+        <x:v>0 / 0</x:v>
+      </x:c>
+      <x:c r="H34" s="287" t="str">
+        <x:v>BUILD SUCCESS — Maven 180/180; Robot 5/5 PASS</x:v>
+      </x:c>
       <x:c r="I34" s="244"/>
       <x:c r="J34" s="244"/>
       <x:c r="K34" s="244"/>
@@ -12377,14 +12670,14 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="16.799999237060547" hidden="0" customHeight="1">
-      <x:c r="A1" s="243" t="str">
+      <x:c r="A1" s="288" t="str">
         <x:v>Requirements / Behavior Traceability</x:v>
       </x:c>
-      <x:c r="B1" s="243"/>
-      <x:c r="C1" s="243"/>
-      <x:c r="D1" s="243"/>
-      <x:c r="E1" s="243"/>
-      <x:c r="F1" s="243"/>
+      <x:c r="B1" s="288"/>
+      <x:c r="C1" s="288"/>
+      <x:c r="D1" s="288"/>
+      <x:c r="E1" s="288"/>
+      <x:c r="F1" s="288"/>
       <x:c r="G1" s="244"/>
       <x:c r="H1" s="244"/>
       <x:c r="I1" s="244"/>
@@ -12394,12 +12687,12 @@
       <x:c r="M1" s="244"/>
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
-      <x:c r="A2" s="244"/>
-      <x:c r="B2" s="244"/>
-      <x:c r="C2" s="244"/>
-      <x:c r="D2" s="244"/>
-      <x:c r="E2" s="244"/>
-      <x:c r="F2" s="244"/>
+      <x:c r="A2" s="287"/>
+      <x:c r="B2" s="287"/>
+      <x:c r="C2" s="287"/>
+      <x:c r="D2" s="287"/>
+      <x:c r="E2" s="287"/>
+      <x:c r="F2" s="287"/>
       <x:c r="G2" s="244"/>
       <x:c r="H2" s="244"/>
       <x:c r="I2" s="244"/>
@@ -12949,12 +13242,12 @@
       <x:c r="M22" s="244"/>
     </x:row>
     <x:row r="23" ht="15" hidden="0" customHeight="1">
-      <x:c r="A23" s="244"/>
-      <x:c r="B23" s="244"/>
-      <x:c r="C23" s="244"/>
-      <x:c r="D23" s="244"/>
-      <x:c r="E23" s="244"/>
-      <x:c r="F23" s="244"/>
+      <x:c r="A23" s="287"/>
+      <x:c r="B23" s="287"/>
+      <x:c r="C23" s="287"/>
+      <x:c r="D23" s="287"/>
+      <x:c r="E23" s="287"/>
+      <x:c r="F23" s="287"/>
       <x:c r="G23" s="244"/>
       <x:c r="H23" s="244"/>
       <x:c r="I23" s="244"/>
@@ -13428,12 +13721,12 @@
       <x:c r="M41" s="244"/>
     </x:row>
     <x:row r="42">
-      <x:c r="A42" s="244"/>
-      <x:c r="B42" s="244"/>
-      <x:c r="C42" s="244"/>
-      <x:c r="D42" s="244"/>
-      <x:c r="E42" s="244"/>
-      <x:c r="F42" s="244"/>
+      <x:c r="A42" s="287"/>
+      <x:c r="B42" s="287"/>
+      <x:c r="C42" s="287"/>
+      <x:c r="D42" s="287"/>
+      <x:c r="E42" s="287"/>
+      <x:c r="F42" s="287"/>
       <x:c r="G42" s="244"/>
       <x:c r="H42" s="244"/>
       <x:c r="I42" s="244"/>
@@ -13929,12 +14222,24 @@
       <x:c r="M60" s="244"/>
     </x:row>
     <x:row r="61">
-      <x:c r="A61" s="244"/>
-      <x:c r="B61" s="244"/>
-      <x:c r="C61" s="244"/>
-      <x:c r="D61" s="244"/>
-      <x:c r="E61" s="244"/>
-      <x:c r="F61" s="244"/>
+      <x:c r="A61" s="287" t="str">
+        <x:v>REQ-WS-AUTH-01</x:v>
+      </x:c>
+      <x:c r="B61" s="287" t="str">
+        <x:v>WebSocket identity ต้องมาจาก authenticated HTTP/session Principal; STOMP login header ต้องไม่ยกระดับสิทธิ์</x:v>
+      </x:c>
+      <x:c r="C61" s="287" t="str">
+        <x:v>TS016</x:v>
+      </x:c>
+      <x:c r="D61" s="287" t="str">
+        <x:v>WSA-001, WSA-002</x:v>
+      </x:c>
+      <x:c r="E61" s="287" t="str">
+        <x:v>WebSocketAuthChannelInterceptor + HttpSessionHandshakeHandler</x:v>
+      </x:c>
+      <x:c r="F61" s="287" t="str">
+        <x:v>Passed - DEF-002 retest</x:v>
+      </x:c>
       <x:c r="G61" s="244"/>
       <x:c r="H61" s="244"/>
       <x:c r="I61" s="244"/>
@@ -13944,12 +14249,24 @@
       <x:c r="M61" s="244"/>
     </x:row>
     <x:row r="62">
-      <x:c r="A62" s="244"/>
-      <x:c r="B62" s="244"/>
-      <x:c r="C62" s="244"/>
-      <x:c r="D62" s="244"/>
-      <x:c r="E62" s="244"/>
-      <x:c r="F62" s="244"/>
+      <x:c r="A62" s="287" t="str">
+        <x:v>REQ-CALL-01</x:v>
+      </x:c>
+      <x:c r="B62" s="287" t="str">
+        <x:v>LEAVE ต้องส่งได้หลังสมาชิกเพิ่งออกจากห้อง แต่ผู้ที่ไม่เคยเป็นสมาชิกต้องถูกปฏิเสธ</x:v>
+      </x:c>
+      <x:c r="C62" s="287" t="str">
+        <x:v>TS016</x:v>
+      </x:c>
+      <x:c r="D62" s="287" t="str">
+        <x:v>CALL-001, CALL-002</x:v>
+      </x:c>
+      <x:c r="E62" s="287" t="str">
+        <x:v>ChatMessageService.relayCallSignal</x:v>
+      </x:c>
+      <x:c r="F62" s="287" t="str">
+        <x:v>Passed - DEF-004 retest</x:v>
+      </x:c>
       <x:c r="G62" s="244"/>
       <x:c r="H62" s="244"/>
       <x:c r="I62" s="244"/>
@@ -13959,12 +14276,24 @@
       <x:c r="M62" s="244"/>
     </x:row>
     <x:row r="63">
-      <x:c r="A63" s="244"/>
-      <x:c r="B63" s="244"/>
-      <x:c r="C63" s="244"/>
-      <x:c r="D63" s="244"/>
-      <x:c r="E63" s="244"/>
-      <x:c r="F63" s="244"/>
+      <x:c r="A63" s="287" t="str">
+        <x:v>REQ-CALL-02</x:v>
+      </x:c>
+      <x:c r="B63" s="287" t="str">
+        <x:v>การปิด/เปิดกล้องต้อง publish MEDIA state และ client ฝั่งรับต้องจัดการ state เพื่ออัปเดต UI</x:v>
+      </x:c>
+      <x:c r="C63" s="287" t="str">
+        <x:v>TS016</x:v>
+      </x:c>
+      <x:c r="D63" s="287" t="str">
+        <x:v>CALL-003, CALL-004</x:v>
+      </x:c>
+      <x:c r="E63" s="287" t="str">
+        <x:v>static/js/call.js + static/js/friend.js</x:v>
+      </x:c>
+      <x:c r="F63" s="287" t="str">
+        <x:v>Passed - DEF-005 retest</x:v>
+      </x:c>
       <x:c r="G63" s="244"/>
       <x:c r="H63" s="244"/>
       <x:c r="I63" s="244"/>
@@ -13974,12 +14303,24 @@
       <x:c r="M63" s="244"/>
     </x:row>
     <x:row r="64">
-      <x:c r="A64" s="244"/>
-      <x:c r="B64" s="244"/>
-      <x:c r="C64" s="244"/>
-      <x:c r="D64" s="244"/>
-      <x:c r="E64" s="244"/>
-      <x:c r="F64" s="244"/>
+      <x:c r="A64" s="287" t="str">
+        <x:v>REQ-E2E-01</x:v>
+      </x:c>
+      <x:c r="B64" s="287" t="str">
+        <x:v>Browser E2E ต้องครอบคลุม login page, password toggle, register navigation, register/login flow และ registration interest persistence</x:v>
+      </x:c>
+      <x:c r="C64" s="287" t="str">
+        <x:v>TS017</x:v>
+      </x:c>
+      <x:c r="D64" s="287" t="str">
+        <x:v>E2E-001 ถึง E2E-005</x:v>
+      </x:c>
+      <x:c r="E64" s="287" t="str">
+        <x:v>Robot Framework + Browser/Playwright</x:v>
+      </x:c>
+      <x:c r="F64" s="287" t="str">
+        <x:v>Passed - E2E 5/5</x:v>
+      </x:c>
       <x:c r="G64" s="244"/>
       <x:c r="H64" s="244"/>
       <x:c r="I64" s="244"/>
@@ -15563,6 +15904,516 @@
       <x:c r="C24" s="47"/>
       <x:c r="D24" s="47"/>
       <x:c r="E24" s="47"/>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="34" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="42" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="50" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="12" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="47" t="str">
+        <x:v>TS016  WebSocket / WebRTC Security &amp; Call Signaling</x:v>
+      </x:c>
+      <x:c r="B1" s="47"/>
+      <x:c r="C1" s="47"/>
+      <x:c r="D1" s="47"/>
+      <x:c r="E1" s="47"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="47"/>
+      <x:c r="B2" s="47"/>
+      <x:c r="C2" s="47"/>
+      <x:c r="D2" s="47"/>
+      <x:c r="E2" s="47"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="47" t="str">
+        <x:v>Scenario ID</x:v>
+      </x:c>
+      <x:c r="B3" s="47" t="str">
+        <x:v>TS016</x:v>
+      </x:c>
+      <x:c r="C3" s="47"/>
+      <x:c r="D3" s="47"/>
+      <x:c r="E3" s="47"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="47" t="str">
+        <x:v>Use Case ID</x:v>
+      </x:c>
+      <x:c r="B4" s="47" t="str">
+        <x:v>UC-WS-01 / UC-CALL-01</x:v>
+      </x:c>
+      <x:c r="C4" s="47"/>
+      <x:c r="D4" s="47"/>
+      <x:c r="E4" s="47"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="47" t="str">
+        <x:v>Module / Unit under Test</x:v>
+      </x:c>
+      <x:c r="B5" s="47" t="str">
+        <x:v>WebSocketAuthChannelInterceptor + ChatMessageService + call.js/friend.js</x:v>
+      </x:c>
+      <x:c r="C5" s="47"/>
+      <x:c r="D5" s="47"/>
+      <x:c r="E5" s="47"/>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="47" t="str">
+        <x:v>Test Level</x:v>
+      </x:c>
+      <x:c r="B6" s="47" t="str">
+        <x:v>Unit Test + Frontend Contract Test</x:v>
+      </x:c>
+      <x:c r="C6" s="47"/>
+      <x:c r="D6" s="47"/>
+      <x:c r="E6" s="47"/>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="47" t="str">
+        <x:v>Test Method</x:v>
+      </x:c>
+      <x:c r="B7" s="47" t="str">
+        <x:v>JUnit 5 + Mockito + static resource contract tests</x:v>
+      </x:c>
+      <x:c r="C7" s="47"/>
+      <x:c r="D7" s="47"/>
+      <x:c r="E7" s="47"/>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="47" t="str">
+        <x:v>Preconditions</x:v>
+      </x:c>
+      <x:c r="B8" s="47" t="str">
+        <x:v>Current tester branch after Piyapon WebSocket integration; HTTP session is authoritative identity source</x:v>
+      </x:c>
+      <x:c r="C8" s="47"/>
+      <x:c r="D8" s="47"/>
+      <x:c r="E8" s="47"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="47" t="str">
+        <x:v>Mocks / Stubs</x:v>
+      </x:c>
+      <x:c r="B9" s="47" t="str">
+        <x:v>MessageChannel, RoomMemberRepository, SimpMessagingTemplate; static JS resources from classpath</x:v>
+      </x:c>
+      <x:c r="C9" s="47"/>
+      <x:c r="D9" s="47"/>
+      <x:c r="E9" s="47"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="47" t="str">
+        <x:v>Test Data / Stub Return</x:v>
+      </x:c>
+      <x:c r="B10" s="47" t="str">
+        <x:v>Authenticated/unauthenticated CONNECT, former/never member LEAVE, camera MEDIA state | Final Maven: 180/180 Pass</x:v>
+      </x:c>
+      <x:c r="C10" s="47"/>
+      <x:c r="D10" s="47"/>
+      <x:c r="E10" s="47"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="47"/>
+      <x:c r="B11" s="47"/>
+      <x:c r="C11" s="47"/>
+      <x:c r="D11" s="47"/>
+      <x:c r="E11" s="47"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="47" t="str">
+        <x:v>Case ID</x:v>
+      </x:c>
+      <x:c r="B12" s="47" t="str">
+        <x:v>Test Condition</x:v>
+      </x:c>
+      <x:c r="C12" s="47" t="str">
+        <x:v>Test Input / Mock Data</x:v>
+      </x:c>
+      <x:c r="D12" s="47" t="str">
+        <x:v>Expected Result</x:v>
+      </x:c>
+      <x:c r="E12" s="47" t="str">
+        <x:v>Status</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="47" t="str">
+        <x:v>WSA-001</x:v>
+      </x:c>
+      <x:c r="B13" s="47" t="str">
+        <x:v>Authenticated Principal is preserved</x:v>
+      </x:c>
+      <x:c r="C13" s="47" t="str">
+        <x:v>CONNECT with existing HTTP/session Principal</x:v>
+      </x:c>
+      <x:c r="D13" s="47" t="str">
+        <x:v>Principal remains unchanged</x:v>
+      </x:c>
+      <x:c r="E13" s="47" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="47" t="str">
+        <x:v>WSA-002</x:v>
+      </x:c>
+      <x:c r="B14" s="47" t="str">
+        <x:v>Unverified STOMP login is rejected as identity</x:v>
+      </x:c>
+      <x:c r="C14" s="47" t="str">
+        <x:v>CONNECT without Principal; login=&lt;claimed UUID&gt;</x:v>
+      </x:c>
+      <x:c r="D14" s="47" t="str">
+        <x:v>No Principal is created from login header</x:v>
+      </x:c>
+      <x:c r="E14" s="47" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="47" t="str">
+        <x:v>CALL-001</x:v>
+      </x:c>
+      <x:c r="B15" s="47" t="str">
+        <x:v>Former member LEAVE</x:v>
+      </x:c>
+      <x:c r="C15" s="47" t="str">
+        <x:v>LEAVE after membership ended; history exists</x:v>
+      </x:c>
+      <x:c r="D15" s="47" t="str">
+        <x:v>Broadcast LEAVE without 403</x:v>
+      </x:c>
+      <x:c r="E15" s="47" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="47" t="str">
+        <x:v>CALL-002</x:v>
+      </x:c>
+      <x:c r="B16" s="47" t="str">
+        <x:v>Never-member LEAVE</x:v>
+      </x:c>
+      <x:c r="C16" s="47" t="str">
+        <x:v>LEAVE with no membership history</x:v>
+      </x:c>
+      <x:c r="D16" s="47" t="str">
+        <x:v>403 FORBIDDEN; no broadcast</x:v>
+      </x:c>
+      <x:c r="E16" s="47" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="47" t="str">
+        <x:v>CALL-003</x:v>
+      </x:c>
+      <x:c r="B17" s="47" t="str">
+        <x:v>Camera MEDIA publish</x:v>
+      </x:c>
+      <x:c r="C17" s="47" t="str">
+        <x:v>toggleCamera while call is active</x:v>
+      </x:c>
+      <x:c r="D17" s="47" t="str">
+        <x:v>Publish MEDIA with videoEnabled state</x:v>
+      </x:c>
+      <x:c r="E17" s="47" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="47" t="str">
+        <x:v>CALL-004</x:v>
+      </x:c>
+      <x:c r="B18" s="47" t="str">
+        <x:v>Incoming MEDIA handling</x:v>
+      </x:c>
+      <x:c r="C18" s="47" t="str">
+        <x:v>Receive MEDIA signal from remote participant</x:v>
+      </x:c>
+      <x:c r="D18" s="47" t="str">
+        <x:v>Client handles state and updates remote video UI</x:v>
+      </x:c>
+      <x:c r="E18" s="47" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="47"/>
+      <x:c r="B19" s="47"/>
+      <x:c r="C19" s="47"/>
+      <x:c r="D19" s="47"/>
+      <x:c r="E19" s="47"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="47"/>
+      <x:c r="B20" s="47"/>
+      <x:c r="C20" s="47"/>
+      <x:c r="D20" s="47"/>
+      <x:c r="E20" s="47"/>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="34" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="42" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="50" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="12" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="47" t="str">
+        <x:v>TS017  Robot Framework Browser E2E</x:v>
+      </x:c>
+      <x:c r="B1" s="47"/>
+      <x:c r="C1" s="47"/>
+      <x:c r="D1" s="47"/>
+      <x:c r="E1" s="47"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="47"/>
+      <x:c r="B2" s="47"/>
+      <x:c r="C2" s="47"/>
+      <x:c r="D2" s="47"/>
+      <x:c r="E2" s="47"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="47" t="str">
+        <x:v>Scenario ID</x:v>
+      </x:c>
+      <x:c r="B3" s="47" t="str">
+        <x:v>TS017</x:v>
+      </x:c>
+      <x:c r="C3" s="47"/>
+      <x:c r="D3" s="47"/>
+      <x:c r="E3" s="47"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="47" t="str">
+        <x:v>Use Case ID</x:v>
+      </x:c>
+      <x:c r="B4" s="47" t="str">
+        <x:v>UC-E2E-01</x:v>
+      </x:c>
+      <x:c r="C4" s="47"/>
+      <x:c r="D4" s="47"/>
+      <x:c r="E4" s="47"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="47" t="str">
+        <x:v>Module / Unit under Test</x:v>
+      </x:c>
+      <x:c r="B5" s="47" t="str">
+        <x:v>Login / Registration / Interest persistence browser flow</x:v>
+      </x:c>
+      <x:c r="C5" s="47"/>
+      <x:c r="D5" s="47"/>
+      <x:c r="E5" s="47"/>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="47" t="str">
+        <x:v>Test Level</x:v>
+      </x:c>
+      <x:c r="B6" s="47" t="str">
+        <x:v>End-to-End / User Flow</x:v>
+      </x:c>
+      <x:c r="C6" s="47"/>
+      <x:c r="D6" s="47"/>
+      <x:c r="E6" s="47"/>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="47" t="str">
+        <x:v>Test Method</x:v>
+      </x:c>
+      <x:c r="B7" s="47" t="str">
+        <x:v>Robot Framework + Browser library / Playwright</x:v>
+      </x:c>
+      <x:c r="C7" s="47"/>
+      <x:c r="D7" s="47"/>
+      <x:c r="E7" s="47"/>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="47" t="str">
+        <x:v>Preconditions</x:v>
+      </x:c>
+      <x:c r="B8" s="47" t="str">
+        <x:v>Spring Boot application running at http://localhost:8080; browser automation environment available</x:v>
+      </x:c>
+      <x:c r="C8" s="47"/>
+      <x:c r="D8" s="47"/>
+      <x:c r="E8" s="47"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="47" t="str">
+        <x:v>Mocks / Stubs</x:v>
+      </x:c>
+      <x:c r="B9" s="47" t="str">
+        <x:v>None — tests interact with the running web application</x:v>
+      </x:c>
+      <x:c r="C9" s="47"/>
+      <x:c r="D9" s="47"/>
+      <x:c r="E9" s="47"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="47" t="str">
+        <x:v>Test Data / Stub Return</x:v>
+      </x:c>
+      <x:c r="B10" s="47" t="str">
+        <x:v>Generated registration/login data and selected interest | Final Robot regression: 5/5 Pass</x:v>
+      </x:c>
+      <x:c r="C10" s="47"/>
+      <x:c r="D10" s="47"/>
+      <x:c r="E10" s="47"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="47"/>
+      <x:c r="B11" s="47"/>
+      <x:c r="C11" s="47"/>
+      <x:c r="D11" s="47"/>
+      <x:c r="E11" s="47"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="47" t="str">
+        <x:v>Case ID</x:v>
+      </x:c>
+      <x:c r="B12" s="47" t="str">
+        <x:v>Test Condition</x:v>
+      </x:c>
+      <x:c r="C12" s="47" t="str">
+        <x:v>Test Input / Mock Data</x:v>
+      </x:c>
+      <x:c r="D12" s="47" t="str">
+        <x:v>Expected Result</x:v>
+      </x:c>
+      <x:c r="E12" s="47" t="str">
+        <x:v>Status</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="47" t="str">
+        <x:v>E2E-001</x:v>
+      </x:c>
+      <x:c r="B13" s="47" t="str">
+        <x:v>Login page loads</x:v>
+      </x:c>
+      <x:c r="C13" s="47" t="str">
+        <x:v>Open /login</x:v>
+      </x:c>
+      <x:c r="D13" s="47" t="str">
+        <x:v>Login page displays successfully</x:v>
+      </x:c>
+      <x:c r="E13" s="47" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="47" t="str">
+        <x:v>E2E-002</x:v>
+      </x:c>
+      <x:c r="B14" s="47" t="str">
+        <x:v>Password visibility toggle</x:v>
+      </x:c>
+      <x:c r="C14" s="47" t="str">
+        <x:v>Click show/hide password</x:v>
+      </x:c>
+      <x:c r="D14" s="47" t="str">
+        <x:v>Password field visibility changes</x:v>
+      </x:c>
+      <x:c r="E14" s="47" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="47" t="str">
+        <x:v>E2E-003</x:v>
+      </x:c>
+      <x:c r="B15" s="47" t="str">
+        <x:v>Register navigation</x:v>
+      </x:c>
+      <x:c r="C15" s="47" t="str">
+        <x:v>Click Register link</x:v>
+      </x:c>
+      <x:c r="D15" s="47" t="str">
+        <x:v>Register page opens</x:v>
+      </x:c>
+      <x:c r="E15" s="47" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="47" t="str">
+        <x:v>E2E-004</x:v>
+      </x:c>
+      <x:c r="B16" s="47" t="str">
+        <x:v>Register and login flow</x:v>
+      </x:c>
+      <x:c r="C16" s="47" t="str">
+        <x:v>Create account then log in</x:v>
+      </x:c>
+      <x:c r="D16" s="47" t="str">
+        <x:v>User reaches /home</x:v>
+      </x:c>
+      <x:c r="E16" s="47" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="47" t="str">
+        <x:v>E2E-005</x:v>
+      </x:c>
+      <x:c r="B17" s="47" t="str">
+        <x:v>Registration interest persistence</x:v>
+      </x:c>
+      <x:c r="C17" s="47" t="str">
+        <x:v>Select interest during registration</x:v>
+      </x:c>
+      <x:c r="D17" s="47" t="str">
+        <x:v>Selected interest remains saved after registration/login</x:v>
+      </x:c>
+      <x:c r="E17" s="47" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="47"/>
+      <x:c r="B18" s="47"/>
+      <x:c r="C18" s="47"/>
+      <x:c r="D18" s="47"/>
+      <x:c r="E18" s="47"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="47"/>
+      <x:c r="B19" s="47"/>
+      <x:c r="C19" s="47"/>
+      <x:c r="D19" s="47"/>
+      <x:c r="E19" s="47"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="47"/>
+      <x:c r="B20" s="47"/>
+      <x:c r="C20" s="47"/>
+      <x:c r="D20" s="47"/>
+      <x:c r="E20" s="47"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -24734,6 +25585,457 @@
       </x:c>
       <x:c r="M226" s="47" t="str">
         <x:v>2026-10-07 19:20:07 +07:00 | 8/8 Pass | BUILD SUCCESS | 15.982 s</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="227">
+      <x:c r="A227" s="47" t="str">
+        <x:v>UC-WS-01</x:v>
+      </x:c>
+      <x:c r="B227" s="47" t="str">
+        <x:v>TS016</x:v>
+      </x:c>
+      <x:c r="C227" s="47" t="str">
+        <x:v>WSA-001</x:v>
+      </x:c>
+      <x:c r="D227" s="47" t="str">
+        <x:v>Authenticated Principal is preserved</x:v>
+      </x:c>
+      <x:c r="E227" s="47" t="str">
+        <x:v>WebSocketAuthChannelInterceptor.preSend</x:v>
+      </x:c>
+      <x:c r="F227" s="47" t="str">
+        <x:v>CONNECT with existing Principal</x:v>
+      </x:c>
+      <x:c r="G227" s="47" t="str">
+        <x:v>Principal from HTTP/session handshake</x:v>
+      </x:c>
+      <x:c r="H227" s="47" t="str">
+        <x:v>Existing Principal remains unchanged</x:v>
+      </x:c>
+      <x:c r="I227" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
+      <x:c r="J227" s="47" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="K227" s="47" t="str">
+        <x:v>Unit test (JUnit 5)</x:v>
+      </x:c>
+      <x:c r="L227" s="47" t="str">
+        <x:v>WebSocketAuthChannelInterceptorTest.connect_withAuthenticatedPrincipal_preservesPrincipal</x:v>
+      </x:c>
+      <x:c r="M227" s="47" t="str">
+        <x:v>2026-10-08 | 2/2 targeted retest Pass | DEF-002 CLOSED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="228">
+      <x:c r="A228" s="47" t="str">
+        <x:v>UC-WS-01</x:v>
+      </x:c>
+      <x:c r="B228" s="47" t="str">
+        <x:v>TS016</x:v>
+      </x:c>
+      <x:c r="C228" s="47" t="str">
+        <x:v>WSA-002</x:v>
+      </x:c>
+      <x:c r="D228" s="47" t="str">
+        <x:v>Unverified STOMP login is not trusted</x:v>
+      </x:c>
+      <x:c r="E228" s="47" t="str">
+        <x:v>WebSocketAuthChannelInterceptor.preSend</x:v>
+      </x:c>
+      <x:c r="F228" s="47" t="str">
+        <x:v>CONNECT without Principal; login=&lt;claimed UUID&gt;</x:v>
+      </x:c>
+      <x:c r="G228" s="47" t="str">
+        <x:v>No authenticated HTTP/session Principal</x:v>
+      </x:c>
+      <x:c r="H228" s="47" t="str">
+        <x:v>result user remains null; login header cannot authenticate client</x:v>
+      </x:c>
+      <x:c r="I228" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
+      <x:c r="J228" s="47" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="K228" s="47" t="str">
+        <x:v>Unit test (JUnit 5)</x:v>
+      </x:c>
+      <x:c r="L228" s="47" t="str">
+        <x:v>WebSocketAuthChannelInterceptorTest.connect_withoutAuthenticatedPrincipal_mustNotTrustLoginHeader</x:v>
+      </x:c>
+      <x:c r="M228" s="47" t="str">
+        <x:v>Reproduced before fix; 2/2 targeted retest Pass | DEF-002 CLOSED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="229">
+      <x:c r="A229" s="47" t="str">
+        <x:v>UC-CALL-01</x:v>
+      </x:c>
+      <x:c r="B229" s="47" t="str">
+        <x:v>TS016</x:v>
+      </x:c>
+      <x:c r="C229" s="47" t="str">
+        <x:v>CALL-001</x:v>
+      </x:c>
+      <x:c r="D229" s="47" t="str">
+        <x:v>Former member LEAVE is relayed</x:v>
+      </x:c>
+      <x:c r="E229" s="47" t="str">
+        <x:v>ChatMessageService.relayCallSignal</x:v>
+      </x:c>
+      <x:c r="F229" s="47" t="str">
+        <x:v>type=LEAVE; active membership absent; historical membership present</x:v>
+      </x:c>
+      <x:c r="G229" s="47" t="str">
+        <x:v>findFirstByRoomIdAndUserIdOrderByJoinedAtDesc -&gt; former member</x:v>
+      </x:c>
+      <x:c r="H229" s="47" t="str">
+        <x:v>No exception; broadcast LEAVE to /topic/rooms/{roomId}/call</x:v>
+      </x:c>
+      <x:c r="I229" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
+      <x:c r="J229" s="47" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="K229" s="47" t="str">
+        <x:v>Unit test (JUnit 5 / Mockito)</x:v>
+      </x:c>
+      <x:c r="L229" s="47" t="str">
+        <x:v>ChatMessageServiceTest.relayCallSignal_leave_afterMembershipEnded_stillBroadcasts</x:v>
+      </x:c>
+      <x:c r="M229" s="47" t="str">
+        <x:v>2026-10-08 | targeted retest Pass | DEF-004 CLOSED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="230">
+      <x:c r="A230" s="47" t="str">
+        <x:v>UC-CALL-01</x:v>
+      </x:c>
+      <x:c r="B230" s="47" t="str">
+        <x:v>TS016</x:v>
+      </x:c>
+      <x:c r="C230" s="47" t="str">
+        <x:v>CALL-002</x:v>
+      </x:c>
+      <x:c r="D230" s="47" t="str">
+        <x:v>Never-member LEAVE is forbidden</x:v>
+      </x:c>
+      <x:c r="E230" s="47" t="str">
+        <x:v>ChatMessageService.relayCallSignal</x:v>
+      </x:c>
+      <x:c r="F230" s="47" t="str">
+        <x:v>type=LEAVE; no active or historical membership</x:v>
+      </x:c>
+      <x:c r="G230" s="47" t="str">
+        <x:v>membership history lookup -&gt; empty</x:v>
+      </x:c>
+      <x:c r="H230" s="47" t="str">
+        <x:v>403 FORBIDDEN; no WebSocket broadcast</x:v>
+      </x:c>
+      <x:c r="I230" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
+      <x:c r="J230" s="47" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="K230" s="47" t="str">
+        <x:v>Unit test (JUnit 5 / Mockito)</x:v>
+      </x:c>
+      <x:c r="L230" s="47" t="str">
+        <x:v>ChatMessageServiceTest.relayCallSignal_leave_neverMember_returnsForbidden</x:v>
+      </x:c>
+      <x:c r="M230" s="47" t="str">
+        <x:v>2026-10-08 | targeted retest Pass | DEF-004 CLOSED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="231">
+      <x:c r="A231" s="47" t="str">
+        <x:v>UC-CALL-01</x:v>
+      </x:c>
+      <x:c r="B231" s="47" t="str">
+        <x:v>TS016</x:v>
+      </x:c>
+      <x:c r="C231" s="47" t="str">
+        <x:v>CALL-003</x:v>
+      </x:c>
+      <x:c r="D231" s="47" t="str">
+        <x:v>Camera toggle publishes MEDIA state</x:v>
+      </x:c>
+      <x:c r="E231" s="47" t="str">
+        <x:v>static/js/call.js</x:v>
+      </x:c>
+      <x:c r="F231" s="47" t="str">
+        <x:v>toggleCamera() with active room/STOMP connection</x:v>
+      </x:c>
+      <x:c r="G231" s="47" t="str">
+        <x:v>read JS resource contract</x:v>
+      </x:c>
+      <x:c r="H231" s="47" t="str">
+        <x:v>camera toggle publishes {type:"MEDIA", payload:{videoEnabled:...}}</x:v>
+      </x:c>
+      <x:c r="I231" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
+      <x:c r="J231" s="47" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="K231" s="47" t="str">
+        <x:v>Frontend contract test</x:v>
+      </x:c>
+      <x:c r="L231" s="47" t="str">
+        <x:v>CallFrontendContractTest.cameraToggle_publishesMediaState</x:v>
+      </x:c>
+      <x:c r="M231" s="47" t="str">
+        <x:v>2026-10-08 20:14:49 +07:00 | 2/2 Pass | DEF-005 CLOSED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="232">
+      <x:c r="A232" s="47" t="str">
+        <x:v>UC-CALL-01</x:v>
+      </x:c>
+      <x:c r="B232" s="47" t="str">
+        <x:v>TS016</x:v>
+      </x:c>
+      <x:c r="C232" s="47" t="str">
+        <x:v>CALL-004</x:v>
+      </x:c>
+      <x:c r="D232" s="47" t="str">
+        <x:v>Incoming MEDIA signal is handled</x:v>
+      </x:c>
+      <x:c r="E232" s="47" t="str">
+        <x:v>static/js/call.js + friend.js</x:v>
+      </x:c>
+      <x:c r="F232" s="47" t="str">
+        <x:v>incoming signal.type = MEDIA</x:v>
+      </x:c>
+      <x:c r="G232" s="47" t="str">
+        <x:v>read JS resource contract</x:v>
+      </x:c>
+      <x:c r="H232" s="47" t="str">
+        <x:v>client handles MEDIA and exposes state for remote video UI</x:v>
+      </x:c>
+      <x:c r="I232" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
+      <x:c r="J232" s="47" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="K232" s="47" t="str">
+        <x:v>Frontend contract test</x:v>
+      </x:c>
+      <x:c r="L232" s="47" t="str">
+        <x:v>CallFrontendContractTest.callJs_handlesIncomingMediaSignal</x:v>
+      </x:c>
+      <x:c r="M232" s="47" t="str">
+        <x:v>2026-10-08 20:14:49 +07:00 | 2/2 Pass | DEF-005 CLOSED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="233">
+      <x:c r="A233" s="47" t="str">
+        <x:v>UC-E2E-01</x:v>
+      </x:c>
+      <x:c r="B233" s="47" t="str">
+        <x:v>TS017</x:v>
+      </x:c>
+      <x:c r="C233" s="47" t="str">
+        <x:v>E2E-001</x:v>
+      </x:c>
+      <x:c r="D233" s="47" t="str">
+        <x:v>Login page loads</x:v>
+      </x:c>
+      <x:c r="E233" s="47" t="str">
+        <x:v>Browser E2E</x:v>
+      </x:c>
+      <x:c r="F233" s="47" t="str">
+        <x:v>Open /login</x:v>
+      </x:c>
+      <x:c r="G233" s="47" t="str">
+        <x:v>Application running at http://localhost:8080</x:v>
+      </x:c>
+      <x:c r="H233" s="47" t="str">
+        <x:v>Login page is displayed successfully</x:v>
+      </x:c>
+      <x:c r="I233" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
+      <x:c r="J233" s="47" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="K233" s="47" t="str">
+        <x:v>Robot Framework Browser/Playwright</x:v>
+      </x:c>
+      <x:c r="L233" s="47" t="str">
+        <x:v>login_smoke.robot — E2E-001 Login Page Loads</x:v>
+      </x:c>
+      <x:c r="M233" s="47" t="str">
+        <x:v>2026-10-08 | Final Robot regression 5/5 Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="234">
+      <x:c r="A234" s="47" t="str">
+        <x:v>UC-E2E-01</x:v>
+      </x:c>
+      <x:c r="B234" s="47" t="str">
+        <x:v>TS017</x:v>
+      </x:c>
+      <x:c r="C234" s="47" t="str">
+        <x:v>E2E-002</x:v>
+      </x:c>
+      <x:c r="D234" s="47" t="str">
+        <x:v>Password visibility can be toggled</x:v>
+      </x:c>
+      <x:c r="E234" s="47" t="str">
+        <x:v>Browser E2E</x:v>
+      </x:c>
+      <x:c r="F234" s="47" t="str">
+        <x:v>Click password show/hide control</x:v>
+      </x:c>
+      <x:c r="G234" s="47" t="str">
+        <x:v>Login page loaded</x:v>
+      </x:c>
+      <x:c r="H234" s="47" t="str">
+        <x:v>Password field visibility changes as expected</x:v>
+      </x:c>
+      <x:c r="I234" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
+      <x:c r="J234" s="47" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="K234" s="47" t="str">
+        <x:v>Robot Framework Browser/Playwright</x:v>
+      </x:c>
+      <x:c r="L234" s="47" t="str">
+        <x:v>login_smoke.robot — E2E-002 Password Can Be Shown And Hidden</x:v>
+      </x:c>
+      <x:c r="M234" s="47" t="str">
+        <x:v>2026-10-08 | Final Robot regression 5/5 Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="235">
+      <x:c r="A235" s="47" t="str">
+        <x:v>UC-E2E-01</x:v>
+      </x:c>
+      <x:c r="B235" s="47" t="str">
+        <x:v>TS017</x:v>
+      </x:c>
+      <x:c r="C235" s="47" t="str">
+        <x:v>E2E-003</x:v>
+      </x:c>
+      <x:c r="D235" s="47" t="str">
+        <x:v>Register link opens registration page</x:v>
+      </x:c>
+      <x:c r="E235" s="47" t="str">
+        <x:v>Browser E2E</x:v>
+      </x:c>
+      <x:c r="F235" s="47" t="str">
+        <x:v>Click Register link from login page</x:v>
+      </x:c>
+      <x:c r="G235" s="47" t="str">
+        <x:v>Login page loaded</x:v>
+      </x:c>
+      <x:c r="H235" s="47" t="str">
+        <x:v>Registration page opens</x:v>
+      </x:c>
+      <x:c r="I235" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
+      <x:c r="J235" s="47" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="K235" s="47" t="str">
+        <x:v>Robot Framework Browser/Playwright</x:v>
+      </x:c>
+      <x:c r="L235" s="47" t="str">
+        <x:v>login_smoke.robot — E2E-003 Register Link Opens Register Page</x:v>
+      </x:c>
+      <x:c r="M235" s="47" t="str">
+        <x:v>2026-10-08 | Final Robot regression 5/5 Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="236">
+      <x:c r="A236" s="47" t="str">
+        <x:v>UC-E2E-01</x:v>
+      </x:c>
+      <x:c r="B236" s="47" t="str">
+        <x:v>TS017</x:v>
+      </x:c>
+      <x:c r="C236" s="47" t="str">
+        <x:v>E2E-004</x:v>
+      </x:c>
+      <x:c r="D236" s="47" t="str">
+        <x:v>Register and login successfully</x:v>
+      </x:c>
+      <x:c r="E236" s="47" t="str">
+        <x:v>Browser E2E</x:v>
+      </x:c>
+      <x:c r="F236" s="47" t="str">
+        <x:v>Create account then submit login credentials</x:v>
+      </x:c>
+      <x:c r="G236" s="47" t="str">
+        <x:v>Application running; generated test account</x:v>
+      </x:c>
+      <x:c r="H236" s="47" t="str">
+        <x:v>User reaches /home after successful login</x:v>
+      </x:c>
+      <x:c r="I236" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
+      <x:c r="J236" s="47" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="K236" s="47" t="str">
+        <x:v>Robot Framework Browser/Playwright</x:v>
+      </x:c>
+      <x:c r="L236" s="47" t="str">
+        <x:v>auth_flow.robot — E2E-004 Register And Login Successfully</x:v>
+      </x:c>
+      <x:c r="M236" s="47" t="str">
+        <x:v>2026-10-08 | Final Robot regression 5/5 Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="237">
+      <x:c r="A237" s="47" t="str">
+        <x:v>UC-E2E-01</x:v>
+      </x:c>
+      <x:c r="B237" s="47" t="str">
+        <x:v>TS017</x:v>
+      </x:c>
+      <x:c r="C237" s="47" t="str">
+        <x:v>E2E-005</x:v>
+      </x:c>
+      <x:c r="D237" s="47" t="str">
+        <x:v>Selected interest persists after registration</x:v>
+      </x:c>
+      <x:c r="E237" s="47" t="str">
+        <x:v>Browser E2E</x:v>
+      </x:c>
+      <x:c r="F237" s="47" t="str">
+        <x:v>Select interest during registration and verify after login</x:v>
+      </x:c>
+      <x:c r="G237" s="47" t="str">
+        <x:v>Application running; generated test account</x:v>
+      </x:c>
+      <x:c r="H237" s="47" t="str">
+        <x:v>Selected interest is saved and returned for new user</x:v>
+      </x:c>
+      <x:c r="I237" s="47" t="str">
+        <x:v>Matched expected result.</x:v>
+      </x:c>
+      <x:c r="J237" s="47" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="K237" s="47" t="str">
+        <x:v>Robot Framework Browser/Playwright</x:v>
+      </x:c>
+      <x:c r="L237" s="47" t="str">
+        <x:v>register_interest.robot — E2E-005 Selected Interest Is Saved After Registration</x:v>
+      </x:c>
+      <x:c r="M237" s="47" t="str">
+        <x:v>2026-10-08 | Final Robot regression 5/5 Pass | DEF-003 CLOSED</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>